<commit_message>
Dados atualizados via Robô: 18/05/2026 17:41
</commit_message>
<xml_diff>
--- a/dados_atuais.xlsx
+++ b/dados_atuais.xlsx
@@ -581,7 +581,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>408,551</t>
+          <t>406,838</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -603,7 +603,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF FÁCIL RF SIMPLES RESP LTDA</t>
+          <t>CAIXA FIC FIF FÁCIL RF SIMPLES RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -638,7 +638,7 @@
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>6.726,533</t>
+          <t>6.646,913</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
@@ -660,7 +660,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF MOVIMENTAÇÕES AUTOMÁTICAS RF SIMPLES RESP LTDA</t>
+          <t>CAIXA FIC FIF MOVIMENTAÇÕES AUTOMÁTICAS RF SIMPLES RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -695,7 +695,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>810,624</t>
+          <t>810,007</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -805,7 +805,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>120,092</t>
+          <t>120,091</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -862,7 +862,7 @@
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>96,153</t>
+          <t>96,136</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -915,7 +915,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>584,603</t>
+          <t>584,596</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -972,7 +972,7 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>61,658</t>
+          <t>61,657</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -1029,7 +1029,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>1.672,750</t>
+          <t>1.672,699</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>28,420</t>
+          <t>28,419</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1310,7 +1310,7 @@
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>79,712</t>
+          <t>79,693</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>140,753</t>
+          <t>140,752</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -1538,7 +1538,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1.756,434</t>
+          <t>1.740,789</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1595,7 +1595,7 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>2.192,986</t>
+          <t>2.192,972</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -1766,7 +1766,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>957,119</t>
+          <t>957,109</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1788,7 +1788,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>CAIXA EXPERT ARX IPCA DEB INCENTIVADAS FIC FIF RF CRED PRIV - RESP LTDA (1) (2)</t>
+          <t>CAIXA EXPERT ARX IPCA DEB INCENTIVADAS FIC FIF RF CRED PRIV - RESP LTDA (2)</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -1798,32 +1798,32 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,10997325</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>-0,001</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>0,00</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>2,89</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>219,622</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
@@ -1841,7 +1841,7 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIF FIC EXPERT SULAMERICA RF CRED PRIV LP - RESP LTDA (1)</t>
+          <t>CAIXA FIF FIC EXPERT SULAMERICA RF CRED PRIV LP - RESP LTDA</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
@@ -1851,32 +1851,32 @@
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F25" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H25" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,22811400</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>-0,001</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>0,62</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>4,85</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>14,63</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>70,980</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -1929,7 +1929,7 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>175,319</t>
+          <t>175,223</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
@@ -2004,7 +2004,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>CAIXA EXPERT VOX DESENV SUSTENTAVEL IS RF CRED PRIV LP - RESP LTDA (1) (2)</t>
+          <t>CAIXA EXPERT VOX DESENV SUSTENTAVEL IS RF CRED PRIV LP - RESP LTDA (2)</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -2014,32 +2014,32 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,02936900</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>-0,001</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>0,52</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>4,97</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>21,758</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
@@ -2057,7 +2057,7 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>CAIXA EXPERT ABSOLUTE CRETA FIC FIF RF CRED PRIV LP - RESP LTDA (1)</t>
+          <t>CAIXA EXPERT ABSOLUTE CRETA FIC FIF RF CRED PRIV LP - RESP LTDA</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
@@ -2067,32 +2067,32 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H29" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,15576700</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>-0,001</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>0,66</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>4,08</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>13,73</t>
         </is>
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>66,353</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -2110,7 +2110,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>CAIXA EXPERT RB ASSET CDI DEB INCENTIVADAS FIC FIF RF CRED PRIV RESP LTDA (1) (2)</t>
+          <t>CAIXA EXPERT RB ASSET CDI DEB INCENTIVADAS FIC FIF RF CRED PRIV RESP LTDA (2)</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -2120,32 +2120,32 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,05776364</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>-0,001</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>0,31</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>2,36</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>332,405</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
@@ -2163,7 +2163,7 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>CAIXA EXPERT VINLAND DEB IN INFRA RF CRED PRIV LP RESP LTDA (1) (2) (3)</t>
+          <t>CAIXA EXPERT VINLAND DEB IN INFRA RF CRED PRIV LP RESP LTDA (2) (3)</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
@@ -2251,7 +2251,7 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>859,898</t>
+          <t>859,833</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
@@ -2304,7 +2304,7 @@
       </c>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>3.241,411</t>
+          <t>3.241,339</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -2418,7 +2418,7 @@
       </c>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>3.113,953</t>
+          <t>3.113,942</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -2475,7 +2475,7 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>125,145</t>
+          <t>125,015</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
@@ -2528,7 +2528,7 @@
       </c>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>550,004</t>
+          <t>549,999</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -2638,7 +2638,7 @@
       </c>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>334,888</t>
+          <t>334,883</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
@@ -2691,7 +2691,7 @@
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>2.373,675</t>
+          <t>2.373,657</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
@@ -2748,7 +2748,7 @@
       </c>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>553,400</t>
+          <t>553,399</t>
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr">
@@ -2805,7 +2805,7 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>15.485,298</t>
+          <t>15.485,082</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -2862,7 +2862,7 @@
       </c>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>1.383,497</t>
+          <t>1.383,496</t>
         </is>
       </c>
       <c r="J43" s="4" t="inlineStr">
@@ -2919,7 +2919,7 @@
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>165,472</t>
+          <t>165,470</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
@@ -3029,7 +3029,7 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>6.013,909</t>
+          <t>5.952,431</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
@@ -3086,7 +3086,7 @@
       </c>
       <c r="I47" s="4" t="inlineStr">
         <is>
-          <t>2.188,952</t>
+          <t>2.188,909</t>
         </is>
       </c>
       <c r="J47" s="4" t="inlineStr">
@@ -3200,7 +3200,7 @@
       </c>
       <c r="I49" s="4" t="inlineStr">
         <is>
-          <t>839,422</t>
+          <t>839,413</t>
         </is>
       </c>
       <c r="J49" s="4" t="inlineStr">
@@ -3257,7 +3257,7 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>15.546,151</t>
+          <t>15.545,914</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
@@ -3314,7 +3314,7 @@
       </c>
       <c r="I51" s="4" t="inlineStr">
         <is>
-          <t>9.466,109</t>
+          <t>9.466,015</t>
         </is>
       </c>
       <c r="J51" s="4" t="inlineStr">
@@ -3371,7 +3371,7 @@
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>20.846,276</t>
+          <t>20.845,858</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr">
@@ -3428,7 +3428,7 @@
       </c>
       <c r="I53" s="4" t="inlineStr">
         <is>
-          <t>13.169,981</t>
+          <t>13.169,776</t>
         </is>
       </c>
       <c r="J53" s="4" t="inlineStr">
@@ -3450,7 +3450,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF RENDA FIXA CURTO PRAZO RESP LTDA</t>
+          <t>CAIXA FIC FIF RENDA FIXA CURTO PRAZO RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -3485,7 +3485,7 @@
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>245,548</t>
+          <t>245,520</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr">
@@ -3503,7 +3503,7 @@
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF FOF SMART CRED PRIV MM LP RESP LTDA (1)</t>
+          <t>CAIXA FIC FIF FOF SMART CRED PRIV MM LP RESP LTDA</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
@@ -3513,32 +3513,32 @@
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E55" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F55" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G55" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H55" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,39931700</t>
+        </is>
+      </c>
+      <c r="E55" s="6" t="inlineStr">
+        <is>
+          <t>-0,007</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="inlineStr">
+        <is>
+          <t>0,60</t>
+        </is>
+      </c>
+      <c r="G55" s="5" t="inlineStr">
+        <is>
+          <t>4,51</t>
+        </is>
+      </c>
+      <c r="H55" s="5" t="inlineStr">
+        <is>
+          <t>14,12</t>
         </is>
       </c>
       <c r="I55" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>68,862</t>
         </is>
       </c>
       <c r="J55" s="4" t="inlineStr">
@@ -3560,7 +3560,7 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC MULTIGESTOR GLOBAL EQUITIES IE (1)</t>
+          <t>CAIXA FIC MULTIGESTOR GLOBAL EQUITIES IE</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -3570,32 +3570,32 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E56" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F56" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G56" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H56" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1.167,25373800</t>
+        </is>
+      </c>
+      <c r="E56" s="7" t="inlineStr">
+        <is>
+          <t>-0,003</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>1,55</t>
+        </is>
+      </c>
+      <c r="G56" s="7" t="inlineStr">
+        <is>
+          <t>-6,97</t>
+        </is>
+      </c>
+      <c r="H56" s="7" t="inlineStr">
+        <is>
+          <t>-2,47</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>35,739</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
@@ -3652,7 +3652,7 @@
       </c>
       <c r="I57" s="4" t="inlineStr">
         <is>
-          <t>328,493</t>
+          <t>540,035</t>
         </is>
       </c>
       <c r="J57" s="4" t="inlineStr">
@@ -3674,7 +3674,7 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF ESTRATÉGIA LIVRE MULTIMERCADO LP RESP LTDA (1)</t>
+          <t>CAIXA FIC FIF ESTRATÉGIA LIVRE MULTIMERCADO LP RESP LTDA</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -3684,32 +3684,32 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E58" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F58" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G58" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H58" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1.632,15053600</t>
+        </is>
+      </c>
+      <c r="E58" s="7" t="inlineStr">
+        <is>
+          <t>-0,006</t>
+        </is>
+      </c>
+      <c r="F58" s="7" t="inlineStr">
+        <is>
+          <t>-0,22</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="inlineStr">
+        <is>
+          <t>4,16</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr">
+        <is>
+          <t>13,39</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>116,889</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
@@ -3766,7 +3766,7 @@
       </c>
       <c r="I59" s="4" t="inlineStr">
         <is>
-          <t>13,423</t>
+          <t>13,348</t>
         </is>
       </c>
       <c r="J59" s="4" t="inlineStr">
@@ -3784,7 +3784,7 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>CAIXA CARTEIRA QUANT DUO FIC FIF MM LP RESP LTDA (1) (2) (3)</t>
+          <t>CAIXA CARTEIRA QUANT DUO FIC FIF MM LP RESP LTDA (2) (3)</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -3837,7 +3837,7 @@
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF FOF SMART LONG SHORT LP RESP LTDA (1)</t>
+          <t>CAIXA FIC FIF FOF SMART LONG SHORT LP RESP LTDA</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
@@ -3847,32 +3847,32 @@
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E61" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F61" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G61" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H61" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,25018500</t>
+        </is>
+      </c>
+      <c r="E61" s="6" t="inlineStr">
+        <is>
+          <t>-0,005</t>
+        </is>
+      </c>
+      <c r="F61" s="6" t="inlineStr">
+        <is>
+          <t>-0,44</t>
+        </is>
+      </c>
+      <c r="G61" s="5" t="inlineStr">
+        <is>
+          <t>2,36</t>
+        </is>
+      </c>
+      <c r="H61" s="5" t="inlineStr">
+        <is>
+          <t>11,60</t>
         </is>
       </c>
       <c r="I61" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>6,666</t>
         </is>
       </c>
       <c r="J61" s="4" t="inlineStr">
@@ -3943,7 +3943,7 @@
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>CAIXA CARTEIRA QUANT QUALI FIC FIF MM LP RESP LTDA (1) (2) (3)</t>
+          <t>CAIXA CARTEIRA QUANT QUALI FIC FIF MM LP RESP LTDA (2) (3)</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
@@ -3996,7 +3996,7 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF FOF SMART LONG BIAS MM RESP LTDA (1)</t>
+          <t>CAIXA FIC FIF FOF SMART LONG BIAS MM RESP LTDA</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -4006,32 +4006,32 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E64" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F64" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G64" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H64" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,44320300</t>
+        </is>
+      </c>
+      <c r="E64" s="7" t="inlineStr">
+        <is>
+          <t>-0,004</t>
+        </is>
+      </c>
+      <c r="F64" s="7" t="inlineStr">
+        <is>
+          <t>-1,73</t>
+        </is>
+      </c>
+      <c r="G64" s="3" t="inlineStr">
+        <is>
+          <t>5,72</t>
+        </is>
+      </c>
+      <c r="H64" s="3" t="inlineStr">
+        <is>
+          <t>21,08</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11,970</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
@@ -4049,7 +4049,7 @@
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>CAIXA CARTEIRA QUANT UNO FIC FIF MM LP RESP LTDA (1) (2) (3)</t>
+          <t>CAIXA CARTEIRA QUANT UNO FIC FIF MM LP RESP LTDA (2) (3)</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
@@ -4159,7 +4159,7 @@
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF ESTRATÉGICO MULTIMERCADO LP RESP LTDA (1)</t>
+          <t>CAIXA FIC FIF ESTRATÉGICO MULTIMERCADO LP RESP LTDA</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
@@ -4169,32 +4169,32 @@
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E67" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F67" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G67" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H67" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>5,32047778</t>
+        </is>
+      </c>
+      <c r="E67" s="6" t="inlineStr">
+        <is>
+          <t>-0,003</t>
+        </is>
+      </c>
+      <c r="F67" s="6" t="inlineStr">
+        <is>
+          <t>-0,21</t>
+        </is>
+      </c>
+      <c r="G67" s="5" t="inlineStr">
+        <is>
+          <t>3,69</t>
+        </is>
+      </c>
+      <c r="H67" s="5" t="inlineStr">
+        <is>
+          <t>13,12</t>
         </is>
       </c>
       <c r="I67" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>33,192</t>
         </is>
       </c>
       <c r="J67" s="4" t="inlineStr">
@@ -4251,7 +4251,7 @@
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>668,164</t>
+          <t>666,467</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr">
@@ -4273,7 +4273,7 @@
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF FOF SMART MULTIESTRATEGIA MM RESP LTDA (1)</t>
+          <t>CAIXA FIC FIF FOF SMART MULTIESTRATEGIA MM RESP LTDA</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
@@ -4283,32 +4283,32 @@
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E69" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F69" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G69" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H69" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>2,85531700</t>
+        </is>
+      </c>
+      <c r="E69" s="6" t="inlineStr">
+        <is>
+          <t>-0,004</t>
+        </is>
+      </c>
+      <c r="F69" s="5" t="inlineStr">
+        <is>
+          <t>0,08</t>
+        </is>
+      </c>
+      <c r="G69" s="5" t="inlineStr">
+        <is>
+          <t>2,22</t>
+        </is>
+      </c>
+      <c r="H69" s="5" t="inlineStr">
+        <is>
+          <t>11,44</t>
         </is>
       </c>
       <c r="I69" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>77,229</t>
         </is>
       </c>
       <c r="J69" s="4" t="inlineStr">
@@ -4422,7 +4422,7 @@
       </c>
       <c r="I71" s="4" t="inlineStr">
         <is>
-          <t>2.330,280</t>
+          <t>2.329,776</t>
         </is>
       </c>
       <c r="J71" s="4" t="inlineStr">
@@ -4501,7 +4501,7 @@
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF FUNCIONARIOS ESTRATEGIA LIVRE MULTIMERCADO LP RESP LTDA (1)</t>
+          <t>CAIXA FIC FIF FUNCIONARIOS ESTRATEGIA LIVRE MULTIMERCADO LP RESP LTDA</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
@@ -4511,32 +4511,32 @@
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E73" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F73" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G73" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H73" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1.652,59401600</t>
+        </is>
+      </c>
+      <c r="E73" s="6" t="inlineStr">
+        <is>
+          <t>-0,003</t>
+        </is>
+      </c>
+      <c r="F73" s="6" t="inlineStr">
+        <is>
+          <t>-0,18</t>
+        </is>
+      </c>
+      <c r="G73" s="5" t="inlineStr">
+        <is>
+          <t>4,49</t>
+        </is>
+      </c>
+      <c r="H73" s="5" t="inlineStr">
+        <is>
+          <t>14,36</t>
         </is>
       </c>
       <c r="I73" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>15,317</t>
         </is>
       </c>
       <c r="J73" s="4" t="inlineStr">
@@ -4554,7 +4554,7 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>CAIXA HASHDEX NASDAQ CRYPTO INDEX FIC FIF MM RESP LTDA (1) (2)</t>
+          <t>CAIXA HASHDEX NASDAQ CRYPTO INDEX FIC FIF MM RESP LTDA (2)</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
@@ -4564,32 +4564,32 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E74" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F74" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G74" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>0,57593472</t>
+        </is>
+      </c>
+      <c r="E74" s="7" t="inlineStr">
+        <is>
+          <t>-0,007</t>
+        </is>
+      </c>
+      <c r="F74" s="3" t="inlineStr">
+        <is>
+          <t>6,16</t>
+        </is>
+      </c>
+      <c r="G74" s="7" t="inlineStr">
+        <is>
+          <t>-20,24</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4,200</t>
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr">
@@ -4607,7 +4607,7 @@
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF CAPITAL PROTEGIDO CESTA AGRO MM (1)</t>
+          <t>CAIXA FIC FIF CAPITAL PROTEGIDO CESTA AGRO MM</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
@@ -4617,32 +4617,32 @@
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E75" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F75" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G75" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H75" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,37874300</t>
+        </is>
+      </c>
+      <c r="E75" s="6" t="inlineStr">
+        <is>
+          <t>-0,003</t>
+        </is>
+      </c>
+      <c r="F75" s="6" t="inlineStr">
+        <is>
+          <t>-1,35</t>
+        </is>
+      </c>
+      <c r="G75" s="5" t="inlineStr">
+        <is>
+          <t>1,66</t>
+        </is>
+      </c>
+      <c r="H75" s="5" t="inlineStr">
+        <is>
+          <t>8,35</t>
         </is>
       </c>
       <c r="I75" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>70,771</t>
         </is>
       </c>
       <c r="J75" s="4" t="inlineStr">
@@ -4660,7 +4660,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>CAIXA CAPITAL PROTEGIDO CÍCLICO III FIC FIF MM LP - RESP LTDA (1)</t>
+          <t>CAIXA CAPITAL PROTEGIDO CÍCLICO III FIC FIF MM LP - RESP LTDA</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -4670,32 +4670,32 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E76" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,53337400</t>
+        </is>
+      </c>
+      <c r="E76" s="7" t="inlineStr">
+        <is>
+          <t>-0,004</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G76" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H76" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>0,00</t>
+        </is>
+      </c>
+      <c r="G76" s="3" t="inlineStr">
+        <is>
+          <t>2,69</t>
+        </is>
+      </c>
+      <c r="H76" s="3" t="inlineStr">
+        <is>
+          <t>18,93</t>
         </is>
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14,513</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr">
@@ -4717,7 +4717,7 @@
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>CAIXA CAPITAL PROTEGIDO IBOVESPA CÍCLICO I FIC FIF MM (1)</t>
+          <t>CAIXA CAPITAL PROTEGIDO IBOVESPA CÍCLICO I FIC FIF MM</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
@@ -4727,32 +4727,32 @@
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E77" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F77" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G77" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H77" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>3,25598300</t>
+        </is>
+      </c>
+      <c r="E77" s="6" t="inlineStr">
+        <is>
+          <t>-0,005</t>
+        </is>
+      </c>
+      <c r="F77" s="5" t="inlineStr">
+        <is>
+          <t>1,19</t>
+        </is>
+      </c>
+      <c r="G77" s="5" t="inlineStr">
+        <is>
+          <t>2,19</t>
+        </is>
+      </c>
+      <c r="H77" s="5" t="inlineStr">
+        <is>
+          <t>7,05</t>
         </is>
       </c>
       <c r="I77" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>155,146</t>
         </is>
       </c>
       <c r="J77" s="4" t="inlineStr">
@@ -4774,7 +4774,7 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIM CAPITAL PROTEGIDO CICLICO II LP - RL (1)</t>
+          <t>CAIXA FIC FIM CAPITAL PROTEGIDO CICLICO II LP - RL</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
@@ -4784,32 +4784,32 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E78" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F78" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G78" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H78" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,47220000</t>
+        </is>
+      </c>
+      <c r="E78" s="7" t="inlineStr">
+        <is>
+          <t>-0,003</t>
+        </is>
+      </c>
+      <c r="F78" s="3" t="inlineStr">
+        <is>
+          <t>1,51</t>
+        </is>
+      </c>
+      <c r="G78" s="3" t="inlineStr">
+        <is>
+          <t>1,80</t>
+        </is>
+      </c>
+      <c r="H78" s="3" t="inlineStr">
+        <is>
+          <t>14,37</t>
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>190,975</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr">
@@ -4827,7 +4827,7 @@
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF EXPERT PIMCO INCOME IE MM LP RESP LTDA (1)</t>
+          <t>CAIXA FIC FIF EXPERT PIMCO INCOME IE MM LP RESP LTDA</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
@@ -4837,32 +4837,32 @@
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E79" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F79" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G79" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H79" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,41230600</t>
+        </is>
+      </c>
+      <c r="E79" s="6" t="inlineStr">
+        <is>
+          <t>-0,003</t>
+        </is>
+      </c>
+      <c r="F79" s="5" t="inlineStr">
+        <is>
+          <t>0,27</t>
+        </is>
+      </c>
+      <c r="G79" s="5" t="inlineStr">
+        <is>
+          <t>2,51</t>
+        </is>
+      </c>
+      <c r="H79" s="5" t="inlineStr">
+        <is>
+          <t>16,08</t>
         </is>
       </c>
       <c r="I79" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>279,219</t>
         </is>
       </c>
       <c r="J79" s="4" t="inlineStr">
@@ -4884,7 +4884,7 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>CAIXA EXPERT GIANT ZARATHUSTRA FIC MULTIMERCADO - RESP LTDA (1)</t>
+          <t>CAIXA EXPERT GIANT ZARATHUSTRA FIC MULTIMERCADO - RESP LTDA</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
@@ -4894,32 +4894,32 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E80" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F80" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G80" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H80" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,31674000</t>
+        </is>
+      </c>
+      <c r="E80" s="7" t="inlineStr">
+        <is>
+          <t>-0,001</t>
+        </is>
+      </c>
+      <c r="F80" s="3" t="inlineStr">
+        <is>
+          <t>0,57</t>
+        </is>
+      </c>
+      <c r="G80" s="3" t="inlineStr">
+        <is>
+          <t>2,59</t>
+        </is>
+      </c>
+      <c r="H80" s="3" t="inlineStr">
+        <is>
+          <t>2,78</t>
         </is>
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13,395</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr">
@@ -4976,7 +4976,7 @@
       </c>
       <c r="I81" s="4" t="inlineStr">
         <is>
-          <t>898,185</t>
+          <t>898,178</t>
         </is>
       </c>
       <c r="J81" s="4" t="inlineStr">
@@ -5033,7 +5033,7 @@
       </c>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t>748,991</t>
+          <t>748,992</t>
         </is>
       </c>
       <c r="J82" s="2" t="inlineStr">
@@ -5055,7 +5055,7 @@
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>FIC FIF CAIXA EXPERT BTG PACTUAL X10 MM LP RESP LTDA (1)</t>
+          <t>FIC FIF CAIXA EXPERT BTG PACTUAL X10 MM LP RESP LTDA</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
@@ -5065,32 +5065,32 @@
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E83" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F83" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G83" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H83" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>6,78432500</t>
+        </is>
+      </c>
+      <c r="E83" s="6" t="inlineStr">
+        <is>
+          <t>-0,004</t>
+        </is>
+      </c>
+      <c r="F83" s="5" t="inlineStr">
+        <is>
+          <t>0,09</t>
+        </is>
+      </c>
+      <c r="G83" s="5" t="inlineStr">
+        <is>
+          <t>5,48</t>
+        </is>
+      </c>
+      <c r="H83" s="5" t="inlineStr">
+        <is>
+          <t>16,73</t>
         </is>
       </c>
       <c r="I83" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>129,587</t>
         </is>
       </c>
       <c r="J83" s="4" t="inlineStr">
@@ -5112,7 +5112,7 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF EXPERT SPX NIMITZ MULTIMERCADO RESP LTDA (1)</t>
+          <t>CAIXA FIC FIF EXPERT SPX NIMITZ MULTIMERCADO RESP LTDA</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
@@ -5122,32 +5122,32 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E84" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F84" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G84" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H84" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,77206600</t>
+        </is>
+      </c>
+      <c r="E84" s="7" t="inlineStr">
+        <is>
+          <t>-0,002</t>
+        </is>
+      </c>
+      <c r="F84" s="3" t="inlineStr">
+        <is>
+          <t>0,72</t>
+        </is>
+      </c>
+      <c r="G84" s="3" t="inlineStr">
+        <is>
+          <t>0,31</t>
+        </is>
+      </c>
+      <c r="H84" s="3" t="inlineStr">
+        <is>
+          <t>10,69</t>
         </is>
       </c>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>176,392</t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr">
@@ -5200,7 +5200,7 @@
       </c>
       <c r="I85" s="4" t="inlineStr">
         <is>
-          <t>97,614</t>
+          <t>97,597</t>
         </is>
       </c>
       <c r="J85" s="4" t="inlineStr">
@@ -5257,7 +5257,7 @@
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>347,120</t>
+          <t>347,118</t>
         </is>
       </c>
       <c r="J86" s="2" t="inlineStr">
@@ -5367,7 +5367,7 @@
       </c>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>10,318</t>
+          <t>10,316</t>
         </is>
       </c>
       <c r="J88" s="2" t="inlineStr">
@@ -5420,7 +5420,7 @@
       </c>
       <c r="I89" s="4" t="inlineStr">
         <is>
-          <t>277,722</t>
+          <t>277,543</t>
         </is>
       </c>
       <c r="J89" s="4" t="inlineStr">
@@ -5477,7 +5477,7 @@
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>445,938</t>
+          <t>445,937</t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr">
@@ -5534,7 +5534,7 @@
       </c>
       <c r="I91" s="4" t="inlineStr">
         <is>
-          <t>58,253</t>
+          <t>58,191</t>
         </is>
       </c>
       <c r="J91" s="4" t="inlineStr">
@@ -5705,7 +5705,7 @@
       </c>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t>92,434</t>
+          <t>92,431</t>
         </is>
       </c>
       <c r="J94" s="2" t="inlineStr">
@@ -5727,7 +5727,7 @@
       </c>
       <c r="B95" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF AÇÕES MULTIGESTOR RESP LTDA (1)</t>
+          <t>CAIXA FIC FIF AÇÕES MULTIGESTOR RESP LTDA</t>
         </is>
       </c>
       <c r="C95" s="4" t="inlineStr">
@@ -5737,32 +5737,32 @@
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E95" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F95" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G95" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H95" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,30185000</t>
+        </is>
+      </c>
+      <c r="E95" s="6" t="inlineStr">
+        <is>
+          <t>-0,024</t>
+        </is>
+      </c>
+      <c r="F95" s="6" t="inlineStr">
+        <is>
+          <t>-4,66</t>
+        </is>
+      </c>
+      <c r="G95" s="5" t="inlineStr">
+        <is>
+          <t>1,14</t>
+        </is>
+      </c>
+      <c r="H95" s="5" t="inlineStr">
+        <is>
+          <t>10,89</t>
         </is>
       </c>
       <c r="I95" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>295,634</t>
         </is>
       </c>
       <c r="J95" s="4" t="inlineStr">
@@ -5819,7 +5819,7 @@
       </c>
       <c r="I96" s="2" t="inlineStr">
         <is>
-          <t>114,110</t>
+          <t>114,109</t>
         </is>
       </c>
       <c r="J96" s="2" t="inlineStr">
@@ -5876,7 +5876,7 @@
       </c>
       <c r="I97" s="4" t="inlineStr">
         <is>
-          <t>133,544</t>
+          <t>133,454</t>
         </is>
       </c>
       <c r="J97" s="4" t="inlineStr">
@@ -5933,7 +5933,7 @@
       </c>
       <c r="I98" s="2" t="inlineStr">
         <is>
-          <t>47,674</t>
+          <t>47,639</t>
         </is>
       </c>
       <c r="J98" s="2" t="inlineStr">
@@ -5986,7 +5986,7 @@
       </c>
       <c r="I99" s="4" t="inlineStr">
         <is>
-          <t>129,900</t>
+          <t>129,793</t>
         </is>
       </c>
       <c r="J99" s="4" t="inlineStr">
@@ -6043,7 +6043,7 @@
       </c>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t>41,489</t>
+          <t>41,414</t>
         </is>
       </c>
       <c r="J100" s="2" t="inlineStr">
@@ -6096,7 +6096,7 @@
       </c>
       <c r="I101" s="4" t="inlineStr">
         <is>
-          <t>677,490</t>
+          <t>677,323</t>
         </is>
       </c>
       <c r="J101" s="4" t="inlineStr">
@@ -6153,7 +6153,7 @@
       </c>
       <c r="I102" s="2" t="inlineStr">
         <is>
-          <t>440,323</t>
+          <t>440,272</t>
         </is>
       </c>
       <c r="J102" s="2" t="inlineStr">
@@ -6263,7 +6263,7 @@
       </c>
       <c r="I104" s="2" t="inlineStr">
         <is>
-          <t>30,199</t>
+          <t>30,188</t>
         </is>
       </c>
       <c r="J104" s="2" t="inlineStr">
@@ -6320,7 +6320,7 @@
       </c>
       <c r="I105" s="4" t="inlineStr">
         <is>
-          <t>1,793</t>
+          <t>1,792</t>
         </is>
       </c>
       <c r="J105" s="4" t="inlineStr">
@@ -6373,7 +6373,7 @@
       </c>
       <c r="I106" s="2" t="inlineStr">
         <is>
-          <t>44,434</t>
+          <t>44,404</t>
         </is>
       </c>
       <c r="J106" s="2" t="inlineStr">
@@ -6430,7 +6430,7 @@
       </c>
       <c r="I107" s="4" t="inlineStr">
         <is>
-          <t>36,469</t>
+          <t>36,461</t>
         </is>
       </c>
       <c r="J107" s="4" t="inlineStr">
@@ -6487,7 +6487,7 @@
       </c>
       <c r="I108" s="2" t="inlineStr">
         <is>
-          <t>910,760</t>
+          <t>910,317</t>
         </is>
       </c>
       <c r="J108" s="2" t="inlineStr">
@@ -6544,7 +6544,7 @@
       </c>
       <c r="I109" s="4" t="inlineStr">
         <is>
-          <t>2,994</t>
+          <t>2,993</t>
         </is>
       </c>
       <c r="J109" s="4" t="inlineStr">
@@ -6650,7 +6650,7 @@
       </c>
       <c r="I111" s="4" t="inlineStr">
         <is>
-          <t>19,765</t>
+          <t>19,390</t>
         </is>
       </c>
       <c r="J111" s="4" t="inlineStr">
@@ -6703,7 +6703,7 @@
       </c>
       <c r="I112" s="2" t="inlineStr">
         <is>
-          <t>269,776</t>
+          <t>269,513</t>
         </is>
       </c>
       <c r="J112" s="2" t="inlineStr">
@@ -6721,7 +6721,7 @@
       </c>
       <c r="B113" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC ACOES EXPERT VERDE AM LONG BIAS - RESP LTDA (1)</t>
+          <t>CAIXA FIC ACOES EXPERT VERDE AM LONG BIAS - RESP LTDA</t>
         </is>
       </c>
       <c r="C113" s="4" t="inlineStr">
@@ -6731,32 +6731,32 @@
       </c>
       <c r="D113" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E113" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F113" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G113" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H113" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1.017,29224100</t>
+        </is>
+      </c>
+      <c r="E113" s="6" t="inlineStr">
+        <is>
+          <t>-0,003</t>
+        </is>
+      </c>
+      <c r="F113" s="6" t="inlineStr">
+        <is>
+          <t>-4,92</t>
+        </is>
+      </c>
+      <c r="G113" s="5" t="inlineStr">
+        <is>
+          <t>3,76</t>
+        </is>
+      </c>
+      <c r="H113" s="5" t="inlineStr">
+        <is>
+          <t>19,30</t>
         </is>
       </c>
       <c r="I113" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>8,171</t>
         </is>
       </c>
       <c r="J113" s="4" t="inlineStr">
@@ -6778,7 +6778,7 @@
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>CAIXA EXPERT CLARITAS VALOR FIC FIF AÇÕES - RESP LTDA (1)</t>
+          <t>CAIXA EXPERT CLARITAS VALOR FIC FIF AÇÕES - RESP LTDA</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
@@ -6788,32 +6788,32 @@
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E114" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F114" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G114" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H114" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1.538,75924600</t>
+        </is>
+      </c>
+      <c r="E114" s="7" t="inlineStr">
+        <is>
+          <t>-0,002</t>
+        </is>
+      </c>
+      <c r="F114" s="7" t="inlineStr">
+        <is>
+          <t>-4,34</t>
+        </is>
+      </c>
+      <c r="G114" s="3" t="inlineStr">
+        <is>
+          <t>2,87</t>
+        </is>
+      </c>
+      <c r="H114" s="3" t="inlineStr">
+        <is>
+          <t>15,06</t>
         </is>
       </c>
       <c r="I114" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>22,409</t>
         </is>
       </c>
       <c r="J114" s="2" t="inlineStr">
@@ -6845,7 +6845,7 @@
       </c>
       <c r="D115" s="4" t="inlineStr">
         <is>
-          <t>172,97549800</t>
+          <t>172,97549798</t>
         </is>
       </c>
       <c r="E115" s="6" t="inlineStr">
@@ -6980,7 +6980,7 @@
       </c>
       <c r="I117" s="4" t="inlineStr">
         <is>
-          <t>1.692,073</t>
+          <t>1.691,330</t>
         </is>
       </c>
       <c r="J117" s="4" t="inlineStr">
@@ -7033,7 +7033,7 @@
       </c>
       <c r="I118" s="2" t="inlineStr">
         <is>
-          <t>730,865</t>
+          <t>730,347</t>
         </is>
       </c>
       <c r="J118" s="2" t="inlineStr">
@@ -7086,7 +7086,7 @@
       </c>
       <c r="I119" s="4" t="inlineStr">
         <is>
-          <t>797,168</t>
+          <t>796,676</t>
         </is>
       </c>
       <c r="J119" s="4" t="inlineStr">
@@ -7245,7 +7245,7 @@
       </c>
       <c r="I122" s="2" t="inlineStr">
         <is>
-          <t>633,334</t>
+          <t>632,633</t>
         </is>
       </c>
       <c r="J122" s="2" t="inlineStr">
@@ -7298,7 +7298,7 @@
       </c>
       <c r="I123" s="4" t="inlineStr">
         <is>
-          <t>477,359</t>
+          <t>476,930</t>
         </is>
       </c>
       <c r="J123" s="4" t="inlineStr">
@@ -7351,7 +7351,7 @@
       </c>
       <c r="I124" s="2" t="inlineStr">
         <is>
-          <t>728,420</t>
+          <t>727,765</t>
         </is>
       </c>
       <c r="J124" s="2" t="inlineStr">
@@ -7369,7 +7369,7 @@
       </c>
       <c r="B125" s="4" t="inlineStr">
         <is>
-          <t>CAIXA AZULZINHA FIC FIF RF SIMPLES - RESP LTDA (2)</t>
+          <t>CAIXA AZULZINHA FIC FIF RF SIMPLES - RESP LTDA (2) (8)</t>
         </is>
       </c>
       <c r="C125" s="4" t="inlineStr">
@@ -7422,7 +7422,7 @@
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF AMETISTA CORP RF SIMPLES RESP LTDA</t>
+          <t>CAIXA FIC FIF AMETISTA CORP RF SIMPLES RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C126" s="2" t="inlineStr">
@@ -7457,7 +7457,7 @@
       </c>
       <c r="I126" s="2" t="inlineStr">
         <is>
-          <t>278,896</t>
+          <t>210,583</t>
         </is>
       </c>
       <c r="J126" s="2" t="inlineStr">
@@ -7514,7 +7514,7 @@
       </c>
       <c r="I127" s="4" t="inlineStr">
         <is>
-          <t>41,349</t>
+          <t>41,348</t>
         </is>
       </c>
       <c r="J127" s="4" t="inlineStr">
@@ -7742,7 +7742,7 @@
       </c>
       <c r="I131" s="4" t="inlineStr">
         <is>
-          <t>7.911,086</t>
+          <t>7.746,819</t>
         </is>
       </c>
       <c r="J131" s="4" t="inlineStr">
@@ -7799,7 +7799,7 @@
       </c>
       <c r="I132" s="2" t="inlineStr">
         <is>
-          <t>15.188,951</t>
+          <t>15.188,427</t>
         </is>
       </c>
       <c r="J132" s="2" t="inlineStr">
@@ -7856,7 +7856,7 @@
       </c>
       <c r="I133" s="4" t="inlineStr">
         <is>
-          <t>3.102,003</t>
+          <t>3.101,995</t>
         </is>
       </c>
       <c r="J133" s="4" t="inlineStr">
@@ -7874,7 +7874,7 @@
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC INST SOBERANO PLUS RF</t>
+          <t>CAIXA FIC INST SOBERANO PLUS RF (8)</t>
         </is>
       </c>
       <c r="C134" s="2" t="inlineStr">
@@ -7884,7 +7884,7 @@
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>1,53832400</t>
+          <t>1,53832366</t>
         </is>
       </c>
       <c r="E134" s="3" t="inlineStr">
@@ -7909,7 +7909,7 @@
       </c>
       <c r="I134" s="2" t="inlineStr">
         <is>
-          <t>351,682</t>
+          <t>349,182</t>
         </is>
       </c>
       <c r="J134" s="2" t="inlineStr">
@@ -8133,7 +8133,7 @@
       </c>
       <c r="I138" s="2" t="inlineStr">
         <is>
-          <t>13.630,096</t>
+          <t>13.358,530</t>
         </is>
       </c>
       <c r="J138" s="2" t="inlineStr">
@@ -8190,7 +8190,7 @@
       </c>
       <c r="I139" s="4" t="inlineStr">
         <is>
-          <t>12.332,869</t>
+          <t>12.332,337</t>
         </is>
       </c>
       <c r="J139" s="4" t="inlineStr">
@@ -8247,7 +8247,7 @@
       </c>
       <c r="I140" s="2" t="inlineStr">
         <is>
-          <t>3.760,319</t>
+          <t>3.760,105</t>
         </is>
       </c>
       <c r="J140" s="2" t="inlineStr">
@@ -8269,7 +8269,7 @@
       </c>
       <c r="B141" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF TURQUESA CORPORATIVO RF CP RESP LTDA</t>
+          <t>CAIXA FIC FIF TURQUESA CORPORATIVO RF CP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C141" s="4" t="inlineStr">
@@ -8304,7 +8304,7 @@
       </c>
       <c r="I141" s="4" t="inlineStr">
         <is>
-          <t>1.405,753</t>
+          <t>1.405,645</t>
         </is>
       </c>
       <c r="J141" s="4" t="inlineStr">
@@ -8326,7 +8326,7 @@
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF AUTOMATICO POLIS RF CURTO PRAZO RESP LTDA</t>
+          <t>CAIXA FIC FIF AUTOMATICO POLIS RF CURTO PRAZO RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C142" s="2" t="inlineStr">
@@ -8361,7 +8361,7 @@
       </c>
       <c r="I142" s="2" t="inlineStr">
         <is>
-          <t>33.663,684</t>
+          <t>33.436,643</t>
         </is>
       </c>
       <c r="J142" s="2" t="inlineStr">
@@ -8379,7 +8379,7 @@
       </c>
       <c r="B143" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF PRÁTICO RF CURTO PRAZO RESP LTDA</t>
+          <t>CAIXA FIC FIF PRÁTICO RF CURTO PRAZO RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C143" s="4" t="inlineStr">
@@ -8414,7 +8414,7 @@
       </c>
       <c r="I143" s="4" t="inlineStr">
         <is>
-          <t>2.913,398</t>
+          <t>2.900,764</t>
         </is>
       </c>
       <c r="J143" s="4" t="inlineStr">
@@ -8436,7 +8436,7 @@
       </c>
       <c r="B144" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF TRANSFERÊNCIA VOLUNTÁRIA RF CP RESP LTDA</t>
+          <t>CAIXA FIC FIF TRANSFERÊNCIA VOLUNTÁRIA RF CP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C144" s="2" t="inlineStr">
@@ -8471,7 +8471,7 @@
       </c>
       <c r="I144" s="2" t="inlineStr">
         <is>
-          <t>14.478,393</t>
+          <t>14.686,376</t>
         </is>
       </c>
       <c r="J144" s="2" t="inlineStr">
@@ -8528,7 +8528,7 @@
       </c>
       <c r="I145" s="4" t="inlineStr">
         <is>
-          <t>9.177,241</t>
+          <t>9.177,239</t>
         </is>
       </c>
       <c r="J145" s="4" t="inlineStr">
@@ -9261,7 +9261,7 @@
       </c>
       <c r="I158" s="2" t="inlineStr">
         <is>
-          <t>13.071,443</t>
+          <t>13.071,442</t>
         </is>
       </c>
       <c r="J158" s="2" t="inlineStr">
@@ -9428,7 +9428,7 @@
       </c>
       <c r="I161" s="4" t="inlineStr">
         <is>
-          <t>1.554,634</t>
+          <t>1.645,842</t>
         </is>
       </c>
       <c r="J161" s="4" t="inlineStr">
@@ -9485,7 +9485,7 @@
       </c>
       <c r="I162" s="2" t="inlineStr">
         <is>
-          <t>24.730,802</t>
+          <t>24.730,801</t>
         </is>
       </c>
       <c r="J162" s="2" t="inlineStr">
@@ -9652,7 +9652,7 @@
       </c>
       <c r="I165" s="4" t="inlineStr">
         <is>
-          <t>301,178</t>
+          <t>301,175</t>
         </is>
       </c>
       <c r="J165" s="4" t="inlineStr">
@@ -9741,7 +9741,7 @@
       </c>
       <c r="D167" s="4" t="inlineStr">
         <is>
-          <t>11,26019000</t>
+          <t>11,26018960</t>
         </is>
       </c>
       <c r="E167" s="5" t="inlineStr">
@@ -9908,7 +9908,7 @@
       </c>
       <c r="D170" s="2" t="inlineStr">
         <is>
-          <t>3,47467000</t>
+          <t>3,47467001</t>
         </is>
       </c>
       <c r="E170" s="7" t="inlineStr">
@@ -9965,7 +9965,7 @@
       </c>
       <c r="D171" s="4" t="inlineStr">
         <is>
-          <t>2,54576900</t>
+          <t>2,54576924</t>
         </is>
       </c>
       <c r="E171" s="6" t="inlineStr">
@@ -10047,7 +10047,7 @@
       </c>
       <c r="I172" s="2" t="inlineStr">
         <is>
-          <t>4.941,247</t>
+          <t>4.940,924</t>
         </is>
       </c>
       <c r="J172" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Dados atualizados via Robô: 19/05/2026 00:13
</commit_message>
<xml_diff>
--- a/dados_atuais.xlsx
+++ b/dados_atuais.xlsx
@@ -703,7 +703,11 @@
           <t>PF | PJ</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/fundo-simples/fic-movimentacoes-automaticas-rf-simples/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -870,7 +874,11 @@
           <t>PF | PJ</t>
         </is>
       </c>
-      <c r="K7" s="4" t="inlineStr"/>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/caixa-fic-plus-rf-credito-privado-lp/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1831,7 +1839,11 @@
           <t>PF</t>
         </is>
       </c>
-      <c r="K24" s="2" t="inlineStr"/>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/debentures-incentivadas/caixa-expert-arx-ipca-deb-incentivadas-rf-cred-priv-lp/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -1884,7 +1896,11 @@
           <t>PF | PJ | RPPS</t>
         </is>
       </c>
-      <c r="K25" s="4" t="inlineStr"/>
+      <c r="K25" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/debentures-incentivadas/caixa-expert-vinlanddebenture-</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1994,7 +2010,11 @@
           <t>PF | PJ</t>
         </is>
       </c>
-      <c r="K27" s="4" t="inlineStr"/>
+      <c r="K27" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/caixa-fif-inflacao-2027/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2153,7 +2173,11 @@
           <t>PF</t>
         </is>
       </c>
-      <c r="K30" s="2" t="inlineStr"/>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/debentures-incentivadas/caixa-expert-rb-asset-deb-incentivadas-cdi-rf-cred-priv/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -2259,7 +2283,11 @@
           <t>PF | PJ</t>
         </is>
       </c>
-      <c r="K32" s="2" t="inlineStr"/>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/caixa-fic-plus-qualificado-rf-credito-privado-lp/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -2483,7 +2511,11 @@
           <t>PF | PJ</t>
         </is>
       </c>
-      <c r="K36" s="2" t="inlineStr"/>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/caixa-fic-renda-fixa-ativa-lp/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -2536,7 +2568,11 @@
           <t>PF</t>
         </is>
       </c>
-      <c r="K37" s="4" t="inlineStr"/>
+      <c r="K37" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/voce/renda-fixa/pos-fixados/ate-100.000/caixa-fic-indexa-tesouro-selic-renda-fixa-lp</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2646,7 +2682,11 @@
           <t>PF</t>
         </is>
       </c>
-      <c r="K39" s="4" t="inlineStr"/>
+      <c r="K39" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/caixa-fic-unique-private-cred-priv-lp/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3493,7 +3533,11 @@
           <t>PF | PJ</t>
         </is>
       </c>
-      <c r="K54" s="2" t="inlineStr"/>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/curto-prazo/fic-automatico-polis-rf-cp/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
@@ -3774,7 +3818,11 @@
           <t>GOV | PF | PJ | RPPS</t>
         </is>
       </c>
-      <c r="K59" s="4" t="inlineStr"/>
+      <c r="K59" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/caixa-fi-indexa-short-dolar-mult-lp/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -3880,7 +3928,11 @@
           <t>PF | PJ</t>
         </is>
       </c>
-      <c r="K61" s="4" t="inlineStr"/>
+      <c r="K61" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/caixa-fic-fof-smart-long-short-mm/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -3933,7 +3985,11 @@
           <t>PF | PJ</t>
         </is>
       </c>
-      <c r="K62" s="2" t="inlineStr"/>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/caixa-fic-fof-smart-long-bias-mm/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
@@ -4039,7 +4095,11 @@
           <t>PF | PJ</t>
         </is>
       </c>
-      <c r="K64" s="2" t="inlineStr"/>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/caixa-fic-fof-smart-long-bias-mm/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
@@ -4650,7 +4710,11 @@
           <t>GOV | PF | PJ | RPPS</t>
         </is>
       </c>
-      <c r="K75" s="4" t="inlineStr"/>
+      <c r="K75" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/caixa_fic_fim_cap_protegido_cesta_agro/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -5155,7 +5219,11 @@
           <t>PF | PJ</t>
         </is>
       </c>
-      <c r="K84" s="2" t="inlineStr"/>
+      <c r="K84" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-caixa-expert-spxmm/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
@@ -5322,7 +5390,11 @@
           <t>GOV | PF | PJ</t>
         </is>
       </c>
-      <c r="K87" s="4" t="inlineStr"/>
+      <c r="K87" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/fi-acoes-brasil-etf-bovespa/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -6051,7 +6123,11 @@
           <t>PF | PJ | RPPS</t>
         </is>
       </c>
-      <c r="K100" s="2" t="inlineStr"/>
+      <c r="K100" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/Caixa-FI-Acoes-Banco-do-Brasil-Plus/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
@@ -6161,7 +6237,11 @@
           <t>GOV | PF | PJ</t>
         </is>
       </c>
-      <c r="K102" s="2" t="inlineStr"/>
+      <c r="K102" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/fia-caixa-seguridade/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
@@ -6328,7 +6408,11 @@
           <t>PF | PJ</t>
         </is>
       </c>
-      <c r="K105" s="4" t="inlineStr"/>
+      <c r="K105" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/fic-fia-dividendos-quantitativo/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -6552,7 +6636,11 @@
           <t>PF | PJ | RPPS</t>
         </is>
       </c>
-      <c r="K109" s="4" t="inlineStr"/>
+      <c r="K109" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/fia-caixa-indexa-iagro/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -6605,7 +6693,11 @@
           <t>PF | PJ | RPPS</t>
         </is>
       </c>
-      <c r="K110" s="2" t="inlineStr"/>
+      <c r="K110" s="2" t="inlineStr">
+        <is>
+          <t>http://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/FIA-Institucional-BDR-nivel-I/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="4" t="inlineStr">
@@ -6658,7 +6750,11 @@
           <t>PF | PJ</t>
         </is>
       </c>
-      <c r="K111" s="4" t="inlineStr"/>
+      <c r="K111" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/fia-caixa-seguridade/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -6711,7 +6807,11 @@
           <t>PF | PJ | RPPS</t>
         </is>
       </c>
-      <c r="K112" s="2" t="inlineStr"/>
+      <c r="K112" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/fia-caixa-eletrobras/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="4" t="inlineStr">
@@ -7412,7 +7512,11 @@
           <t>PJ</t>
         </is>
       </c>
-      <c r="K125" s="4" t="inlineStr"/>
+      <c r="K125" s="4" t="inlineStr">
+        <is>
+          <t>http://site.extra.caixa.gov.br/fundos-investimento/fundo-simples/fic-azulzinha-rf-simples/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -7864,7 +7968,11 @@
           <t>PJ</t>
         </is>
       </c>
-      <c r="K133" s="4" t="inlineStr"/>
+      <c r="K133" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/referenciados/fi-safira-corporativo-rf-lp</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -7917,7 +8025,11 @@
           <t>PJ</t>
         </is>
       </c>
-      <c r="K134" s="2" t="inlineStr"/>
+      <c r="K134" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-institucional-soberano-plus-rf-lp/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="4" t="inlineStr">
@@ -8369,7 +8481,11 @@
           <t>GOV</t>
         </is>
       </c>
-      <c r="K142" s="2" t="inlineStr"/>
+      <c r="K142" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/curto-prazo/fic-automatico-polis-rf-cp/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="4" t="inlineStr">
@@ -8536,7 +8652,11 @@
           <t>RPPS</t>
         </is>
       </c>
-      <c r="K145" s="4" t="inlineStr"/>
+      <c r="K145" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fi-brasil-matriz-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -8703,7 +8823,11 @@
           <t>RPPS</t>
         </is>
       </c>
-      <c r="K148" s="2" t="inlineStr"/>
+      <c r="K148" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/brasil-IPCA/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="4" t="inlineStr">
@@ -9383,7 +9507,11 @@
           <t>RPPS</t>
         </is>
       </c>
-      <c r="K160" s="2" t="inlineStr"/>
+      <c r="K160" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-caixa-brasil-idka-pre2a-rf-lp/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="4" t="inlineStr">
@@ -9607,7 +9735,11 @@
           <t>RPPS</t>
         </is>
       </c>
-      <c r="K164" s="2" t="inlineStr"/>
+      <c r="K164" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/estrategia-livre-mm-lp/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Dados atualizados via Robô: 19/05/2026 01:34
</commit_message>
<xml_diff>
--- a/dados_atuais.xlsx
+++ b/dados_atuais.xlsx
@@ -3562,7 +3562,7 @@
       </c>
       <c r="E55" s="6" t="inlineStr">
         <is>
-          <t>-0,007</t>
+          <t>-0,078</t>
         </is>
       </c>
       <c r="F55" s="5" t="inlineStr">
@@ -3619,7 +3619,7 @@
       </c>
       <c r="E56" s="7" t="inlineStr">
         <is>
-          <t>-0,003</t>
+          <t>-0,443</t>
         </is>
       </c>
       <c r="F56" s="3" t="inlineStr">
@@ -5814,7 +5814,7 @@
       </c>
       <c r="E95" s="6" t="inlineStr">
         <is>
-          <t>-0,024</t>
+          <t>-0,035</t>
         </is>
       </c>
       <c r="F95" s="6" t="inlineStr">
@@ -9692,7 +9692,7 @@
       </c>
       <c r="B164" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF BRASIL ESTRATÉGIA LIVRE MM LP RESP LTDA (1)</t>
+          <t>CAIXA FIC FIF BRASIL ESTRATÉGIA LIVRE MM LP RESP LTDA</t>
         </is>
       </c>
       <c r="C164" s="2" t="inlineStr">
@@ -9702,32 +9702,32 @@
       </c>
       <c r="D164" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E164" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F164" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G164" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H164" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1.541,83184800</t>
+        </is>
+      </c>
+      <c r="E164" s="7" t="inlineStr">
+        <is>
+          <t>-0,299</t>
+        </is>
+      </c>
+      <c r="F164" s="7" t="inlineStr">
+        <is>
+          <t>-0,50</t>
+        </is>
+      </c>
+      <c r="G164" s="3" t="inlineStr">
+        <is>
+          <t>3,87</t>
+        </is>
+      </c>
+      <c r="H164" s="3" t="inlineStr">
+        <is>
+          <t>13,07</t>
         </is>
       </c>
       <c r="I164" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>131,786</t>
         </is>
       </c>
       <c r="J164" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Dados atualizados via Robô: 19/05/2026 02:21
</commit_message>
<xml_diff>
--- a/dados_atuais.xlsx
+++ b/dados_atuais.xlsx
@@ -546,7 +546,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIF E-SIMPLES RENDA FIXA LP RESP LTDA</t>
+          <t>CAIXA FIF E-SIMPLES RENDA FIXA LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -717,7 +717,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF GERAÇÃO JOVEM CRED PRIV RF LP RESP LTDA</t>
+          <t>CAIXA FIC FIF GERAÇÃO JOVEM CRED PRIV RF LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -774,7 +774,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF RELACIONAMENTO PERSONAL RF LP RESP LTDA</t>
+          <t>CAIXA FIC FIF RELACIONAMENTO PERSONAL RF LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -831,7 +831,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>CAIXA MASTER PLUS FIF RF CRED PRIV LP RESP LTDA</t>
+          <t>CAIXA MASTER PLUS FIF RF CRED PRIV LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -888,7 +888,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF IDEAL RF LP RESP LTDA</t>
+          <t>CAIXA FIC FIF IDEAL RF LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -945,7 +945,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF E-FUNDO RF LP RESP LTDA</t>
+          <t>CAIXA FIC FIF E-FUNDO RF LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -1002,7 +1002,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF EXCLUSIVO FUNC RF CREDITO PRIVADO LP RESP LTDA</t>
+          <t>CAIXA FIC FIF EXCLUSIVO FUNC RF CREDITO PRIVADO LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF ABSOLUTO PRE RF LP RESP LTDA</t>
+          <t>CAIXA FIC FIF ABSOLUTO PRE RF LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -1112,7 +1112,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF CAPITAL IND PREÇOS RF LP RESP LTDA</t>
+          <t>CAIXA FIC FIF CAPITAL IND PREÇOS RF LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1169,7 +1169,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF EMPREENDER RF LP RESP LTDA</t>
+          <t>CAIXA FIC FIF EMPREENDER RF LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -1226,7 +1226,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF SOBERANO RF LP RESP LTDA</t>
+          <t>CAIXA FIC FIF SOBERANO RF LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF FOCO IND PREÇOS RF LP RESP LTDA</t>
+          <t>CAIXA FIC FIF FOCO IND PREÇOS RF LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -1340,7 +1340,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF CLÁSSICO RF LP RESP LTDA</t>
+          <t>CAIXA FIC FIF CLÁSSICO RF LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1397,7 +1397,7 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF DESENVOLVER RF LP RESP LTDA</t>
+          <t>CAIXA FIC FIF DESENVOLVER RF LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
@@ -1454,7 +1454,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF OBJETIVO PRE RF LP RESP LTDA</t>
+          <t>CAIXA FIC FIF OBJETIVO PRE RF LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1511,7 +1511,7 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF OAB RF CRÉD PRIV LP RESP LTDA</t>
+          <t>CAIXA FIC FIF OAB RF CRÉD PRIV LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -1568,7 +1568,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF EXECUTIVO RF LP RESP LTDA</t>
+          <t>CAIXA FIC FIF EXECUTIVO RF LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1625,7 +1625,7 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC RELACIONAMENTO IDEAL RF LP</t>
+          <t>CAIXA FIC RELACIONAMENTO IDEAL RF LP (8)</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
@@ -1682,7 +1682,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF PERFORMANCE IMA-B RF LP RESP LTDA</t>
+          <t>CAIXA FIC FIF PERFORMANCE IMA-B RF LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -1739,7 +1739,7 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIFINVESTIDOR RF LP RESP LTDA</t>
+          <t>CAIXA FIC FIFINVESTIDOR RF LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
@@ -1806,32 +1806,32 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>1,10997325</t>
+          <t>1,10691900</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>-0,001</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
+          <t>-0,276</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>-0,28</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>2,61</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t>0,00</t>
         </is>
       </c>
-      <c r="G24" s="3" t="inlineStr">
-        <is>
-          <t>2,89</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>219,622</t>
+          <t>219,018</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
@@ -1863,32 +1863,32 @@
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>1,22811400</t>
-        </is>
-      </c>
-      <c r="E25" s="6" t="inlineStr">
-        <is>
-          <t>-0,001</t>
+          <t>1,22877200</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>0,052</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>0,62</t>
+          <t>0,67</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>4,85</t>
+          <t>4,91</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr">
         <is>
-          <t>14,63</t>
+          <t>14,69</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>70,980</t>
+          <t>71,018</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -1910,7 +1910,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF PLUS QUALI RF CREDI PRIV LP RESP LTDA</t>
+          <t>CAIXA FIC FIF PLUS QUALI RF CREDI PRIV LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1967,7 +1967,7 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIF INFLACAO PRIVATE 2027 RF LONGO PRAZO</t>
+          <t>CAIXA FIF INFLACAO PRIVATE 2027 RF LONGO PRAZO (8)</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
@@ -2034,22 +2034,22 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>1,02936900</t>
-        </is>
-      </c>
-      <c r="E28" s="7" t="inlineStr">
-        <is>
-          <t>-0,001</t>
+          <t>1,02990900</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>0,051</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>0,52</t>
+          <t>0,57</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>4,97</t>
+          <t>5,03</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -2059,7 +2059,7 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>21,758</t>
+          <t>21,769</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
@@ -2087,32 +2087,32 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>1,15576700</t>
-        </is>
-      </c>
-      <c r="E29" s="6" t="inlineStr">
-        <is>
-          <t>-0,001</t>
+          <t>1,15651000</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>0,062</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>0,66</t>
+          <t>0,73</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>4,08</t>
+          <t>4,14</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr">
         <is>
-          <t>13,73</t>
+          <t>13,81</t>
         </is>
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>66,353</t>
+          <t>66,395</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -2140,22 +2140,22 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>1,05776364</t>
-        </is>
-      </c>
-      <c r="E30" s="7" t="inlineStr">
-        <is>
-          <t>-0,001</t>
+          <t>1,05784500</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>0,006</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>0,31</t>
+          <t>0,32</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>2,36</t>
+          <t>2,37</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -2165,7 +2165,7 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>332,405</t>
+          <t>332,430</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
@@ -2240,7 +2240,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIF QUALIFICADO RF CRED PRIV LP - RESP LTDA</t>
+          <t>CAIXA FIF QUALIFICADO RF CRED PRIV LP - RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -2297,7 +2297,7 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF EXPERTISE RF CRED PRIV LP RESP LTDA</t>
+          <t>CAIXA FIC FIF EXPERTISE RF CRED PRIV LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
@@ -2354,7 +2354,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF SELEÇÃO RF RESP LTDA</t>
+          <t>CAIXA FIC FIF SELEÇÃO RF RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -2411,7 +2411,7 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF PERSONAL RF LP RESP LTDA</t>
+          <t>CAIXA FIC FIF PERSONAL RF LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
@@ -2468,7 +2468,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF RENDA FIXA ATIVA LP RESP LTDA</t>
+          <t>CAIXA FIC FIF RENDA FIXA ATIVA LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -2525,7 +2525,7 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>CAIXA INDEXA TESOURO SELIC FIC FIF RF LP - RESP LTDA</t>
+          <t>CAIXA INDEXA TESOURO SELIC FIC FIF RF LP - RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
@@ -2582,7 +2582,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF SUPREMO RF LP RESP LTDA</t>
+          <t>CAIXA FIC FIF SUPREMO RF LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2639,7 +2639,7 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF UNIQUE RF CRED PRIV LP - RL</t>
+          <t>CAIXA FIC FIF UNIQUE RF CRED PRIV LP - RL (8)</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
@@ -2696,7 +2696,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF ESPECIAL RF LP RESP LTDA</t>
+          <t>CAIXA FIC FIF ESPECIAL RF LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -2753,7 +2753,7 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIF FIDELIDADE PRIVATE RF LP - RESP LTDA</t>
+          <t>CAIXA FIF FIDELIDADE PRIVATE RF LP - RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
@@ -2810,7 +2810,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF MAXI RENDA FIXA CRED PRIV LP - RESP LTDA</t>
+          <t>CAIXA FIC FIF MAXI RENDA FIXA CRED PRIV LP - RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIF FIDELIDADE II RF CRÉD PRIV LP</t>
+          <t>CAIXA FIF FIDELIDADE II RF CRÉD PRIV LP (8)</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
@@ -2924,7 +2924,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF BETA RF REF DI LP RESP LTDA</t>
+          <t>CAIXA FIC FIF BETA RF REF DI LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -2981,7 +2981,7 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>CAIXA SIGMA FUNCIONARIOS FIC FIF RF REF DI LP - RESP LTDA (2) (3)</t>
+          <t>CAIXA SIGMA FUNCIONARIOS FIC FIF RF REF DI LP - RESP LTDA (2) (3) (8)</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
@@ -3034,7 +3034,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF GIRO IMEDIATO RF REF DI LP RESP LTDA</t>
+          <t>CAIXA FIC FIF GIRO IMEDIATO RF REF DI LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -3091,7 +3091,7 @@
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF PLENO REF DI LP RESP LTDA</t>
+          <t>CAIXA FIC FIF PLENO REF DI LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
@@ -3148,7 +3148,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC OMEGA REF DI RF LONGO PRAZO</t>
+          <t>CAIXA FIC OMEGA REF DI RF LONGO PRAZO (8)</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -3205,7 +3205,7 @@
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF PREFERENCIAL REF DI LP RESP LTDA</t>
+          <t>CAIXA FIC FIF PREFERENCIAL REF DI LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
@@ -3262,7 +3262,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF SIGMA RF REF DI LP RESP LTDA</t>
+          <t>CAIXA FIC FIF SIGMA RF REF DI LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -3319,7 +3319,7 @@
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF RUBI RF REF DI LP RESP LTDA</t>
+          <t>CAIXA FIC FIF RUBI RF REF DI LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
@@ -3376,7 +3376,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF MEGA RF REFERENC DI LONGO PRAZO - RESP LTDA</t>
+          <t>CAIXA FIC FIF MEGA RF REFERENC DI LONGO PRAZO - RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -3433,7 +3433,7 @@
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF TOP PRIVATE RF REF DI LP RESP LTDA</t>
+          <t>CAIXA FIC FIF TOP PRIVATE RF REF DI LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
@@ -3557,32 +3557,32 @@
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>1,39931700</t>
-        </is>
-      </c>
-      <c r="E55" s="6" t="inlineStr">
-        <is>
-          <t>-0,078</t>
+          <t>1,40124300</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>0,058</t>
         </is>
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>0,60</t>
+          <t>0,74</t>
         </is>
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
-          <t>4,51</t>
+          <t>4,66</t>
         </is>
       </c>
       <c r="H55" s="5" t="inlineStr">
         <is>
-          <t>14,12</t>
+          <t>14,28</t>
         </is>
       </c>
       <c r="I55" s="4" t="inlineStr">
         <is>
-          <t>68,862</t>
+          <t>68,957</t>
         </is>
       </c>
       <c r="J55" s="4" t="inlineStr">
@@ -3614,32 +3614,32 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>1.167,25373800</t>
-        </is>
-      </c>
-      <c r="E56" s="7" t="inlineStr">
-        <is>
-          <t>-0,443</t>
+          <t>1.184,51723600</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>1,028</t>
         </is>
       </c>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>1,55</t>
+          <t>3,05</t>
         </is>
       </c>
       <c r="G56" s="7" t="inlineStr">
         <is>
-          <t>-6,97</t>
+          <t>-5,60</t>
         </is>
       </c>
       <c r="H56" s="7" t="inlineStr">
         <is>
-          <t>-2,47</t>
+          <t>-1,03</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>35,739</t>
+          <t>36,268</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
@@ -3661,7 +3661,7 @@
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIF MULTIMERCADO RV 30 LP RESP LTDA</t>
+          <t>CAIXA FIF MULTIMERCADO RV 30 LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
@@ -3728,32 +3728,32 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>1.632,15053600</t>
+          <t>1.627,36844900</t>
         </is>
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
-          <t>-0,006</t>
+          <t>-0,299</t>
         </is>
       </c>
       <c r="F58" s="7" t="inlineStr">
         <is>
-          <t>-0,22</t>
+          <t>-0,51</t>
         </is>
       </c>
       <c r="G58" s="3" t="inlineStr">
         <is>
-          <t>4,16</t>
+          <t>3,85</t>
         </is>
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>13,39</t>
+          <t>13,06</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>116,889</t>
+          <t>116,546</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
@@ -3775,7 +3775,7 @@
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIF INDEXA SHORT DOLAR MM LP RESP LTDA</t>
+          <t>CAIXA FIF INDEXA SHORT DOLAR MM LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
@@ -3895,32 +3895,32 @@
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>1,25018500</t>
+          <t>1,24779700</t>
         </is>
       </c>
       <c r="E61" s="6" t="inlineStr">
         <is>
-          <t>-0,005</t>
+          <t>-0,196</t>
         </is>
       </c>
       <c r="F61" s="6" t="inlineStr">
         <is>
-          <t>-0,44</t>
+          <t>-0,63</t>
         </is>
       </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
-          <t>2,36</t>
+          <t>2,16</t>
         </is>
       </c>
       <c r="H61" s="5" t="inlineStr">
         <is>
-          <t>11,60</t>
+          <t>11,39</t>
         </is>
       </c>
       <c r="I61" s="4" t="inlineStr">
         <is>
-          <t>6,666</t>
+          <t>6,654</t>
         </is>
       </c>
       <c r="J61" s="4" t="inlineStr">
@@ -3942,7 +3942,7 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC LONG BIAS MM</t>
+          <t>CAIXA FIC LONG BIAS MM (8)</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -4062,32 +4062,32 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>1,44320300</t>
+          <t>1,43008500</t>
         </is>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>-0,004</t>
+          <t>-0,913</t>
         </is>
       </c>
       <c r="F64" s="7" t="inlineStr">
         <is>
-          <t>-1,73</t>
+          <t>-2,62</t>
         </is>
       </c>
       <c r="G64" s="3" t="inlineStr">
         <is>
-          <t>5,72</t>
+          <t>4,76</t>
         </is>
       </c>
       <c r="H64" s="3" t="inlineStr">
         <is>
-          <t>21,08</t>
+          <t>19,98</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>11,970</t>
+          <t>11,861</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
@@ -4162,7 +4162,7 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIF INDEXA EURO MM LONGO PRAZO RESP LTDA</t>
+          <t>CAIXA FIF INDEXA EURO MM LONGO PRAZO RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -4229,32 +4229,32 @@
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>5,32047778</t>
+          <t>5,30784700</t>
         </is>
       </c>
       <c r="E67" s="6" t="inlineStr">
         <is>
-          <t>-0,003</t>
+          <t>-0,240</t>
         </is>
       </c>
       <c r="F67" s="6" t="inlineStr">
         <is>
-          <t>-0,21</t>
+          <t>-0,44</t>
         </is>
       </c>
       <c r="G67" s="5" t="inlineStr">
         <is>
-          <t>3,69</t>
+          <t>3,44</t>
         </is>
       </c>
       <c r="H67" s="5" t="inlineStr">
         <is>
-          <t>13,12</t>
+          <t>12,85</t>
         </is>
       </c>
       <c r="I67" s="4" t="inlineStr">
         <is>
-          <t>33,192</t>
+          <t>33,114</t>
         </is>
       </c>
       <c r="J67" s="4" t="inlineStr">
@@ -4276,7 +4276,7 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIF INDEXA OURO MULTIMERCADO LP RESP LTDA</t>
+          <t>CAIXA FIF INDEXA OURO MULTIMERCADO LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
@@ -4343,32 +4343,32 @@
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>2,85531700</t>
+          <t>2,84411900</t>
         </is>
       </c>
       <c r="E69" s="6" t="inlineStr">
         <is>
-          <t>-0,004</t>
-        </is>
-      </c>
-      <c r="F69" s="5" t="inlineStr">
-        <is>
-          <t>0,08</t>
+          <t>-0,396</t>
+        </is>
+      </c>
+      <c r="F69" s="6" t="inlineStr">
+        <is>
+          <t>-0,30</t>
         </is>
       </c>
       <c r="G69" s="5" t="inlineStr">
         <is>
-          <t>2,22</t>
+          <t>1,82</t>
         </is>
       </c>
       <c r="H69" s="5" t="inlineStr">
         <is>
-          <t>11,44</t>
+          <t>11,01</t>
         </is>
       </c>
       <c r="I69" s="4" t="inlineStr">
         <is>
-          <t>77,229</t>
+          <t>76,927</t>
         </is>
       </c>
       <c r="J69" s="4" t="inlineStr">
@@ -4390,7 +4390,7 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF HEDGE MULTIMERCADO LONGO PRAZO RESP LTDA</t>
+          <t>CAIXA FIC FIF HEDGE MULTIMERCADO LONGO PRAZO RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
@@ -4447,7 +4447,7 @@
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIF INDEXA BOLSA AMERICANA MM LP RESP LTDA</t>
+          <t>CAIXA FIF INDEXA BOLSA AMERICANA MM LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
@@ -4504,7 +4504,7 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF JUROS E MOEDAS MM PLUS LP RESP LTDA</t>
+          <t>CAIXA FIC FIF JUROS E MOEDAS MM PLUS LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
@@ -4571,32 +4571,32 @@
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>1.652,59401600</t>
+          <t>1.647,85915600</t>
         </is>
       </c>
       <c r="E73" s="6" t="inlineStr">
         <is>
-          <t>-0,003</t>
+          <t>-0,289</t>
         </is>
       </c>
       <c r="F73" s="6" t="inlineStr">
         <is>
-          <t>-0,18</t>
+          <t>-0,47</t>
         </is>
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>4,49</t>
+          <t>4,19</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
         <is>
-          <t>14,36</t>
+          <t>14,03</t>
         </is>
       </c>
       <c r="I73" s="4" t="inlineStr">
         <is>
-          <t>15,317</t>
+          <t>15,273</t>
         </is>
       </c>
       <c r="J73" s="4" t="inlineStr">
@@ -4624,22 +4624,22 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>0,57593472</t>
+          <t>0,56806700</t>
         </is>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>-0,007</t>
+          <t>-1,373</t>
         </is>
       </c>
       <c r="F74" s="3" t="inlineStr">
         <is>
-          <t>6,16</t>
+          <t>4,71</t>
         </is>
       </c>
       <c r="G74" s="7" t="inlineStr">
         <is>
-          <t>-20,24</t>
+          <t>-21,33</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
@@ -4649,7 +4649,7 @@
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>4,200</t>
+          <t>4,142</t>
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr">
@@ -4677,32 +4677,32 @@
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>1,37874300</t>
+          <t>1,37535500</t>
         </is>
       </c>
       <c r="E75" s="6" t="inlineStr">
         <is>
-          <t>-0,003</t>
+          <t>-0,249</t>
         </is>
       </c>
       <c r="F75" s="6" t="inlineStr">
         <is>
-          <t>-1,35</t>
+          <t>-1,59</t>
         </is>
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>1,66</t>
+          <t>1,41</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
         <is>
-          <t>8,35</t>
+          <t>8,08</t>
         </is>
       </c>
       <c r="I75" s="4" t="inlineStr">
         <is>
-          <t>70,771</t>
+          <t>70,597</t>
         </is>
       </c>
       <c r="J75" s="4" t="inlineStr">
@@ -4734,32 +4734,32 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>1,53337400</t>
+          <t>1,53191100</t>
         </is>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>-0,004</t>
-        </is>
-      </c>
-      <c r="F76" s="2" t="inlineStr">
-        <is>
-          <t>0,00</t>
+          <t>-0,100</t>
+        </is>
+      </c>
+      <c r="F76" s="7" t="inlineStr">
+        <is>
+          <t>-0,10</t>
         </is>
       </c>
       <c r="G76" s="3" t="inlineStr">
         <is>
-          <t>2,69</t>
+          <t>2,59</t>
         </is>
       </c>
       <c r="H76" s="3" t="inlineStr">
         <is>
-          <t>18,93</t>
+          <t>18,82</t>
         </is>
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>14,513</t>
+          <t>14,499</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr">
@@ -4791,32 +4791,32 @@
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>3,25598300</t>
+          <t>3,23396800</t>
         </is>
       </c>
       <c r="E77" s="6" t="inlineStr">
         <is>
-          <t>-0,005</t>
+          <t>-0,681</t>
         </is>
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>1,19</t>
+          <t>0,50</t>
         </is>
       </c>
       <c r="G77" s="5" t="inlineStr">
         <is>
-          <t>2,19</t>
+          <t>1,50</t>
         </is>
       </c>
       <c r="H77" s="5" t="inlineStr">
         <is>
-          <t>7,05</t>
+          <t>6,33</t>
         </is>
       </c>
       <c r="I77" s="4" t="inlineStr">
         <is>
-          <t>155,146</t>
+          <t>154,097</t>
         </is>
       </c>
       <c r="J77" s="4" t="inlineStr">
@@ -4848,32 +4848,32 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>1,47220000</t>
-        </is>
-      </c>
-      <c r="E78" s="7" t="inlineStr">
-        <is>
-          <t>-0,003</t>
+          <t>1,47794200</t>
+        </is>
+      </c>
+      <c r="E78" s="3" t="inlineStr">
+        <is>
+          <t>0,386</t>
         </is>
       </c>
       <c r="F78" s="3" t="inlineStr">
         <is>
-          <t>1,51</t>
+          <t>1,90</t>
         </is>
       </c>
       <c r="G78" s="3" t="inlineStr">
         <is>
-          <t>1,80</t>
+          <t>2,19</t>
         </is>
       </c>
       <c r="H78" s="3" t="inlineStr">
         <is>
-          <t>14,37</t>
+          <t>14,82</t>
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>190,975</t>
+          <t>191,720</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr">
@@ -4958,32 +4958,32 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>1,31674000</t>
+          <t>1,30889800</t>
         </is>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
-          <t>-0,001</t>
-        </is>
-      </c>
-      <c r="F80" s="3" t="inlineStr">
-        <is>
-          <t>0,57</t>
+          <t>-0,597</t>
+        </is>
+      </c>
+      <c r="F80" s="7" t="inlineStr">
+        <is>
+          <t>-0,02</t>
         </is>
       </c>
       <c r="G80" s="3" t="inlineStr">
         <is>
-          <t>2,59</t>
+          <t>1,97</t>
         </is>
       </c>
       <c r="H80" s="3" t="inlineStr">
         <is>
-          <t>2,78</t>
+          <t>2,17</t>
         </is>
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>13,395</t>
+          <t>13,313</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr">
@@ -5005,7 +5005,7 @@
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF ALOCAÇÃO MACRO MM LONGO PRAZO RESP LTDA</t>
+          <t>CAIXA FIC FIF ALOCAÇÃO MACRO MM LONGO PRAZO RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
@@ -5062,7 +5062,7 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF JUROS E MOEDAS MM LP RESP LTDA</t>
+          <t>CAIXA FIC FIF JUROS E MOEDAS MM LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
@@ -5186,32 +5186,32 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>1,77206600</t>
-        </is>
-      </c>
-      <c r="E84" s="7" t="inlineStr">
-        <is>
-          <t>-0,002</t>
+          <t>1,77462000</t>
+        </is>
+      </c>
+      <c r="E84" s="3" t="inlineStr">
+        <is>
+          <t>0,142</t>
         </is>
       </c>
       <c r="F84" s="3" t="inlineStr">
         <is>
-          <t>0,72</t>
+          <t>0,86</t>
         </is>
       </c>
       <c r="G84" s="3" t="inlineStr">
         <is>
-          <t>0,31</t>
+          <t>0,45</t>
         </is>
       </c>
       <c r="H84" s="3" t="inlineStr">
         <is>
-          <t>10,69</t>
+          <t>10,85</t>
         </is>
       </c>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t>176,392</t>
+          <t>176,646</t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr">
@@ -5233,7 +5233,7 @@
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF INDEXA DOLAR CAMBIAL RESP LTDA</t>
+          <t>CAIXA FIC FIF INDEXA DOLAR CAMBIAL RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
@@ -5290,7 +5290,7 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIF AÇÕES DIVIDENDOS RESP LTDA</t>
+          <t>CAIXA FIF AÇÕES DIVIDENDOS RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
@@ -5347,7 +5347,7 @@
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF AÇÕES E-FUNDOS IBOVESPA RESP LTDA</t>
+          <t>CAIXA FIC FIF AÇÕES E-FUNDOS IBOVESPA RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
@@ -5404,7 +5404,7 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>CAIXA ATENA FIC FIF AÇÕES FUNCIONÁRIOS LIVRE QUANT RESP LTDA</t>
+          <t>CAIXA ATENA FIC FIF AÇÕES FUNCIONÁRIOS LIVRE QUANT RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
@@ -5457,7 +5457,7 @@
       </c>
       <c r="B89" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIF AÇÕES BDR NÍVEL I RESP LTDA</t>
+          <t>CAIXA FIF AÇÕES BDR NÍVEL I RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C89" s="4" t="inlineStr">
@@ -5514,7 +5514,7 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIF AÇÕES SMALL CAPS ATIVO RESP LTDA</t>
+          <t>CAIXA FIF AÇÕES SMALL CAPS ATIVO RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
@@ -5571,7 +5571,7 @@
       </c>
       <c r="B91" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIF AÇÕES CONSUMO RESP LTDA</t>
+          <t>CAIXA FIF AÇÕES CONSUMO RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C91" s="4" t="inlineStr">
@@ -5628,7 +5628,7 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIF ACOES SUSTENTABILIDADE EMPRESARIAL ISE - IS RESP LTDA</t>
+          <t>CAIXA FIF ACOES SUSTENTABILIDADE EMPRESARIAL ISE - IS RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
@@ -5685,7 +5685,7 @@
       </c>
       <c r="B93" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIF ACOES PETROBRAS PLUS RESP LTDA</t>
+          <t>CAIXA FIF ACOES PETROBRAS PLUS RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C93" s="4" t="inlineStr">
@@ -5742,7 +5742,7 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF AÇÕES IBOVESPA RESP LTDA</t>
+          <t>CAIXA FIC FIF AÇÕES IBOVESPA RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
@@ -5809,32 +5809,32 @@
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
-          <t>1,30185000</t>
+          <t>1,28764700</t>
         </is>
       </c>
       <c r="E95" s="6" t="inlineStr">
         <is>
-          <t>-0,035</t>
+          <t>-1,125</t>
         </is>
       </c>
       <c r="F95" s="6" t="inlineStr">
         <is>
-          <t>-4,66</t>
+          <t>-5,70</t>
         </is>
       </c>
       <c r="G95" s="5" t="inlineStr">
         <is>
-          <t>1,14</t>
+          <t>0,04</t>
         </is>
       </c>
       <c r="H95" s="5" t="inlineStr">
         <is>
-          <t>10,89</t>
+          <t>9,68</t>
         </is>
       </c>
       <c r="I95" s="4" t="inlineStr">
         <is>
-          <t>295,634</t>
+          <t>292,409</t>
         </is>
       </c>
       <c r="J95" s="4" t="inlineStr">
@@ -5856,7 +5856,7 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIF AÇÕES CONSTRUÇÃO CIVIL RESP LTDA</t>
+          <t>CAIXA FIF AÇÕES CONSTRUÇÃO CIVIL RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
@@ -5913,7 +5913,7 @@
       </c>
       <c r="B97" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIF AÇÕES INFRAESTRUTURA RESP LTDA</t>
+          <t>CAIXA FIF AÇÕES INFRAESTRUTURA RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C97" s="4" t="inlineStr">
@@ -5970,7 +5970,7 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>CAIXA ATENA FIC FIF AÇÕES LIVRE QUANT RESP LTDA</t>
+          <t>CAIXA ATENA FIC FIF AÇÕES LIVRE QUANT RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
@@ -6023,7 +6023,7 @@
       </c>
       <c r="B99" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIF AÇÕES PETROBRAS PRÉ-SAL RESP LTDA</t>
+          <t>CAIXA FIF AÇÕES PETROBRAS PRÉ-SAL RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C99" s="4" t="inlineStr">
@@ -6080,7 +6080,7 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIF ACOES BANCO DO BRASIL PLUS RESP LTDA</t>
+          <t>CAIXA FIF ACOES BANCO DO BRASIL PLUS RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
@@ -6137,7 +6137,7 @@
       </c>
       <c r="B101" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIF AÇÕES VALE DO RIO DOCE RESP LTDA</t>
+          <t>CAIXA FIF AÇÕES VALE DO RIO DOCE RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C101" s="4" t="inlineStr">
@@ -6194,7 +6194,7 @@
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIF ACOES SEGURIDADE RESP LTDA</t>
+          <t>CAIXA FIF ACOES SEGURIDADE RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
@@ -6251,7 +6251,7 @@
       </c>
       <c r="B103" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIF AÇÕES IBRX ATIVO RESP LTDA</t>
+          <t>CAIXA FIF AÇÕES IBRX ATIVO RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C103" s="4" t="inlineStr">
@@ -6308,7 +6308,7 @@
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIF ACOES INDEXA SETOR FINANCEIRO RESP LTDA</t>
+          <t>CAIXA FIF ACOES INDEXA SETOR FINANCEIRO RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
@@ -6365,7 +6365,7 @@
       </c>
       <c r="B105" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF ACOES DIVIDENDOS QUANTITATIVO RESP LTDA</t>
+          <t>CAIXA FIC FIF ACOES DIVIDENDOS QUANTITATIVO RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C105" s="4" t="inlineStr">
@@ -6422,7 +6422,7 @@
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIF ACOES INDEXA PIBB IBRX 50 RESP LTDA</t>
+          <t>CAIXA FIF ACOES INDEXA PIBB IBRX 50 RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
@@ -6479,7 +6479,7 @@
       </c>
       <c r="B107" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIF ACOES IBOVESPA ATIVO RESP LTDA</t>
+          <t>CAIXA FIF ACOES IBOVESPA ATIVO RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C107" s="4" t="inlineStr">
@@ -6536,7 +6536,7 @@
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIF AÇÕES PETROBRÁS RESP LTDA</t>
+          <t>CAIXA FIF AÇÕES PETROBRÁS RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
@@ -6593,7 +6593,7 @@
       </c>
       <c r="B109" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIF ACOES INDEXA IAGRO RESP LTDA</t>
+          <t>CAIXA FIF ACOES INDEXA IAGRO RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C109" s="4" t="inlineStr">
@@ -6650,7 +6650,7 @@
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF ACOES COMPROMISSO BDR NIVEL I RESP LTDA</t>
+          <t>CAIXA FIC FIF ACOES COMPROMISSO BDR NIVEL I RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
@@ -6707,7 +6707,7 @@
       </c>
       <c r="B111" s="4" t="inlineStr">
         <is>
-          <t>CAIXA SEGURIDADE II FIF ACOES - RESP LTDA</t>
+          <t>CAIXA SEGURIDADE II FIF ACOES - RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C111" s="4" t="inlineStr">
@@ -6764,7 +6764,7 @@
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIF ACOES ELETROBRAS RESP LTDA</t>
+          <t>CAIXA FIF ACOES ELETROBRAS RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C112" s="2" t="inlineStr">
@@ -6831,32 +6831,32 @@
       </c>
       <c r="D113" s="4" t="inlineStr">
         <is>
-          <t>1.017,29224100</t>
+          <t>1.011,74473600</t>
         </is>
       </c>
       <c r="E113" s="6" t="inlineStr">
         <is>
-          <t>-0,003</t>
+          <t>-0,548</t>
         </is>
       </c>
       <c r="F113" s="6" t="inlineStr">
         <is>
-          <t>-4,92</t>
+          <t>-5,44</t>
         </is>
       </c>
       <c r="G113" s="5" t="inlineStr">
         <is>
-          <t>3,76</t>
+          <t>3,20</t>
         </is>
       </c>
       <c r="H113" s="5" t="inlineStr">
         <is>
-          <t>19,30</t>
+          <t>18,65</t>
         </is>
       </c>
       <c r="I113" s="4" t="inlineStr">
         <is>
-          <t>8,171</t>
+          <t>8,126</t>
         </is>
       </c>
       <c r="J113" s="4" t="inlineStr">
@@ -6888,32 +6888,32 @@
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>1.538,75924600</t>
+          <t>1.528,30147000</t>
         </is>
       </c>
       <c r="E114" s="7" t="inlineStr">
         <is>
-          <t>-0,002</t>
+          <t>-0,682</t>
         </is>
       </c>
       <c r="F114" s="7" t="inlineStr">
         <is>
-          <t>-4,34</t>
+          <t>-4,99</t>
         </is>
       </c>
       <c r="G114" s="3" t="inlineStr">
         <is>
-          <t>2,87</t>
+          <t>2,17</t>
         </is>
       </c>
       <c r="H114" s="3" t="inlineStr">
         <is>
-          <t>15,06</t>
+          <t>14,28</t>
         </is>
       </c>
       <c r="I114" s="2" t="inlineStr">
         <is>
-          <t>22,409</t>
+          <t>22,256</t>
         </is>
       </c>
       <c r="J114" s="2" t="inlineStr">
@@ -6935,7 +6935,7 @@
       </c>
       <c r="B115" s="4" t="inlineStr">
         <is>
-          <t>CAIXA ETF IBOVESPA FUNDO DE ÍNDICE RESP LTDA</t>
+          <t>CAIXA ETF IBOVESPA FUNDO DE ÍNDICE RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C115" s="4" t="inlineStr">
@@ -6992,7 +6992,7 @@
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FMP-FGTS ELETROBRAS MIGRACAO</t>
+          <t>CAIXA FMP-FGTS ELETROBRAS MIGRACAO (8)</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
@@ -7045,7 +7045,7 @@
       </c>
       <c r="B117" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FMP-FGTS ELETROBRAS RESP LTDA</t>
+          <t>CAIXA FMP-FGTS ELETROBRAS RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C117" s="4" t="inlineStr">
@@ -7098,7 +7098,7 @@
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FMP-FGTS PETROBRÁS IV RESP LTDA</t>
+          <t>CAIXA FMP-FGTS PETROBRÁS IV RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
@@ -7151,7 +7151,7 @@
       </c>
       <c r="B119" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FMP-FGTS VALE RIO DOCE II RESP LTDA</t>
+          <t>CAIXA FMP-FGTS VALE RIO DOCE II RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C119" s="4" t="inlineStr">
@@ -7204,7 +7204,7 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FMP-FGTS CL ABSOLUTO RESP LTDA</t>
+          <t>CAIXA FMP-FGTS CL ABSOLUTO RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
@@ -7257,7 +7257,7 @@
       </c>
       <c r="B121" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FMP-FGTS VALE RIO DOCE MIGRAÇÃO RESP LTDA</t>
+          <t>CAIXA FMP-FGTS VALE RIO DOCE MIGRAÇÃO RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C121" s="4" t="inlineStr">
@@ -7310,7 +7310,7 @@
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FMP-FGTS PETROBRÁS II RESP LTDA</t>
+          <t>CAIXA FMP-FGTS PETROBRÁS II RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
@@ -7363,7 +7363,7 @@
       </c>
       <c r="B123" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FMP-FGTS VALE RIO DOCE I RESP LTDA</t>
+          <t>CAIXA FMP-FGTS VALE RIO DOCE I RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C123" s="4" t="inlineStr">
@@ -7416,7 +7416,7 @@
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FMP-FGTS PETROBRÁS III RESP LTDA</t>
+          <t>CAIXA FMP-FGTS PETROBRÁS III RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
@@ -7583,7 +7583,7 @@
       </c>
       <c r="B127" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF EQUILIBRIO MPE RF LP RESP LTDA</t>
+          <t>CAIXA FIC FIF EQUILIBRIO MPE RF LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C127" s="4" t="inlineStr">
@@ -7640,7 +7640,7 @@
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIF SAUDE SUPLEMENTAR ANS RF LP - RESP LTDA</t>
+          <t>CAIXA FIF SAUDE SUPLEMENTAR ANS RF LP - RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C128" s="2" t="inlineStr">
@@ -7697,7 +7697,7 @@
       </c>
       <c r="B129" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF TITULO PUBLICO MPE RF LP RESP LTDA</t>
+          <t>CAIXA FIC FIF TITULO PUBLICO MPE RF LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C129" s="4" t="inlineStr">
@@ -7754,7 +7754,7 @@
       </c>
       <c r="B130" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF PATRIMONIO IND.DE PRECOS RF LP RESP LTDA</t>
+          <t>CAIXA FIC FIF PATRIMONIO IND.DE PRECOS RF LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C130" s="2" t="inlineStr">
@@ -7811,7 +7811,7 @@
       </c>
       <c r="B131" s="4" t="inlineStr">
         <is>
-          <t>CAIXA GIRO EMPRESAS FIC FIF RF REF DI LP RESP LTDA</t>
+          <t>CAIXA GIRO EMPRESAS FIC FIF RF REF DI LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C131" s="4" t="inlineStr">
@@ -7868,7 +7868,7 @@
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIF DIAMANTE CORP RF CRED PRIV LP - RESP LTDA</t>
+          <t>CAIXA FIF DIAMANTE CORP RF CRED PRIV LP - RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C132" s="2" t="inlineStr">
@@ -7925,7 +7925,7 @@
       </c>
       <c r="B133" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIF SAFIRA CORPORATIVO RF LP - RESP LTDA</t>
+          <t>CAIXA FIF SAFIRA CORPORATIVO RF LP - RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C133" s="4" t="inlineStr">
@@ -8039,7 +8039,7 @@
       </c>
       <c r="B135" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIF SAUDE SUPLEMENTAR ANS II RF LP - RESP LTDA</t>
+          <t>CAIXA FIF SAUDE SUPLEMENTAR ANS II RF LP - RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C135" s="4" t="inlineStr">
@@ -8096,7 +8096,7 @@
       </c>
       <c r="B136" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIF CNI RF LP - RESP LTDA</t>
+          <t>CAIXA FIF CNI RF LP - RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C136" s="2" t="inlineStr">
@@ -8153,7 +8153,7 @@
       </c>
       <c r="B137" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIF SEBRAE RF LP RESP LTDA</t>
+          <t>CAIXA FIF SEBRAE RF LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C137" s="4" t="inlineStr">
@@ -8210,7 +8210,7 @@
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF GIRO MPE REF DI LP RESP LTDA</t>
+          <t>CAIXA FIC FIF GIRO MPE REF DI LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C138" s="2" t="inlineStr">
@@ -8267,7 +8267,7 @@
       </c>
       <c r="B139" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIF TOPAZIO CORP RF REFERENC DI - RESP LTDA</t>
+          <t>CAIXA FIF TOPAZIO CORP RF REFERENC DI - RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C139" s="4" t="inlineStr">
@@ -8324,7 +8324,7 @@
       </c>
       <c r="B140" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC ESMERALDA CORP RF REF DI CRED PRIV LP - RESP LTDA</t>
+          <t>CAIXA FIC ESMERALDA CORP RF REF DI CRED PRIV LP - RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C140" s="2" t="inlineStr">
@@ -8609,7 +8609,7 @@
       </c>
       <c r="B145" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIF BRASIL MATRIZ RF RESP LTDA</t>
+          <t>CAIXA FIF BRASIL MATRIZ RF RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C145" s="4" t="inlineStr">
@@ -8666,7 +8666,7 @@
       </c>
       <c r="B146" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF BRASIL GESTÃO ESTRATÉGICA RF RESP LTDA</t>
+          <t>CAIXA FIC FIF BRASIL GESTÃO ESTRATÉGICA RF RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C146" s="2" t="inlineStr">
@@ -8723,7 +8723,7 @@
       </c>
       <c r="B147" s="4" t="inlineStr">
         <is>
-          <t>CAIXA BRASIL INFLAÇÃO ATIVA FIF RF CRED PRIV RESP LTDA</t>
+          <t>CAIXA BRASIL INFLAÇÃO ATIVA FIF RF CRED PRIV RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C147" s="4" t="inlineStr">
@@ -8780,7 +8780,7 @@
       </c>
       <c r="B148" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF BRASIL RENDA FIXA ATIVA LP RESP LTDA</t>
+          <t>CAIXA FIC FIF BRASIL RENDA FIXA ATIVA LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C148" s="2" t="inlineStr">
@@ -8837,7 +8837,7 @@
       </c>
       <c r="B149" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FI BRASIL IRF-M 1 TP RF</t>
+          <t>CAIXA FI BRASIL IRF-M 1 TP RF (8)</t>
         </is>
       </c>
       <c r="C149" s="4" t="inlineStr">
@@ -8894,7 +8894,7 @@
       </c>
       <c r="B150" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIF BRASIL IDKA IPCA 2A TIT PUB RF LP RESP LTDA</t>
+          <t>CAIXA FIF BRASIL IDKA IPCA 2A TIT PUB RF LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C150" s="2" t="inlineStr">
@@ -8951,7 +8951,7 @@
       </c>
       <c r="B151" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIF BRASIL IRF-M TP RF LP - RESP LTDA</t>
+          <t>CAIXA FIF BRASIL IRF-M TP RF LP - RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C151" s="4" t="inlineStr">
@@ -9008,7 +9008,7 @@
       </c>
       <c r="B152" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FI BRASIL IMA-B TP RF LP</t>
+          <t>CAIXA FI BRASIL IMA-B TP RF LP (8)</t>
         </is>
       </c>
       <c r="C152" s="2" t="inlineStr">
@@ -9065,7 +9065,7 @@
       </c>
       <c r="B153" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIF BRASIL IMA-B 5 TP RF LP - RESP LTDA</t>
+          <t>CAIXA FIF BRASIL IMA-B 5 TP RF LP - RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C153" s="4" t="inlineStr">
@@ -9122,7 +9122,7 @@
       </c>
       <c r="B154" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIF BRASIL IMA GERAL TP RF LP - RESP LTDA</t>
+          <t>CAIXA FIF BRASIL IMA GERAL TP RF LP - RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C154" s="2" t="inlineStr">
@@ -9179,7 +9179,7 @@
       </c>
       <c r="B155" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIF RS TITULOS PUBLICOS RF LP - RESP LTDA</t>
+          <t>CAIXA FIF RS TITULOS PUBLICOS RF LP - RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C155" s="4" t="inlineStr">
@@ -9236,7 +9236,7 @@
       </c>
       <c r="B156" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIF BRASIL IMA-B 5+ TP RF LP - RESP LTDA</t>
+          <t>CAIXA FIF BRASIL IMA-B 5+ TP RF LP - RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C156" s="2" t="inlineStr">
@@ -9293,7 +9293,7 @@
       </c>
       <c r="B157" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FI BRASIL IRF-M 1+ TP RF LP</t>
+          <t>CAIXA FI BRASIL IRF-M 1+ TP RF LP (8)</t>
         </is>
       </c>
       <c r="C157" s="4" t="inlineStr">
@@ -9350,7 +9350,7 @@
       </c>
       <c r="B158" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIF BRASIL TITULOS PUBLICOS RF LP - RESP LTDA</t>
+          <t>CAIXA FIF BRASIL TITULOS PUBLICOS RF LP - RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C158" s="2" t="inlineStr">
@@ -9407,7 +9407,7 @@
       </c>
       <c r="B159" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIF ALIANÇA TP RF CURTO PRAZO - RESP LTDA</t>
+          <t>CAIXA FIF ALIANÇA TP RF CURTO PRAZO - RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C159" s="4" t="inlineStr">
@@ -9464,7 +9464,7 @@
       </c>
       <c r="B160" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF BRASIL IDKA PRE 2A RF LP RESP LTDA</t>
+          <t>CAIXA FIC FIF BRASIL IDKA PRE 2A RF LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C160" s="2" t="inlineStr">
@@ -9521,7 +9521,7 @@
       </c>
       <c r="B161" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF BRASIL DISPONIBILIDADES SIMPLES RF RESP LTDA</t>
+          <t>CAIXA FIC FIF BRASIL DISPONIBILIDADES SIMPLES RF RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C161" s="4" t="inlineStr">
@@ -9578,7 +9578,7 @@
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF BRASIL RF REFER DI LONGO PRAZO RESP LTDA</t>
+          <t>CAIXA FIC FIF BRASIL RF REFER DI LONGO PRAZO RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C162" s="2" t="inlineStr">
@@ -9635,7 +9635,7 @@
       </c>
       <c r="B163" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF NOVO BRASIL RF IMA-B LP RESP LTDA</t>
+          <t>CAIXA FIC FIF NOVO BRASIL RF IMA-B LP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C163" s="4" t="inlineStr">
@@ -9749,7 +9749,7 @@
       </c>
       <c r="B165" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIF AÇOES BRASIL IBOVESPA RESP LTDA</t>
+          <t>CAIXA FIF AÇOES BRASIL IBOVESPA RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C165" s="4" t="inlineStr">
@@ -9806,7 +9806,7 @@
       </c>
       <c r="B166" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIF AÇÕES BRASIL ETF IBOVESPA RESP LTDA</t>
+          <t>CAIXA FIF AÇÕES BRASIL ETF IBOVESPA RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C166" s="2" t="inlineStr">
@@ -9863,7 +9863,7 @@
       </c>
       <c r="B167" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIF AÇÕES INSTITUCIONAL BDR NIVEL I RESP LTDA</t>
+          <t>CAIXA FIF AÇÕES INSTITUCIONAL BDR NIVEL I RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C167" s="4" t="inlineStr">
@@ -9920,7 +9920,7 @@
       </c>
       <c r="B168" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIF ACOES BRASIL IBX-50 RESP LTDA</t>
+          <t>CAIXA FIF ACOES BRASIL IBX-50 RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C168" s="2" t="inlineStr">
@@ -9977,7 +9977,7 @@
       </c>
       <c r="B169" s="4" t="inlineStr">
         <is>
-          <t>CAIXA ATENA FIC FIF AÇÕES BRASIL LIVRE QUANT RESP LTDA</t>
+          <t>CAIXA ATENA FIC FIF AÇÕES BRASIL LIVRE QUANT RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C169" s="4" t="inlineStr">
@@ -10030,7 +10030,7 @@
       </c>
       <c r="B170" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC ACOES EXPERT VINCI VALOR DIVIDENDOS RPPS RESP LTDA</t>
+          <t>CAIXA FIC ACOES EXPERT VINCI VALOR DIVIDENDOS RPPS RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C170" s="2" t="inlineStr">
@@ -10087,7 +10087,7 @@
       </c>
       <c r="B171" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC ACOES EXPERT VINCI VALOR RPPS RESP LTDA</t>
+          <t>CAIXA FIC ACOES EXPERT VINCI VALOR RPPS RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C171" s="4" t="inlineStr">
@@ -10144,7 +10144,7 @@
       </c>
       <c r="B172" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIF EXTRAMERCADO COMUM IRFM-1 RF RESP LTDA</t>
+          <t>CAIXA FIF EXTRAMERCADO COMUM IRFM-1 RF RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C172" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Dados atualizados via Robô: 19/05/2026 04:16
</commit_message>
<xml_diff>
--- a/dados_atuais.xlsx
+++ b/dados_atuais.xlsx
@@ -1944,11 +1944,7 @@
           <t>PF | PJ | TODOS</t>
         </is>
       </c>
-      <c r="K23" s="4" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-investidor-rf-longo-prazo</t>
-        </is>
-      </c>
+      <c r="K23" s="4" t="inlineStr"/>
       <c r="L23" s="4" t="inlineStr"/>
       <c r="M23" s="4" t="inlineStr"/>
       <c r="N23" s="4" t="inlineStr"/>
@@ -1964,7 +1960,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>CAIXA EXPERT ARX IPCA DEB INCENTIVADAS FIC FIF RF CRED PRIV - RESP LTDA (1) (2)</t>
+          <t>CAIXA EXPERT ARX IPCA DEB INCENTIVADAS FIC FIF RF CRED PRIV - RESP LTDA</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -2027,7 +2023,7 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIF FIC EXPERT SULAMERICA RF CRED PRIV LP - RESP LTDA (1)</t>
+          <t>CAIXA FIF FIC EXPERT SULAMERICA RF CRED PRIV LP - RESP LTDA</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
@@ -2216,7 +2212,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>CAIXA EXPERT VOX DESENV SUSTENTAVEL IS RF CRED PRIV LP - RESP LTDA (1) (2)</t>
+          <t>CAIXA EXPERT VOX DESENV SUSTENTAVEL IS RF CRED PRIV LP - RESP LTDA</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -2275,7 +2271,7 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>CAIXA EXPERT ABSOLUTE CRETA FIC FIF RF CRED PRIV LP - RESP LTDA (1)</t>
+          <t>CAIXA EXPERT ABSOLUTE CRETA FIC FIF RF CRED PRIV LP - RESP LTDA</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
@@ -2334,7 +2330,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>CAIXA EXPERT RB ASSET CDI DEB INCENTIVADAS FIC FIF RF CRED PRIV RESP LTDA (1) (2)</t>
+          <t>CAIXA EXPERT RB ASSET CDI DEB INCENTIVADAS FIC FIF RF CRED PRIV RESP LTDA</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -2397,7 +2393,7 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>CAIXA EXPERT VINLAND DEB IN INFRA RF CRED PRIV LP RESP LTDA (1) (2) (3)</t>
+          <t>CAIXA EXPERT VINLAND DEB IN INFRA RF CRED PRIV LP RESP LTDA</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
@@ -3275,7 +3271,7 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>CAIXA SIGMA FUNCIONARIOS FIC FIF RF REF DI LP - RESP LTDA (2) (3)</t>
+          <t>CAIXA SIGMA FUNCIONARIOS FIC FIF RF REF DI LP - RESP LTDA</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
@@ -3901,7 +3897,7 @@
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF FOF SMART CRED PRIV MM LP RESP LTDA (1)</t>
+          <t>CAIXA FIC FIF FOF SMART CRED PRIV MM LP RESP LTDA</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
@@ -3964,7 +3960,7 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC MULTIGESTOR GLOBAL EQUITIES IE (1)</t>
+          <t>CAIXA FIC MULTIGESTOR GLOBAL EQUITIES IE</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -4090,7 +4086,7 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF ESTRATÉGIA LIVRE MULTIMERCADO LP RESP LTDA (1)</t>
+          <t>CAIXA FIC FIF ESTRATÉGIA LIVRE MULTIMERCADO LP RESP LTDA</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -4216,7 +4212,7 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>CAIXA CARTEIRA QUANT DUO FIC FIF MM LP RESP LTDA (1) (2) (3)</t>
+          <t>CAIXA CARTEIRA QUANT DUO FIC FIF MM LP RESP LTDA</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -4275,7 +4271,7 @@
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF FOF SMART LONG SHORT LP RESP LTDA (1)</t>
+          <t>CAIXA FIC FIF FOF SMART LONG SHORT LP RESP LTDA</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
@@ -4401,7 +4397,7 @@
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>CAIXA CARTEIRA QUANT QUALI FIC FIF MM LP RESP LTDA (1) (2) (3)</t>
+          <t>CAIXA CARTEIRA QUANT QUALI FIC FIF MM LP RESP LTDA</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
@@ -4460,7 +4456,7 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF FOF SMART LONG BIAS MM RESP LTDA (1)</t>
+          <t>CAIXA FIC FIF FOF SMART LONG BIAS MM RESP LTDA</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -4523,7 +4519,7 @@
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>CAIXA CARTEIRA QUANT UNO FIC FIF MM LP RESP LTDA (1) (2) (3)</t>
+          <t>CAIXA CARTEIRA QUANT UNO FIC FIF MM LP RESP LTDA</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
@@ -4645,7 +4641,7 @@
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF ESTRATÉGICO MULTIMERCADO LP RESP LTDA (1)</t>
+          <t>CAIXA FIC FIF ESTRATÉGICO MULTIMERCADO LP RESP LTDA</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
@@ -4771,7 +4767,7 @@
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF FOF SMART MULTIESTRATEGIA MM RESP LTDA (1)</t>
+          <t>CAIXA FIC FIF FOF SMART MULTIESTRATEGIA MM RESP LTDA</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
@@ -5023,7 +5019,7 @@
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF FUNCIONARIOS ESTRATEGIA LIVRE MULTIMERCADO LP RESP LTDA (1)</t>
+          <t>CAIXA FIC FIF FUNCIONARIOS ESTRATEGIA LIVRE MULTIMERCADO LP RESP LTDA</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
@@ -5082,7 +5078,7 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>CAIXA HASHDEX NASDAQ CRYPTO INDEX FIC FIF MM RESP LTDA (1) (2)</t>
+          <t>CAIXA HASHDEX NASDAQ CRYPTO INDEX FIC FIF MM RESP LTDA</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
@@ -5141,7 +5137,7 @@
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF CAPITAL PROTEGIDO CESTA AGRO MM (1)</t>
+          <t>CAIXA FIC FIF CAPITAL PROTEGIDO CESTA AGRO MM</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
@@ -5204,7 +5200,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>CAIXA CAPITAL PROTEGIDO CÍCLICO III FIC FIF MM LP - RESP LTDA (1)</t>
+          <t>CAIXA CAPITAL PROTEGIDO CÍCLICO III FIC FIF MM LP - RESP LTDA</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -5267,7 +5263,7 @@
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>CAIXA CAPITAL PROTEGIDO IBOVESPA CÍCLICO I FIC FIF MM (1)</t>
+          <t>CAIXA CAPITAL PROTEGIDO IBOVESPA CÍCLICO I FIC FIF MM</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
@@ -5330,7 +5326,7 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIM CAPITAL PROTEGIDO CICLICO II LP - RL (1)</t>
+          <t>CAIXA FIC FIM CAPITAL PROTEGIDO CICLICO II LP - RL</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
@@ -5393,7 +5389,7 @@
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF EXPERT PIMCO INCOME IE MM LP RESP LTDA (1)</t>
+          <t>CAIXA FIC FIF EXPERT PIMCO INCOME IE MM LP RESP LTDA</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
@@ -5456,7 +5452,7 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>CAIXA EXPERT GIANT ZARATHUSTRA FIC MULTIMERCADO - RESP LTDA (1)</t>
+          <t>CAIXA EXPERT GIANT ZARATHUSTRA FIC MULTIMERCADO - RESP LTDA</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
@@ -5645,7 +5641,7 @@
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>FIC FIF CAIXA EXPERT BTG PACTUAL X10 MM LP RESP LTDA (1)</t>
+          <t>FIC FIF CAIXA EXPERT BTG PACTUAL X10 MM LP RESP LTDA</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
@@ -5708,7 +5704,7 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF EXPERT SPX NIMITZ MULTIMERCADO RESP LTDA (1)</t>
+          <t>CAIXA FIC FIF EXPERT SPX NIMITZ MULTIMERCADO RESP LTDA</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
@@ -6397,7 +6393,7 @@
       </c>
       <c r="B95" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF AÇÕES MULTIGESTOR RESP LTDA (1)</t>
+          <t>CAIXA FIC FIF AÇÕES MULTIGESTOR RESP LTDA</t>
         </is>
       </c>
       <c r="C95" s="4" t="inlineStr">
@@ -7381,11 +7377,7 @@
           <t>PF | PJ | RPPS</t>
         </is>
       </c>
-      <c r="K110" s="2" t="inlineStr">
-        <is>
-          <t>http://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/FIA-Institucional-BDR-nivel-I/Paginas/default.aspx</t>
-        </is>
-      </c>
+      <c r="K110" s="2" t="inlineStr"/>
       <c r="L110" s="2" t="inlineStr"/>
       <c r="M110" s="2" t="inlineStr"/>
       <c r="N110" s="2" t="inlineStr"/>
@@ -7527,7 +7519,7 @@
       </c>
       <c r="B113" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC ACOES EXPERT VERDE AM LONG BIAS - RESP LTDA (1)</t>
+          <t>CAIXA FIC ACOES EXPERT VERDE AM LONG BIAS - RESP LTDA</t>
         </is>
       </c>
       <c r="C113" s="4" t="inlineStr">
@@ -7590,7 +7582,7 @@
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>CAIXA EXPERT CLARITAS VALOR FIC FIF AÇÕES - RESP LTDA (1)</t>
+          <t>CAIXA EXPERT CLARITAS VALOR FIC FIF AÇÕES - RESP LTDA</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
@@ -8247,7 +8239,7 @@
       </c>
       <c r="B125" s="4" t="inlineStr">
         <is>
-          <t>CAIXA AZULZINHA FIC FIF RF SIMPLES - RESP LTDA (2)</t>
+          <t>CAIXA AZULZINHA FIC FIF RF SIMPLES - RESP LTDA</t>
         </is>
       </c>
       <c r="C125" s="4" t="inlineStr">
@@ -10704,7 +10696,7 @@
       </c>
       <c r="B164" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF BRASIL ESTRATÉGIA LIVRE MM LP RESP LTDA (1)</t>
+          <t>CAIXA FIC FIF BRASIL ESTRATÉGIA LIVRE MM LP RESP LTDA</t>
         </is>
       </c>
       <c r="C164" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Dados atualizados via Robô: 19/05/2026 04:55
</commit_message>
<xml_diff>
--- a/dados_atuais.xlsx
+++ b/dados_atuais.xlsx
@@ -479,8 +479,8 @@
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="30" customWidth="1" min="10" max="10"/>
     <col width="60" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="22" customWidth="1" min="15" max="15"/>
     <col width="18" customWidth="1" min="16" max="16"/>
@@ -882,12 +882,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-relacionamento-personal-rf-longo-prazo</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr"/>
-      <c r="M6" s="2" t="inlineStr"/>
-      <c r="N6" s="2" t="inlineStr"/>
-      <c r="O6" s="2" t="inlineStr"/>
-      <c r="P6" s="2" t="inlineStr"/>
-      <c r="Q6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>10.577.509/0001-55</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>0.7</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -1071,12 +1095,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/e-fundos/renda-fixa-longo-prazo</t>
         </is>
       </c>
-      <c r="L9" s="4" t="inlineStr"/>
-      <c r="M9" s="4" t="inlineStr"/>
-      <c r="N9" s="4" t="inlineStr"/>
-      <c r="O9" s="4" t="inlineStr"/>
-      <c r="P9" s="4" t="inlineStr"/>
-      <c r="Q9" s="4" t="inlineStr"/>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>15.154.422/0001-99</t>
+        </is>
+      </c>
+      <c r="M9" s="4" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N9" s="4" t="inlineStr">
+        <is>
+          <t>0.7</t>
+        </is>
+      </c>
+      <c r="O9" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P9" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q9" s="4" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1319,12 +1367,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-empreender-rf-longo-prazo/</t>
         </is>
       </c>
-      <c r="L13" s="4" t="inlineStr"/>
-      <c r="M13" s="4" t="inlineStr"/>
-      <c r="N13" s="4" t="inlineStr"/>
-      <c r="O13" s="4" t="inlineStr"/>
-      <c r="P13" s="4" t="inlineStr"/>
-      <c r="Q13" s="4" t="inlineStr"/>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>00.068.305/0001-35</t>
+        </is>
+      </c>
+      <c r="M13" s="4" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N13" s="4" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="O13" s="4" t="inlineStr">
+        <is>
+          <t>50.0</t>
+        </is>
+      </c>
+      <c r="P13" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q13" s="4" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1571,12 +1643,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-desenvolver-rf-longo-prazo/</t>
         </is>
       </c>
-      <c r="L17" s="4" t="inlineStr"/>
-      <c r="M17" s="4" t="inlineStr"/>
-      <c r="N17" s="4" t="inlineStr"/>
-      <c r="O17" s="4" t="inlineStr"/>
-      <c r="P17" s="4" t="inlineStr"/>
-      <c r="Q17" s="4" t="inlineStr"/>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>16.877.609/0001-83</t>
+        </is>
+      </c>
+      <c r="M17" s="4" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N17" s="4" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="O17" s="4" t="inlineStr">
+        <is>
+          <t>500.0</t>
+        </is>
+      </c>
+      <c r="P17" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q17" s="4" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1634,12 +1730,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-objetivo-pre-rf-longo-prazo/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L18" s="2" t="inlineStr"/>
-      <c r="M18" s="2" t="inlineStr"/>
-      <c r="N18" s="2" t="inlineStr"/>
-      <c r="O18" s="2" t="inlineStr"/>
-      <c r="P18" s="2" t="inlineStr"/>
-      <c r="Q18" s="2" t="inlineStr"/>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>14.120.511/0001-51</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>0.7</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q18" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -1886,12 +2006,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-performance-ima-b-renda-fixa-longo-prazo/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L22" s="2" t="inlineStr"/>
-      <c r="M22" s="2" t="inlineStr"/>
-      <c r="N22" s="2" t="inlineStr"/>
-      <c r="O22" s="2" t="inlineStr"/>
-      <c r="P22" s="2" t="inlineStr"/>
-      <c r="Q22" s="2" t="inlineStr"/>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>10.577.516/0001-57</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q22" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -2500,12 +2644,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/caixa-fic-plus-qualificado-rf-credito-privado-lp/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L32" s="2" t="inlineStr"/>
-      <c r="M32" s="2" t="inlineStr"/>
-      <c r="N32" s="2" t="inlineStr"/>
-      <c r="O32" s="2" t="inlineStr"/>
-      <c r="P32" s="2" t="inlineStr"/>
-      <c r="Q32" s="2" t="inlineStr"/>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>10.551.353/0001-33</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>20000.0</t>
+        </is>
+      </c>
+      <c r="P32" s="2" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q32" s="2" t="inlineStr">
+        <is>
+          <t>D+04 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -2563,12 +2731,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-expertise-rf-credito-privado-longo-prazo</t>
         </is>
       </c>
-      <c r="L33" s="4" t="inlineStr"/>
-      <c r="M33" s="4" t="inlineStr"/>
-      <c r="N33" s="4" t="inlineStr"/>
-      <c r="O33" s="4" t="inlineStr"/>
-      <c r="P33" s="4" t="inlineStr"/>
-      <c r="Q33" s="4" t="inlineStr"/>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t>10.646.888/0001-98</t>
+        </is>
+      </c>
+      <c r="M33" s="4" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N33" s="4" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="O33" s="4" t="inlineStr">
+        <is>
+          <t>20000.0</t>
+        </is>
+      </c>
+      <c r="P33" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q33" s="4" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2626,12 +2818,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-selecao-rf-longo-prazo</t>
         </is>
       </c>
-      <c r="L34" s="2" t="inlineStr"/>
-      <c r="M34" s="2" t="inlineStr"/>
-      <c r="N34" s="2" t="inlineStr"/>
-      <c r="O34" s="2" t="inlineStr"/>
-      <c r="P34" s="2" t="inlineStr"/>
-      <c r="Q34" s="2" t="inlineStr"/>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>03.737.207/0001-31</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="O34" s="2" t="inlineStr">
+        <is>
+          <t>30000.0</t>
+        </is>
+      </c>
+      <c r="P34" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q34" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -2815,12 +3031,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/voce/renda-fixa/pos-fixados/ate-100.000/caixa-fic-indexa-tesouro-selic-renda-fixa-lp</t>
         </is>
       </c>
-      <c r="L37" s="4" t="inlineStr"/>
-      <c r="M37" s="4" t="inlineStr"/>
-      <c r="N37" s="4" t="inlineStr"/>
-      <c r="O37" s="4" t="inlineStr"/>
-      <c r="P37" s="4" t="inlineStr"/>
-      <c r="Q37" s="4" t="inlineStr"/>
+      <c r="L37" s="4" t="inlineStr">
+        <is>
+          <t>17.687.735/0001-38</t>
+        </is>
+      </c>
+      <c r="M37" s="4" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="N37" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="O37" s="4" t="inlineStr">
+        <is>
+          <t>50000.0</t>
+        </is>
+      </c>
+      <c r="P37" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q37" s="4" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -3130,12 +3370,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-maxi-rf-credito-privado-longo-prazo/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L42" s="2" t="inlineStr"/>
-      <c r="M42" s="2" t="inlineStr"/>
-      <c r="N42" s="2" t="inlineStr"/>
-      <c r="O42" s="2" t="inlineStr"/>
-      <c r="P42" s="2" t="inlineStr"/>
-      <c r="Q42" s="2" t="inlineStr"/>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>17.322.725/0001-07</t>
+        </is>
+      </c>
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="O42" s="2" t="inlineStr">
+        <is>
+          <t>50000.0</t>
+        </is>
+      </c>
+      <c r="P42" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q42" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
@@ -3441,12 +3705,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/referenciados/fic-pleno-ref-di-longo-prazo</t>
         </is>
       </c>
-      <c r="L47" s="4" t="inlineStr"/>
-      <c r="M47" s="4" t="inlineStr"/>
-      <c r="N47" s="4" t="inlineStr"/>
-      <c r="O47" s="4" t="inlineStr"/>
-      <c r="P47" s="4" t="inlineStr"/>
-      <c r="Q47" s="4" t="inlineStr"/>
+      <c r="L47" s="4" t="inlineStr">
+        <is>
+          <t>10.740.508/0001-80</t>
+        </is>
+      </c>
+      <c r="M47" s="4" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="N47" s="4" t="inlineStr">
+        <is>
+          <t>0.7</t>
+        </is>
+      </c>
+      <c r="O47" s="4" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="P47" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q47" s="4" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3567,12 +3855,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/referenciados/fic-preferencial-ref-di-longo-prazo</t>
         </is>
       </c>
-      <c r="L49" s="4" t="inlineStr"/>
-      <c r="M49" s="4" t="inlineStr"/>
-      <c r="N49" s="4" t="inlineStr"/>
-      <c r="O49" s="4" t="inlineStr"/>
-      <c r="P49" s="4" t="inlineStr"/>
-      <c r="Q49" s="4" t="inlineStr"/>
+      <c r="L49" s="4" t="inlineStr">
+        <is>
+          <t>03.737.211/0001-08</t>
+        </is>
+      </c>
+      <c r="M49" s="4" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="N49" s="4" t="inlineStr">
+        <is>
+          <t>0.6</t>
+        </is>
+      </c>
+      <c r="O49" s="4" t="inlineStr">
+        <is>
+          <t>30000.0</t>
+        </is>
+      </c>
+      <c r="P49" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q49" s="4" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3882,12 +4194,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/curto-prazo/fic-automatico-polis-rf-cp/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L54" s="2" t="inlineStr"/>
-      <c r="M54" s="2" t="inlineStr"/>
-      <c r="N54" s="2" t="inlineStr"/>
-      <c r="O54" s="2" t="inlineStr"/>
-      <c r="P54" s="2" t="inlineStr"/>
-      <c r="Q54" s="2" t="inlineStr"/>
+      <c r="L54" s="2" t="inlineStr">
+        <is>
+          <t>39.594.941/0001-36</t>
+        </is>
+      </c>
+      <c r="M54" s="2" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="N54" s="2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="O54" s="2" t="inlineStr">
+        <is>
+          <t>10000.0</t>
+        </is>
+      </c>
+      <c r="P54" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q54" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
@@ -4197,12 +4533,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/multimercado/caixa-fi-indexa-short-dolar-mult-lp/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L59" s="4" t="inlineStr"/>
-      <c r="M59" s="4" t="inlineStr"/>
-      <c r="N59" s="4" t="inlineStr"/>
-      <c r="O59" s="4" t="inlineStr"/>
-      <c r="P59" s="4" t="inlineStr"/>
-      <c r="Q59" s="4" t="inlineStr"/>
+      <c r="L59" s="4" t="inlineStr">
+        <is>
+          <t>29.157.511/0001-01</t>
+        </is>
+      </c>
+      <c r="M59" s="4" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N59" s="4" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="O59" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P59" s="4" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q59" s="4" t="inlineStr">
+        <is>
+          <t>D+01 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -4752,12 +5112,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fi-ouro-multimercado-longo-prazo</t>
         </is>
       </c>
-      <c r="L68" s="2" t="inlineStr"/>
-      <c r="M68" s="2" t="inlineStr"/>
-      <c r="N68" s="2" t="inlineStr"/>
-      <c r="O68" s="2" t="inlineStr"/>
-      <c r="P68" s="2" t="inlineStr"/>
-      <c r="Q68" s="2" t="inlineStr"/>
+      <c r="L68" s="2" t="inlineStr">
+        <is>
+          <t>16.916.060/0001-99</t>
+        </is>
+      </c>
+      <c r="M68" s="2" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N68" s="2" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="O68" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P68" s="2" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q68" s="2" t="inlineStr">
+        <is>
+          <t>D+02 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
@@ -4878,12 +5262,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/multimercado/caixa-fic-hedge-multimercado-lp/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L70" s="2" t="inlineStr"/>
-      <c r="M70" s="2" t="inlineStr"/>
-      <c r="N70" s="2" t="inlineStr"/>
-      <c r="O70" s="2" t="inlineStr"/>
-      <c r="P70" s="2" t="inlineStr"/>
-      <c r="Q70" s="2" t="inlineStr"/>
+      <c r="L70" s="2" t="inlineStr">
+        <is>
+          <t>30.068.135/0001-50</t>
+        </is>
+      </c>
+      <c r="M70" s="2" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N70" s="2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="O70" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P70" s="2" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q70" s="2" t="inlineStr">
+        <is>
+          <t>D+01 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
@@ -5626,12 +6034,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fi-juros-moedas-multimercado-longo-prazo</t>
         </is>
       </c>
-      <c r="L82" s="2" t="inlineStr"/>
-      <c r="M82" s="2" t="inlineStr"/>
-      <c r="N82" s="2" t="inlineStr"/>
-      <c r="O82" s="2" t="inlineStr"/>
-      <c r="P82" s="2" t="inlineStr"/>
-      <c r="Q82" s="2" t="inlineStr"/>
+      <c r="L82" s="2" t="inlineStr">
+        <is>
+          <t>14.120.520/0001-42</t>
+        </is>
+      </c>
+      <c r="M82" s="2" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N82" s="2" t="inlineStr">
+        <is>
+          <t>0.7</t>
+        </is>
+      </c>
+      <c r="O82" s="2" t="inlineStr">
+        <is>
+          <t>10000.0</t>
+        </is>
+      </c>
+      <c r="P82" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q82" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
@@ -5815,12 +6247,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/cambiais/fic-cambial-dolar/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L85" s="4" t="inlineStr"/>
-      <c r="M85" s="4" t="inlineStr"/>
-      <c r="N85" s="4" t="inlineStr"/>
-      <c r="O85" s="4" t="inlineStr"/>
-      <c r="P85" s="4" t="inlineStr"/>
-      <c r="Q85" s="4" t="inlineStr"/>
+      <c r="L85" s="4" t="inlineStr">
+        <is>
+          <t>05.114.733/0001-70</t>
+        </is>
+      </c>
+      <c r="M85" s="4" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N85" s="4" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="O85" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P85" s="4" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q85" s="4" t="inlineStr">
+        <is>
+          <t>D+01 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -5878,12 +6334,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/fi-acoes-dividendos</t>
         </is>
       </c>
-      <c r="L86" s="2" t="inlineStr"/>
-      <c r="M86" s="2" t="inlineStr"/>
-      <c r="N86" s="2" t="inlineStr"/>
-      <c r="O86" s="2" t="inlineStr"/>
-      <c r="P86" s="2" t="inlineStr"/>
-      <c r="Q86" s="2" t="inlineStr"/>
+      <c r="L86" s="2" t="inlineStr">
+        <is>
+          <t>05.900.798/0001-41</t>
+        </is>
+      </c>
+      <c r="M86" s="2" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N86" s="2" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="O86" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P86" s="2" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q86" s="2" t="inlineStr">
+        <is>
+          <t>D+03 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
@@ -6063,12 +6543,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/fi-acoes-bdr-nivel-1</t>
         </is>
       </c>
-      <c r="L89" s="4" t="inlineStr"/>
-      <c r="M89" s="4" t="inlineStr"/>
-      <c r="N89" s="4" t="inlineStr"/>
-      <c r="O89" s="4" t="inlineStr"/>
-      <c r="P89" s="4" t="inlineStr"/>
-      <c r="Q89" s="4" t="inlineStr"/>
+      <c r="L89" s="4" t="inlineStr">
+        <is>
+          <t>17.503.172/0001-80</t>
+        </is>
+      </c>
+      <c r="M89" s="4" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N89" s="4" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="O89" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P89" s="4" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q89" s="4" t="inlineStr">
+        <is>
+          <t>D+03 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -6126,12 +6630,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/fi-acoes-small-caps-ativo</t>
         </is>
       </c>
-      <c r="L90" s="2" t="inlineStr"/>
-      <c r="M90" s="2" t="inlineStr"/>
-      <c r="N90" s="2" t="inlineStr"/>
-      <c r="O90" s="2" t="inlineStr"/>
-      <c r="P90" s="2" t="inlineStr"/>
-      <c r="Q90" s="2" t="inlineStr"/>
+      <c r="L90" s="2" t="inlineStr">
+        <is>
+          <t>15.154.220/0001-47</t>
+        </is>
+      </c>
+      <c r="M90" s="2" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N90" s="2" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="O90" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P90" s="2" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q90" s="2" t="inlineStr">
+        <is>
+          <t>D+03 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
@@ -6189,12 +6717,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/fi-acoes-consumo</t>
         </is>
       </c>
-      <c r="L91" s="4" t="inlineStr"/>
-      <c r="M91" s="4" t="inlineStr"/>
-      <c r="N91" s="4" t="inlineStr"/>
-      <c r="O91" s="4" t="inlineStr"/>
-      <c r="P91" s="4" t="inlineStr"/>
-      <c r="Q91" s="4" t="inlineStr"/>
+      <c r="L91" s="4" t="inlineStr">
+        <is>
+          <t>10.577.512/0001-79</t>
+        </is>
+      </c>
+      <c r="M91" s="4" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N91" s="4" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+      <c r="O91" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P91" s="4" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q91" s="4" t="inlineStr">
+        <is>
+          <t>D+03 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -6252,12 +6804,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/fi-acoes-ise</t>
         </is>
       </c>
-      <c r="L92" s="2" t="inlineStr"/>
-      <c r="M92" s="2" t="inlineStr"/>
-      <c r="N92" s="2" t="inlineStr"/>
-      <c r="O92" s="2" t="inlineStr"/>
-      <c r="P92" s="2" t="inlineStr"/>
-      <c r="Q92" s="2" t="inlineStr"/>
+      <c r="L92" s="2" t="inlineStr">
+        <is>
+          <t>08.070.838/0001-63</t>
+        </is>
+      </c>
+      <c r="M92" s="2" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N92" s="2" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="O92" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P92" s="2" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q92" s="2" t="inlineStr">
+        <is>
+          <t>D+03 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
@@ -6315,12 +6891,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/fia-caixa-petrobras-plus/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L93" s="4" t="inlineStr"/>
-      <c r="M93" s="4" t="inlineStr"/>
-      <c r="N93" s="4" t="inlineStr"/>
-      <c r="O93" s="4" t="inlineStr"/>
-      <c r="P93" s="4" t="inlineStr"/>
-      <c r="Q93" s="4" t="inlineStr"/>
+      <c r="L93" s="4" t="inlineStr">
+        <is>
+          <t>30.068.205/0001-70</t>
+        </is>
+      </c>
+      <c r="M93" s="4" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N93" s="4" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="O93" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P93" s="4" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q93" s="4" t="inlineStr">
+        <is>
+          <t>D+03 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -6378,12 +6978,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/fi-acoes-ibovespa</t>
         </is>
       </c>
-      <c r="L94" s="2" t="inlineStr"/>
-      <c r="M94" s="2" t="inlineStr"/>
-      <c r="N94" s="2" t="inlineStr"/>
-      <c r="O94" s="2" t="inlineStr"/>
-      <c r="P94" s="2" t="inlineStr"/>
-      <c r="Q94" s="2" t="inlineStr"/>
+      <c r="L94" s="2" t="inlineStr">
+        <is>
+          <t>01.525.057/0001-77</t>
+        </is>
+      </c>
+      <c r="M94" s="2" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N94" s="2" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="O94" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P94" s="2" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q94" s="2" t="inlineStr">
+        <is>
+          <t>D+03 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
@@ -6504,12 +7128,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/fi-acoes-construcao-civil</t>
         </is>
       </c>
-      <c r="L96" s="2" t="inlineStr"/>
-      <c r="M96" s="2" t="inlineStr"/>
-      <c r="N96" s="2" t="inlineStr"/>
-      <c r="O96" s="2" t="inlineStr"/>
-      <c r="P96" s="2" t="inlineStr"/>
-      <c r="Q96" s="2" t="inlineStr"/>
+      <c r="L96" s="2" t="inlineStr">
+        <is>
+          <t>10.551.375/0001-01</t>
+        </is>
+      </c>
+      <c r="M96" s="2" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N96" s="2" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="O96" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P96" s="2" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q96" s="2" t="inlineStr">
+        <is>
+          <t>D+03 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
@@ -6567,12 +7215,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/fi-acoes-infraestrutura</t>
         </is>
       </c>
-      <c r="L97" s="4" t="inlineStr"/>
-      <c r="M97" s="4" t="inlineStr"/>
-      <c r="N97" s="4" t="inlineStr"/>
-      <c r="O97" s="4" t="inlineStr"/>
-      <c r="P97" s="4" t="inlineStr"/>
-      <c r="Q97" s="4" t="inlineStr"/>
+      <c r="L97" s="4" t="inlineStr">
+        <is>
+          <t>10.551.382/0001-03</t>
+        </is>
+      </c>
+      <c r="M97" s="4" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N97" s="4" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="O97" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P97" s="4" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q97" s="4" t="inlineStr">
+        <is>
+          <t>D+03 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -6625,13 +7297,41 @@
           <t>PF | PJ</t>
         </is>
       </c>
-      <c r="K98" s="2" t="inlineStr"/>
-      <c r="L98" s="2" t="inlineStr"/>
-      <c r="M98" s="2" t="inlineStr"/>
-      <c r="N98" s="2" t="inlineStr"/>
-      <c r="O98" s="2" t="inlineStr"/>
-      <c r="P98" s="2" t="inlineStr"/>
-      <c r="Q98" s="2" t="inlineStr"/>
+      <c r="K98" s="2" t="inlineStr">
+        <is>
+          <t>http://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/FIC-FIA-acoes-livres/Paginas/default.aspx</t>
+        </is>
+      </c>
+      <c r="L98" s="2" t="inlineStr">
+        <is>
+          <t>22.791.154/0001-81</t>
+        </is>
+      </c>
+      <c r="M98" s="2" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N98" s="2" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="O98" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P98" s="2" t="inlineStr">
+        <is>
+          <t>D+13 (du)</t>
+        </is>
+      </c>
+      <c r="Q98" s="2" t="inlineStr">
+        <is>
+          <t>D+15 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
@@ -6689,12 +7389,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/fi-acoes-petrobras-pre-sal</t>
         </is>
       </c>
-      <c r="L99" s="4" t="inlineStr"/>
-      <c r="M99" s="4" t="inlineStr"/>
-      <c r="N99" s="4" t="inlineStr"/>
-      <c r="O99" s="4" t="inlineStr"/>
-      <c r="P99" s="4" t="inlineStr"/>
-      <c r="Q99" s="4" t="inlineStr"/>
+      <c r="L99" s="4" t="inlineStr">
+        <is>
+          <t>11.060.594/0001-42</t>
+        </is>
+      </c>
+      <c r="M99" s="4" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N99" s="4" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="O99" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P99" s="4" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q99" s="4" t="inlineStr">
+        <is>
+          <t>D+03 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -6752,12 +7476,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/Caixa-FI-Acoes-Banco-do-Brasil-Plus/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L100" s="2" t="inlineStr"/>
-      <c r="M100" s="2" t="inlineStr"/>
-      <c r="N100" s="2" t="inlineStr"/>
-      <c r="O100" s="2" t="inlineStr"/>
-      <c r="P100" s="2" t="inlineStr"/>
-      <c r="Q100" s="2" t="inlineStr"/>
+      <c r="L100" s="2" t="inlineStr">
+        <is>
+          <t>30.068.271/0001-40</t>
+        </is>
+      </c>
+      <c r="M100" s="2" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N100" s="2" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="O100" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P100" s="2" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q100" s="2" t="inlineStr">
+        <is>
+          <t>D+03 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
@@ -6815,12 +7563,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/fi-acoes-vale-rio-doce</t>
         </is>
       </c>
-      <c r="L101" s="4" t="inlineStr"/>
-      <c r="M101" s="4" t="inlineStr"/>
-      <c r="N101" s="4" t="inlineStr"/>
-      <c r="O101" s="4" t="inlineStr"/>
-      <c r="P101" s="4" t="inlineStr"/>
-      <c r="Q101" s="4" t="inlineStr"/>
+      <c r="L101" s="4" t="inlineStr">
+        <is>
+          <t>04.885.820/0001-69</t>
+        </is>
+      </c>
+      <c r="M101" s="4" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N101" s="4" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="O101" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P101" s="4" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q101" s="4" t="inlineStr">
+        <is>
+          <t>D+03 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -6941,12 +7713,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/fi-acoes-ibrx-ativo</t>
         </is>
       </c>
-      <c r="L103" s="4" t="inlineStr"/>
-      <c r="M103" s="4" t="inlineStr"/>
-      <c r="N103" s="4" t="inlineStr"/>
-      <c r="O103" s="4" t="inlineStr"/>
-      <c r="P103" s="4" t="inlineStr"/>
-      <c r="Q103" s="4" t="inlineStr"/>
+      <c r="L103" s="4" t="inlineStr">
+        <is>
+          <t>05.164.370/0001-88</t>
+        </is>
+      </c>
+      <c r="M103" s="4" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N103" s="4" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="O103" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P103" s="4" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q103" s="4" t="inlineStr">
+        <is>
+          <t>D+03 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -7004,12 +7800,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/caixa-fia-indexa-setor-financeiro/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L104" s="2" t="inlineStr"/>
-      <c r="M104" s="2" t="inlineStr"/>
-      <c r="N104" s="2" t="inlineStr"/>
-      <c r="O104" s="2" t="inlineStr"/>
-      <c r="P104" s="2" t="inlineStr"/>
-      <c r="Q104" s="2" t="inlineStr"/>
+      <c r="L104" s="2" t="inlineStr">
+        <is>
+          <t>40.209.029/0001-00</t>
+        </is>
+      </c>
+      <c r="M104" s="2" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N104" s="2" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="O104" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P104" s="2" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q104" s="2" t="inlineStr">
+        <is>
+          <t>D+03 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
@@ -7067,12 +7887,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/fic-fia-dividendos-quantitativo/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L105" s="4" t="inlineStr"/>
-      <c r="M105" s="4" t="inlineStr"/>
-      <c r="N105" s="4" t="inlineStr"/>
-      <c r="O105" s="4" t="inlineStr"/>
-      <c r="P105" s="4" t="inlineStr"/>
-      <c r="Q105" s="4" t="inlineStr"/>
+      <c r="L105" s="4" t="inlineStr">
+        <is>
+          <t>42.120.405/0001-03</t>
+        </is>
+      </c>
+      <c r="M105" s="4" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N105" s="4" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="O105" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P105" s="4" t="inlineStr">
+        <is>
+          <t>D+13 (du)</t>
+        </is>
+      </c>
+      <c r="Q105" s="4" t="inlineStr">
+        <is>
+          <t>D+15 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -7130,12 +7974,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/fi-acoes-pibb-sem-opcao-de-venda</t>
         </is>
       </c>
-      <c r="L106" s="2" t="inlineStr"/>
-      <c r="M106" s="2" t="inlineStr"/>
-      <c r="N106" s="2" t="inlineStr"/>
-      <c r="O106" s="2" t="inlineStr"/>
-      <c r="P106" s="2" t="inlineStr"/>
-      <c r="Q106" s="2" t="inlineStr"/>
+      <c r="L106" s="2" t="inlineStr">
+        <is>
+          <t>05.164.361/0001-97</t>
+        </is>
+      </c>
+      <c r="M106" s="2" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N106" s="2" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="O106" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P106" s="2" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q106" s="2" t="inlineStr">
+        <is>
+          <t>D+03 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="4" t="inlineStr">
@@ -7193,12 +8061,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/fi-acoes-ibovespa-ativo</t>
         </is>
       </c>
-      <c r="L107" s="4" t="inlineStr"/>
-      <c r="M107" s="4" t="inlineStr"/>
-      <c r="N107" s="4" t="inlineStr"/>
-      <c r="O107" s="4" t="inlineStr"/>
-      <c r="P107" s="4" t="inlineStr"/>
-      <c r="Q107" s="4" t="inlineStr"/>
+      <c r="L107" s="4" t="inlineStr">
+        <is>
+          <t>08.046.355/0001-23</t>
+        </is>
+      </c>
+      <c r="M107" s="4" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N107" s="4" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="O107" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P107" s="4" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q107" s="4" t="inlineStr">
+        <is>
+          <t>D+03 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -7256,12 +8148,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/fi-acoes-petrobras</t>
         </is>
       </c>
-      <c r="L108" s="2" t="inlineStr"/>
-      <c r="M108" s="2" t="inlineStr"/>
-      <c r="N108" s="2" t="inlineStr"/>
-      <c r="O108" s="2" t="inlineStr"/>
-      <c r="P108" s="2" t="inlineStr"/>
-      <c r="Q108" s="2" t="inlineStr"/>
+      <c r="L108" s="2" t="inlineStr">
+        <is>
+          <t>03.914.671/0001-56</t>
+        </is>
+      </c>
+      <c r="M108" s="2" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N108" s="2" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="O108" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P108" s="2" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q108" s="2" t="inlineStr">
+        <is>
+          <t>D+03 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="4" t="inlineStr">
@@ -7319,12 +8235,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/fia-caixa-indexa-iagro/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L109" s="4" t="inlineStr"/>
-      <c r="M109" s="4" t="inlineStr"/>
-      <c r="N109" s="4" t="inlineStr"/>
-      <c r="O109" s="4" t="inlineStr"/>
-      <c r="P109" s="4" t="inlineStr"/>
-      <c r="Q109" s="4" t="inlineStr"/>
+      <c r="L109" s="4" t="inlineStr">
+        <is>
+          <t>45.443.601/0001-07</t>
+        </is>
+      </c>
+      <c r="M109" s="4" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N109" s="4" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="O109" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P109" s="4" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q109" s="4" t="inlineStr">
+        <is>
+          <t>D+03 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -7377,13 +8317,41 @@
           <t>PF | PJ | RPPS</t>
         </is>
       </c>
-      <c r="K110" s="2" t="inlineStr"/>
-      <c r="L110" s="2" t="inlineStr"/>
-      <c r="M110" s="2" t="inlineStr"/>
-      <c r="N110" s="2" t="inlineStr"/>
-      <c r="O110" s="2" t="inlineStr"/>
-      <c r="P110" s="2" t="inlineStr"/>
-      <c r="Q110" s="2" t="inlineStr"/>
+      <c r="K110" s="2" t="inlineStr">
+        <is>
+          <t>http://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/FIA-Institucional-BDR-nivel-I/Paginas/default.aspx</t>
+        </is>
+      </c>
+      <c r="L110" s="2" t="inlineStr">
+        <is>
+          <t>43.760.251/0001-87</t>
+        </is>
+      </c>
+      <c r="M110" s="2" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N110" s="2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="O110" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P110" s="2" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q110" s="2" t="inlineStr">
+        <is>
+          <t>D+03 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="4" t="inlineStr">
@@ -7441,12 +8409,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/fia-caixa-seguridade/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L111" s="4" t="inlineStr"/>
-      <c r="M111" s="4" t="inlineStr"/>
-      <c r="N111" s="4" t="inlineStr"/>
-      <c r="O111" s="4" t="inlineStr"/>
-      <c r="P111" s="4" t="inlineStr"/>
-      <c r="Q111" s="4" t="inlineStr"/>
+      <c r="L111" s="4" t="inlineStr">
+        <is>
+          <t>59.815.671/0001-53</t>
+        </is>
+      </c>
+      <c r="M111" s="4" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N111" s="4" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="O111" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P111" s="4" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q111" s="4" t="inlineStr">
+        <is>
+          <t>D+03 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -7504,12 +8496,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/fia-caixa-eletrobras/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L112" s="2" t="inlineStr"/>
-      <c r="M112" s="2" t="inlineStr"/>
-      <c r="N112" s="2" t="inlineStr"/>
-      <c r="O112" s="2" t="inlineStr"/>
-      <c r="P112" s="2" t="inlineStr"/>
-      <c r="Q112" s="2" t="inlineStr"/>
+      <c r="L112" s="2" t="inlineStr">
+        <is>
+          <t>45.443.475/0001-90</t>
+        </is>
+      </c>
+      <c r="M112" s="2" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N112" s="2" t="inlineStr">
+        <is>
+          <t>0.45</t>
+        </is>
+      </c>
+      <c r="O112" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P112" s="2" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q112" s="2" t="inlineStr">
+        <is>
+          <t>D+03 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="4" t="inlineStr">
@@ -7810,13 +8826,41 @@
           <t>PF</t>
         </is>
       </c>
-      <c r="K117" s="4" t="inlineStr"/>
-      <c r="L117" s="4" t="inlineStr"/>
-      <c r="M117" s="4" t="inlineStr"/>
-      <c r="N117" s="4" t="inlineStr"/>
-      <c r="O117" s="4" t="inlineStr"/>
-      <c r="P117" s="4" t="inlineStr"/>
-      <c r="Q117" s="4" t="inlineStr"/>
+      <c r="K117" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/mutuos-privatizacao/fmp-fgts-eletrobras</t>
+        </is>
+      </c>
+      <c r="L117" s="4" t="inlineStr">
+        <is>
+          <t>45.160.183/0001-40</t>
+        </is>
+      </c>
+      <c r="M117" s="4" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N117" s="4" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="O117" s="4" t="inlineStr">
+        <is>
+          <t>200.0</t>
+        </is>
+      </c>
+      <c r="P117" s="4" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q117" s="4" t="inlineStr">
+        <is>
+          <t>D+05 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -7869,13 +8913,41 @@
           <t>PF</t>
         </is>
       </c>
-      <c r="K118" s="2" t="inlineStr"/>
-      <c r="L118" s="2" t="inlineStr"/>
-      <c r="M118" s="2" t="inlineStr"/>
-      <c r="N118" s="2" t="inlineStr"/>
-      <c r="O118" s="2" t="inlineStr"/>
-      <c r="P118" s="2" t="inlineStr"/>
-      <c r="Q118" s="2" t="inlineStr"/>
+      <c r="K118" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/mutuos-privatizacao/fmp-fgts-petrobas-4</t>
+        </is>
+      </c>
+      <c r="L118" s="2" t="inlineStr">
+        <is>
+          <t>03.555.959/0001-81</t>
+        </is>
+      </c>
+      <c r="M118" s="2" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N118" s="2" t="inlineStr">
+        <is>
+          <t>0.95</t>
+        </is>
+      </c>
+      <c r="O118" s="2" t="inlineStr">
+        <is>
+          <t>300.0</t>
+        </is>
+      </c>
+      <c r="P118" s="2" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q118" s="2" t="inlineStr">
+        <is>
+          <t>D+05 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="4" t="inlineStr">
@@ -7987,13 +9059,41 @@
           <t>PF</t>
         </is>
       </c>
-      <c r="K120" s="2" t="inlineStr"/>
-      <c r="L120" s="2" t="inlineStr"/>
-      <c r="M120" s="2" t="inlineStr"/>
-      <c r="N120" s="2" t="inlineStr"/>
-      <c r="O120" s="2" t="inlineStr"/>
-      <c r="P120" s="2" t="inlineStr"/>
-      <c r="Q120" s="2" t="inlineStr"/>
+      <c r="K120" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/mutuos-privatizacao/fmp-fgts-cl-absoluto</t>
+        </is>
+      </c>
+      <c r="L120" s="2" t="inlineStr">
+        <is>
+          <t>04.602.186/0001-00</t>
+        </is>
+      </c>
+      <c r="M120" s="2" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N120" s="2" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="O120" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P120" s="2" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q120" s="2" t="inlineStr">
+        <is>
+          <t>D+05 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="4" t="inlineStr">
@@ -8105,13 +9205,41 @@
           <t>PF</t>
         </is>
       </c>
-      <c r="K122" s="2" t="inlineStr"/>
-      <c r="L122" s="2" t="inlineStr"/>
-      <c r="M122" s="2" t="inlineStr"/>
-      <c r="N122" s="2" t="inlineStr"/>
-      <c r="O122" s="2" t="inlineStr"/>
-      <c r="P122" s="2" t="inlineStr"/>
-      <c r="Q122" s="2" t="inlineStr"/>
+      <c r="K122" s="2" t="inlineStr">
+        <is>
+          <t>http://www.caixa.gov.br/fundos-investimento/mutuos-privatizacao/fmp-fgts-petrobas-2</t>
+        </is>
+      </c>
+      <c r="L122" s="2" t="inlineStr">
+        <is>
+          <t>03.915.910/0001-92</t>
+        </is>
+      </c>
+      <c r="M122" s="2" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N122" s="2" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="O122" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P122" s="2" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q122" s="2" t="inlineStr">
+        <is>
+          <t>D+05 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="4" t="inlineStr">
@@ -8223,13 +9351,41 @@
           <t>PF</t>
         </is>
       </c>
-      <c r="K124" s="2" t="inlineStr"/>
-      <c r="L124" s="2" t="inlineStr"/>
-      <c r="M124" s="2" t="inlineStr"/>
-      <c r="N124" s="2" t="inlineStr"/>
-      <c r="O124" s="2" t="inlineStr"/>
-      <c r="P124" s="2" t="inlineStr"/>
-      <c r="Q124" s="2" t="inlineStr"/>
+      <c r="K124" s="2" t="inlineStr">
+        <is>
+          <t>http://www.caixa.gov.br/fundos-investimento/mutuos-privatizacao/fmp-fgts-petrobas-3</t>
+        </is>
+      </c>
+      <c r="L124" s="2" t="inlineStr">
+        <is>
+          <t>03.915.903/0001-90</t>
+        </is>
+      </c>
+      <c r="M124" s="2" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N124" s="2" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="O124" s="2" t="inlineStr">
+        <is>
+          <t>10000.0</t>
+        </is>
+      </c>
+      <c r="P124" s="2" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q124" s="2" t="inlineStr">
+        <is>
+          <t>D+05 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="4" t="inlineStr">
@@ -8413,12 +9569,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/caixa-equilibrio-mpe-rf-lp/</t>
         </is>
       </c>
-      <c r="L127" s="4" t="inlineStr"/>
-      <c r="M127" s="4" t="inlineStr"/>
-      <c r="N127" s="4" t="inlineStr"/>
-      <c r="O127" s="4" t="inlineStr"/>
-      <c r="P127" s="4" t="inlineStr"/>
-      <c r="Q127" s="4" t="inlineStr"/>
+      <c r="L127" s="4" t="inlineStr">
+        <is>
+          <t>07.986.172/0001-25</t>
+        </is>
+      </c>
+      <c r="M127" s="4" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N127" s="4" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="O127" s="4" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="P127" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q127" s="4" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -8476,12 +9656,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fi-saude-suplementar-anf-rf</t>
         </is>
       </c>
-      <c r="L128" s="2" t="inlineStr"/>
-      <c r="M128" s="2" t="inlineStr"/>
-      <c r="N128" s="2" t="inlineStr"/>
-      <c r="O128" s="2" t="inlineStr"/>
-      <c r="P128" s="2" t="inlineStr"/>
-      <c r="Q128" s="2" t="inlineStr"/>
+      <c r="L128" s="2" t="inlineStr">
+        <is>
+          <t>09.181.268/0001-41</t>
+        </is>
+      </c>
+      <c r="M128" s="2" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="N128" s="2" t="inlineStr">
+        <is>
+          <t>0.35</t>
+        </is>
+      </c>
+      <c r="O128" s="2" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="P128" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q128" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="4" t="inlineStr">
@@ -8539,12 +9743,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/caixa-fic-tp-mpe-rf-lp/</t>
         </is>
       </c>
-      <c r="L129" s="4" t="inlineStr"/>
-      <c r="M129" s="4" t="inlineStr"/>
-      <c r="N129" s="4" t="inlineStr"/>
-      <c r="O129" s="4" t="inlineStr"/>
-      <c r="P129" s="4" t="inlineStr"/>
-      <c r="Q129" s="4" t="inlineStr"/>
+      <c r="L129" s="4" t="inlineStr">
+        <is>
+          <t>15.154.429/0001-00</t>
+        </is>
+      </c>
+      <c r="M129" s="4" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="N129" s="4" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="O129" s="4" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="P129" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q129" s="4" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -8602,12 +9830,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-patrimonio-indice-precos-rf-longo-prazo</t>
         </is>
       </c>
-      <c r="L130" s="2" t="inlineStr"/>
-      <c r="M130" s="2" t="inlineStr"/>
-      <c r="N130" s="2" t="inlineStr"/>
-      <c r="O130" s="2" t="inlineStr"/>
-      <c r="P130" s="2" t="inlineStr"/>
-      <c r="Q130" s="2" t="inlineStr"/>
+      <c r="L130" s="2" t="inlineStr">
+        <is>
+          <t>03.191.874/0001-61</t>
+        </is>
+      </c>
+      <c r="M130" s="2" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N130" s="2" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="O130" s="2" t="inlineStr">
+        <is>
+          <t>100000.0</t>
+        </is>
+      </c>
+      <c r="P130" s="2" t="inlineStr">
+        <is>
+          <t>D+3 (du)</t>
+        </is>
+      </c>
+      <c r="Q130" s="2" t="inlineStr">
+        <is>
+          <t>D+03 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="4" t="inlineStr">
@@ -8665,12 +9917,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/referenciados/fic-giro-empresas-ref-di-longo-prazo/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L131" s="4" t="inlineStr"/>
-      <c r="M131" s="4" t="inlineStr"/>
-      <c r="N131" s="4" t="inlineStr"/>
-      <c r="O131" s="4" t="inlineStr"/>
-      <c r="P131" s="4" t="inlineStr"/>
-      <c r="Q131" s="4" t="inlineStr"/>
+      <c r="L131" s="4" t="inlineStr">
+        <is>
+          <t>16.916.063/0001-22</t>
+        </is>
+      </c>
+      <c r="M131" s="4" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="N131" s="4" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="O131" s="4" t="inlineStr">
+        <is>
+          <t>500000.0</t>
+        </is>
+      </c>
+      <c r="P131" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q131" s="4" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -8791,12 +10067,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/referenciados/fi-safira-corporativo-rf-lp</t>
         </is>
       </c>
-      <c r="L133" s="4" t="inlineStr"/>
-      <c r="M133" s="4" t="inlineStr"/>
-      <c r="N133" s="4" t="inlineStr"/>
-      <c r="O133" s="4" t="inlineStr"/>
-      <c r="P133" s="4" t="inlineStr"/>
-      <c r="Q133" s="4" t="inlineStr"/>
+      <c r="L133" s="4" t="inlineStr">
+        <is>
+          <t>10.384.413/0001-70</t>
+        </is>
+      </c>
+      <c r="M133" s="4" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="N133" s="4" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="O133" s="4" t="inlineStr">
+        <is>
+          <t>1000000.0</t>
+        </is>
+      </c>
+      <c r="P133" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q133" s="4" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -8917,12 +10217,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fi-saude-suplementar-ans-ii-rf-longo-prazo</t>
         </is>
       </c>
-      <c r="L135" s="4" t="inlineStr"/>
-      <c r="M135" s="4" t="inlineStr"/>
-      <c r="N135" s="4" t="inlineStr"/>
-      <c r="O135" s="4" t="inlineStr"/>
-      <c r="P135" s="4" t="inlineStr"/>
-      <c r="Q135" s="4" t="inlineStr"/>
+      <c r="L135" s="4" t="inlineStr">
+        <is>
+          <t>09.548.725/0001-93</t>
+        </is>
+      </c>
+      <c r="M135" s="4" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="N135" s="4" t="inlineStr">
+        <is>
+          <t>0.07</t>
+        </is>
+      </c>
+      <c r="O135" s="4" t="inlineStr">
+        <is>
+          <t>10000000.0</t>
+        </is>
+      </c>
+      <c r="P135" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q135" s="4" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -9043,12 +10367,32 @@
           <t>https://www.caixa.gov.br/fundos-investimento/empresa/renda-fixa/fi-sebrae-rf-longo-prazo/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L137" s="4" t="inlineStr"/>
-      <c r="M137" s="4" t="inlineStr"/>
+      <c r="L137" s="4" t="inlineStr">
+        <is>
+          <t>03.737.227/0001-02</t>
+        </is>
+      </c>
+      <c r="M137" s="4" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
       <c r="N137" s="4" t="inlineStr"/>
-      <c r="O137" s="4" t="inlineStr"/>
-      <c r="P137" s="4" t="inlineStr"/>
-      <c r="Q137" s="4" t="inlineStr"/>
+      <c r="O137" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P137" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q137" s="4" t="inlineStr">
+        <is>
+          <t>D+01 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -9673,12 +11017,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/brasil-IPCA</t>
         </is>
       </c>
-      <c r="L147" s="4" t="inlineStr"/>
-      <c r="M147" s="4" t="inlineStr"/>
-      <c r="N147" s="4" t="inlineStr"/>
-      <c r="O147" s="4" t="inlineStr"/>
-      <c r="P147" s="4" t="inlineStr"/>
-      <c r="Q147" s="4" t="inlineStr"/>
+      <c r="L147" s="4" t="inlineStr">
+        <is>
+          <t>21.918.896/0001-62</t>
+        </is>
+      </c>
+      <c r="M147" s="4" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N147" s="4" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="O147" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P147" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q147" s="4" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -10492,12 +11860,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-caixa-brasil-idka-pre2a-rf-lp/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L160" s="2" t="inlineStr"/>
-      <c r="M160" s="2" t="inlineStr"/>
-      <c r="N160" s="2" t="inlineStr"/>
-      <c r="O160" s="2" t="inlineStr"/>
-      <c r="P160" s="2" t="inlineStr"/>
-      <c r="Q160" s="2" t="inlineStr"/>
+      <c r="L160" s="2" t="inlineStr">
+        <is>
+          <t>45.163.710/0001-70</t>
+        </is>
+      </c>
+      <c r="M160" s="2" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N160" s="2" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="O160" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P160" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q160" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="4" t="inlineStr">
@@ -11244,12 +12636,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fi-extramercado-comum-irfm-1-rf/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L172" s="2" t="inlineStr"/>
-      <c r="M172" s="2" t="inlineStr"/>
-      <c r="N172" s="2" t="inlineStr"/>
-      <c r="O172" s="2" t="inlineStr"/>
-      <c r="P172" s="2" t="inlineStr"/>
-      <c r="Q172" s="2" t="inlineStr"/>
+      <c r="L172" s="2" t="inlineStr">
+        <is>
+          <t>14.507.897/0001-59</t>
+        </is>
+      </c>
+      <c r="M172" s="2" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="N172" s="2" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="O172" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P172" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q172" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Dados atualizados via Robô: 19/05/2026 05:46
</commit_message>
<xml_diff>
--- a/dados_atuais.xlsx
+++ b/dados_atuais.xlsx
@@ -693,12 +693,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/fundo-simples/fic-facil-rf-simples</t>
         </is>
       </c>
-      <c r="L3" s="4" t="inlineStr"/>
-      <c r="M3" s="4" t="inlineStr"/>
-      <c r="N3" s="4" t="inlineStr"/>
-      <c r="O3" s="4" t="inlineStr"/>
-      <c r="P3" s="4" t="inlineStr"/>
-      <c r="Q3" s="4" t="inlineStr"/>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t>05.114.716/0001-33</t>
+        </is>
+      </c>
+      <c r="M3" s="4" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="N3" s="4" t="inlineStr">
+        <is>
+          <t>1.7</t>
+        </is>
+      </c>
+      <c r="O3" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P3" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q3" s="4" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -756,12 +780,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/fundo-simples/fic-movimentacoes-automaticas-rf-simples/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr"/>
-      <c r="M4" s="2" t="inlineStr"/>
-      <c r="N4" s="2" t="inlineStr"/>
-      <c r="O4" s="2" t="inlineStr"/>
-      <c r="P4" s="2" t="inlineStr"/>
-      <c r="Q4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>14.508.652/0001-46</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>1.7</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -969,12 +1017,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/caixa-fic-plus-rf-credito-privado-lp/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L7" s="4" t="inlineStr"/>
-      <c r="M7" s="4" t="inlineStr"/>
-      <c r="N7" s="4" t="inlineStr"/>
-      <c r="O7" s="4" t="inlineStr"/>
-      <c r="P7" s="4" t="inlineStr"/>
-      <c r="Q7" s="4" t="inlineStr"/>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>40.194.309/0001-84</t>
+        </is>
+      </c>
+      <c r="M7" s="4" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N7" s="4" t="inlineStr">
+        <is>
+          <t>0.7</t>
+        </is>
+      </c>
+      <c r="O7" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P7" s="4" t="inlineStr">
+        <is>
+          <t>D+14 (du)</t>
+        </is>
+      </c>
+      <c r="Q7" s="4" t="inlineStr">
+        <is>
+          <t>D+15 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1032,12 +1104,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-ideal-rf-longo-prazo</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr"/>
-      <c r="M8" s="2" t="inlineStr"/>
-      <c r="N8" s="2" t="inlineStr"/>
-      <c r="O8" s="2" t="inlineStr"/>
-      <c r="P8" s="2" t="inlineStr"/>
-      <c r="Q8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>68.623.479/0001-56</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q8" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -1241,12 +1337,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-absoluto-pre-rf-longo-prazo</t>
         </is>
       </c>
-      <c r="L11" s="4" t="inlineStr"/>
-      <c r="M11" s="4" t="inlineStr"/>
-      <c r="N11" s="4" t="inlineStr"/>
-      <c r="O11" s="4" t="inlineStr"/>
-      <c r="P11" s="4" t="inlineStr"/>
-      <c r="Q11" s="4" t="inlineStr"/>
+      <c r="L11" s="4" t="inlineStr">
+        <is>
+          <t>02.201.164/0001-02</t>
+        </is>
+      </c>
+      <c r="M11" s="4" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N11" s="4" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="O11" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P11" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q11" s="4" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1304,12 +1424,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-capital-indice-de-precos-rf-longo-prazo</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr"/>
-      <c r="M12" s="2" t="inlineStr"/>
-      <c r="N12" s="2" t="inlineStr"/>
-      <c r="O12" s="2" t="inlineStr"/>
-      <c r="P12" s="2" t="inlineStr"/>
-      <c r="Q12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>03.218.183/0001-04</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>D+3 (du)</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr">
+        <is>
+          <t>D+03 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1454,12 +1598,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-soberano-rf-longo-prazo</t>
         </is>
       </c>
-      <c r="L14" s="2" t="inlineStr"/>
-      <c r="M14" s="2" t="inlineStr"/>
-      <c r="N14" s="2" t="inlineStr"/>
-      <c r="O14" s="2" t="inlineStr"/>
-      <c r="P14" s="2" t="inlineStr"/>
-      <c r="Q14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>02.323.746/0001-61</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>50.0</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1517,12 +1685,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-foco-indice-precos-rf-longo-prazo</t>
         </is>
       </c>
-      <c r="L15" s="4" t="inlineStr"/>
-      <c r="M15" s="4" t="inlineStr"/>
-      <c r="N15" s="4" t="inlineStr"/>
-      <c r="O15" s="4" t="inlineStr"/>
-      <c r="P15" s="4" t="inlineStr"/>
-      <c r="Q15" s="4" t="inlineStr"/>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>09.548.729/0001-71</t>
+        </is>
+      </c>
+      <c r="M15" s="4" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N15" s="4" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="O15" s="4" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
+      <c r="P15" s="4" t="inlineStr">
+        <is>
+          <t>D+3 (du)</t>
+        </is>
+      </c>
+      <c r="Q15" s="4" t="inlineStr">
+        <is>
+          <t>D+03 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1580,12 +1772,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-classico-rf-longo-prazo</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr"/>
-      <c r="M16" s="2" t="inlineStr"/>
-      <c r="N16" s="2" t="inlineStr"/>
-      <c r="O16" s="2" t="inlineStr"/>
-      <c r="P16" s="2" t="inlineStr"/>
-      <c r="Q16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>01.165.796/0001-03</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q16" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -1817,12 +2033,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-oab-rf-credito-privado-longo-prazo</t>
         </is>
       </c>
-      <c r="L19" s="4" t="inlineStr"/>
-      <c r="M19" s="4" t="inlineStr"/>
-      <c r="N19" s="4" t="inlineStr"/>
-      <c r="O19" s="4" t="inlineStr"/>
-      <c r="P19" s="4" t="inlineStr"/>
-      <c r="Q19" s="4" t="inlineStr"/>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>14.120.488/0001-03</t>
+        </is>
+      </c>
+      <c r="M19" s="4" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N19" s="4" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="O19" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P19" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q19" s="4" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1880,12 +2120,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-executivo-rf-longo-prazo</t>
         </is>
       </c>
-      <c r="L20" s="2" t="inlineStr"/>
-      <c r="M20" s="2" t="inlineStr"/>
-      <c r="N20" s="2" t="inlineStr"/>
-      <c r="O20" s="2" t="inlineStr"/>
-      <c r="P20" s="2" t="inlineStr"/>
-      <c r="Q20" s="2" t="inlineStr"/>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>01.165.781/0001-37</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q20" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -1943,12 +2207,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-relacionamento-ideal-rf-longo-prazo</t>
         </is>
       </c>
-      <c r="L21" s="4" t="inlineStr"/>
-      <c r="M21" s="4" t="inlineStr"/>
-      <c r="N21" s="4" t="inlineStr"/>
-      <c r="O21" s="4" t="inlineStr"/>
-      <c r="P21" s="4" t="inlineStr"/>
-      <c r="Q21" s="4" t="inlineStr"/>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>10.577.505/0001-77</t>
+        </is>
+      </c>
+      <c r="M21" s="4" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N21" s="4" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="O21" s="4" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="P21" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q21" s="4" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2152,12 +2440,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/debentures-incentivadas/caixa-expert-arx-ipca-deb-incentivadas-rf-cred-priv-lp/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L24" s="2" t="inlineStr"/>
-      <c r="M24" s="2" t="inlineStr"/>
-      <c r="N24" s="2" t="inlineStr"/>
-      <c r="O24" s="2" t="inlineStr"/>
-      <c r="P24" s="2" t="inlineStr"/>
-      <c r="Q24" s="2" t="inlineStr"/>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>60.138.811/0001-85</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>10000.0</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>D+14 (du)</t>
+        </is>
+      </c>
+      <c r="Q24" s="2" t="inlineStr">
+        <is>
+          <t>D+16 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -2215,12 +2527,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/debentures-incentivadas/caixa-expert-vinlanddebenture-</t>
         </is>
       </c>
-      <c r="L25" s="4" t="inlineStr"/>
-      <c r="M25" s="4" t="inlineStr"/>
-      <c r="N25" s="4" t="inlineStr"/>
-      <c r="O25" s="4" t="inlineStr"/>
-      <c r="P25" s="4" t="inlineStr"/>
-      <c r="Q25" s="4" t="inlineStr"/>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>58.113.332/0001-62</t>
+        </is>
+      </c>
+      <c r="M25" s="4" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N25" s="4" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="O25" s="4" t="inlineStr">
+        <is>
+          <t>10000.0</t>
+        </is>
+      </c>
+      <c r="P25" s="4" t="inlineStr">
+        <is>
+          <t>D+13 (du)</t>
+        </is>
+      </c>
+      <c r="Q25" s="4" t="inlineStr">
+        <is>
+          <t>D+15 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2341,12 +2677,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/caixa-fif-inflacao-2027/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L27" s="4" t="inlineStr"/>
-      <c r="M27" s="4" t="inlineStr"/>
-      <c r="N27" s="4" t="inlineStr"/>
-      <c r="O27" s="4" t="inlineStr"/>
-      <c r="P27" s="4" t="inlineStr"/>
-      <c r="Q27" s="4" t="inlineStr"/>
+      <c r="L27" s="4" t="inlineStr">
+        <is>
+          <t>56.349.290/0001-38</t>
+        </is>
+      </c>
+      <c r="M27" s="4" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N27" s="4" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="O27" s="4" t="inlineStr">
+        <is>
+          <t>10000.0</t>
+        </is>
+      </c>
+      <c r="P27" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q27" s="4" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2400,12 +2760,36 @@
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr"/>
-      <c r="L28" s="2" t="inlineStr"/>
-      <c r="M28" s="2" t="inlineStr"/>
-      <c r="N28" s="2" t="inlineStr"/>
-      <c r="O28" s="2" t="inlineStr"/>
-      <c r="P28" s="2" t="inlineStr"/>
-      <c r="Q28" s="2" t="inlineStr"/>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>63.455.348/0001-93</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>0.17</t>
+        </is>
+      </c>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="P28" s="2" t="inlineStr">
+        <is>
+          <t>D+5 (du)</t>
+        </is>
+      </c>
+      <c r="Q28" s="2" t="inlineStr">
+        <is>
+          <t>D+07 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -2459,12 +2843,36 @@
         </is>
       </c>
       <c r="K29" s="4" t="inlineStr"/>
-      <c r="L29" s="4" t="inlineStr"/>
-      <c r="M29" s="4" t="inlineStr"/>
-      <c r="N29" s="4" t="inlineStr"/>
-      <c r="O29" s="4" t="inlineStr"/>
-      <c r="P29" s="4" t="inlineStr"/>
-      <c r="Q29" s="4" t="inlineStr"/>
+      <c r="L29" s="4" t="inlineStr">
+        <is>
+          <t>59.861.817/0001-05</t>
+        </is>
+      </c>
+      <c r="M29" s="4" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N29" s="4" t="inlineStr">
+        <is>
+          <t>0.29</t>
+        </is>
+      </c>
+      <c r="O29" s="4" t="inlineStr">
+        <is>
+          <t>10000.0</t>
+        </is>
+      </c>
+      <c r="P29" s="4" t="inlineStr">
+        <is>
+          <t>D+22 (du)</t>
+        </is>
+      </c>
+      <c r="Q29" s="4" t="inlineStr">
+        <is>
+          <t>D+24 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2522,12 +2930,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/debentures-incentivadas/caixa-expert-rb-asset-deb-incentivadas-cdi-rf-cred-priv/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L30" s="2" t="inlineStr"/>
-      <c r="M30" s="2" t="inlineStr"/>
-      <c r="N30" s="2" t="inlineStr"/>
-      <c r="O30" s="2" t="inlineStr"/>
-      <c r="P30" s="2" t="inlineStr"/>
-      <c r="Q30" s="2" t="inlineStr"/>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>62.890.286/0001-85</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>10000.0</t>
+        </is>
+      </c>
+      <c r="P30" s="2" t="inlineStr">
+        <is>
+          <t>D+14 (du)</t>
+        </is>
+      </c>
+      <c r="Q30" s="2" t="inlineStr">
+        <is>
+          <t>D+16 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -2581,12 +3013,32 @@
         </is>
       </c>
       <c r="K31" s="4" t="inlineStr"/>
-      <c r="L31" s="4" t="inlineStr"/>
-      <c r="M31" s="4" t="inlineStr"/>
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t>65.789.297/0001-61</t>
+        </is>
+      </c>
+      <c r="M31" s="4" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
       <c r="N31" s="4" t="inlineStr"/>
-      <c r="O31" s="4" t="inlineStr"/>
-      <c r="P31" s="4" t="inlineStr"/>
-      <c r="Q31" s="4" t="inlineStr"/>
+      <c r="O31" s="4" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="P31" s="4" t="inlineStr">
+        <is>
+          <t>D+21 (du)</t>
+        </is>
+      </c>
+      <c r="Q31" s="4" t="inlineStr">
+        <is>
+          <t>D+23 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2905,12 +3357,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-personal-rf-longo-prazo</t>
         </is>
       </c>
-      <c r="L35" s="4" t="inlineStr"/>
-      <c r="M35" s="4" t="inlineStr"/>
-      <c r="N35" s="4" t="inlineStr"/>
-      <c r="O35" s="4" t="inlineStr"/>
-      <c r="P35" s="4" t="inlineStr"/>
-      <c r="Q35" s="4" t="inlineStr"/>
+      <c r="L35" s="4" t="inlineStr">
+        <is>
+          <t>02.201.163/0001-68</t>
+        </is>
+      </c>
+      <c r="M35" s="4" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N35" s="4" t="inlineStr">
+        <is>
+          <t>0.6</t>
+        </is>
+      </c>
+      <c r="O35" s="4" t="inlineStr">
+        <is>
+          <t>50000.0</t>
+        </is>
+      </c>
+      <c r="P35" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q35" s="4" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2968,12 +3444,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/caixa-fic-renda-fixa-ativa-lp/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L36" s="2" t="inlineStr"/>
-      <c r="M36" s="2" t="inlineStr"/>
-      <c r="N36" s="2" t="inlineStr"/>
-      <c r="O36" s="2" t="inlineStr"/>
-      <c r="P36" s="2" t="inlineStr"/>
-      <c r="Q36" s="2" t="inlineStr"/>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>35.536.542/0001-68</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N36" s="2" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="O36" s="2" t="inlineStr">
+        <is>
+          <t>50000.0</t>
+        </is>
+      </c>
+      <c r="P36" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q36" s="2" t="inlineStr">
+        <is>
+          <t>D+01 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -3118,12 +3618,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-supremo-rf-longo-prazo</t>
         </is>
       </c>
-      <c r="L38" s="2" t="inlineStr"/>
-      <c r="M38" s="2" t="inlineStr"/>
-      <c r="N38" s="2" t="inlineStr"/>
-      <c r="O38" s="2" t="inlineStr"/>
-      <c r="P38" s="2" t="inlineStr"/>
-      <c r="Q38" s="2" t="inlineStr"/>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>07.986.178/0001-00</t>
+        </is>
+      </c>
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N38" s="2" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="O38" s="2" t="inlineStr">
+        <is>
+          <t>70000.0</t>
+        </is>
+      </c>
+      <c r="P38" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q38" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
@@ -3181,12 +3705,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/caixa-fic-unique-private-cred-priv-lp/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L39" s="4" t="inlineStr"/>
-      <c r="M39" s="4" t="inlineStr"/>
-      <c r="N39" s="4" t="inlineStr"/>
-      <c r="O39" s="4" t="inlineStr"/>
-      <c r="P39" s="4" t="inlineStr"/>
-      <c r="Q39" s="4" t="inlineStr"/>
+      <c r="L39" s="4" t="inlineStr">
+        <is>
+          <t>55.986.292/0001-75</t>
+        </is>
+      </c>
+      <c r="M39" s="4" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N39" s="4" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="O39" s="4" t="inlineStr">
+        <is>
+          <t>100000.0</t>
+        </is>
+      </c>
+      <c r="P39" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q39" s="4" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3244,12 +3792,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-especial-rf-longo-prazo/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L40" s="2" t="inlineStr"/>
-      <c r="M40" s="2" t="inlineStr"/>
-      <c r="N40" s="2" t="inlineStr"/>
-      <c r="O40" s="2" t="inlineStr"/>
-      <c r="P40" s="2" t="inlineStr"/>
-      <c r="Q40" s="2" t="inlineStr"/>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>03.737.190/0001-12</t>
+        </is>
+      </c>
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N40" s="2" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="O40" s="2" t="inlineStr">
+        <is>
+          <t>100000.0</t>
+        </is>
+      </c>
+      <c r="P40" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q40" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
@@ -3307,12 +3879,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fi-fidelidade-private-rf-longo-prazo/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L41" s="4" t="inlineStr"/>
-      <c r="M41" s="4" t="inlineStr"/>
-      <c r="N41" s="4" t="inlineStr"/>
-      <c r="O41" s="4" t="inlineStr"/>
-      <c r="P41" s="4" t="inlineStr"/>
-      <c r="Q41" s="4" t="inlineStr"/>
+      <c r="L41" s="4" t="inlineStr">
+        <is>
+          <t>09.181.287/0001-78</t>
+        </is>
+      </c>
+      <c r="M41" s="4" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N41" s="4" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="O41" s="4" t="inlineStr">
+        <is>
+          <t>200000.0</t>
+        </is>
+      </c>
+      <c r="P41" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q41" s="4" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3457,12 +4053,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fi-fidelidade-ii-rf-credito-privado-longo-prazo/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L43" s="4" t="inlineStr"/>
-      <c r="M43" s="4" t="inlineStr"/>
-      <c r="N43" s="4" t="inlineStr"/>
-      <c r="O43" s="4" t="inlineStr"/>
-      <c r="P43" s="4" t="inlineStr"/>
-      <c r="Q43" s="4" t="inlineStr"/>
+      <c r="L43" s="4" t="inlineStr">
+        <is>
+          <t>10.322.668/0001-09</t>
+        </is>
+      </c>
+      <c r="M43" s="4" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N43" s="4" t="inlineStr">
+        <is>
+          <t>0.05</t>
+        </is>
+      </c>
+      <c r="O43" s="4" t="inlineStr">
+        <is>
+          <t>1000000.0</t>
+        </is>
+      </c>
+      <c r="P43" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q43" s="4" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3520,12 +4140,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/referenciados/fic-beta-ref-di-lp</t>
         </is>
       </c>
-      <c r="L44" s="2" t="inlineStr"/>
-      <c r="M44" s="2" t="inlineStr"/>
-      <c r="N44" s="2" t="inlineStr"/>
-      <c r="O44" s="2" t="inlineStr"/>
-      <c r="P44" s="2" t="inlineStr"/>
-      <c r="Q44" s="2" t="inlineStr"/>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>00.834.072/0001-34</t>
+        </is>
+      </c>
+      <c r="M44" s="2" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="N44" s="2" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="O44" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P44" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q44" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
@@ -3579,12 +4223,36 @@
         </is>
       </c>
       <c r="K45" s="4" t="inlineStr"/>
-      <c r="L45" s="4" t="inlineStr"/>
-      <c r="M45" s="4" t="inlineStr"/>
-      <c r="N45" s="4" t="inlineStr"/>
-      <c r="O45" s="4" t="inlineStr"/>
-      <c r="P45" s="4" t="inlineStr"/>
-      <c r="Q45" s="4" t="inlineStr"/>
+      <c r="L45" s="4" t="inlineStr">
+        <is>
+          <t>66.034.762/0001-17</t>
+        </is>
+      </c>
+      <c r="M45" s="4" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="N45" s="4" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="O45" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P45" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q45" s="4" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3642,12 +4310,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/referenciados/fic-giro-imediato-ref-di-longo-prazo</t>
         </is>
       </c>
-      <c r="L46" s="2" t="inlineStr"/>
-      <c r="M46" s="2" t="inlineStr"/>
-      <c r="N46" s="2" t="inlineStr"/>
-      <c r="O46" s="2" t="inlineStr"/>
-      <c r="P46" s="2" t="inlineStr"/>
-      <c r="Q46" s="2" t="inlineStr"/>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>17.502.869/0001-37</t>
+        </is>
+      </c>
+      <c r="M46" s="2" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="N46" s="2" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="O46" s="2" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="P46" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q46" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
@@ -3792,12 +4484,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/referenciados/fic-omega-ref-di-longo-prazo/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L48" s="2" t="inlineStr"/>
-      <c r="M48" s="2" t="inlineStr"/>
-      <c r="N48" s="2" t="inlineStr"/>
-      <c r="O48" s="2" t="inlineStr"/>
-      <c r="P48" s="2" t="inlineStr"/>
-      <c r="Q48" s="2" t="inlineStr"/>
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>55.036.101/0001-04</t>
+        </is>
+      </c>
+      <c r="M48" s="2" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="N48" s="2" t="inlineStr">
+        <is>
+          <t>0.15</t>
+        </is>
+      </c>
+      <c r="O48" s="2" t="inlineStr">
+        <is>
+          <t>10000.0</t>
+        </is>
+      </c>
+      <c r="P48" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q48" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
@@ -3942,12 +4658,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/referenciados/fic-sigma-ref-di-longo-prazo</t>
         </is>
       </c>
-      <c r="L50" s="2" t="inlineStr"/>
-      <c r="M50" s="2" t="inlineStr"/>
-      <c r="N50" s="2" t="inlineStr"/>
-      <c r="O50" s="2" t="inlineStr"/>
-      <c r="P50" s="2" t="inlineStr"/>
-      <c r="Q50" s="2" t="inlineStr"/>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>10.731.794/0001-17</t>
+        </is>
+      </c>
+      <c r="M50" s="2" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="N50" s="2" t="inlineStr">
+        <is>
+          <t>0.35</t>
+        </is>
+      </c>
+      <c r="O50" s="2" t="inlineStr">
+        <is>
+          <t>5000.0</t>
+        </is>
+      </c>
+      <c r="P50" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q50" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
@@ -4005,12 +4745,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/referenciados/fic-rubi-ref-di-longo-prazo/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L51" s="4" t="inlineStr"/>
-      <c r="M51" s="4" t="inlineStr"/>
-      <c r="N51" s="4" t="inlineStr"/>
-      <c r="O51" s="4" t="inlineStr"/>
-      <c r="P51" s="4" t="inlineStr"/>
-      <c r="Q51" s="4" t="inlineStr"/>
+      <c r="L51" s="4" t="inlineStr">
+        <is>
+          <t>10.646.885/0001-54</t>
+        </is>
+      </c>
+      <c r="M51" s="4" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="N51" s="4" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="O51" s="4" t="inlineStr">
+        <is>
+          <t>100000.0</t>
+        </is>
+      </c>
+      <c r="P51" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q51" s="4" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -4131,12 +4895,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/referenciados/fic-top-private-ref-di-longo-prazo/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L53" s="4" t="inlineStr"/>
-      <c r="M53" s="4" t="inlineStr"/>
-      <c r="N53" s="4" t="inlineStr"/>
-      <c r="O53" s="4" t="inlineStr"/>
-      <c r="P53" s="4" t="inlineStr"/>
-      <c r="Q53" s="4" t="inlineStr"/>
+      <c r="L53" s="4" t="inlineStr">
+        <is>
+          <t>19.769.018/0001-80</t>
+        </is>
+      </c>
+      <c r="M53" s="4" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="N53" s="4" t="inlineStr">
+        <is>
+          <t>0.15</t>
+        </is>
+      </c>
+      <c r="O53" s="4" t="inlineStr">
+        <is>
+          <t>100000.0</t>
+        </is>
+      </c>
+      <c r="P53" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q53" s="4" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -4281,12 +5069,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-fof-smart-credito-privado-multimercado-longo-prazo/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L55" s="4" t="inlineStr"/>
-      <c r="M55" s="4" t="inlineStr"/>
-      <c r="N55" s="4" t="inlineStr"/>
-      <c r="O55" s="4" t="inlineStr"/>
-      <c r="P55" s="4" t="inlineStr"/>
-      <c r="Q55" s="4" t="inlineStr"/>
+      <c r="L55" s="4" t="inlineStr">
+        <is>
+          <t>51.943.346/0001-64</t>
+        </is>
+      </c>
+      <c r="M55" s="4" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N55" s="4" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="O55" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P55" s="4" t="inlineStr">
+        <is>
+          <t>D+46 (du)</t>
+        </is>
+      </c>
+      <c r="Q55" s="4" t="inlineStr">
+        <is>
+          <t>D+48 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -4344,12 +5156,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/multimercado/caixa-multigestor-global-equities-invest-ext/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L56" s="2" t="inlineStr"/>
-      <c r="M56" s="2" t="inlineStr"/>
-      <c r="N56" s="2" t="inlineStr"/>
-      <c r="O56" s="2" t="inlineStr"/>
-      <c r="P56" s="2" t="inlineStr"/>
-      <c r="Q56" s="2" t="inlineStr"/>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>39.528.038/0001-77</t>
+        </is>
+      </c>
+      <c r="M56" s="2" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N56" s="2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="O56" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P56" s="2" t="inlineStr">
+        <is>
+          <t>D+7 (du)</t>
+        </is>
+      </c>
+      <c r="Q56" s="2" t="inlineStr">
+        <is>
+          <t>D+12 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
@@ -4470,12 +5306,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/multimercado/estrategia-livre-mm-lp</t>
         </is>
       </c>
-      <c r="L58" s="2" t="inlineStr"/>
-      <c r="M58" s="2" t="inlineStr"/>
-      <c r="N58" s="2" t="inlineStr"/>
-      <c r="O58" s="2" t="inlineStr"/>
-      <c r="P58" s="2" t="inlineStr"/>
-      <c r="Q58" s="2" t="inlineStr"/>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>34.660.276/0001-18</t>
+        </is>
+      </c>
+      <c r="M58" s="2" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N58" s="2" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="O58" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P58" s="2" t="inlineStr">
+        <is>
+          <t>D+13 (du)</t>
+        </is>
+      </c>
+      <c r="Q58" s="2" t="inlineStr">
+        <is>
+          <t>D+15 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
@@ -4616,12 +5476,36 @@
         </is>
       </c>
       <c r="K60" s="2" t="inlineStr"/>
-      <c r="L60" s="2" t="inlineStr"/>
-      <c r="M60" s="2" t="inlineStr"/>
-      <c r="N60" s="2" t="inlineStr"/>
-      <c r="O60" s="2" t="inlineStr"/>
-      <c r="P60" s="2" t="inlineStr"/>
-      <c r="Q60" s="2" t="inlineStr"/>
+      <c r="L60" s="2" t="inlineStr">
+        <is>
+          <t>65.795.043/0001-56</t>
+        </is>
+      </c>
+      <c r="M60" s="2" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N60" s="2" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="O60" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P60" s="2" t="inlineStr">
+        <is>
+          <t>D+8 (du)</t>
+        </is>
+      </c>
+      <c r="Q60" s="2" t="inlineStr">
+        <is>
+          <t>D+10 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
@@ -4679,12 +5563,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/multimercado/caixa-fic-fof-smart-long-short-mm/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L61" s="4" t="inlineStr"/>
-      <c r="M61" s="4" t="inlineStr"/>
-      <c r="N61" s="4" t="inlineStr"/>
-      <c r="O61" s="4" t="inlineStr"/>
-      <c r="P61" s="4" t="inlineStr"/>
-      <c r="Q61" s="4" t="inlineStr"/>
+      <c r="L61" s="4" t="inlineStr">
+        <is>
+          <t>51.408.738/0001-23</t>
+        </is>
+      </c>
+      <c r="M61" s="4" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N61" s="4" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="O61" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P61" s="4" t="inlineStr">
+        <is>
+          <t>D+24 (du)</t>
+        </is>
+      </c>
+      <c r="Q61" s="4" t="inlineStr">
+        <is>
+          <t>D+26 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -4742,12 +5650,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/multimercado/caixa-fic-fof-smart-long-bias-mm/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L62" s="2" t="inlineStr"/>
-      <c r="M62" s="2" t="inlineStr"/>
-      <c r="N62" s="2" t="inlineStr"/>
-      <c r="O62" s="2" t="inlineStr"/>
-      <c r="P62" s="2" t="inlineStr"/>
-      <c r="Q62" s="2" t="inlineStr"/>
+      <c r="L62" s="2" t="inlineStr">
+        <is>
+          <t>54.439.846/0001-51</t>
+        </is>
+      </c>
+      <c r="M62" s="2" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N62" s="2" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="O62" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P62" s="2" t="inlineStr">
+        <is>
+          <t>D+13 (du)</t>
+        </is>
+      </c>
+      <c r="Q62" s="2" t="inlineStr">
+        <is>
+          <t>D+15 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
@@ -4801,12 +5733,36 @@
         </is>
       </c>
       <c r="K63" s="4" t="inlineStr"/>
-      <c r="L63" s="4" t="inlineStr"/>
-      <c r="M63" s="4" t="inlineStr"/>
-      <c r="N63" s="4" t="inlineStr"/>
-      <c r="O63" s="4" t="inlineStr"/>
-      <c r="P63" s="4" t="inlineStr"/>
-      <c r="Q63" s="4" t="inlineStr"/>
+      <c r="L63" s="4" t="inlineStr">
+        <is>
+          <t>65.795.384/0001-21</t>
+        </is>
+      </c>
+      <c r="M63" s="4" t="inlineStr">
+        <is>
+          <t>Agressivo</t>
+        </is>
+      </c>
+      <c r="N63" s="4" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="O63" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P63" s="4" t="inlineStr">
+        <is>
+          <t>D+14 (du)</t>
+        </is>
+      </c>
+      <c r="Q63" s="4" t="inlineStr">
+        <is>
+          <t>D+16 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -4864,12 +5820,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/multimercado/caixa-fic-fof-smart-long-bias-mm/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L64" s="2" t="inlineStr"/>
-      <c r="M64" s="2" t="inlineStr"/>
-      <c r="N64" s="2" t="inlineStr"/>
-      <c r="O64" s="2" t="inlineStr"/>
-      <c r="P64" s="2" t="inlineStr"/>
-      <c r="Q64" s="2" t="inlineStr"/>
+      <c r="L64" s="2" t="inlineStr">
+        <is>
+          <t>51.408.950/0001-90</t>
+        </is>
+      </c>
+      <c r="M64" s="2" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N64" s="2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="O64" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P64" s="2" t="inlineStr">
+        <is>
+          <t>D+24 (du)</t>
+        </is>
+      </c>
+      <c r="Q64" s="2" t="inlineStr">
+        <is>
+          <t>D+26 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
@@ -4923,12 +5903,36 @@
         </is>
       </c>
       <c r="K65" s="4" t="inlineStr"/>
-      <c r="L65" s="4" t="inlineStr"/>
-      <c r="M65" s="4" t="inlineStr"/>
-      <c r="N65" s="4" t="inlineStr"/>
-      <c r="O65" s="4" t="inlineStr"/>
-      <c r="P65" s="4" t="inlineStr"/>
-      <c r="Q65" s="4" t="inlineStr"/>
+      <c r="L65" s="4" t="inlineStr">
+        <is>
+          <t>65.794.476/0001-97</t>
+        </is>
+      </c>
+      <c r="M65" s="4" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N65" s="4" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="O65" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P65" s="4" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q65" s="4" t="inlineStr">
+        <is>
+          <t>D+03 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -4986,12 +5990,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fi-euro-multimercado-longo-prazo/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L66" s="2" t="inlineStr"/>
-      <c r="M66" s="2" t="inlineStr"/>
-      <c r="N66" s="2" t="inlineStr"/>
-      <c r="O66" s="2" t="inlineStr"/>
-      <c r="P66" s="2" t="inlineStr"/>
-      <c r="Q66" s="2" t="inlineStr"/>
+      <c r="L66" s="2" t="inlineStr">
+        <is>
+          <t>54.483.566/0001-40</t>
+        </is>
+      </c>
+      <c r="M66" s="2" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N66" s="2" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="O66" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P66" s="2" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q66" s="2" t="inlineStr">
+        <is>
+          <t>D+03 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
@@ -5049,12 +6077,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-estrategico-multimercado-longo-prazo</t>
         </is>
       </c>
-      <c r="L67" s="4" t="inlineStr"/>
-      <c r="M67" s="4" t="inlineStr"/>
-      <c r="N67" s="4" t="inlineStr"/>
-      <c r="O67" s="4" t="inlineStr"/>
-      <c r="P67" s="4" t="inlineStr"/>
-      <c r="Q67" s="4" t="inlineStr"/>
+      <c r="L67" s="4" t="inlineStr">
+        <is>
+          <t>03.737.200/0001-10</t>
+        </is>
+      </c>
+      <c r="M67" s="4" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N67" s="4" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="O67" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P67" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q67" s="4" t="inlineStr">
+        <is>
+          <t>D+01 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -5199,12 +6251,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-multigestor</t>
         </is>
       </c>
-      <c r="L69" s="4" t="inlineStr"/>
-      <c r="M69" s="4" t="inlineStr"/>
-      <c r="N69" s="4" t="inlineStr"/>
-      <c r="O69" s="4" t="inlineStr"/>
-      <c r="P69" s="4" t="inlineStr"/>
-      <c r="Q69" s="4" t="inlineStr"/>
+      <c r="L69" s="4" t="inlineStr">
+        <is>
+          <t>18.007.710/0001-09</t>
+        </is>
+      </c>
+      <c r="M69" s="4" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N69" s="4" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="O69" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P69" s="4" t="inlineStr">
+        <is>
+          <t>D+24 (du)</t>
+        </is>
+      </c>
+      <c r="Q69" s="4" t="inlineStr">
+        <is>
+          <t>D+26 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -5349,12 +6425,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fi-bolsa-americana-multimercado-lp</t>
         </is>
       </c>
-      <c r="L71" s="4" t="inlineStr"/>
-      <c r="M71" s="4" t="inlineStr"/>
-      <c r="N71" s="4" t="inlineStr"/>
-      <c r="O71" s="4" t="inlineStr"/>
-      <c r="P71" s="4" t="inlineStr"/>
-      <c r="Q71" s="4" t="inlineStr"/>
+      <c r="L71" s="4" t="inlineStr">
+        <is>
+          <t>30.036.235/0001-02</t>
+        </is>
+      </c>
+      <c r="M71" s="4" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N71" s="4" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="O71" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P71" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q71" s="4" t="inlineStr">
+        <is>
+          <t>D+01 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -5412,12 +6512,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/multimercado/caixa-fic-juros-e-moedas-multimercado-plus-lp/</t>
         </is>
       </c>
-      <c r="L72" s="2" t="inlineStr"/>
-      <c r="M72" s="2" t="inlineStr"/>
-      <c r="N72" s="2" t="inlineStr"/>
-      <c r="O72" s="2" t="inlineStr"/>
-      <c r="P72" s="2" t="inlineStr"/>
-      <c r="Q72" s="2" t="inlineStr"/>
+      <c r="L72" s="2" t="inlineStr">
+        <is>
+          <t>29.157.485/0001-03</t>
+        </is>
+      </c>
+      <c r="M72" s="2" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N72" s="2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="O72" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P72" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q72" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
@@ -5471,12 +6595,36 @@
         </is>
       </c>
       <c r="K73" s="4" t="inlineStr"/>
-      <c r="L73" s="4" t="inlineStr"/>
-      <c r="M73" s="4" t="inlineStr"/>
-      <c r="N73" s="4" t="inlineStr"/>
-      <c r="O73" s="4" t="inlineStr"/>
-      <c r="P73" s="4" t="inlineStr"/>
-      <c r="Q73" s="4" t="inlineStr"/>
+      <c r="L73" s="4" t="inlineStr">
+        <is>
+          <t>35.536.472/0001-48</t>
+        </is>
+      </c>
+      <c r="M73" s="4" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N73" s="4" t="inlineStr">
+        <is>
+          <t>0.6</t>
+        </is>
+      </c>
+      <c r="O73" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P73" s="4" t="inlineStr">
+        <is>
+          <t>D+13 (du)</t>
+        </is>
+      </c>
+      <c r="Q73" s="4" t="inlineStr">
+        <is>
+          <t>D+15 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -5529,13 +6677,41 @@
           <t>PF | PJ</t>
         </is>
       </c>
-      <c r="K74" s="2" t="inlineStr"/>
-      <c r="L74" s="2" t="inlineStr"/>
-      <c r="M74" s="2" t="inlineStr"/>
-      <c r="N74" s="2" t="inlineStr"/>
-      <c r="O74" s="2" t="inlineStr"/>
-      <c r="P74" s="2" t="inlineStr"/>
-      <c r="Q74" s="2" t="inlineStr"/>
+      <c r="K74" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/caixa-hashdex-nasdaq-crypto-fic-fif-mm</t>
+        </is>
+      </c>
+      <c r="L74" s="2" t="inlineStr">
+        <is>
+          <t>62.769.135/0001-73</t>
+        </is>
+      </c>
+      <c r="M74" s="2" t="inlineStr">
+        <is>
+          <t>Agressivo</t>
+        </is>
+      </c>
+      <c r="N74" s="2" t="inlineStr">
+        <is>
+          <t>0.7</t>
+        </is>
+      </c>
+      <c r="O74" s="2" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
+      <c r="P74" s="2" t="inlineStr">
+        <is>
+          <t>D+3 (du)</t>
+        </is>
+      </c>
+      <c r="Q74" s="2" t="inlineStr">
+        <is>
+          <t>D+08 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
@@ -5593,12 +6769,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/multimercado/caixa_fic_fim_cap_protegido_cesta_agro/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L75" s="4" t="inlineStr"/>
-      <c r="M75" s="4" t="inlineStr"/>
-      <c r="N75" s="4" t="inlineStr"/>
-      <c r="O75" s="4" t="inlineStr"/>
-      <c r="P75" s="4" t="inlineStr"/>
-      <c r="Q75" s="4" t="inlineStr"/>
+      <c r="L75" s="4" t="inlineStr">
+        <is>
+          <t>42.229.068/0001-97</t>
+        </is>
+      </c>
+      <c r="M75" s="4" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="N75" s="4" t="inlineStr">
+        <is>
+          <t>0.9</t>
+        </is>
+      </c>
+      <c r="O75" s="4" t="inlineStr">
+        <is>
+          <t>5000.0</t>
+        </is>
+      </c>
+      <c r="P75" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q75" s="4" t="inlineStr">
+        <is>
+          <t>D+02 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -5656,12 +6856,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-capital-protegido-ciclico-iii-multimercado-lp/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L76" s="2" t="inlineStr"/>
-      <c r="M76" s="2" t="inlineStr"/>
-      <c r="N76" s="2" t="inlineStr"/>
-      <c r="O76" s="2" t="inlineStr"/>
-      <c r="P76" s="2" t="inlineStr"/>
-      <c r="Q76" s="2" t="inlineStr"/>
+      <c r="L76" s="2" t="inlineStr">
+        <is>
+          <t>44.683.343/0001-73</t>
+        </is>
+      </c>
+      <c r="M76" s="2" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="N76" s="2" t="inlineStr">
+        <is>
+          <t>0.9</t>
+        </is>
+      </c>
+      <c r="O76" s="2" t="inlineStr">
+        <is>
+          <t>5000.0</t>
+        </is>
+      </c>
+      <c r="P76" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q76" s="2" t="inlineStr">
+        <is>
+          <t>D+02 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
@@ -5719,12 +6943,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-capital-protegido-ibovespa-ciclico-1-multimercado</t>
         </is>
       </c>
-      <c r="L77" s="4" t="inlineStr"/>
-      <c r="M77" s="4" t="inlineStr"/>
-      <c r="N77" s="4" t="inlineStr"/>
-      <c r="O77" s="4" t="inlineStr"/>
-      <c r="P77" s="4" t="inlineStr"/>
-      <c r="Q77" s="4" t="inlineStr"/>
+      <c r="L77" s="4" t="inlineStr">
+        <is>
+          <t>14.239.659/0001-00</t>
+        </is>
+      </c>
+      <c r="M77" s="4" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="N77" s="4" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+      <c r="O77" s="4" t="inlineStr">
+        <is>
+          <t>5000.0</t>
+        </is>
+      </c>
+      <c r="P77" s="4" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q77" s="4" t="inlineStr">
+        <is>
+          <t>D+03 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -5782,12 +7030,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-capital-protegido-ciclico-ii-multimercado-lp/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L78" s="2" t="inlineStr"/>
-      <c r="M78" s="2" t="inlineStr"/>
-      <c r="N78" s="2" t="inlineStr"/>
-      <c r="O78" s="2" t="inlineStr"/>
-      <c r="P78" s="2" t="inlineStr"/>
-      <c r="Q78" s="2" t="inlineStr"/>
+      <c r="L78" s="2" t="inlineStr">
+        <is>
+          <t>45.443.651/0001-94</t>
+        </is>
+      </c>
+      <c r="M78" s="2" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="N78" s="2" t="inlineStr">
+        <is>
+          <t>0.9</t>
+        </is>
+      </c>
+      <c r="O78" s="2" t="inlineStr">
+        <is>
+          <t>5000.0</t>
+        </is>
+      </c>
+      <c r="P78" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q78" s="2" t="inlineStr">
+        <is>
+          <t>D+02 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
@@ -5845,12 +7117,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/multimercado/caixa-expert-pimco-income-ie-fic-multimercado/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L79" s="4" t="inlineStr"/>
-      <c r="M79" s="4" t="inlineStr"/>
-      <c r="N79" s="4" t="inlineStr"/>
-      <c r="O79" s="4" t="inlineStr"/>
-      <c r="P79" s="4" t="inlineStr"/>
-      <c r="Q79" s="4" t="inlineStr"/>
+      <c r="L79" s="4" t="inlineStr">
+        <is>
+          <t>51.659.921/0001-00</t>
+        </is>
+      </c>
+      <c r="M79" s="4" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N79" s="4" t="inlineStr">
+        <is>
+          <t>0.93</t>
+        </is>
+      </c>
+      <c r="O79" s="4" t="inlineStr">
+        <is>
+          <t>10000.0</t>
+        </is>
+      </c>
+      <c r="P79" s="4" t="inlineStr">
+        <is>
+          <t>D+3 (du)</t>
+        </is>
+      </c>
+      <c r="Q79" s="4" t="inlineStr">
+        <is>
+          <t>D+08 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -5908,12 +7204,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/multimercado/expert-giant-zarathustra-fic-multimercado</t>
         </is>
       </c>
-      <c r="L80" s="2" t="inlineStr"/>
-      <c r="M80" s="2" t="inlineStr"/>
-      <c r="N80" s="2" t="inlineStr"/>
-      <c r="O80" s="2" t="inlineStr"/>
-      <c r="P80" s="2" t="inlineStr"/>
-      <c r="Q80" s="2" t="inlineStr"/>
+      <c r="L80" s="2" t="inlineStr">
+        <is>
+          <t>40.209.061/0001-88</t>
+        </is>
+      </c>
+      <c r="M80" s="2" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N80" s="2" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="O80" s="2" t="inlineStr">
+        <is>
+          <t>10000.0</t>
+        </is>
+      </c>
+      <c r="P80" s="2" t="inlineStr">
+        <is>
+          <t>D+22 (du)</t>
+        </is>
+      </c>
+      <c r="Q80" s="2" t="inlineStr">
+        <is>
+          <t>D+25 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
@@ -5971,12 +7291,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-alocacao-macro-multimercado-longo-prazo/</t>
         </is>
       </c>
-      <c r="L81" s="4" t="inlineStr"/>
-      <c r="M81" s="4" t="inlineStr"/>
-      <c r="N81" s="4" t="inlineStr"/>
-      <c r="O81" s="4" t="inlineStr"/>
-      <c r="P81" s="4" t="inlineStr"/>
-      <c r="Q81" s="4" t="inlineStr"/>
+      <c r="L81" s="4" t="inlineStr">
+        <is>
+          <t>08.070.841/0001-87</t>
+        </is>
+      </c>
+      <c r="M81" s="4" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N81" s="4" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="O81" s="4" t="inlineStr">
+        <is>
+          <t>10000.0</t>
+        </is>
+      </c>
+      <c r="P81" s="4" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q81" s="4" t="inlineStr">
+        <is>
+          <t>D+03 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -6121,12 +7465,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/multimercado/btg-pactual-x10-multimercado-longo-prazo/</t>
         </is>
       </c>
-      <c r="L83" s="4" t="inlineStr"/>
-      <c r="M83" s="4" t="inlineStr"/>
-      <c r="N83" s="4" t="inlineStr"/>
-      <c r="O83" s="4" t="inlineStr"/>
-      <c r="P83" s="4" t="inlineStr"/>
-      <c r="Q83" s="4" t="inlineStr"/>
+      <c r="L83" s="4" t="inlineStr">
+        <is>
+          <t>17.433.039/0001-03</t>
+        </is>
+      </c>
+      <c r="M83" s="4" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N83" s="4" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="O83" s="4" t="inlineStr">
+        <is>
+          <t>10000.0</t>
+        </is>
+      </c>
+      <c r="P83" s="4" t="inlineStr">
+        <is>
+          <t>D+8 (du)</t>
+        </is>
+      </c>
+      <c r="Q83" s="4" t="inlineStr">
+        <is>
+          <t>D+10 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -6184,12 +7552,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-caixa-expert-spxmm/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L84" s="2" t="inlineStr"/>
-      <c r="M84" s="2" t="inlineStr"/>
-      <c r="N84" s="2" t="inlineStr"/>
-      <c r="O84" s="2" t="inlineStr"/>
-      <c r="P84" s="2" t="inlineStr"/>
-      <c r="Q84" s="2" t="inlineStr"/>
+      <c r="L84" s="2" t="inlineStr">
+        <is>
+          <t>34.660.453/0001-66</t>
+        </is>
+      </c>
+      <c r="M84" s="2" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N84" s="2" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="O84" s="2" t="inlineStr">
+        <is>
+          <t>10000.0</t>
+        </is>
+      </c>
+      <c r="P84" s="2" t="inlineStr">
+        <is>
+          <t>D+22 (du)</t>
+        </is>
+      </c>
+      <c r="Q84" s="2" t="inlineStr">
+        <is>
+          <t>D+24 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
@@ -6421,12 +7813,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/fi-acoes-brasil-etf-bovespa/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L87" s="4" t="inlineStr"/>
-      <c r="M87" s="4" t="inlineStr"/>
-      <c r="N87" s="4" t="inlineStr"/>
-      <c r="O87" s="4" t="inlineStr"/>
-      <c r="P87" s="4" t="inlineStr"/>
-      <c r="Q87" s="4" t="inlineStr"/>
+      <c r="L87" s="4" t="inlineStr">
+        <is>
+          <t>01.525.057/0001-77</t>
+        </is>
+      </c>
+      <c r="M87" s="4" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N87" s="4" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="O87" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P87" s="4" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q87" s="4" t="inlineStr">
+        <is>
+          <t>D+03 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -6480,12 +7896,36 @@
         </is>
       </c>
       <c r="K88" s="2" t="inlineStr"/>
-      <c r="L88" s="2" t="inlineStr"/>
-      <c r="M88" s="2" t="inlineStr"/>
-      <c r="N88" s="2" t="inlineStr"/>
-      <c r="O88" s="2" t="inlineStr"/>
-      <c r="P88" s="2" t="inlineStr"/>
-      <c r="Q88" s="2" t="inlineStr"/>
+      <c r="L88" s="2" t="inlineStr">
+        <is>
+          <t>35.536.497/0001-41</t>
+        </is>
+      </c>
+      <c r="M88" s="2" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N88" s="2" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="O88" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P88" s="2" t="inlineStr">
+        <is>
+          <t>D+13 (du)</t>
+        </is>
+      </c>
+      <c r="Q88" s="2" t="inlineStr">
+        <is>
+          <t>D+15 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
@@ -7065,12 +8505,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/fic-fia-multigestor/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L95" s="4" t="inlineStr"/>
-      <c r="M95" s="4" t="inlineStr"/>
-      <c r="N95" s="4" t="inlineStr"/>
-      <c r="O95" s="4" t="inlineStr"/>
-      <c r="P95" s="4" t="inlineStr"/>
-      <c r="Q95" s="4" t="inlineStr"/>
+      <c r="L95" s="4" t="inlineStr">
+        <is>
+          <t>30.068.224/0001-04</t>
+        </is>
+      </c>
+      <c r="M95" s="4" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N95" s="4" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="O95" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P95" s="4" t="inlineStr">
+        <is>
+          <t>D+23 (du)</t>
+        </is>
+      </c>
+      <c r="Q95" s="4" t="inlineStr">
+        <is>
+          <t>D+25 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -7650,12 +9114,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/fia-caixa-seguridade/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L102" s="2" t="inlineStr"/>
-      <c r="M102" s="2" t="inlineStr"/>
-      <c r="N102" s="2" t="inlineStr"/>
-      <c r="O102" s="2" t="inlineStr"/>
-      <c r="P102" s="2" t="inlineStr"/>
-      <c r="Q102" s="2" t="inlineStr"/>
+      <c r="L102" s="2" t="inlineStr">
+        <is>
+          <t>30.068.049/0001-47</t>
+        </is>
+      </c>
+      <c r="M102" s="2" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N102" s="2" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="O102" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P102" s="2" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q102" s="2" t="inlineStr">
+        <is>
+          <t>D+03 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
@@ -8583,12 +10071,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/CAIXA-Expert-Verde-Am-Long-Bias-FIC-Acoes/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L113" s="4" t="inlineStr"/>
-      <c r="M113" s="4" t="inlineStr"/>
-      <c r="N113" s="4" t="inlineStr"/>
-      <c r="O113" s="4" t="inlineStr"/>
-      <c r="P113" s="4" t="inlineStr"/>
-      <c r="Q113" s="4" t="inlineStr"/>
+      <c r="L113" s="4" t="inlineStr">
+        <is>
+          <t>30.068.071/0001-97</t>
+        </is>
+      </c>
+      <c r="M113" s="4" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N113" s="4" t="inlineStr">
+        <is>
+          <t>0.7</t>
+        </is>
+      </c>
+      <c r="O113" s="4" t="inlineStr">
+        <is>
+          <t>10000.0</t>
+        </is>
+      </c>
+      <c r="P113" s="4" t="inlineStr">
+        <is>
+          <t>D+22 (du)</t>
+        </is>
+      </c>
+      <c r="Q113" s="4" t="inlineStr">
+        <is>
+          <t>D+24 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -8646,12 +10158,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/caixa-expert-claritas-valor-fic-acoes/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L114" s="2" t="inlineStr"/>
-      <c r="M114" s="2" t="inlineStr"/>
-      <c r="N114" s="2" t="inlineStr"/>
-      <c r="O114" s="2" t="inlineStr"/>
-      <c r="P114" s="2" t="inlineStr"/>
-      <c r="Q114" s="2" t="inlineStr"/>
+      <c r="L114" s="2" t="inlineStr">
+        <is>
+          <t>30.068.060/0001-07</t>
+        </is>
+      </c>
+      <c r="M114" s="2" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N114" s="2" t="inlineStr">
+        <is>
+          <t>0.6</t>
+        </is>
+      </c>
+      <c r="O114" s="2" t="inlineStr">
+        <is>
+          <t>10000.0</t>
+        </is>
+      </c>
+      <c r="P114" s="2" t="inlineStr">
+        <is>
+          <t>D+23 (du)</t>
+        </is>
+      </c>
+      <c r="Q114" s="2" t="inlineStr">
+        <is>
+          <t>D+25 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="4" t="inlineStr">
@@ -8767,13 +10303,41 @@
           <t>PF</t>
         </is>
       </c>
-      <c r="K116" s="2" t="inlineStr"/>
-      <c r="L116" s="2" t="inlineStr"/>
-      <c r="M116" s="2" t="inlineStr"/>
-      <c r="N116" s="2" t="inlineStr"/>
-      <c r="O116" s="2" t="inlineStr"/>
-      <c r="P116" s="2" t="inlineStr"/>
-      <c r="Q116" s="2" t="inlineStr"/>
+      <c r="K116" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/mutuos-privatizacao/fmp-fgts-eletrobras-migracao</t>
+        </is>
+      </c>
+      <c r="L116" s="2" t="inlineStr">
+        <is>
+          <t>45.443.366/0001-73</t>
+        </is>
+      </c>
+      <c r="M116" s="2" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N116" s="2" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="O116" s="2" t="inlineStr">
+        <is>
+          <t>200.0</t>
+        </is>
+      </c>
+      <c r="P116" s="2" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q116" s="2" t="inlineStr">
+        <is>
+          <t>D+05 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="4" t="inlineStr">
@@ -9000,13 +10564,41 @@
           <t>PF</t>
         </is>
       </c>
-      <c r="K119" s="4" t="inlineStr"/>
-      <c r="L119" s="4" t="inlineStr"/>
-      <c r="M119" s="4" t="inlineStr"/>
-      <c r="N119" s="4" t="inlineStr"/>
-      <c r="O119" s="4" t="inlineStr"/>
-      <c r="P119" s="4" t="inlineStr"/>
-      <c r="Q119" s="4" t="inlineStr"/>
+      <c r="K119" s="4" t="inlineStr">
+        <is>
+          <t>http://www.caixa.gov.br/fundos-investimento/mutuos-privatizacao/fmp-fgts-vale-do-rio-doce-2</t>
+        </is>
+      </c>
+      <c r="L119" s="4" t="inlineStr">
+        <is>
+          <t>04.885.824/0001-47</t>
+        </is>
+      </c>
+      <c r="M119" s="4" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N119" s="4" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="O119" s="4" t="inlineStr">
+        <is>
+          <t>10000.0</t>
+        </is>
+      </c>
+      <c r="P119" s="4" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q119" s="4" t="inlineStr">
+        <is>
+          <t>D+05 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -9146,13 +10738,41 @@
           <t>PF</t>
         </is>
       </c>
-      <c r="K121" s="4" t="inlineStr"/>
-      <c r="L121" s="4" t="inlineStr"/>
-      <c r="M121" s="4" t="inlineStr"/>
-      <c r="N121" s="4" t="inlineStr"/>
-      <c r="O121" s="4" t="inlineStr"/>
-      <c r="P121" s="4" t="inlineStr"/>
-      <c r="Q121" s="4" t="inlineStr"/>
+      <c r="K121" s="4" t="inlineStr">
+        <is>
+          <t>http://www.caixa.gov.br/fundos-investimento/mutuos-privatizacao/fmp-fgts-vale-do-rio-doce-migracao</t>
+        </is>
+      </c>
+      <c r="L121" s="4" t="inlineStr">
+        <is>
+          <t>04.885.832/0001-93</t>
+        </is>
+      </c>
+      <c r="M121" s="4" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N121" s="4" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="O121" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P121" s="4" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q121" s="4" t="inlineStr">
+        <is>
+          <t>D+05 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -9292,13 +10912,41 @@
           <t>PF</t>
         </is>
       </c>
-      <c r="K123" s="4" t="inlineStr"/>
-      <c r="L123" s="4" t="inlineStr"/>
-      <c r="M123" s="4" t="inlineStr"/>
-      <c r="N123" s="4" t="inlineStr"/>
-      <c r="O123" s="4" t="inlineStr"/>
-      <c r="P123" s="4" t="inlineStr"/>
-      <c r="Q123" s="4" t="inlineStr"/>
+      <c r="K123" s="4" t="inlineStr">
+        <is>
+          <t>http://www.caixa.gov.br/fundos-investimento/mutuos-privatizacao/fmp-fgts-vale-do-rio-doce-2</t>
+        </is>
+      </c>
+      <c r="L123" s="4" t="inlineStr">
+        <is>
+          <t>04.885.824/0001-47</t>
+        </is>
+      </c>
+      <c r="M123" s="4" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N123" s="4" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="O123" s="4" t="inlineStr">
+        <is>
+          <t>10000.0</t>
+        </is>
+      </c>
+      <c r="P123" s="4" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q123" s="4" t="inlineStr">
+        <is>
+          <t>D+05 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -9443,12 +11091,36 @@
           <t>http://site.extra.caixa.gov.br/fundos-investimento/fundo-simples/fic-azulzinha-rf-simples/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L125" s="4" t="inlineStr"/>
-      <c r="M125" s="4" t="inlineStr"/>
-      <c r="N125" s="4" t="inlineStr"/>
-      <c r="O125" s="4" t="inlineStr"/>
-      <c r="P125" s="4" t="inlineStr"/>
-      <c r="Q125" s="4" t="inlineStr"/>
+      <c r="L125" s="4" t="inlineStr">
+        <is>
+          <t>61.160.298/0001-91</t>
+        </is>
+      </c>
+      <c r="M125" s="4" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="N125" s="4" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="O125" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P125" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q125" s="4" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -10004,12 +11676,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/empresa/renda-fixa/credito-privado/caixa-fi-diamante-corporativo-rf-cred-priv-lp</t>
         </is>
       </c>
-      <c r="L132" s="2" t="inlineStr"/>
-      <c r="M132" s="2" t="inlineStr"/>
-      <c r="N132" s="2" t="inlineStr"/>
-      <c r="O132" s="2" t="inlineStr"/>
-      <c r="P132" s="2" t="inlineStr"/>
-      <c r="Q132" s="2" t="inlineStr"/>
+      <c r="L132" s="2" t="inlineStr">
+        <is>
+          <t>29.157.520/0001-94</t>
+        </is>
+      </c>
+      <c r="M132" s="2" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="N132" s="2" t="inlineStr">
+        <is>
+          <t>0.12</t>
+        </is>
+      </c>
+      <c r="O132" s="2" t="inlineStr">
+        <is>
+          <t>1000000.0</t>
+        </is>
+      </c>
+      <c r="P132" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q132" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="4" t="inlineStr">
@@ -10154,12 +11850,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-institucional-soberano-plus-rf-lp/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L134" s="2" t="inlineStr"/>
-      <c r="M134" s="2" t="inlineStr"/>
-      <c r="N134" s="2" t="inlineStr"/>
-      <c r="O134" s="2" t="inlineStr"/>
-      <c r="P134" s="2" t="inlineStr"/>
-      <c r="Q134" s="2" t="inlineStr"/>
+      <c r="L134" s="2" t="inlineStr">
+        <is>
+          <t>42.196.029/0001-30</t>
+        </is>
+      </c>
+      <c r="M134" s="2" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N134" s="2" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="O134" s="2" t="inlineStr">
+        <is>
+          <t>5000000.0</t>
+        </is>
+      </c>
+      <c r="P134" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q134" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="4" t="inlineStr">
@@ -10304,12 +12024,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/empresa/renda-fixa/fi-cni-rf-longo-prazo/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L136" s="2" t="inlineStr"/>
-      <c r="M136" s="2" t="inlineStr"/>
-      <c r="N136" s="2" t="inlineStr"/>
-      <c r="O136" s="2" t="inlineStr"/>
-      <c r="P136" s="2" t="inlineStr"/>
-      <c r="Q136" s="2" t="inlineStr"/>
+      <c r="L136" s="2" t="inlineStr">
+        <is>
+          <t>05.164.366/0001-10</t>
+        </is>
+      </c>
+      <c r="M136" s="2" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N136" s="2" t="inlineStr">
+        <is>
+          <t>0.07</t>
+        </is>
+      </c>
+      <c r="O136" s="2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="P136" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q136" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="4" t="inlineStr">
@@ -10450,12 +12194,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/referenciados/fic-giro-mpe-ref-di-longo-prazo/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L138" s="2" t="inlineStr"/>
-      <c r="M138" s="2" t="inlineStr"/>
-      <c r="N138" s="2" t="inlineStr"/>
-      <c r="O138" s="2" t="inlineStr"/>
-      <c r="P138" s="2" t="inlineStr"/>
-      <c r="Q138" s="2" t="inlineStr"/>
+      <c r="L138" s="2" t="inlineStr">
+        <is>
+          <t>10.551.370/0001-70</t>
+        </is>
+      </c>
+      <c r="M138" s="2" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="N138" s="2" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="O138" s="2" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="P138" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q138" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="4" t="inlineStr">
@@ -10513,12 +12281,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/referenciados/fic-topazio-rf-ref-di-lp/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L139" s="4" t="inlineStr"/>
-      <c r="M139" s="4" t="inlineStr"/>
-      <c r="N139" s="4" t="inlineStr"/>
-      <c r="O139" s="4" t="inlineStr"/>
-      <c r="P139" s="4" t="inlineStr"/>
-      <c r="Q139" s="4" t="inlineStr"/>
+      <c r="L139" s="4" t="inlineStr">
+        <is>
+          <t>11.061.230/0001-87</t>
+        </is>
+      </c>
+      <c r="M139" s="4" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="N139" s="4" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="O139" s="4" t="inlineStr">
+        <is>
+          <t>1000000.0</t>
+        </is>
+      </c>
+      <c r="P139" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q139" s="4" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -10576,12 +12368,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/referenciados/fic-esmeralda-corp-ref-di/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L140" s="2" t="inlineStr"/>
-      <c r="M140" s="2" t="inlineStr"/>
-      <c r="N140" s="2" t="inlineStr"/>
-      <c r="O140" s="2" t="inlineStr"/>
-      <c r="P140" s="2" t="inlineStr"/>
-      <c r="Q140" s="2" t="inlineStr"/>
+      <c r="L140" s="2" t="inlineStr">
+        <is>
+          <t>52.699.555/0001-77</t>
+        </is>
+      </c>
+      <c r="M140" s="2" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="N140" s="2" t="inlineStr">
+        <is>
+          <t>0.12</t>
+        </is>
+      </c>
+      <c r="O140" s="2" t="inlineStr">
+        <is>
+          <t>1000000.0</t>
+        </is>
+      </c>
+      <c r="P140" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q140" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="4" t="inlineStr">
@@ -10639,12 +12455,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/voce/renda-fixa/fic-turquesa-corporativo-curto-prazo</t>
         </is>
       </c>
-      <c r="L141" s="4" t="inlineStr"/>
-      <c r="M141" s="4" t="inlineStr"/>
-      <c r="N141" s="4" t="inlineStr"/>
-      <c r="O141" s="4" t="inlineStr"/>
-      <c r="P141" s="4" t="inlineStr"/>
-      <c r="Q141" s="4" t="inlineStr"/>
+      <c r="L141" s="4" t="inlineStr">
+        <is>
+          <t>30.068.141/0001-07</t>
+        </is>
+      </c>
+      <c r="M141" s="4" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="N141" s="4" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="O141" s="4" t="inlineStr">
+        <is>
+          <t>3000000.0</t>
+        </is>
+      </c>
+      <c r="P141" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q141" s="4" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -10702,12 +12542,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/curto-prazo/fic-automatico-polis-rf-cp/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L142" s="2" t="inlineStr"/>
-      <c r="M142" s="2" t="inlineStr"/>
-      <c r="N142" s="2" t="inlineStr"/>
-      <c r="O142" s="2" t="inlineStr"/>
-      <c r="P142" s="2" t="inlineStr"/>
-      <c r="Q142" s="2" t="inlineStr"/>
+      <c r="L142" s="2" t="inlineStr">
+        <is>
+          <t>50.803.936/0001-29</t>
+        </is>
+      </c>
+      <c r="M142" s="2" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="N142" s="2" t="inlineStr">
+        <is>
+          <t>1.7</t>
+        </is>
+      </c>
+      <c r="O142" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P142" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q142" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="4" t="inlineStr">
@@ -10765,12 +12629,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/curto-prazo/fic-pratico-curto-prazo</t>
         </is>
       </c>
-      <c r="L143" s="4" t="inlineStr"/>
-      <c r="M143" s="4" t="inlineStr"/>
-      <c r="N143" s="4" t="inlineStr"/>
-      <c r="O143" s="4" t="inlineStr"/>
-      <c r="P143" s="4" t="inlineStr"/>
-      <c r="Q143" s="4" t="inlineStr"/>
+      <c r="L143" s="4" t="inlineStr">
+        <is>
+          <t>00.834.074/0001-23</t>
+        </is>
+      </c>
+      <c r="M143" s="4" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="N143" s="4" t="inlineStr">
+        <is>
+          <t>1.7</t>
+        </is>
+      </c>
+      <c r="O143" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P143" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q143" s="4" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -10891,12 +12779,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fi-brasil-matriz-rf/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L145" s="4" t="inlineStr"/>
-      <c r="M145" s="4" t="inlineStr"/>
-      <c r="N145" s="4" t="inlineStr"/>
-      <c r="O145" s="4" t="inlineStr"/>
-      <c r="P145" s="4" t="inlineStr"/>
-      <c r="Q145" s="4" t="inlineStr"/>
+      <c r="L145" s="4" t="inlineStr">
+        <is>
+          <t>23.215.008/0001-70</t>
+        </is>
+      </c>
+      <c r="M145" s="4" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="N145" s="4" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="O145" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P145" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q145" s="4" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -10954,12 +12866,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/caixa-fic-brasil-gestao-estrategica-rf</t>
         </is>
       </c>
-      <c r="L146" s="2" t="inlineStr"/>
-      <c r="M146" s="2" t="inlineStr"/>
-      <c r="N146" s="2" t="inlineStr"/>
-      <c r="O146" s="2" t="inlineStr"/>
-      <c r="P146" s="2" t="inlineStr"/>
-      <c r="Q146" s="2" t="inlineStr"/>
+      <c r="L146" s="2" t="inlineStr">
+        <is>
+          <t>23.215.097/0001-55</t>
+        </is>
+      </c>
+      <c r="M146" s="2" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N146" s="2" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="O146" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P146" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q146" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="4" t="inlineStr">
@@ -11104,12 +13040,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/brasil-IPCA/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L148" s="2" t="inlineStr"/>
-      <c r="M148" s="2" t="inlineStr"/>
-      <c r="N148" s="2" t="inlineStr"/>
-      <c r="O148" s="2" t="inlineStr"/>
-      <c r="P148" s="2" t="inlineStr"/>
-      <c r="Q148" s="2" t="inlineStr"/>
+      <c r="L148" s="2" t="inlineStr">
+        <is>
+          <t>35.536.532/0001-22</t>
+        </is>
+      </c>
+      <c r="M148" s="2" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N148" s="2" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="O148" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P148" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q148" s="2" t="inlineStr">
+        <is>
+          <t>D+01 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="4" t="inlineStr">
@@ -11167,12 +13127,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fi-brasil-irfm-1-titulos-publicos-rf</t>
         </is>
       </c>
-      <c r="L149" s="4" t="inlineStr"/>
-      <c r="M149" s="4" t="inlineStr"/>
-      <c r="N149" s="4" t="inlineStr"/>
-      <c r="O149" s="4" t="inlineStr"/>
-      <c r="P149" s="4" t="inlineStr"/>
-      <c r="Q149" s="4" t="inlineStr"/>
+      <c r="L149" s="4" t="inlineStr">
+        <is>
+          <t>10.740.670/0001-06</t>
+        </is>
+      </c>
+      <c r="M149" s="4" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="N149" s="4" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="O149" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P149" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q149" s="4" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -11293,12 +13277,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/brasil-irf-m-titulos-publicos-renda-fixa-longo-prazo</t>
         </is>
       </c>
-      <c r="L151" s="4" t="inlineStr"/>
-      <c r="M151" s="4" t="inlineStr"/>
-      <c r="N151" s="4" t="inlineStr"/>
-      <c r="O151" s="4" t="inlineStr"/>
-      <c r="P151" s="4" t="inlineStr"/>
-      <c r="Q151" s="4" t="inlineStr"/>
+      <c r="L151" s="4" t="inlineStr">
+        <is>
+          <t>10.740.670/0001-06</t>
+        </is>
+      </c>
+      <c r="M151" s="4" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="N151" s="4" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="O151" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P151" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q151" s="4" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -11356,12 +13364,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fi-brasil-ima-b-titulos-rf-longo-prazo</t>
         </is>
       </c>
-      <c r="L152" s="2" t="inlineStr"/>
-      <c r="M152" s="2" t="inlineStr"/>
-      <c r="N152" s="2" t="inlineStr"/>
-      <c r="O152" s="2" t="inlineStr"/>
-      <c r="P152" s="2" t="inlineStr"/>
-      <c r="Q152" s="2" t="inlineStr"/>
+      <c r="L152" s="2" t="inlineStr">
+        <is>
+          <t>10.740.658/0001-93</t>
+        </is>
+      </c>
+      <c r="M152" s="2" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N152" s="2" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="O152" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P152" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q152" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="4" t="inlineStr">
@@ -11419,12 +13451,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fi-brasil-ima-b-5-titulos-publicos-rf-longo-prazo</t>
         </is>
       </c>
-      <c r="L153" s="4" t="inlineStr"/>
-      <c r="M153" s="4" t="inlineStr"/>
-      <c r="N153" s="4" t="inlineStr"/>
-      <c r="O153" s="4" t="inlineStr"/>
-      <c r="P153" s="4" t="inlineStr"/>
-      <c r="Q153" s="4" t="inlineStr"/>
+      <c r="L153" s="4" t="inlineStr">
+        <is>
+          <t>10.740.658/0001-93</t>
+        </is>
+      </c>
+      <c r="M153" s="4" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N153" s="4" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="O153" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P153" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q153" s="4" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -11482,12 +13538,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fi-brasil-ima-geral-tp-rf-longo-prazo</t>
         </is>
       </c>
-      <c r="L154" s="2" t="inlineStr"/>
-      <c r="M154" s="2" t="inlineStr"/>
-      <c r="N154" s="2" t="inlineStr"/>
-      <c r="O154" s="2" t="inlineStr"/>
-      <c r="P154" s="2" t="inlineStr"/>
-      <c r="Q154" s="2" t="inlineStr"/>
+      <c r="L154" s="2" t="inlineStr">
+        <is>
+          <t>11.061.217/0001-28</t>
+        </is>
+      </c>
+      <c r="M154" s="2" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N154" s="2" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="O154" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P154" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q154" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="4" t="inlineStr">
@@ -11608,12 +13688,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fi-brasil-ima-b-5_mais-titulos-publicos-rf-lp/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L156" s="2" t="inlineStr"/>
-      <c r="M156" s="2" t="inlineStr"/>
-      <c r="N156" s="2" t="inlineStr"/>
-      <c r="O156" s="2" t="inlineStr"/>
-      <c r="P156" s="2" t="inlineStr"/>
-      <c r="Q156" s="2" t="inlineStr"/>
+      <c r="L156" s="2" t="inlineStr">
+        <is>
+          <t>10.740.658/0001-93</t>
+        </is>
+      </c>
+      <c r="M156" s="2" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N156" s="2" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="O156" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P156" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q156" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="4" t="inlineStr">
@@ -11671,12 +13775,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fi-brasil-irfm-1-titulos-publicos-rf-longo-prazo/</t>
         </is>
       </c>
-      <c r="L157" s="4" t="inlineStr"/>
-      <c r="M157" s="4" t="inlineStr"/>
-      <c r="N157" s="4" t="inlineStr"/>
-      <c r="O157" s="4" t="inlineStr"/>
-      <c r="P157" s="4" t="inlineStr"/>
-      <c r="Q157" s="4" t="inlineStr"/>
+      <c r="L157" s="4" t="inlineStr">
+        <is>
+          <t>10.740.670/0001-06</t>
+        </is>
+      </c>
+      <c r="M157" s="4" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="N157" s="4" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="O157" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P157" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q157" s="4" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -11734,12 +13862,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fi-brasil-titulos-publicos-rf-longo-prazo</t>
         </is>
       </c>
-      <c r="L158" s="2" t="inlineStr"/>
-      <c r="M158" s="2" t="inlineStr"/>
-      <c r="N158" s="2" t="inlineStr"/>
-      <c r="O158" s="2" t="inlineStr"/>
-      <c r="P158" s="2" t="inlineStr"/>
-      <c r="Q158" s="2" t="inlineStr"/>
+      <c r="L158" s="2" t="inlineStr">
+        <is>
+          <t>05.164.356/0001-84</t>
+        </is>
+      </c>
+      <c r="M158" s="2" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="N158" s="2" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="O158" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P158" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q158" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="4" t="inlineStr">
@@ -11797,12 +13949,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-alianca-rf</t>
         </is>
       </c>
-      <c r="L159" s="4" t="inlineStr"/>
-      <c r="M159" s="4" t="inlineStr"/>
-      <c r="N159" s="4" t="inlineStr"/>
-      <c r="O159" s="4" t="inlineStr"/>
-      <c r="P159" s="4" t="inlineStr"/>
-      <c r="Q159" s="4" t="inlineStr"/>
+      <c r="L159" s="4" t="inlineStr">
+        <is>
+          <t>05.164.358/0001-73</t>
+        </is>
+      </c>
+      <c r="M159" s="4" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="N159" s="4" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="O159" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P159" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q159" s="4" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -11947,12 +14123,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/brasil-disponibilidades</t>
         </is>
       </c>
-      <c r="L161" s="4" t="inlineStr"/>
-      <c r="M161" s="4" t="inlineStr"/>
-      <c r="N161" s="4" t="inlineStr"/>
-      <c r="O161" s="4" t="inlineStr"/>
-      <c r="P161" s="4" t="inlineStr"/>
-      <c r="Q161" s="4" t="inlineStr"/>
+      <c r="L161" s="4" t="inlineStr">
+        <is>
+          <t>14.508.643/0001-55</t>
+        </is>
+      </c>
+      <c r="M161" s="4" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="N161" s="4" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="O161" s="4" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
+      <c r="P161" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q161" s="4" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -12073,12 +14273,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-novo-brasil-ima-b-rf-longo-prazo</t>
         </is>
       </c>
-      <c r="L163" s="4" t="inlineStr"/>
-      <c r="M163" s="4" t="inlineStr"/>
-      <c r="N163" s="4" t="inlineStr"/>
-      <c r="O163" s="4" t="inlineStr"/>
-      <c r="P163" s="4" t="inlineStr"/>
-      <c r="Q163" s="4" t="inlineStr"/>
+      <c r="L163" s="4" t="inlineStr">
+        <is>
+          <t>10.646.895/0001-90</t>
+        </is>
+      </c>
+      <c r="M163" s="4" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N163" s="4" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="O163" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P163" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Q163" s="4" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -12136,12 +14360,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/multimercado/estrategia-livre-mm-lp/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L164" s="2" t="inlineStr"/>
-      <c r="M164" s="2" t="inlineStr"/>
-      <c r="N164" s="2" t="inlineStr"/>
-      <c r="O164" s="2" t="inlineStr"/>
-      <c r="P164" s="2" t="inlineStr"/>
-      <c r="Q164" s="2" t="inlineStr"/>
+      <c r="L164" s="2" t="inlineStr">
+        <is>
+          <t>34.660.276/0001-18</t>
+        </is>
+      </c>
+      <c r="M164" s="2" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="N164" s="2" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="O164" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P164" s="2" t="inlineStr">
+        <is>
+          <t>D+13 (du)</t>
+        </is>
+      </c>
+      <c r="Q164" s="2" t="inlineStr">
+        <is>
+          <t>D+15 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="4" t="inlineStr">
@@ -12199,12 +14447,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/fi-acoes-brasil-ibovespa/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L165" s="4" t="inlineStr"/>
-      <c r="M165" s="4" t="inlineStr"/>
-      <c r="N165" s="4" t="inlineStr"/>
-      <c r="O165" s="4" t="inlineStr"/>
-      <c r="P165" s="4" t="inlineStr"/>
-      <c r="Q165" s="4" t="inlineStr"/>
+      <c r="L165" s="4" t="inlineStr">
+        <is>
+          <t>13.058.816/0001-18</t>
+        </is>
+      </c>
+      <c r="M165" s="4" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N165" s="4" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="O165" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P165" s="4" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q165" s="4" t="inlineStr">
+        <is>
+          <t>D+03 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
@@ -12262,12 +14534,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/fi-acoes-brasil-etf-bovespa</t>
         </is>
       </c>
-      <c r="L166" s="2" t="inlineStr"/>
-      <c r="M166" s="2" t="inlineStr"/>
-      <c r="N166" s="2" t="inlineStr"/>
-      <c r="O166" s="2" t="inlineStr"/>
-      <c r="P166" s="2" t="inlineStr"/>
-      <c r="Q166" s="2" t="inlineStr"/>
+      <c r="L166" s="2" t="inlineStr">
+        <is>
+          <t>15.154.236/0001-50</t>
+        </is>
+      </c>
+      <c r="M166" s="2" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N166" s="2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="O166" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P166" s="2" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q166" s="2" t="inlineStr">
+        <is>
+          <t>D+03 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="4" t="inlineStr">
@@ -12325,12 +14621,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/FIA-Institucional-BDR-nivel-I/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L167" s="4" t="inlineStr"/>
-      <c r="M167" s="4" t="inlineStr"/>
-      <c r="N167" s="4" t="inlineStr"/>
-      <c r="O167" s="4" t="inlineStr"/>
-      <c r="P167" s="4" t="inlineStr"/>
-      <c r="Q167" s="4" t="inlineStr"/>
+      <c r="L167" s="4" t="inlineStr">
+        <is>
+          <t>17.502.937/0001-68</t>
+        </is>
+      </c>
+      <c r="M167" s="4" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N167" s="4" t="inlineStr">
+        <is>
+          <t>0.7</t>
+        </is>
+      </c>
+      <c r="O167" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P167" s="4" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q167" s="4" t="inlineStr">
+        <is>
+          <t>D+03 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
@@ -12388,12 +14708,36 @@
           <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/fi-acoes-brasil-ibx-50</t>
         </is>
       </c>
-      <c r="L168" s="2" t="inlineStr"/>
-      <c r="M168" s="2" t="inlineStr"/>
-      <c r="N168" s="2" t="inlineStr"/>
-      <c r="O168" s="2" t="inlineStr"/>
-      <c r="P168" s="2" t="inlineStr"/>
-      <c r="Q168" s="2" t="inlineStr"/>
+      <c r="L168" s="2" t="inlineStr">
+        <is>
+          <t>03.737.217/0001-77</t>
+        </is>
+      </c>
+      <c r="M168" s="2" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N168" s="2" t="inlineStr">
+        <is>
+          <t>0.7</t>
+        </is>
+      </c>
+      <c r="O168" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P168" s="2" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="Q168" s="2" t="inlineStr">
+        <is>
+          <t>D+03 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="4" t="inlineStr">
@@ -12446,13 +14790,41 @@
           <t>RPPS</t>
         </is>
       </c>
-      <c r="K169" s="4" t="inlineStr"/>
-      <c r="L169" s="4" t="inlineStr"/>
-      <c r="M169" s="4" t="inlineStr"/>
-      <c r="N169" s="4" t="inlineStr"/>
-      <c r="O169" s="4" t="inlineStr"/>
-      <c r="P169" s="4" t="inlineStr"/>
-      <c r="Q169" s="4" t="inlineStr"/>
+      <c r="K169" s="4" t="inlineStr">
+        <is>
+          <t>http://www.caixa.gov.br/fundos-investimento/fundos-de-acoes/FIC-FIA-Brasil-Acoes-Livres/Paginas/default.aspx</t>
+        </is>
+      </c>
+      <c r="L169" s="4" t="inlineStr">
+        <is>
+          <t>30.068.169/0001-44</t>
+        </is>
+      </c>
+      <c r="M169" s="4" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="N169" s="4" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="O169" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="P169" s="4" t="inlineStr">
+        <is>
+          <t>D+13 (du)</t>
+        </is>
+      </c>
+      <c r="Q169" s="4" t="inlineStr">
+        <is>
+          <t>D+15 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
@@ -12510,12 +14882,32 @@
           <t>https://www.caixa.gov.br/fundos-investimento/rpps/caixa-fic-acoes-vinci-valor-dividendos-rpps</t>
         </is>
       </c>
-      <c r="L170" s="2" t="inlineStr"/>
-      <c r="M170" s="2" t="inlineStr"/>
+      <c r="L170" s="2" t="inlineStr">
+        <is>
+          <t>15.154.441/0001-15</t>
+        </is>
+      </c>
+      <c r="M170" s="2" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
       <c r="N170" s="2" t="inlineStr"/>
-      <c r="O170" s="2" t="inlineStr"/>
-      <c r="P170" s="2" t="inlineStr"/>
-      <c r="Q170" s="2" t="inlineStr"/>
+      <c r="O170" s="2" t="inlineStr">
+        <is>
+          <t>10000.0</t>
+        </is>
+      </c>
+      <c r="P170" s="2" t="inlineStr">
+        <is>
+          <t>D+30 (du)</t>
+        </is>
+      </c>
+      <c r="Q170" s="2" t="inlineStr">
+        <is>
+          <t>D+32 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="4" t="inlineStr">
@@ -12573,12 +14965,32 @@
           <t>https://www.caixa.gov.br/fundos-investimento/rpps/caixa-fic-acoes-vinci-valor-rpps</t>
         </is>
       </c>
-      <c r="L171" s="4" t="inlineStr"/>
-      <c r="M171" s="4" t="inlineStr"/>
+      <c r="L171" s="4" t="inlineStr">
+        <is>
+          <t>14.507.699/0001-95</t>
+        </is>
+      </c>
+      <c r="M171" s="4" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
       <c r="N171" s="4" t="inlineStr"/>
-      <c r="O171" s="4" t="inlineStr"/>
-      <c r="P171" s="4" t="inlineStr"/>
-      <c r="Q171" s="4" t="inlineStr"/>
+      <c r="O171" s="4" t="inlineStr">
+        <is>
+          <t>10000.0</t>
+        </is>
+      </c>
+      <c r="P171" s="4" t="inlineStr">
+        <is>
+          <t>D+21 (du)</t>
+        </is>
+      </c>
+      <c r="Q171" s="4" t="inlineStr">
+        <is>
+          <t>D+23 (du)</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Dados atualizados via Robô: 01/06/2026 01:21
</commit_message>
<xml_diff>
--- a/dados_atuais.xlsx
+++ b/dados_atuais.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W172"/>
+  <dimension ref="A1:X172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -491,6 +491,7 @@
     <col width="15" customWidth="1" min="21" max="21"/>
     <col width="15" customWidth="1" min="22" max="22"/>
     <col width="15" customWidth="1" min="23" max="23"/>
+    <col width="15" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -607,6 +608,11 @@
       <c r="W1" s="1" t="inlineStr">
         <is>
           <t>doc_carta</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>doc_boletim</t>
         </is>
       </c>
     </row>
@@ -678,6 +684,7 @@
       <c r="U2" s="2" t="inlineStr"/>
       <c r="V2" s="2" t="inlineStr"/>
       <c r="W2" s="2" t="inlineStr"/>
+      <c r="X2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -795,6 +802,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_88.pdf</t>
         </is>
       </c>
+      <c r="X3" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_88.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -912,6 +924,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5823.pdf</t>
         </is>
       </c>
+      <c r="X4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5823.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -969,18 +986,71 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-geracao-jovem-rf-credito-privado-longo-prazo</t>
         </is>
       </c>
-      <c r="L5" s="4" t="inlineStr"/>
-      <c r="M5" s="4" t="inlineStr"/>
-      <c r="N5" s="4" t="inlineStr"/>
-      <c r="O5" s="4" t="inlineStr"/>
-      <c r="P5" s="4" t="inlineStr"/>
-      <c r="Q5" s="4" t="inlineStr"/>
-      <c r="R5" s="4" t="inlineStr"/>
-      <c r="S5" s="4" t="inlineStr"/>
-      <c r="T5" s="4" t="inlineStr"/>
-      <c r="U5" s="4" t="inlineStr"/>
-      <c r="V5" s="4" t="inlineStr"/>
-      <c r="W5" s="4" t="inlineStr"/>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>10.577.485/0001-34</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="inlineStr">
+        <is>
+          <t>5570</t>
+        </is>
+      </c>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="O5" s="4" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="P5" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="Q5" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="R5" s="4" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
+      <c r="S5" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5570.pdf</t>
+        </is>
+      </c>
+      <c r="T5" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5570.pdf</t>
+        </is>
+      </c>
+      <c r="U5" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5570.pdf</t>
+        </is>
+      </c>
+      <c r="V5" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5570.pdf</t>
+        </is>
+      </c>
+      <c r="W5" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5570.pdf</t>
+        </is>
+      </c>
+      <c r="X5" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5570.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1098,6 +1168,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5565.pdf</t>
         </is>
       </c>
+      <c r="X6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5565.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -1215,6 +1290,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6532.pdf</t>
         </is>
       </c>
+      <c r="X7" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6532.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1332,6 +1412,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_59.pdf</t>
         </is>
       </c>
+      <c r="X8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_59.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -1449,6 +1534,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5834.pdf</t>
         </is>
       </c>
+      <c r="X9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5834.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1502,18 +1592,71 @@
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr"/>
-      <c r="L10" s="2" t="inlineStr"/>
-      <c r="M10" s="2" t="inlineStr"/>
-      <c r="N10" s="2" t="inlineStr"/>
-      <c r="O10" s="2" t="inlineStr"/>
-      <c r="P10" s="2" t="inlineStr"/>
-      <c r="Q10" s="2" t="inlineStr"/>
-      <c r="R10" s="2" t="inlineStr"/>
-      <c r="S10" s="2" t="inlineStr"/>
-      <c r="T10" s="2" t="inlineStr"/>
-      <c r="U10" s="2" t="inlineStr"/>
-      <c r="V10" s="2" t="inlineStr"/>
-      <c r="W10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>15.154.319/0001-49</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>5972</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="Q10" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="R10" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
+      <c r="S10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5972.pdf</t>
+        </is>
+      </c>
+      <c r="T10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5972.pdf</t>
+        </is>
+      </c>
+      <c r="U10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5972.pdf</t>
+        </is>
+      </c>
+      <c r="V10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5972.pdf</t>
+        </is>
+      </c>
+      <c r="W10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5972.pdf</t>
+        </is>
+      </c>
+      <c r="X10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5972.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -1631,6 +1774,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_86.pdf</t>
         </is>
       </c>
+      <c r="X11" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_86.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1748,6 +1896,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_87.pdf</t>
         </is>
       </c>
+      <c r="X12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_87.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1865,6 +2018,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_54.pdf</t>
         </is>
       </c>
+      <c r="X13" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_54.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1982,6 +2140,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_57.pdf</t>
         </is>
       </c>
+      <c r="X14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_57.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -2099,6 +2262,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5414.pdf</t>
         </is>
       </c>
+      <c r="X15" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5414.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -2216,6 +2384,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_85.pdf</t>
         </is>
       </c>
+      <c r="X16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_85.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -2333,6 +2506,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5892.pdf</t>
         </is>
       </c>
+      <c r="X17" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5892.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2450,6 +2628,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5576.pdf</t>
         </is>
       </c>
+      <c r="X18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5576.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -2567,6 +2750,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5970.pdf</t>
         </is>
       </c>
+      <c r="X19" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5970.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2684,6 +2872,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_58.pdf</t>
         </is>
       </c>
+      <c r="X20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_58.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -2801,6 +2994,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5566.pdf</t>
         </is>
       </c>
+      <c r="X21" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5566.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2918,6 +3116,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5571.pdf</t>
         </is>
       </c>
+      <c r="X22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5571.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -2970,19 +3173,76 @@
           <t>PF | PJ | TODOS</t>
         </is>
       </c>
-      <c r="K23" s="4" t="inlineStr"/>
-      <c r="L23" s="4" t="inlineStr"/>
-      <c r="M23" s="4" t="inlineStr"/>
-      <c r="N23" s="4" t="inlineStr"/>
-      <c r="O23" s="4" t="inlineStr"/>
-      <c r="P23" s="4" t="inlineStr"/>
-      <c r="Q23" s="4" t="inlineStr"/>
-      <c r="R23" s="4" t="inlineStr"/>
-      <c r="S23" s="4" t="inlineStr"/>
-      <c r="T23" s="4" t="inlineStr"/>
-      <c r="U23" s="4" t="inlineStr"/>
-      <c r="V23" s="4" t="inlineStr"/>
-      <c r="W23" s="4" t="inlineStr"/>
+      <c r="K23" s="4" t="inlineStr">
+        <is>
+          <t>http://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-investidor-rf-longo-prazo</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>03.164.294/0001-85</t>
+        </is>
+      </c>
+      <c r="M23" s="4" t="inlineStr">
+        <is>
+          <t>89</t>
+        </is>
+      </c>
+      <c r="N23" s="4" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="O23" s="4" t="inlineStr">
+        <is>
+          <t>0.85</t>
+        </is>
+      </c>
+      <c r="P23" s="4" t="inlineStr">
+        <is>
+          <t>5000.0</t>
+        </is>
+      </c>
+      <c r="Q23" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="R23" s="4" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
+      <c r="S23" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_0089.pdf</t>
+        </is>
+      </c>
+      <c r="T23" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_0089.pdf</t>
+        </is>
+      </c>
+      <c r="U23" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_0089.pdf</t>
+        </is>
+      </c>
+      <c r="V23" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_0089.pdf</t>
+        </is>
+      </c>
+      <c r="W23" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_89.pdf</t>
+        </is>
+      </c>
+      <c r="X23" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_89.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -3100,6 +3360,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_7938.pdf</t>
         </is>
       </c>
+      <c r="X24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_7938.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -3217,6 +3482,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_7931.pdf</t>
         </is>
       </c>
+      <c r="X25" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_7931.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -3274,18 +3544,71 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-plus-qualificado-rf-credito-privado-longo-prazo/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L26" s="2" t="inlineStr"/>
-      <c r="M26" s="2" t="inlineStr"/>
-      <c r="N26" s="2" t="inlineStr"/>
-      <c r="O26" s="2" t="inlineStr"/>
-      <c r="P26" s="2" t="inlineStr"/>
-      <c r="Q26" s="2" t="inlineStr"/>
-      <c r="R26" s="2" t="inlineStr"/>
-      <c r="S26" s="2" t="inlineStr"/>
-      <c r="T26" s="2" t="inlineStr"/>
-      <c r="U26" s="2" t="inlineStr"/>
-      <c r="V26" s="2" t="inlineStr"/>
-      <c r="W26" s="2" t="inlineStr"/>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>40.194.314/0001-97</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>6533</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>0.55</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>10000.0</t>
+        </is>
+      </c>
+      <c r="Q26" s="2" t="inlineStr">
+        <is>
+          <t>D+14 (du)</t>
+        </is>
+      </c>
+      <c r="R26" s="2" t="inlineStr">
+        <is>
+          <t>D+15 (du)</t>
+        </is>
+      </c>
+      <c r="S26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6533.pdf</t>
+        </is>
+      </c>
+      <c r="T26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_6533.pdf</t>
+        </is>
+      </c>
+      <c r="U26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_6533.pdf</t>
+        </is>
+      </c>
+      <c r="V26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_6533.pdf</t>
+        </is>
+      </c>
+      <c r="W26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6533.pdf</t>
+        </is>
+      </c>
+      <c r="X26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6533.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -3403,6 +3726,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_7887.pdf</t>
         </is>
       </c>
+      <c r="X27" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_7887.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -3516,6 +3844,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_7987.pdf</t>
         </is>
       </c>
+      <c r="X28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_7987.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -3629,6 +3962,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_7940.pdf</t>
         </is>
       </c>
+      <c r="X29" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_7940.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -3746,6 +4084,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_7978.pdf</t>
         </is>
       </c>
+      <c r="X30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_7978.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -3855,6 +4198,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_7999.pdf</t>
         </is>
       </c>
+      <c r="X31" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_7999.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -3972,6 +4320,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5154.pdf</t>
         </is>
       </c>
+      <c r="X32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5154.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -4089,6 +4442,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5156.pdf</t>
         </is>
       </c>
+      <c r="X33" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5156.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -4206,6 +4564,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5401.pdf</t>
         </is>
       </c>
+      <c r="X34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5401.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -4323,6 +4686,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_83.pdf</t>
         </is>
       </c>
+      <c r="X35" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_83.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -4440,6 +4808,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6482.pdf</t>
         </is>
       </c>
+      <c r="X36" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6482.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -4557,6 +4930,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5940.pdf</t>
         </is>
       </c>
+      <c r="X37" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5940.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -4674,6 +5052,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5406.pdf</t>
         </is>
       </c>
+      <c r="X38" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5406.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
@@ -4791,6 +5174,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_7916.pdf</t>
         </is>
       </c>
+      <c r="X39" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_7916.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -4908,6 +5296,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_84.pdf</t>
         </is>
       </c>
+      <c r="X40" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_84.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
@@ -5025,6 +5418,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5408.pdf</t>
         </is>
       </c>
+      <c r="X41" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5408.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -5142,6 +5540,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5908.pdf</t>
         </is>
       </c>
+      <c r="X42" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5908.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
@@ -5259,6 +5662,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5410.pdf</t>
         </is>
       </c>
+      <c r="X43" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5410.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -5376,6 +5784,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_56.pdf</t>
         </is>
       </c>
+      <c r="X44" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_56.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
@@ -5489,6 +5902,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_8500.pdf</t>
         </is>
       </c>
+      <c r="X45" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_8500.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -5606,6 +6024,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5930.pdf</t>
         </is>
       </c>
+      <c r="X46" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5930.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
@@ -5723,6 +6146,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5498.pdf</t>
         </is>
       </c>
+      <c r="X47" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5498.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -5840,6 +6268,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_7914.pdf</t>
         </is>
       </c>
+      <c r="X48" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_7914.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
@@ -5957,6 +6390,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5402.pdf</t>
         </is>
       </c>
+      <c r="X49" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5402.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -6074,6 +6512,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5171.pdf</t>
         </is>
       </c>
+      <c r="X50" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5171.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
@@ -6191,6 +6634,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5157.pdf</t>
         </is>
       </c>
+      <c r="X51" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5157.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -6248,18 +6696,71 @@
           <t>https://www.caixa.gov.br/fundos-investimento/referenciados/fic-mega-ref-di-longo-prazo/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L52" s="2" t="inlineStr"/>
-      <c r="M52" s="2" t="inlineStr"/>
-      <c r="N52" s="2" t="inlineStr"/>
-      <c r="O52" s="2" t="inlineStr"/>
-      <c r="P52" s="2" t="inlineStr"/>
-      <c r="Q52" s="2" t="inlineStr"/>
-      <c r="R52" s="2" t="inlineStr"/>
-      <c r="S52" s="2" t="inlineStr"/>
-      <c r="T52" s="2" t="inlineStr"/>
-      <c r="U52" s="2" t="inlineStr"/>
-      <c r="V52" s="2" t="inlineStr"/>
-      <c r="W52" s="2" t="inlineStr"/>
+      <c r="L52" s="2" t="inlineStr">
+        <is>
+          <t>10.322.633/0001-70</t>
+        </is>
+      </c>
+      <c r="M52" s="2" t="inlineStr">
+        <is>
+          <t>5411</t>
+        </is>
+      </c>
+      <c r="N52" s="2" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="O52" s="2" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="P52" s="2" t="inlineStr">
+        <is>
+          <t>50000.0</t>
+        </is>
+      </c>
+      <c r="Q52" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="R52" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
+      <c r="S52" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5411.pdf</t>
+        </is>
+      </c>
+      <c r="T52" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5411.pdf</t>
+        </is>
+      </c>
+      <c r="U52" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5411.pdf</t>
+        </is>
+      </c>
+      <c r="V52" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5411.pdf</t>
+        </is>
+      </c>
+      <c r="W52" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5411.pdf</t>
+        </is>
+      </c>
+      <c r="X52" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5411.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
@@ -6377,6 +6878,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5969.pdf</t>
         </is>
       </c>
+      <c r="X53" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5969.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -6494,6 +7000,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6520.pdf</t>
         </is>
       </c>
+      <c r="X54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6520.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
@@ -6611,6 +7122,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_7880.pdf</t>
         </is>
       </c>
+      <c r="X55" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_7880.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -6726,6 +7242,11 @@
       <c r="W56" s="2" t="inlineStr">
         <is>
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6518.pdf</t>
+        </is>
+      </c>
+      <c r="X56" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6518.pdf</t>
         </is>
       </c>
     </row>
@@ -6797,6 +7318,7 @@
       <c r="U57" s="4" t="inlineStr"/>
       <c r="V57" s="4" t="inlineStr"/>
       <c r="W57" s="4" t="inlineStr"/>
+      <c r="X57" s="4" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -6914,6 +7436,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6439.pdf</t>
         </is>
       </c>
+      <c r="X58" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6439.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
@@ -7031,6 +7558,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6446.pdf</t>
         </is>
       </c>
+      <c r="X59" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6446.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -7144,6 +7676,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_7990.pdf</t>
         </is>
       </c>
+      <c r="X60" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_7990.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
@@ -7261,6 +7798,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_7877.pdf</t>
         </is>
       </c>
+      <c r="X61" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_7877.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -7378,6 +7920,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6950.pdf</t>
         </is>
       </c>
+      <c r="X62" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6950.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
@@ -7491,6 +8038,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_7991.pdf</t>
         </is>
       </c>
+      <c r="X63" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_7991.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -7608,6 +8160,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_7876.pdf</t>
         </is>
       </c>
+      <c r="X64" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_7876.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
@@ -7721,6 +8278,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_7992.pdf</t>
         </is>
       </c>
+      <c r="X65" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_7992.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -7838,6 +8400,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_7910.pdf</t>
         </is>
       </c>
+      <c r="X66" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_7910.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
@@ -7955,6 +8522,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5490.pdf</t>
         </is>
       </c>
+      <c r="X67" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5490.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -8072,6 +8644,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5902.pdf</t>
         </is>
       </c>
+      <c r="X68" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5902.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
@@ -8189,6 +8766,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5954.pdf</t>
         </is>
       </c>
+      <c r="X69" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5954.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -8306,6 +8888,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6399.pdf</t>
         </is>
       </c>
+      <c r="X70" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6399.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
@@ -8423,6 +9010,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6999.pdf</t>
         </is>
       </c>
+      <c r="X71" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6999.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -8540,6 +9132,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6353.pdf</t>
         </is>
       </c>
+      <c r="X72" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6353.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
@@ -8653,6 +9250,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6479.pdf</t>
         </is>
       </c>
+      <c r="X73" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6479.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -8770,6 +9372,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_7980.pdf</t>
         </is>
       </c>
+      <c r="X74" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_7980.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
@@ -8887,6 +9494,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5475.pdf</t>
         </is>
       </c>
+      <c r="X75" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5475.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -9004,6 +9616,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6608.pdf</t>
         </is>
       </c>
+      <c r="X76" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6608.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
@@ -9121,6 +9738,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6621.pdf</t>
         </is>
       </c>
+      <c r="X77" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6621.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -9238,6 +9860,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6623.pdf</t>
         </is>
       </c>
+      <c r="X78" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6623.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
@@ -9355,6 +9982,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6475.pdf</t>
         </is>
       </c>
+      <c r="X79" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6475.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -9472,6 +10104,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5492.pdf</t>
         </is>
       </c>
+      <c r="X80" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5492.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
@@ -9589,6 +10226,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5582.pdf</t>
         </is>
       </c>
+      <c r="X81" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5582.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -9706,6 +10348,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5911.pdf</t>
         </is>
       </c>
+      <c r="X82" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5911.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
@@ -9823,6 +10470,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_7875.pdf</t>
         </is>
       </c>
+      <c r="X83" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_7875.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -9940,6 +10592,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6535.pdf</t>
         </is>
       </c>
+      <c r="X84" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6535.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
@@ -10057,6 +10714,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5403.pdf</t>
         </is>
       </c>
+      <c r="X85" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5403.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -10174,6 +10836,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5390.pdf</t>
         </is>
       </c>
+      <c r="X86" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5390.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
@@ -10291,6 +10958,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_53.pdf</t>
         </is>
       </c>
+      <c r="X87" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_53.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -10404,6 +11076,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6478.pdf</t>
         </is>
       </c>
+      <c r="X88" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6478.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
@@ -10521,6 +11198,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5928.pdf</t>
         </is>
       </c>
+      <c r="X89" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5928.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -10638,6 +11320,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5841.pdf</t>
         </is>
       </c>
+      <c r="X90" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5841.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
@@ -10755,6 +11442,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5567.pdf</t>
         </is>
       </c>
+      <c r="X91" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5567.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -10872,6 +11564,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5395.pdf</t>
         </is>
       </c>
+      <c r="X92" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5395.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
@@ -10989,6 +11686,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6420.pdf</t>
         </is>
       </c>
+      <c r="X93" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6420.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -11106,6 +11808,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_53.pdf</t>
         </is>
       </c>
+      <c r="X94" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_53.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
@@ -11223,6 +11930,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6421.pdf</t>
         </is>
       </c>
+      <c r="X95" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6421.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -11340,6 +12052,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5397.pdf</t>
         </is>
       </c>
+      <c r="X96" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5397.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
@@ -11457,6 +12174,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5398.pdf</t>
         </is>
       </c>
+      <c r="X97" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5398.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -11574,6 +12296,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5978.pdf</t>
         </is>
       </c>
+      <c r="X98" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5978.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
@@ -11691,6 +12418,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5420.pdf</t>
         </is>
       </c>
+      <c r="X99" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5420.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -11808,6 +12540,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6447.pdf</t>
         </is>
       </c>
+      <c r="X100" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6447.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
@@ -11925,6 +12662,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5301.pdf</t>
         </is>
       </c>
+      <c r="X101" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5301.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -12042,6 +12784,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6499.pdf</t>
         </is>
       </c>
+      <c r="X102" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6499.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
@@ -12159,6 +12906,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5392.pdf</t>
         </is>
       </c>
+      <c r="X103" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5392.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -12276,6 +13028,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6530.pdf</t>
         </is>
       </c>
+      <c r="X104" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6530.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
@@ -12393,6 +13150,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6591.pdf</t>
         </is>
       </c>
+      <c r="X105" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6591.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -12510,6 +13272,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5393.pdf</t>
         </is>
       </c>
+      <c r="X106" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5393.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="4" t="inlineStr">
@@ -12627,6 +13394,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5394.pdf</t>
         </is>
       </c>
+      <c r="X107" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5394.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -12744,6 +13516,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_48.pdf</t>
         </is>
       </c>
+      <c r="X108" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_48.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="4" t="inlineStr">
@@ -12861,6 +13638,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6620.pdf</t>
         </is>
       </c>
+      <c r="X109" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6620.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -12978,6 +13760,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6593.pdf</t>
         </is>
       </c>
+      <c r="X110" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6593.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="4" t="inlineStr">
@@ -13095,6 +13882,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_7971.pdf</t>
         </is>
       </c>
+      <c r="X111" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_7971.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -13212,6 +14004,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6602.pdf</t>
         </is>
       </c>
+      <c r="X112" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6602.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="4" t="inlineStr">
@@ -13329,6 +14126,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6994.pdf</t>
         </is>
       </c>
+      <c r="X113" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6994.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -13446,6 +14248,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6397.pdf</t>
         </is>
       </c>
+      <c r="X114" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6397.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="4" t="inlineStr">
@@ -13503,18 +14310,71 @@
           <t>https://www.caixa.gov.br/fundos-investimento/fundos-de-indices/etf-ibovespa-fundo-de-indice/</t>
         </is>
       </c>
-      <c r="L115" s="4" t="inlineStr"/>
-      <c r="M115" s="4" t="inlineStr"/>
-      <c r="N115" s="4" t="inlineStr"/>
-      <c r="O115" s="4" t="inlineStr"/>
-      <c r="P115" s="4" t="inlineStr"/>
-      <c r="Q115" s="4" t="inlineStr"/>
-      <c r="R115" s="4" t="inlineStr"/>
-      <c r="S115" s="4" t="inlineStr"/>
-      <c r="T115" s="4" t="inlineStr"/>
-      <c r="U115" s="4" t="inlineStr"/>
-      <c r="V115" s="4" t="inlineStr"/>
-      <c r="W115" s="4" t="inlineStr"/>
+      <c r="L115" s="4" t="inlineStr">
+        <is>
+          <t>15.154.236/0001-50</t>
+        </is>
+      </c>
+      <c r="M115" s="4" t="inlineStr">
+        <is>
+          <t>5842</t>
+        </is>
+      </c>
+      <c r="N115" s="4" t="inlineStr">
+        <is>
+          <t>Arrojado</t>
+        </is>
+      </c>
+      <c r="O115" s="4" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="P115" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="Q115" s="4" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="R115" s="4" t="inlineStr">
+        <is>
+          <t>D+03 (du)</t>
+        </is>
+      </c>
+      <c r="S115" s="4" t="inlineStr">
+        <is>
+          <t>http://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5842.pdf</t>
+        </is>
+      </c>
+      <c r="T115" s="4" t="inlineStr">
+        <is>
+          <t>http://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5842.pdf</t>
+        </is>
+      </c>
+      <c r="U115" s="4" t="inlineStr">
+        <is>
+          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5842.pdf</t>
+        </is>
+      </c>
+      <c r="V115" s="4" t="inlineStr">
+        <is>
+          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_5842.pdf</t>
+        </is>
+      </c>
+      <c r="W115" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5842.pdf</t>
+        </is>
+      </c>
+      <c r="X115" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5842.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -13632,6 +14492,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6601.pdf</t>
         </is>
       </c>
+      <c r="X116" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6601.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="4" t="inlineStr">
@@ -13749,6 +14614,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6600.pdf</t>
         </is>
       </c>
+      <c r="X117" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6600.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -13866,6 +14736,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5204.pdf</t>
         </is>
       </c>
+      <c r="X118" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5204.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="4" t="inlineStr">
@@ -13983,6 +14858,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5205.pdf</t>
         </is>
       </c>
+      <c r="X119" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5205.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -14100,6 +14980,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5251.pdf</t>
         </is>
       </c>
+      <c r="X120" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5251.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="4" t="inlineStr">
@@ -14217,6 +15102,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5253.pdf</t>
         </is>
       </c>
+      <c r="X121" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5253.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -14334,6 +15224,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5202.pdf</t>
         </is>
       </c>
+      <c r="X122" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5202.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="4" t="inlineStr">
@@ -14451,6 +15346,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5205.pdf</t>
         </is>
       </c>
+      <c r="X123" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5205.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -14568,6 +15468,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5203.pdf</t>
         </is>
       </c>
+      <c r="X124" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5203.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="4" t="inlineStr">
@@ -14685,6 +15590,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_7972.pdf</t>
         </is>
       </c>
+      <c r="X125" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_7972.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -14742,18 +15652,71 @@
           <t>https://www.caixa.gov.br/fundos-investimento/fundo-simples/fic-ametista-corporativo-rf-simples/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L126" s="2" t="inlineStr"/>
-      <c r="M126" s="2" t="inlineStr"/>
-      <c r="N126" s="2" t="inlineStr"/>
-      <c r="O126" s="2" t="inlineStr"/>
-      <c r="P126" s="2" t="inlineStr"/>
-      <c r="Q126" s="2" t="inlineStr"/>
-      <c r="R126" s="2" t="inlineStr"/>
-      <c r="S126" s="2" t="inlineStr"/>
-      <c r="T126" s="2" t="inlineStr"/>
-      <c r="U126" s="2" t="inlineStr"/>
-      <c r="V126" s="2" t="inlineStr"/>
-      <c r="W126" s="2" t="inlineStr"/>
+      <c r="L126" s="2" t="inlineStr">
+        <is>
+          <t>51.255.391/0001-26</t>
+        </is>
+      </c>
+      <c r="M126" s="2" t="inlineStr">
+        <is>
+          <t>7861</t>
+        </is>
+      </c>
+      <c r="N126" s="2" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="O126" s="2" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="P126" s="2" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="Q126" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="R126" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
+      <c r="S126" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_7861.pdf</t>
+        </is>
+      </c>
+      <c r="T126" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_7861.pdf</t>
+        </is>
+      </c>
+      <c r="U126" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_7861.pdf</t>
+        </is>
+      </c>
+      <c r="V126" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_7861.pdf</t>
+        </is>
+      </c>
+      <c r="W126" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_7861.pdf</t>
+        </is>
+      </c>
+      <c r="X126" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_7861.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="4" t="inlineStr">
@@ -14871,6 +15834,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5405.pdf</t>
         </is>
       </c>
+      <c r="X127" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5405.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -14988,6 +15956,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5080.pdf</t>
         </is>
       </c>
+      <c r="X128" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5080.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="4" t="inlineStr">
@@ -15105,6 +16078,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5833.pdf</t>
         </is>
       </c>
+      <c r="X129" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5833.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -15222,6 +16200,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_46.pdf</t>
         </is>
       </c>
+      <c r="X130" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_46.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="4" t="inlineStr">
@@ -15339,6 +16322,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5901.pdf</t>
         </is>
       </c>
+      <c r="X131" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5901.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -15456,6 +16444,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6445.pdf</t>
         </is>
       </c>
+      <c r="X132" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6445.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="4" t="inlineStr">
@@ -15573,6 +16566,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5148.pdf</t>
         </is>
       </c>
+      <c r="X133" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5148.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -15690,6 +16688,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6606.pdf</t>
         </is>
       </c>
+      <c r="X134" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6606.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="4" t="inlineStr">
@@ -15807,6 +16810,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5132.pdf</t>
         </is>
       </c>
+      <c r="X135" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5132.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -15924,6 +16932,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5066.pdf</t>
         </is>
       </c>
+      <c r="X136" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5066.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="4" t="inlineStr">
@@ -16037,6 +17050,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5053.pdf</t>
         </is>
       </c>
+      <c r="X137" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5053.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -16154,6 +17172,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5948.pdf</t>
         </is>
       </c>
+      <c r="X138" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5948.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="4" t="inlineStr">
@@ -16271,6 +17294,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5189.pdf</t>
         </is>
       </c>
+      <c r="X139" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5189.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -16388,6 +17416,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6996.pdf</t>
         </is>
       </c>
+      <c r="X140" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6996.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="4" t="inlineStr">
@@ -16505,6 +17538,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5946.pdf</t>
         </is>
       </c>
+      <c r="X141" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5946.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -16622,6 +17660,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_7869.pdf</t>
         </is>
       </c>
+      <c r="X142" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_7869.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="4" t="inlineStr">
@@ -16739,6 +17782,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_55.pdf</t>
         </is>
       </c>
+      <c r="X143" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_55.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -16796,18 +17844,71 @@
           <t>https://www.caixa.gov.br/fundos-investimento/curto-prazo/fic-transferencias-voluntarias-curto-prazo</t>
         </is>
       </c>
-      <c r="L144" s="2" t="inlineStr"/>
-      <c r="M144" s="2" t="inlineStr"/>
-      <c r="N144" s="2" t="inlineStr"/>
-      <c r="O144" s="2" t="inlineStr"/>
-      <c r="P144" s="2" t="inlineStr"/>
-      <c r="Q144" s="2" t="inlineStr"/>
-      <c r="R144" s="2" t="inlineStr"/>
-      <c r="S144" s="2" t="inlineStr"/>
-      <c r="T144" s="2" t="inlineStr"/>
-      <c r="U144" s="2" t="inlineStr"/>
-      <c r="V144" s="2" t="inlineStr"/>
-      <c r="W144" s="2" t="inlineStr"/>
+      <c r="L144" s="2" t="inlineStr">
+        <is>
+          <t>10.740.552/0001-90</t>
+        </is>
+      </c>
+      <c r="M144" s="2" t="inlineStr">
+        <is>
+          <t>5413</t>
+        </is>
+      </c>
+      <c r="N144" s="2" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="O144" s="2" t="inlineStr">
+        <is>
+          <t>1.7</t>
+        </is>
+      </c>
+      <c r="P144" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="Q144" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="R144" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
+      <c r="S144" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5413.pdf</t>
+        </is>
+      </c>
+      <c r="T144" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5413.pdf</t>
+        </is>
+      </c>
+      <c r="U144" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5413.pdf</t>
+        </is>
+      </c>
+      <c r="V144" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5413.pdf</t>
+        </is>
+      </c>
+      <c r="W144" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5413.pdf</t>
+        </is>
+      </c>
+      <c r="X144" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5413.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="4" t="inlineStr">
@@ -16925,6 +18026,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5982.pdf</t>
         </is>
       </c>
+      <c r="X145" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5982.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -17042,6 +18148,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5993.pdf</t>
         </is>
       </c>
+      <c r="X146" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5993.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="4" t="inlineStr">
@@ -17159,6 +18270,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5975.pdf</t>
         </is>
       </c>
+      <c r="X147" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5975.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -17276,6 +18392,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6481.pdf</t>
         </is>
       </c>
+      <c r="X148" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6481.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="4" t="inlineStr">
@@ -17393,6 +18514,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5824.pdf</t>
         </is>
       </c>
+      <c r="X149" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5824.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -17450,18 +18576,71 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fi-brasil-idka-ipca-2a-rf-longo-prazo</t>
         </is>
       </c>
-      <c r="L150" s="2" t="inlineStr"/>
-      <c r="M150" s="2" t="inlineStr"/>
-      <c r="N150" s="2" t="inlineStr"/>
-      <c r="O150" s="2" t="inlineStr"/>
-      <c r="P150" s="2" t="inlineStr"/>
-      <c r="Q150" s="2" t="inlineStr"/>
-      <c r="R150" s="2" t="inlineStr"/>
-      <c r="S150" s="2" t="inlineStr"/>
-      <c r="T150" s="2" t="inlineStr"/>
-      <c r="U150" s="2" t="inlineStr"/>
-      <c r="V150" s="2" t="inlineStr"/>
-      <c r="W150" s="2" t="inlineStr"/>
+      <c r="L150" s="2" t="inlineStr">
+        <is>
+          <t>14.386.926/0001-71</t>
+        </is>
+      </c>
+      <c r="M150" s="2" t="inlineStr">
+        <is>
+          <t>5825</t>
+        </is>
+      </c>
+      <c r="N150" s="2" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="O150" s="2" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="P150" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="Q150" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="R150" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
+      <c r="S150" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5825.pdf</t>
+        </is>
+      </c>
+      <c r="T150" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5825.pdf</t>
+        </is>
+      </c>
+      <c r="U150" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5825.pdf</t>
+        </is>
+      </c>
+      <c r="V150" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5825.pdf</t>
+        </is>
+      </c>
+      <c r="W150" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5825.pdf</t>
+        </is>
+      </c>
+      <c r="X150" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5825.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="4" t="inlineStr">
@@ -17579,6 +18758,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5824.pdf</t>
         </is>
       </c>
+      <c r="X151" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5824.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -17696,6 +18880,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5184.pdf</t>
         </is>
       </c>
+      <c r="X152" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5184.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="4" t="inlineStr">
@@ -17813,6 +19002,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5184.pdf</t>
         </is>
       </c>
+      <c r="X153" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5184.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -17928,6 +19122,11 @@
       <c r="W154" s="2" t="inlineStr">
         <is>
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5188.pdf</t>
+        </is>
+      </c>
+      <c r="X154" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5188.pdf</t>
         </is>
       </c>
     </row>
@@ -17999,6 +19198,7 @@
       <c r="U155" s="4" t="inlineStr"/>
       <c r="V155" s="4" t="inlineStr"/>
       <c r="W155" s="4" t="inlineStr"/>
+      <c r="X155" s="4" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -18116,6 +19316,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5184.pdf</t>
         </is>
       </c>
+      <c r="X156" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5184.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="4" t="inlineStr">
@@ -18233,6 +19438,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5824.pdf</t>
         </is>
       </c>
+      <c r="X157" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5824.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -18350,6 +19560,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5404.pdf</t>
         </is>
       </c>
+      <c r="X158" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5404.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="4" t="inlineStr">
@@ -18467,6 +19682,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5461.pdf</t>
         </is>
       </c>
+      <c r="X159" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5461.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -18584,6 +19804,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6634.pdf</t>
         </is>
       </c>
+      <c r="X160" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6634.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="4" t="inlineStr">
@@ -18699,6 +19924,11 @@
       <c r="W161" s="4" t="inlineStr">
         <is>
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5826.pdf</t>
+        </is>
+      </c>
+      <c r="X161" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5826.pdf</t>
         </is>
       </c>
     </row>
@@ -18770,6 +20000,7 @@
       <c r="U162" s="2" t="inlineStr"/>
       <c r="V162" s="2" t="inlineStr"/>
       <c r="W162" s="2" t="inlineStr"/>
+      <c r="X162" s="2" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" s="4" t="inlineStr">
@@ -18887,6 +20118,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5168.pdf</t>
         </is>
       </c>
+      <c r="X163" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5168.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -19004,6 +20240,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6439.pdf</t>
         </is>
       </c>
+      <c r="X164" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6439.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="4" t="inlineStr">
@@ -19121,6 +20362,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5445.pdf</t>
         </is>
       </c>
+      <c r="X165" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5445.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
@@ -19238,6 +20484,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5842.pdf</t>
         </is>
       </c>
+      <c r="X166" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5842.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="4" t="inlineStr">
@@ -19355,6 +20606,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5929.pdf</t>
         </is>
       </c>
+      <c r="X167" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5929.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
@@ -19472,6 +20728,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5396.pdf</t>
         </is>
       </c>
+      <c r="X168" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5396.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="4" t="inlineStr">
@@ -19589,6 +20850,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6425.pdf</t>
         </is>
       </c>
+      <c r="X169" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6425.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
@@ -19702,6 +20968,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6160.pdf</t>
         </is>
       </c>
+      <c r="X170" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6160.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="4" t="inlineStr">
@@ -19815,6 +21086,11 @@
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5563.pdf</t>
         </is>
       </c>
+      <c r="X171" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5563.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
@@ -19930,6 +21206,11 @@
       <c r="W172" s="2" t="inlineStr">
         <is>
           <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5487.pdf</t>
+        </is>
+      </c>
+      <c r="X172" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5487.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dados atualizados via Robô: 01/06/2026 13:30
</commit_message>
<xml_diff>
--- a/dados_atuais.xlsx
+++ b/dados_atuais.xlsx
@@ -5676,62 +5676,58 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF BETA RF REF DI LP RESP LTDA</t>
+          <t>CAIXA SIGMA FUNCIONARIOS FIC FIF RF REF DI LP - RESP LTDA</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>02/10/1995</t>
+          <t>08/04/2026</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>30,23758400</t>
-        </is>
-      </c>
-      <c r="E44" s="3" t="inlineStr">
-        <is>
-          <t>0,048</t>
-        </is>
-      </c>
-      <c r="F44" s="3" t="inlineStr">
-        <is>
-          <t>0,96</t>
-        </is>
-      </c>
-      <c r="G44" s="3" t="inlineStr">
-        <is>
-          <t>5,08</t>
-        </is>
-      </c>
-      <c r="H44" s="3" t="inlineStr">
-        <is>
-          <t>13,21</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>165,211</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>PF | TODOS</t>
-        </is>
-      </c>
-      <c r="K44" s="2" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/fundos-investimento/referenciados/fic-beta-ref-di-lp</t>
-        </is>
-      </c>
+          <t>PF</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr"/>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>00.834.072/0001-34</t>
+          <t>66.034.762/0001-17</t>
         </is>
       </c>
       <c r="M44" s="2" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>8500</t>
         </is>
       </c>
       <c r="N44" s="2" t="inlineStr">
@@ -5741,7 +5737,7 @@
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>0.2</t>
         </is>
       </c>
       <c r="P44" s="2" t="inlineStr">
@@ -5761,32 +5757,32 @@
       </c>
       <c r="S44" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_0056.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_8500.pdf</t>
         </is>
       </c>
       <c r="T44" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_0056.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_8500.pdf</t>
         </is>
       </c>
       <c r="U44" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_0056.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_8500.pdf</t>
         </is>
       </c>
       <c r="V44" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_0056.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_8500.pdf</t>
         </is>
       </c>
       <c r="W44" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_56.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_8500.pdf</t>
         </is>
       </c>
       <c r="X44" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_56.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_8500.pdf</t>
         </is>
       </c>
     </row>
@@ -5798,58 +5794,62 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>CAIXA SIGMA FUNCIONARIOS FIC FIF RF REF DI LP - RESP LTDA</t>
+          <t>CAIXA FIC FIF BETA RF REF DI LP RESP LTDA</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>08/04/2026</t>
+          <t>02/10/1995</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E45" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F45" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G45" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H45" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>30,23758400</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>0,048</t>
+        </is>
+      </c>
+      <c r="F45" s="5" t="inlineStr">
+        <is>
+          <t>0,96</t>
+        </is>
+      </c>
+      <c r="G45" s="5" t="inlineStr">
+        <is>
+          <t>5,08</t>
+        </is>
+      </c>
+      <c r="H45" s="5" t="inlineStr">
+        <is>
+          <t>13,21</t>
         </is>
       </c>
       <c r="I45" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>165,211</t>
         </is>
       </c>
       <c r="J45" s="4" t="inlineStr">
         <is>
-          <t>PF</t>
-        </is>
-      </c>
-      <c r="K45" s="4" t="inlineStr"/>
+          <t>PF | TODOS</t>
+        </is>
+      </c>
+      <c r="K45" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/referenciados/fic-beta-ref-di-lp</t>
+        </is>
+      </c>
       <c r="L45" s="4" t="inlineStr">
         <is>
-          <t>66.034.762/0001-17</t>
+          <t>00.834.072/0001-34</t>
         </is>
       </c>
       <c r="M45" s="4" t="inlineStr">
         <is>
-          <t>8500</t>
+          <t>56</t>
         </is>
       </c>
       <c r="N45" s="4" t="inlineStr">
@@ -5859,7 +5859,7 @@
       </c>
       <c r="O45" s="4" t="inlineStr">
         <is>
-          <t>0.2</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="P45" s="4" t="inlineStr">
@@ -5879,32 +5879,32 @@
       </c>
       <c r="S45" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_8500.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_0056.pdf</t>
         </is>
       </c>
       <c r="T45" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_8500.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_0056.pdf</t>
         </is>
       </c>
       <c r="U45" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_8500.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_0056.pdf</t>
         </is>
       </c>
       <c r="V45" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_8500.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_0056.pdf</t>
         </is>
       </c>
       <c r="W45" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_8500.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_56.pdf</t>
         </is>
       </c>
       <c r="X45" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_8500.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_56.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dados atualizados via Robô: 01/06/2026 18:58
</commit_message>
<xml_diff>
--- a/dados_atuais.xlsx
+++ b/dados_atuais.xlsx
@@ -659,7 +659,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>407,706</t>
+          <t>402,851</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -729,7 +729,7 @@
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>6.783,321</t>
+          <t>6.646,794</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
@@ -851,7 +851,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>876,296</t>
+          <t>886,956</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -973,7 +973,7 @@
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>11,649</t>
+          <t>11,550</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
@@ -1095,7 +1095,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>120,046</t>
+          <t>119,002</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>97,403</t>
+          <t>96,504</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -1339,7 +1339,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>586,164</t>
+          <t>581,391</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -1461,7 +1461,7 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>61,836</t>
+          <t>61,339</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>1.674,712</t>
+          <t>1.661,172</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -1701,7 +1701,7 @@
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>123,417</t>
+          <t>122,783</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>28,382</t>
+          <t>28,033</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1838,12 +1838,12 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>03.218.183/0001-04</t>
+          <t>03.191.874/0001-61</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>46</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1853,12 +1853,12 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>0.3</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>0.01</t>
+          <t>100000.0</t>
         </is>
       </c>
       <c r="Q12" s="2" t="inlineStr">
@@ -1873,32 +1873,32 @@
       </c>
       <c r="S12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_0087.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_0046.pdf</t>
         </is>
       </c>
       <c r="T12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_0087.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_0046.pdf</t>
         </is>
       </c>
       <c r="U12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_0087.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_0046.pdf</t>
         </is>
       </c>
       <c r="V12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_87.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_46.pdf</t>
         </is>
       </c>
       <c r="W12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_87.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_46.pdf</t>
         </is>
       </c>
       <c r="X12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_87.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_46.pdf</t>
         </is>
       </c>
     </row>
@@ -1945,7 +1945,7 @@
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>40,715</t>
+          <t>40,384</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
@@ -2067,7 +2067,7 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>64,881</t>
+          <t>64,363</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -2189,7 +2189,7 @@
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>79,838</t>
+          <t>79,084</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -2311,7 +2311,7 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>27,956</t>
+          <t>27,719</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>1,659</t>
+          <t>1,646</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -2555,7 +2555,7 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>139,380</t>
+          <t>138,691</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -2677,7 +2677,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1.801,377</t>
+          <t>1.771,652</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -2712,7 +2712,7 @@
       </c>
       <c r="P19" s="4" t="inlineStr">
         <is>
-          <t>0.01</t>
+          <t>1000.0</t>
         </is>
       </c>
       <c r="Q19" s="4" t="inlineStr">
@@ -2799,7 +2799,7 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>2.192,556</t>
+          <t>2.175,893</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -2921,7 +2921,7 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>13,227</t>
+          <t>13,106</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -3043,7 +3043,7 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>66,747</t>
+          <t>66,269</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -3165,7 +3165,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>957,410</t>
+          <t>948,894</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -3262,32 +3262,32 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,11446441</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>-0,039</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>0,39</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>3,31</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>212,664</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
@@ -3384,32 +3384,32 @@
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F25" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H25" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,23544100</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>-0,001</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>1,22</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>5,48</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>14,65</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>71,169</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -3531,7 +3531,7 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>175,484</t>
+          <t>173,953</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
@@ -3653,7 +3653,7 @@
       </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>40,304</t>
+          <t>39,867</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -3750,32 +3750,32 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,03539400</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>-0,001</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>1,11</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>5,59</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>21,752</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
@@ -3868,32 +3868,32 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H29" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,16411800</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>-0,001</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>1,39</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>4,83</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>13,88</t>
         </is>
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>66,448</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -3986,32 +3986,32 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,06921896</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>0,149</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>1,40</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>3,47</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>311,054</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
@@ -4160,7 +4160,7 @@
       <c r="O31" s="4" t="inlineStr"/>
       <c r="P31" s="4" t="inlineStr">
         <is>
-          <t>1000.0</t>
+          <t>10000.0</t>
         </is>
       </c>
       <c r="Q31" s="4" t="inlineStr">
@@ -4247,7 +4247,7 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>861,613</t>
+          <t>851,672</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
@@ -4369,7 +4369,7 @@
       </c>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>3.249,946</t>
+          <t>3.222,999</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -4491,7 +4491,7 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>21,281</t>
+          <t>21,029</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
@@ -4613,7 +4613,7 @@
       </c>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>3.114,091</t>
+          <t>3.090,447</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -4735,7 +4735,7 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>125,785</t>
+          <t>124,407</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
@@ -4857,7 +4857,7 @@
       </c>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>592,393</t>
+          <t>588,678</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -4979,7 +4979,7 @@
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>122,631</t>
+          <t>121,489</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
@@ -5101,7 +5101,7 @@
       </c>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>347,289</t>
+          <t>344,859</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
@@ -5223,7 +5223,7 @@
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>2.387,379</t>
+          <t>2.369,834</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
@@ -5345,7 +5345,7 @@
       </c>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>556,112</t>
+          <t>551,459</t>
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr">
@@ -5467,7 +5467,7 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>15.558,982</t>
+          <t>15.431,671</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -5502,7 +5502,7 @@
       </c>
       <c r="P42" s="2" t="inlineStr">
         <is>
-          <t>50000.0</t>
+          <t>200000.0</t>
         </is>
       </c>
       <c r="Q42" s="2" t="inlineStr">
@@ -5589,7 +5589,7 @@
       </c>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>1.390,430</t>
+          <t>1.384,208</t>
         </is>
       </c>
       <c r="J43" s="4" t="inlineStr">
@@ -5829,7 +5829,7 @@
       </c>
       <c r="I45" s="4" t="inlineStr">
         <is>
-          <t>165,211</t>
+          <t>163,886</t>
         </is>
       </c>
       <c r="J45" s="4" t="inlineStr">
@@ -5951,7 +5951,7 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>6.060,253</t>
+          <t>5.941,253</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
@@ -6073,7 +6073,7 @@
       </c>
       <c r="I47" s="4" t="inlineStr">
         <is>
-          <t>2.185,880</t>
+          <t>2.168,505</t>
         </is>
       </c>
       <c r="J47" s="4" t="inlineStr">
@@ -6195,7 +6195,7 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>63,837</t>
+          <t>63,321</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
@@ -6317,7 +6317,7 @@
       </c>
       <c r="I49" s="4" t="inlineStr">
         <is>
-          <t>838,049</t>
+          <t>830,131</t>
         </is>
       </c>
       <c r="J49" s="4" t="inlineStr">
@@ -6439,7 +6439,7 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>15.819,078</t>
+          <t>15.719,475</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
@@ -6474,7 +6474,7 @@
       </c>
       <c r="P50" s="2" t="inlineStr">
         <is>
-          <t>5000.0</t>
+          <t>50000.0</t>
         </is>
       </c>
       <c r="Q50" s="2" t="inlineStr">
@@ -6561,7 +6561,7 @@
       </c>
       <c r="I51" s="4" t="inlineStr">
         <is>
-          <t>9.472,413</t>
+          <t>9.412,983</t>
         </is>
       </c>
       <c r="J51" s="4" t="inlineStr">
@@ -6596,7 +6596,7 @@
       </c>
       <c r="P51" s="4" t="inlineStr">
         <is>
-          <t>100000.0</t>
+          <t>200000.0</t>
         </is>
       </c>
       <c r="Q51" s="4" t="inlineStr">
@@ -6683,7 +6683,7 @@
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>21.145,854</t>
+          <t>20.988,542</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr">
@@ -6718,7 +6718,7 @@
       </c>
       <c r="P52" s="2" t="inlineStr">
         <is>
-          <t>50000.0</t>
+          <t>300000.0</t>
         </is>
       </c>
       <c r="Q52" s="2" t="inlineStr">
@@ -6805,7 +6805,7 @@
       </c>
       <c r="I53" s="4" t="inlineStr">
         <is>
-          <t>13.384,828</t>
+          <t>13.310,330</t>
         </is>
       </c>
       <c r="J53" s="4" t="inlineStr">
@@ -6840,7 +6840,7 @@
       </c>
       <c r="P53" s="4" t="inlineStr">
         <is>
-          <t>100000.0</t>
+          <t>1000000.0</t>
         </is>
       </c>
       <c r="Q53" s="4" t="inlineStr">
@@ -6927,7 +6927,7 @@
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>247,206</t>
+          <t>245,506</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr">
@@ -6940,71 +6940,19 @@
           <t>https://www.caixa.gov.br/fundos-investimento/curto-prazo/fic-automatico-polis-rf-cp/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L54" s="2" t="inlineStr">
-        <is>
-          <t>39.594.941/0001-36</t>
-        </is>
-      </c>
-      <c r="M54" s="2" t="inlineStr">
-        <is>
-          <t>6520</t>
-        </is>
-      </c>
-      <c r="N54" s="2" t="inlineStr">
-        <is>
-          <t>Conservador</t>
-        </is>
-      </c>
-      <c r="O54" s="2" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
-      </c>
-      <c r="P54" s="2" t="inlineStr">
-        <is>
-          <t>10000.0</t>
-        </is>
-      </c>
-      <c r="Q54" s="2" t="inlineStr">
-        <is>
-          <t>D+0 (du)</t>
-        </is>
-      </c>
-      <c r="R54" s="2" t="inlineStr">
-        <is>
-          <t>D+00 (du)</t>
-        </is>
-      </c>
-      <c r="S54" s="2" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_6520.pdf</t>
-        </is>
-      </c>
-      <c r="T54" s="2" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_6520.pdf</t>
-        </is>
-      </c>
-      <c r="U54" s="2" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_6520.pdf</t>
-        </is>
-      </c>
-      <c r="V54" s="2" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_6520.pdf</t>
-        </is>
-      </c>
-      <c r="W54" s="2" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6520.pdf</t>
-        </is>
-      </c>
-      <c r="X54" s="2" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6520.pdf</t>
-        </is>
-      </c>
+      <c r="L54" s="2" t="inlineStr"/>
+      <c r="M54" s="2" t="inlineStr"/>
+      <c r="N54" s="2" t="inlineStr"/>
+      <c r="O54" s="2" t="inlineStr"/>
+      <c r="P54" s="2" t="inlineStr"/>
+      <c r="Q54" s="2" t="inlineStr"/>
+      <c r="R54" s="2" t="inlineStr"/>
+      <c r="S54" s="2" t="inlineStr"/>
+      <c r="T54" s="2" t="inlineStr"/>
+      <c r="U54" s="2" t="inlineStr"/>
+      <c r="V54" s="2" t="inlineStr"/>
+      <c r="W54" s="2" t="inlineStr"/>
+      <c r="X54" s="2" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
@@ -7024,32 +6972,32 @@
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1,40949900</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F55" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G55" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H55" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>0,000</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="inlineStr">
+        <is>
+          <t>1,33</t>
+        </is>
+      </c>
+      <c r="G55" s="5" t="inlineStr">
+        <is>
+          <t>5,27</t>
+        </is>
+      </c>
+      <c r="H55" s="5" t="inlineStr">
+        <is>
+          <t>14,31</t>
         </is>
       </c>
       <c r="I55" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>67,622</t>
         </is>
       </c>
       <c r="J55" s="4" t="inlineStr">
@@ -7146,32 +7094,32 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E56" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F56" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G56" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H56" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1.193,19101100</t>
+        </is>
+      </c>
+      <c r="E56" s="6" t="inlineStr">
+        <is>
+          <t>-0,002</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>3,81</t>
+        </is>
+      </c>
+      <c r="G56" s="6" t="inlineStr">
+        <is>
+          <t>-4,90</t>
+        </is>
+      </c>
+      <c r="H56" s="6" t="inlineStr">
+        <is>
+          <t>-0,75</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>36,431</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
@@ -7293,7 +7241,7 @@
       </c>
       <c r="I57" s="4" t="inlineStr">
         <is>
-          <t>327,947</t>
+          <t>540,035</t>
         </is>
       </c>
       <c r="J57" s="4" t="inlineStr">
@@ -7338,32 +7286,32 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E58" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F58" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G58" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H58" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1.637,20394000</t>
+        </is>
+      </c>
+      <c r="E58" s="6" t="inlineStr">
+        <is>
+          <t>-0,114</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>0,08</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="inlineStr">
+        <is>
+          <t>4,48</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr">
+        <is>
+          <t>13,07</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>114,507</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
@@ -7485,7 +7433,7 @@
       </c>
       <c r="I59" s="4" t="inlineStr">
         <is>
-          <t>12,847</t>
+          <t>12,674</t>
         </is>
       </c>
       <c r="J59" s="4" t="inlineStr">
@@ -7700,32 +7648,32 @@
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E61" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F61" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G61" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H61" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,25386200</t>
+        </is>
+      </c>
+      <c r="E61" s="7" t="inlineStr">
+        <is>
+          <t>-0,005</t>
+        </is>
+      </c>
+      <c r="F61" s="7" t="inlineStr">
+        <is>
+          <t>-0,15</t>
+        </is>
+      </c>
+      <c r="G61" s="5" t="inlineStr">
+        <is>
+          <t>2,66</t>
+        </is>
+      </c>
+      <c r="H61" s="5" t="inlineStr">
+        <is>
+          <t>10,74</t>
         </is>
       </c>
       <c r="I61" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>6,430</t>
         </is>
       </c>
       <c r="J61" s="4" t="inlineStr">
@@ -8062,32 +8010,32 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E64" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F64" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G64" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H64" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,42327300</t>
+        </is>
+      </c>
+      <c r="E64" s="6" t="inlineStr">
+        <is>
+          <t>-0,004</t>
+        </is>
+      </c>
+      <c r="F64" s="6" t="inlineStr">
+        <is>
+          <t>-3,09</t>
+        </is>
+      </c>
+      <c r="G64" s="3" t="inlineStr">
+        <is>
+          <t>4,26</t>
+        </is>
+      </c>
+      <c r="H64" s="3" t="inlineStr">
+        <is>
+          <t>17,44</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11,840</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
@@ -8327,7 +8275,7 @@
       </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>3,754</t>
+          <t>3,753</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr">
@@ -8424,32 +8372,32 @@
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E67" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F67" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G67" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H67" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>5,33686931</t>
+        </is>
+      </c>
+      <c r="E67" s="7" t="inlineStr">
+        <is>
+          <t>-0,114</t>
+        </is>
+      </c>
+      <c r="F67" s="5" t="inlineStr">
+        <is>
+          <t>0,09</t>
+        </is>
+      </c>
+      <c r="G67" s="5" t="inlineStr">
+        <is>
+          <t>4,01</t>
+        </is>
+      </c>
+      <c r="H67" s="5" t="inlineStr">
+        <is>
+          <t>12,82</t>
         </is>
       </c>
       <c r="I67" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>32,833</t>
         </is>
       </c>
       <c r="J67" s="4" t="inlineStr">
@@ -8571,7 +8519,7 @@
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>639,783</t>
+          <t>628,367</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr">
@@ -8668,32 +8616,32 @@
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E69" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F69" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G69" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H69" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>2,86271200</t>
+        </is>
+      </c>
+      <c r="E69" s="7" t="inlineStr">
+        <is>
+          <t>-0,004</t>
+        </is>
+      </c>
+      <c r="F69" s="5" t="inlineStr">
+        <is>
+          <t>0,34</t>
+        </is>
+      </c>
+      <c r="G69" s="5" t="inlineStr">
+        <is>
+          <t>2,49</t>
+        </is>
+      </c>
+      <c r="H69" s="5" t="inlineStr">
+        <is>
+          <t>10,66</t>
         </is>
       </c>
       <c r="I69" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>74,533</t>
         </is>
       </c>
       <c r="J69" s="4" t="inlineStr">
@@ -8815,7 +8763,7 @@
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>29,006</t>
+          <t>28,806</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
@@ -8937,7 +8885,7 @@
       </c>
       <c r="I71" s="4" t="inlineStr">
         <is>
-          <t>2.402,829</t>
+          <t>2.388,736</t>
         </is>
       </c>
       <c r="J71" s="4" t="inlineStr">
@@ -9059,7 +9007,7 @@
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>21,994</t>
+          <t>21,850</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr">
@@ -9156,32 +9104,32 @@
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E73" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F73" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G73" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H73" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1.658,37370000</t>
+        </is>
+      </c>
+      <c r="E73" s="7" t="inlineStr">
+        <is>
+          <t>-0,110</t>
+        </is>
+      </c>
+      <c r="F73" s="5" t="inlineStr">
+        <is>
+          <t>0,16</t>
+        </is>
+      </c>
+      <c r="G73" s="5" t="inlineStr">
+        <is>
+          <t>4,86</t>
+        </is>
+      </c>
+      <c r="H73" s="5" t="inlineStr">
+        <is>
+          <t>14,05</t>
         </is>
       </c>
       <c r="I73" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14,674</t>
         </is>
       </c>
       <c r="J73" s="4" t="inlineStr">
@@ -9274,32 +9222,32 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E74" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F74" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G74" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>0,52057047</t>
+        </is>
+      </c>
+      <c r="E74" s="6" t="inlineStr">
+        <is>
+          <t>-0,007</t>
+        </is>
+      </c>
+      <c r="F74" s="6" t="inlineStr">
+        <is>
+          <t>-4,04</t>
+        </is>
+      </c>
+      <c r="G74" s="6" t="inlineStr">
+        <is>
+          <t>-27,90</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3,876</t>
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr">
@@ -9396,32 +9344,32 @@
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E75" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F75" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G75" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H75" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>3,27988400</t>
+        </is>
+      </c>
+      <c r="E75" s="5" t="inlineStr">
+        <is>
+          <t>0,532</t>
+        </is>
+      </c>
+      <c r="F75" s="5" t="inlineStr">
+        <is>
+          <t>1,93</t>
+        </is>
+      </c>
+      <c r="G75" s="5" t="inlineStr">
+        <is>
+          <t>2,94</t>
+        </is>
+      </c>
+      <c r="H75" s="5" t="inlineStr">
+        <is>
+          <t>8,54</t>
         </is>
       </c>
       <c r="I75" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>156,216</t>
         </is>
       </c>
       <c r="J75" s="4" t="inlineStr">
@@ -9518,32 +9466,32 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E76" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F76" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G76" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H76" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,54915500</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="inlineStr">
+        <is>
+          <t>0,003</t>
+        </is>
+      </c>
+      <c r="F76" s="3" t="inlineStr">
+        <is>
+          <t>1,01</t>
+        </is>
+      </c>
+      <c r="G76" s="3" t="inlineStr">
+        <is>
+          <t>3,75</t>
+        </is>
+      </c>
+      <c r="H76" s="3" t="inlineStr">
+        <is>
+          <t>20,28</t>
         </is>
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14,594</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr">
@@ -9640,32 +9588,32 @@
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E77" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F77" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G77" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H77" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,37383500</t>
+        </is>
+      </c>
+      <c r="E77" s="7" t="inlineStr">
+        <is>
+          <t>-0,660</t>
+        </is>
+      </c>
+      <c r="F77" s="7" t="inlineStr">
+        <is>
+          <t>-1,70</t>
+        </is>
+      </c>
+      <c r="G77" s="5" t="inlineStr">
+        <is>
+          <t>1,30</t>
+        </is>
+      </c>
+      <c r="H77" s="5" t="inlineStr">
+        <is>
+          <t>7,37</t>
         </is>
       </c>
       <c r="I77" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>70,402</t>
         </is>
       </c>
       <c r="J77" s="4" t="inlineStr">
@@ -9762,32 +9710,32 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E78" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F78" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G78" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H78" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,50209900</t>
+        </is>
+      </c>
+      <c r="E78" s="3" t="inlineStr">
+        <is>
+          <t>0,180</t>
+        </is>
+      </c>
+      <c r="F78" s="3" t="inlineStr">
+        <is>
+          <t>3,57</t>
+        </is>
+      </c>
+      <c r="G78" s="3" t="inlineStr">
+        <is>
+          <t>3,86</t>
+        </is>
+      </c>
+      <c r="H78" s="3" t="inlineStr">
+        <is>
+          <t>16,32</t>
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>194,763</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr">
@@ -9797,7 +9745,7 @@
       </c>
       <c r="K78" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-capital-protegido-ciclico-ii-multimercado-lp/Paginas/default.aspx</t>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/caixa-fic-fim-cap-protegido-ciclico-ii</t>
         </is>
       </c>
       <c r="L78" s="2" t="inlineStr">
@@ -9884,32 +9832,32 @@
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E79" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F79" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G79" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H79" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,77828200</t>
+        </is>
+      </c>
+      <c r="E79" s="7" t="inlineStr">
+        <is>
+          <t>-0,002</t>
+        </is>
+      </c>
+      <c r="F79" s="5" t="inlineStr">
+        <is>
+          <t>1,07</t>
+        </is>
+      </c>
+      <c r="G79" s="5" t="inlineStr">
+        <is>
+          <t>0,66</t>
+        </is>
+      </c>
+      <c r="H79" s="5" t="inlineStr">
+        <is>
+          <t>10,09</t>
         </is>
       </c>
       <c r="I79" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>176,122</t>
         </is>
       </c>
       <c r="J79" s="4" t="inlineStr">
@@ -10031,7 +9979,7 @@
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>902,819</t>
+          <t>898,155</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr">
@@ -10153,7 +10101,7 @@
       </c>
       <c r="I81" s="4" t="inlineStr">
         <is>
-          <t>747,266</t>
+          <t>745,586</t>
         </is>
       </c>
       <c r="J81" s="4" t="inlineStr">
@@ -10250,32 +10198,32 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E82" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F82" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G82" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H82" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>6,82921600</t>
+        </is>
+      </c>
+      <c r="E82" s="6" t="inlineStr">
+        <is>
+          <t>-0,004</t>
+        </is>
+      </c>
+      <c r="F82" s="3" t="inlineStr">
+        <is>
+          <t>0,75</t>
+        </is>
+      </c>
+      <c r="G82" s="3" t="inlineStr">
+        <is>
+          <t>6,18</t>
+        </is>
+      </c>
+      <c r="H82" s="3" t="inlineStr">
+        <is>
+          <t>16,85</t>
         </is>
       </c>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>128,939</t>
         </is>
       </c>
       <c r="J82" s="2" t="inlineStr">
@@ -10372,32 +10320,32 @@
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E83" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F83" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G83" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H83" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,42390900</t>
+        </is>
+      </c>
+      <c r="E83" s="7" t="inlineStr">
+        <is>
+          <t>-0,003</t>
+        </is>
+      </c>
+      <c r="F83" s="5" t="inlineStr">
+        <is>
+          <t>1,09</t>
+        </is>
+      </c>
+      <c r="G83" s="5" t="inlineStr">
+        <is>
+          <t>3,35</t>
+        </is>
+      </c>
+      <c r="H83" s="5" t="inlineStr">
+        <is>
+          <t>16,21</t>
         </is>
       </c>
       <c r="I83" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>281,056</t>
         </is>
       </c>
       <c r="J83" s="4" t="inlineStr">
@@ -10494,32 +10442,32 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E84" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F84" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G84" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H84" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,32775300</t>
+        </is>
+      </c>
+      <c r="E84" s="6" t="inlineStr">
+        <is>
+          <t>-0,002</t>
+        </is>
+      </c>
+      <c r="F84" s="3" t="inlineStr">
+        <is>
+          <t>1,41</t>
+        </is>
+      </c>
+      <c r="G84" s="3" t="inlineStr">
+        <is>
+          <t>3,44</t>
+        </is>
+      </c>
+      <c r="H84" s="3" t="inlineStr">
+        <is>
+          <t>3,06</t>
         </is>
       </c>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13,382</t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr">
@@ -10641,7 +10589,7 @@
       </c>
       <c r="I85" s="4" t="inlineStr">
         <is>
-          <t>96,762</t>
+          <t>96,616</t>
         </is>
       </c>
       <c r="J85" s="4" t="inlineStr">
@@ -10763,7 +10711,7 @@
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>340,588</t>
+          <t>340,536</t>
         </is>
       </c>
       <c r="J86" s="2" t="inlineStr">
@@ -11007,7 +10955,7 @@
       </c>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>10,300</t>
+          <t>10,297</t>
         </is>
       </c>
       <c r="J88" s="2" t="inlineStr">
@@ -11125,7 +11073,7 @@
       </c>
       <c r="I89" s="4" t="inlineStr">
         <is>
-          <t>283,484</t>
+          <t>283,357</t>
         </is>
       </c>
       <c r="J89" s="4" t="inlineStr">
@@ -11247,7 +11195,7 @@
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>446,677</t>
+          <t>446,580</t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr">
@@ -11491,7 +11439,7 @@
       </c>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>2,130</t>
+          <t>2,126</t>
         </is>
       </c>
       <c r="J92" s="2" t="inlineStr">
@@ -11613,7 +11561,7 @@
       </c>
       <c r="I93" s="4" t="inlineStr">
         <is>
-          <t>76,584</t>
+          <t>76,536</t>
         </is>
       </c>
       <c r="J93" s="4" t="inlineStr">
@@ -11735,7 +11683,7 @@
       </c>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t>90,397</t>
+          <t>90,378</t>
         </is>
       </c>
       <c r="J94" s="2" t="inlineStr">
@@ -11832,32 +11780,32 @@
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E95" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F95" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G95" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H95" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,27967300</t>
+        </is>
+      </c>
+      <c r="E95" s="7" t="inlineStr">
+        <is>
+          <t>-0,045</t>
+        </is>
+      </c>
+      <c r="F95" s="7" t="inlineStr">
+        <is>
+          <t>-6,28</t>
+        </is>
+      </c>
+      <c r="G95" s="7" t="inlineStr">
+        <is>
+          <t>-0,57</t>
+        </is>
+      </c>
+      <c r="H95" s="5" t="inlineStr">
+        <is>
+          <t>7,69</t>
         </is>
       </c>
       <c r="I95" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>289,458</t>
         </is>
       </c>
       <c r="J95" s="4" t="inlineStr">
@@ -11979,7 +11927,7 @@
       </c>
       <c r="I96" s="2" t="inlineStr">
         <is>
-          <t>114,891</t>
+          <t>114,886</t>
         </is>
       </c>
       <c r="J96" s="2" t="inlineStr">
@@ -12101,7 +12049,7 @@
       </c>
       <c r="I97" s="4" t="inlineStr">
         <is>
-          <t>127,209</t>
+          <t>127,196</t>
         </is>
       </c>
       <c r="J97" s="4" t="inlineStr">
@@ -12223,7 +12171,7 @@
       </c>
       <c r="I98" s="2" t="inlineStr">
         <is>
-          <t>48,093</t>
+          <t>48,074</t>
         </is>
       </c>
       <c r="J98" s="2" t="inlineStr">
@@ -12345,7 +12293,7 @@
       </c>
       <c r="I99" s="4" t="inlineStr">
         <is>
-          <t>119,528</t>
+          <t>119,373</t>
         </is>
       </c>
       <c r="J99" s="4" t="inlineStr">
@@ -12467,7 +12415,7 @@
       </c>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t>40,929</t>
+          <t>40,893</t>
         </is>
       </c>
       <c r="J100" s="2" t="inlineStr">
@@ -12589,7 +12537,7 @@
       </c>
       <c r="I101" s="4" t="inlineStr">
         <is>
-          <t>668,903</t>
+          <t>668,752</t>
         </is>
       </c>
       <c r="J101" s="4" t="inlineStr">
@@ -12711,7 +12659,7 @@
       </c>
       <c r="I102" s="2" t="inlineStr">
         <is>
-          <t>446,282</t>
+          <t>446,175</t>
         </is>
       </c>
       <c r="J102" s="2" t="inlineStr">
@@ -13321,7 +13269,7 @@
       </c>
       <c r="I107" s="4" t="inlineStr">
         <is>
-          <t>35,566</t>
+          <t>35,541</t>
         </is>
       </c>
       <c r="J107" s="4" t="inlineStr">
@@ -13443,7 +13391,7 @@
       </c>
       <c r="I108" s="2" t="inlineStr">
         <is>
-          <t>835,509</t>
+          <t>834,938</t>
         </is>
       </c>
       <c r="J108" s="2" t="inlineStr">
@@ -13565,7 +13513,7 @@
       </c>
       <c r="I109" s="4" t="inlineStr">
         <is>
-          <t>2,908</t>
+          <t>2,906</t>
         </is>
       </c>
       <c r="J109" s="4" t="inlineStr">
@@ -13809,7 +13757,7 @@
       </c>
       <c r="I111" s="4" t="inlineStr">
         <is>
-          <t>19,715</t>
+          <t>19,698</t>
         </is>
       </c>
       <c r="J111" s="4" t="inlineStr">
@@ -13931,7 +13879,7 @@
       </c>
       <c r="I112" s="2" t="inlineStr">
         <is>
-          <t>274,449</t>
+          <t>274,269</t>
         </is>
       </c>
       <c r="J112" s="2" t="inlineStr">
@@ -14028,32 +13976,32 @@
       </c>
       <c r="D113" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E113" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F113" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G113" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H113" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1.003,15033500</t>
+        </is>
+      </c>
+      <c r="E113" s="7" t="inlineStr">
+        <is>
+          <t>-0,003</t>
+        </is>
+      </c>
+      <c r="F113" s="7" t="inlineStr">
+        <is>
+          <t>-6,24</t>
+        </is>
+      </c>
+      <c r="G113" s="5" t="inlineStr">
+        <is>
+          <t>2,32</t>
+        </is>
+      </c>
+      <c r="H113" s="5" t="inlineStr">
+        <is>
+          <t>16,31</t>
         </is>
       </c>
       <c r="I113" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>7,913</t>
         </is>
       </c>
       <c r="J113" s="4" t="inlineStr">
@@ -14150,32 +14098,32 @@
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E114" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F114" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G114" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H114" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1.505,83720300</t>
+        </is>
+      </c>
+      <c r="E114" s="6" t="inlineStr">
+        <is>
+          <t>-0,002</t>
+        </is>
+      </c>
+      <c r="F114" s="6" t="inlineStr">
+        <is>
+          <t>-6,39</t>
+        </is>
+      </c>
+      <c r="G114" s="3" t="inlineStr">
+        <is>
+          <t>0,67</t>
+        </is>
+      </c>
+      <c r="H114" s="3" t="inlineStr">
+        <is>
+          <t>10,99</t>
         </is>
       </c>
       <c r="I114" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>21,900</t>
         </is>
       </c>
       <c r="J114" s="2" t="inlineStr">
@@ -14272,7 +14220,7 @@
       </c>
       <c r="D115" s="4" t="inlineStr">
         <is>
-          <t>169,55922300</t>
+          <t>169,55922343</t>
         </is>
       </c>
       <c r="E115" s="7" t="inlineStr">
@@ -14541,7 +14489,7 @@
       </c>
       <c r="I117" s="4" t="inlineStr">
         <is>
-          <t>1.616,184</t>
+          <t>1.615,388</t>
         </is>
       </c>
       <c r="J117" s="4" t="inlineStr">
@@ -14785,7 +14733,7 @@
       </c>
       <c r="I119" s="4" t="inlineStr">
         <is>
-          <t>785,583</t>
+          <t>785,107</t>
         </is>
       </c>
       <c r="J119" s="4" t="inlineStr">
@@ -14795,17 +14743,17 @@
       </c>
       <c r="K119" s="4" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/fundos-investimento/mutuos-privatizacao/fmp-fgts-vale-do-rio-doce-1</t>
+          <t>http://www.caixa.gov.br/fundos-investimento/mutuos-privatizacao/fmp-fgts-vale-do-rio-doce-2</t>
         </is>
       </c>
       <c r="L119" s="4" t="inlineStr">
         <is>
-          <t>04.885.818/0001-90</t>
+          <t>04.885.824/0001-47</t>
         </is>
       </c>
       <c r="M119" s="4" t="inlineStr">
         <is>
-          <t>5205</t>
+          <t>5206</t>
         </is>
       </c>
       <c r="N119" s="4" t="inlineStr">
@@ -14815,12 +14763,12 @@
       </c>
       <c r="O119" s="4" t="inlineStr">
         <is>
-          <t>1.9</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="P119" s="4" t="inlineStr">
         <is>
-          <t>0.01</t>
+          <t>10000.0</t>
         </is>
       </c>
       <c r="Q119" s="4" t="inlineStr">
@@ -14835,32 +14783,32 @@
       </c>
       <c r="S119" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5205.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5206.pdf</t>
         </is>
       </c>
       <c r="T119" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5205.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5206.pdf</t>
         </is>
       </c>
       <c r="U119" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5205.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5206.pdf</t>
         </is>
       </c>
       <c r="V119" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_5205.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_5206.pdf</t>
         </is>
       </c>
       <c r="W119" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5205.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5206.pdf</t>
         </is>
       </c>
       <c r="X119" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5205.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5206.pdf</t>
         </is>
       </c>
     </row>
@@ -14907,7 +14855,7 @@
       </c>
       <c r="I120" s="2" t="inlineStr">
         <is>
-          <t>113,591</t>
+          <t>113,569</t>
         </is>
       </c>
       <c r="J120" s="2" t="inlineStr">
@@ -15151,7 +15099,7 @@
       </c>
       <c r="I122" s="2" t="inlineStr">
         <is>
-          <t>582,688</t>
+          <t>581,978</t>
         </is>
       </c>
       <c r="J122" s="2" t="inlineStr">
@@ -15273,7 +15221,7 @@
       </c>
       <c r="I123" s="4" t="inlineStr">
         <is>
-          <t>470,938</t>
+          <t>470,848</t>
         </is>
       </c>
       <c r="J123" s="4" t="inlineStr">
@@ -15283,17 +15231,17 @@
       </c>
       <c r="K123" s="4" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/fundos-investimento/mutuos-privatizacao/fmp-fgts-vale-do-rio-doce-1</t>
+          <t>http://www.caixa.gov.br/fundos-investimento/mutuos-privatizacao/fmp-fgts-vale-do-rio-doce-2</t>
         </is>
       </c>
       <c r="L123" s="4" t="inlineStr">
         <is>
-          <t>04.885.818/0001-90</t>
+          <t>04.885.824/0001-47</t>
         </is>
       </c>
       <c r="M123" s="4" t="inlineStr">
         <is>
-          <t>5205</t>
+          <t>5206</t>
         </is>
       </c>
       <c r="N123" s="4" t="inlineStr">
@@ -15303,12 +15251,12 @@
       </c>
       <c r="O123" s="4" t="inlineStr">
         <is>
-          <t>1.9</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="P123" s="4" t="inlineStr">
         <is>
-          <t>0.01</t>
+          <t>10000.0</t>
         </is>
       </c>
       <c r="Q123" s="4" t="inlineStr">
@@ -15323,32 +15271,32 @@
       </c>
       <c r="S123" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5205.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5206.pdf</t>
         </is>
       </c>
       <c r="T123" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5205.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5206.pdf</t>
         </is>
       </c>
       <c r="U123" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5205.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5206.pdf</t>
         </is>
       </c>
       <c r="V123" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_5205.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_5206.pdf</t>
         </is>
       </c>
       <c r="W123" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5205.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5206.pdf</t>
         </is>
       </c>
       <c r="X123" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5205.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5206.pdf</t>
         </is>
       </c>
     </row>
@@ -15395,7 +15343,7 @@
       </c>
       <c r="I124" s="2" t="inlineStr">
         <is>
-          <t>670,495</t>
+          <t>669,850</t>
         </is>
       </c>
       <c r="J124" s="2" t="inlineStr">
@@ -15639,7 +15587,7 @@
       </c>
       <c r="I126" s="2" t="inlineStr">
         <is>
-          <t>215,263</t>
+          <t>196,696</t>
         </is>
       </c>
       <c r="J126" s="2" t="inlineStr">
@@ -15761,7 +15709,7 @@
       </c>
       <c r="I127" s="4" t="inlineStr">
         <is>
-          <t>41,338</t>
+          <t>41,030</t>
         </is>
       </c>
       <c r="J127" s="4" t="inlineStr">
@@ -15883,7 +15831,7 @@
       </c>
       <c r="I128" s="2" t="inlineStr">
         <is>
-          <t>791,217</t>
+          <t>784,325</t>
         </is>
       </c>
       <c r="J128" s="2" t="inlineStr">
@@ -16005,7 +15953,7 @@
       </c>
       <c r="I129" s="4" t="inlineStr">
         <is>
-          <t>18,924</t>
+          <t>18,812</t>
         </is>
       </c>
       <c r="J129" s="4" t="inlineStr">
@@ -16127,7 +16075,7 @@
       </c>
       <c r="I130" s="2" t="inlineStr">
         <is>
-          <t>94,973</t>
+          <t>94,369</t>
         </is>
       </c>
       <c r="J130" s="2" t="inlineStr">
@@ -16249,7 +16197,7 @@
       </c>
       <c r="I131" s="4" t="inlineStr">
         <is>
-          <t>7.939,338</t>
+          <t>7.710,838</t>
         </is>
       </c>
       <c r="J131" s="4" t="inlineStr">
@@ -16371,7 +16319,7 @@
       </c>
       <c r="I132" s="2" t="inlineStr">
         <is>
-          <t>15.867,048</t>
+          <t>15.793,725</t>
         </is>
       </c>
       <c r="J132" s="2" t="inlineStr">
@@ -16406,7 +16354,7 @@
       </c>
       <c r="P132" s="2" t="inlineStr">
         <is>
-          <t>1000000.0</t>
+          <t>3000000.0</t>
         </is>
       </c>
       <c r="Q132" s="2" t="inlineStr">
@@ -16493,7 +16441,7 @@
       </c>
       <c r="I133" s="4" t="inlineStr">
         <is>
-          <t>3.045,452</t>
+          <t>3.031,660</t>
         </is>
       </c>
       <c r="J133" s="4" t="inlineStr">
@@ -16528,7 +16476,7 @@
       </c>
       <c r="P133" s="4" t="inlineStr">
         <is>
-          <t>1000000.0</t>
+          <t>3000000.0</t>
         </is>
       </c>
       <c r="Q133" s="4" t="inlineStr">
@@ -16590,7 +16538,7 @@
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>1,54654300</t>
+          <t>1,54654296</t>
         </is>
       </c>
       <c r="E134" s="3" t="inlineStr">
@@ -16737,7 +16685,7 @@
       </c>
       <c r="I135" s="4" t="inlineStr">
         <is>
-          <t>285,149</t>
+          <t>284,379</t>
         </is>
       </c>
       <c r="J135" s="4" t="inlineStr">
@@ -16859,7 +16807,7 @@
       </c>
       <c r="I136" s="2" t="inlineStr">
         <is>
-          <t>4.013,008</t>
+          <t>4.011,477</t>
         </is>
       </c>
       <c r="J136" s="2" t="inlineStr">
@@ -16981,7 +16929,7 @@
       </c>
       <c r="I137" s="4" t="inlineStr">
         <is>
-          <t>4.781,473</t>
+          <t>4.780,987</t>
         </is>
       </c>
       <c r="J137" s="4" t="inlineStr">
@@ -17099,7 +17047,7 @@
       </c>
       <c r="I138" s="2" t="inlineStr">
         <is>
-          <t>13.989,956</t>
+          <t>13.597,824</t>
         </is>
       </c>
       <c r="J138" s="2" t="inlineStr">
@@ -17221,7 +17169,7 @@
       </c>
       <c r="I139" s="4" t="inlineStr">
         <is>
-          <t>12.515,793</t>
+          <t>12.463,903</t>
         </is>
       </c>
       <c r="J139" s="4" t="inlineStr">
@@ -17256,7 +17204,7 @@
       </c>
       <c r="P139" s="4" t="inlineStr">
         <is>
-          <t>1000000.0</t>
+          <t>3000000.0</t>
         </is>
       </c>
       <c r="Q139" s="4" t="inlineStr">
@@ -17343,7 +17291,7 @@
       </c>
       <c r="I140" s="2" t="inlineStr">
         <is>
-          <t>3.596,587</t>
+          <t>3.582,717</t>
         </is>
       </c>
       <c r="J140" s="2" t="inlineStr">
@@ -17378,7 +17326,7 @@
       </c>
       <c r="P140" s="2" t="inlineStr">
         <is>
-          <t>1000000.0</t>
+          <t>3000000.0</t>
         </is>
       </c>
       <c r="Q140" s="2" t="inlineStr">
@@ -17465,7 +17413,7 @@
       </c>
       <c r="I141" s="4" t="inlineStr">
         <is>
-          <t>1.468,990</t>
+          <t>1.461,203</t>
         </is>
       </c>
       <c r="J141" s="4" t="inlineStr">
@@ -17587,7 +17535,7 @@
       </c>
       <c r="I142" s="2" t="inlineStr">
         <is>
-          <t>33.690,972</t>
+          <t>31.773,754</t>
         </is>
       </c>
       <c r="J142" s="2" t="inlineStr">
@@ -17709,7 +17657,7 @@
       </c>
       <c r="I143" s="4" t="inlineStr">
         <is>
-          <t>3.007,512</t>
+          <t>2.804,769</t>
         </is>
       </c>
       <c r="J143" s="4" t="inlineStr">
@@ -17831,7 +17779,7 @@
       </c>
       <c r="I144" s="2" t="inlineStr">
         <is>
-          <t>16.519,133</t>
+          <t>16.634,401</t>
         </is>
       </c>
       <c r="J144" s="2" t="inlineStr">
@@ -18456,12 +18404,12 @@
       </c>
       <c r="L149" s="4" t="inlineStr">
         <is>
-          <t>14.508.605/0001-00</t>
+          <t>10.740.670/0001-06</t>
         </is>
       </c>
       <c r="M149" s="4" t="inlineStr">
         <is>
-          <t>5824</t>
+          <t>5464</t>
         </is>
       </c>
       <c r="N149" s="4" t="inlineStr">
@@ -18491,32 +18439,32 @@
       </c>
       <c r="S149" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5824.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5464.pdf</t>
         </is>
       </c>
       <c r="T149" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5824.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5464.pdf</t>
         </is>
       </c>
       <c r="U149" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5824.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5464.pdf</t>
         </is>
       </c>
       <c r="V149" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5824.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5464.pdf</t>
         </is>
       </c>
       <c r="W149" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5824.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5464.pdf</t>
         </is>
       </c>
       <c r="X149" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5824.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5464.pdf</t>
         </is>
       </c>
     </row>
@@ -18700,12 +18648,12 @@
       </c>
       <c r="L151" s="4" t="inlineStr">
         <is>
-          <t>14.508.605/0001-00</t>
+          <t>10.740.670/0001-06</t>
         </is>
       </c>
       <c r="M151" s="4" t="inlineStr">
         <is>
-          <t>5824</t>
+          <t>5464</t>
         </is>
       </c>
       <c r="N151" s="4" t="inlineStr">
@@ -18735,32 +18683,32 @@
       </c>
       <c r="S151" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5824.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5464.pdf</t>
         </is>
       </c>
       <c r="T151" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5824.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5464.pdf</t>
         </is>
       </c>
       <c r="U151" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5824.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5464.pdf</t>
         </is>
       </c>
       <c r="V151" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5824.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5464.pdf</t>
         </is>
       </c>
       <c r="W151" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5824.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5464.pdf</t>
         </is>
       </c>
       <c r="X151" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5824.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5464.pdf</t>
         </is>
       </c>
     </row>
@@ -19365,7 +19313,7 @@
       </c>
       <c r="I157" s="4" t="inlineStr">
         <is>
-          <t>720,376</t>
+          <t>720,375</t>
         </is>
       </c>
       <c r="J157" s="4" t="inlineStr">
@@ -19380,12 +19328,12 @@
       </c>
       <c r="L157" s="4" t="inlineStr">
         <is>
-          <t>14.508.605/0001-00</t>
+          <t>10.740.670/0001-06</t>
         </is>
       </c>
       <c r="M157" s="4" t="inlineStr">
         <is>
-          <t>5824</t>
+          <t>5464</t>
         </is>
       </c>
       <c r="N157" s="4" t="inlineStr">
@@ -19415,32 +19363,32 @@
       </c>
       <c r="S157" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5824.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5464.pdf</t>
         </is>
       </c>
       <c r="T157" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5824.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5464.pdf</t>
         </is>
       </c>
       <c r="U157" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5824.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5464.pdf</t>
         </is>
       </c>
       <c r="V157" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5824.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5464.pdf</t>
         </is>
       </c>
       <c r="W157" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5824.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5464.pdf</t>
         </is>
       </c>
       <c r="X157" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5824.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5464.pdf</t>
         </is>
       </c>
     </row>
@@ -19487,7 +19435,7 @@
       </c>
       <c r="I158" s="2" t="inlineStr">
         <is>
-          <t>12.901,464</t>
+          <t>12.901,293</t>
         </is>
       </c>
       <c r="J158" s="2" t="inlineStr">
@@ -19502,12 +19450,12 @@
       </c>
       <c r="L158" s="2" t="inlineStr">
         <is>
-          <t>03.737.206/0001-97</t>
+          <t>05.164.356/0001-84</t>
         </is>
       </c>
       <c r="M158" s="2" t="inlineStr">
         <is>
-          <t>5404</t>
+          <t>5462</t>
         </is>
       </c>
       <c r="N158" s="2" t="inlineStr">
@@ -19537,32 +19485,32 @@
       </c>
       <c r="S158" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5404.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5462.pdf</t>
         </is>
       </c>
       <c r="T158" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5404.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5462.pdf</t>
         </is>
       </c>
       <c r="U158" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5404.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5462.pdf</t>
         </is>
       </c>
       <c r="V158" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5404.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5462.pdf</t>
         </is>
       </c>
       <c r="W158" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5404.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5462.pdf</t>
         </is>
       </c>
       <c r="X158" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5404.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5462.pdf</t>
         </is>
       </c>
     </row>
@@ -19609,7 +19557,7 @@
       </c>
       <c r="I159" s="4" t="inlineStr">
         <is>
-          <t>4.621,489</t>
+          <t>4.621,477</t>
         </is>
       </c>
       <c r="J159" s="4" t="inlineStr">
@@ -19853,7 +19801,7 @@
       </c>
       <c r="I161" s="4" t="inlineStr">
         <is>
-          <t>1.750,478</t>
+          <t>1.543,199</t>
         </is>
       </c>
       <c r="J161" s="4" t="inlineStr">
@@ -19975,7 +19923,7 @@
       </c>
       <c r="I162" s="2" t="inlineStr">
         <is>
-          <t>23.815,568</t>
+          <t>23.815,493</t>
         </is>
       </c>
       <c r="J162" s="2" t="inlineStr">
@@ -20289,7 +20237,7 @@
       </c>
       <c r="I165" s="4" t="inlineStr">
         <is>
-          <t>295,252</t>
+          <t>295,234</t>
         </is>
       </c>
       <c r="J165" s="4" t="inlineStr">
@@ -20508,7 +20456,7 @@
       </c>
       <c r="D167" s="4" t="inlineStr">
         <is>
-          <t>11,49497800</t>
+          <t>11,49497823</t>
         </is>
       </c>
       <c r="E167" s="5" t="inlineStr">
@@ -20874,7 +20822,7 @@
       </c>
       <c r="D170" s="2" t="inlineStr">
         <is>
-          <t>3,41371100</t>
+          <t>3,41371062</t>
         </is>
       </c>
       <c r="E170" s="6" t="inlineStr">
@@ -20992,7 +20940,7 @@
       </c>
       <c r="D171" s="4" t="inlineStr">
         <is>
-          <t>2,48907700</t>
+          <t>2,48907659</t>
         </is>
       </c>
       <c r="E171" s="7" t="inlineStr">
@@ -21135,7 +21083,7 @@
       </c>
       <c r="I172" s="2" t="inlineStr">
         <is>
-          <t>4.929,702</t>
+          <t>4.880,670</t>
         </is>
       </c>
       <c r="J172" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Dados atualizados via Robô: 12/06/2026 02:36
</commit_message>
<xml_diff>
--- a/dados_atuais.xlsx
+++ b/dados_atuais.xlsx
@@ -3262,22 +3262,22 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>1,10173366</t>
-        </is>
-      </c>
-      <c r="E24" s="7" t="inlineStr">
-        <is>
-          <t>-0,001</t>
+          <t>1,10380800</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>0,186</t>
         </is>
       </c>
       <c r="F24" s="7" t="inlineStr">
         <is>
-          <t>-1,14</t>
+          <t>-0,95</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>2,13</t>
+          <t>2,32</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -3287,7 +3287,7 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>203,565</t>
+          <t>203,949</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
@@ -3384,32 +3384,32 @@
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>1,24015200</t>
-        </is>
-      </c>
-      <c r="E25" s="6" t="inlineStr">
-        <is>
-          <t>-0,001</t>
+          <t>1,24082700</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>0,053</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>0,32</t>
+          <t>0,37</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>5,88</t>
+          <t>5,94</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr">
         <is>
-          <t>14,54</t>
+          <t>14,61</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>71,144</t>
+          <t>71,182</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -3750,22 +3750,22 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>1,03873100</t>
-        </is>
-      </c>
-      <c r="E28" s="7" t="inlineStr">
-        <is>
-          <t>-0,001</t>
+          <t>1,03996200</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>0,056</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>0,26</t>
+          <t>0,37</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>5,93</t>
+          <t>6,05</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -3775,7 +3775,7 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>21,933</t>
+          <t>21,959</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
@@ -3868,32 +3868,32 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>1,17052700</t>
-        </is>
-      </c>
-      <c r="E29" s="6" t="inlineStr">
-        <is>
-          <t>-0,001</t>
+          <t>1,17114000</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>0,051</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>0,45</t>
+          <t>0,51</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>5,41</t>
+          <t>5,46</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr">
         <is>
-          <t>13,99</t>
+          <t>14,05</t>
         </is>
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>66,479</t>
+          <t>66,514</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -3986,22 +3986,22 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>1,07281439</t>
-        </is>
-      </c>
-      <c r="E30" s="7" t="inlineStr">
-        <is>
-          <t>-0,001</t>
+          <t>1,07439400</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>0,145</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>0,33</t>
+          <t>0,48</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>3,82</t>
+          <t>3,97</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -4011,7 +4011,7 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>305,940</t>
+          <t>306,390</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
@@ -6972,32 +6972,32 @@
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>1,41608300</t>
-        </is>
-      </c>
-      <c r="E55" s="4" t="inlineStr">
-        <is>
-          <t>0,000</t>
+          <t>1,41627200</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>0,013</t>
         </is>
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>0,39</t>
+          <t>0,40</t>
         </is>
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
-          <t>5,76</t>
+          <t>5,78</t>
         </is>
       </c>
       <c r="H55" s="5" t="inlineStr">
         <is>
-          <t>14,35</t>
+          <t>14,36</t>
         </is>
       </c>
       <c r="I55" s="4" t="inlineStr">
         <is>
-          <t>67,801</t>
+          <t>67,810</t>
         </is>
       </c>
       <c r="J55" s="4" t="inlineStr">
@@ -7094,32 +7094,32 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>1.218,68940700</t>
+          <t>1.207,29403300</t>
         </is>
       </c>
       <c r="E56" s="7" t="inlineStr">
         <is>
-          <t>-0,002</t>
+          <t>-0,937</t>
         </is>
       </c>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>1,25</t>
+          <t>0,30</t>
         </is>
       </c>
       <c r="G56" s="7" t="inlineStr">
         <is>
-          <t>-2,87</t>
+          <t>-3,78</t>
         </is>
       </c>
       <c r="H56" s="3" t="inlineStr">
         <is>
-          <t>1,51</t>
+          <t>0,56</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>37,155</t>
+          <t>36,808</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
@@ -7286,32 +7286,32 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>1.617,46323900</t>
+          <t>1.614,86272800</t>
         </is>
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
-          <t>-0,006</t>
+          <t>-0,166</t>
         </is>
       </c>
       <c r="F58" s="7" t="inlineStr">
         <is>
-          <t>-1,20</t>
+          <t>-1,36</t>
         </is>
       </c>
       <c r="G58" s="3" t="inlineStr">
         <is>
-          <t>3,22</t>
+          <t>3,05</t>
         </is>
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>11,18</t>
+          <t>11,00</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>113,173</t>
+          <t>112,991</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
@@ -7648,32 +7648,32 @@
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>1,24518700</t>
+          <t>1,24466400</t>
         </is>
       </c>
       <c r="E61" s="6" t="inlineStr">
         <is>
-          <t>-0,005</t>
+          <t>-0,047</t>
         </is>
       </c>
       <c r="F61" s="6" t="inlineStr">
         <is>
-          <t>-0,50</t>
+          <t>-0,54</t>
         </is>
       </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
-          <t>1,95</t>
+          <t>1,91</t>
         </is>
       </c>
       <c r="H61" s="5" t="inlineStr">
         <is>
-          <t>9,44</t>
+          <t>9,39</t>
         </is>
       </c>
       <c r="I61" s="4" t="inlineStr">
         <is>
-          <t>6,272</t>
+          <t>6,269</t>
         </is>
       </c>
       <c r="J61" s="4" t="inlineStr">
@@ -8010,32 +8010,32 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>1,38982100</t>
+          <t>1,37630800</t>
         </is>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>-0,004</t>
+          <t>-0,977</t>
         </is>
       </c>
       <c r="F64" s="7" t="inlineStr">
         <is>
-          <t>-2,15</t>
+          <t>-3,10</t>
         </is>
       </c>
       <c r="G64" s="3" t="inlineStr">
         <is>
-          <t>1,81</t>
+          <t>0,82</t>
         </is>
       </c>
       <c r="H64" s="3" t="inlineStr">
         <is>
-          <t>14,52</t>
+          <t>13,41</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>11,523</t>
+          <t>11,411</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
@@ -8372,32 +8372,32 @@
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>5,27698843</t>
+          <t>5,26976600</t>
         </is>
       </c>
       <c r="E67" s="6" t="inlineStr">
         <is>
-          <t>-0,003</t>
+          <t>-0,140</t>
         </is>
       </c>
       <c r="F67" s="6" t="inlineStr">
         <is>
-          <t>-1,12</t>
+          <t>-1,25</t>
         </is>
       </c>
       <c r="G67" s="5" t="inlineStr">
         <is>
-          <t>2,84</t>
+          <t>2,70</t>
         </is>
       </c>
       <c r="H67" s="5" t="inlineStr">
         <is>
-          <t>11,02</t>
+          <t>10,87</t>
         </is>
       </c>
       <c r="I67" s="4" t="inlineStr">
         <is>
-          <t>32,492</t>
+          <t>32,447</t>
         </is>
       </c>
       <c r="J67" s="4" t="inlineStr">
@@ -8616,32 +8616,32 @@
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>2,83240800</t>
+          <t>2,82738400</t>
         </is>
       </c>
       <c r="E69" s="6" t="inlineStr">
         <is>
-          <t>-0,004</t>
+          <t>-0,181</t>
         </is>
       </c>
       <c r="F69" s="6" t="inlineStr">
         <is>
-          <t>-1,07</t>
+          <t>-1,24</t>
         </is>
       </c>
       <c r="G69" s="5" t="inlineStr">
         <is>
-          <t>1,40</t>
+          <t>1,22</t>
         </is>
       </c>
       <c r="H69" s="5" t="inlineStr">
         <is>
-          <t>9,05</t>
+          <t>8,85</t>
         </is>
       </c>
       <c r="I69" s="4" t="inlineStr">
         <is>
-          <t>73,514</t>
+          <t>73,384</t>
         </is>
       </c>
       <c r="J69" s="4" t="inlineStr">
@@ -9104,32 +9104,32 @@
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>1.638,96341700</t>
+          <t>1.636,33252700</t>
         </is>
       </c>
       <c r="E73" s="6" t="inlineStr">
         <is>
-          <t>-0,003</t>
+          <t>-0,163</t>
         </is>
       </c>
       <c r="F73" s="6" t="inlineStr">
         <is>
-          <t>-1,17</t>
+          <t>-1,32</t>
         </is>
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>3,63</t>
+          <t>3,46</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
         <is>
-          <t>12,15</t>
+          <t>11,97</t>
         </is>
       </c>
       <c r="I73" s="4" t="inlineStr">
         <is>
-          <t>14,384</t>
+          <t>14,361</t>
         </is>
       </c>
       <c r="J73" s="4" t="inlineStr">
@@ -9222,22 +9222,22 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>0,45575376</t>
+          <t>0,45277400</t>
         </is>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>-0,005</t>
+          <t>-0,659</t>
         </is>
       </c>
       <c r="F74" s="7" t="inlineStr">
         <is>
-          <t>-13,50</t>
+          <t>-14,06</t>
         </is>
       </c>
       <c r="G74" s="7" t="inlineStr">
         <is>
-          <t>-36,88</t>
+          <t>-37,29</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
@@ -9247,7 +9247,7 @@
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>3,609</t>
+          <t>3,585</t>
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr">
@@ -9344,32 +9344,32 @@
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>3,27918200</t>
+          <t>3,24636900</t>
         </is>
       </c>
       <c r="E75" s="6" t="inlineStr">
         <is>
-          <t>-0,005</t>
+          <t>-1,006</t>
         </is>
       </c>
       <c r="F75" s="6" t="inlineStr">
         <is>
-          <t>-0,02</t>
+          <t>-1,02</t>
         </is>
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2,92</t>
+          <t>1,89</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
         <is>
-          <t>10,40</t>
+          <t>9,30</t>
         </is>
       </c>
       <c r="I75" s="4" t="inlineStr">
         <is>
-          <t>156,182</t>
+          <t>154,619</t>
         </is>
       </c>
       <c r="J75" s="4" t="inlineStr">
@@ -9466,12 +9466,12 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>1,52179200</t>
-        </is>
-      </c>
-      <c r="E76" s="7" t="inlineStr">
-        <is>
-          <t>-0,004</t>
+          <t>1,52188600</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="inlineStr">
+        <is>
+          <t>0,001</t>
         </is>
       </c>
       <c r="F76" s="7" t="inlineStr">
@@ -9481,17 +9481,17 @@
       </c>
       <c r="G76" s="3" t="inlineStr">
         <is>
-          <t>1,91</t>
+          <t>1,92</t>
         </is>
       </c>
       <c r="H76" s="3" t="inlineStr">
         <is>
-          <t>18,98</t>
+          <t>18,99</t>
         </is>
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>14,336</t>
+          <t>14,337</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr">
@@ -9588,32 +9588,32 @@
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>1,37835200</t>
-        </is>
-      </c>
-      <c r="E77" s="6" t="inlineStr">
-        <is>
-          <t>-0,003</t>
+          <t>1,37872300</t>
+        </is>
+      </c>
+      <c r="E77" s="5" t="inlineStr">
+        <is>
+          <t>0,023</t>
         </is>
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>0,32</t>
+          <t>0,35</t>
         </is>
       </c>
       <c r="G77" s="5" t="inlineStr">
         <is>
-          <t>1,63</t>
+          <t>1,66</t>
         </is>
       </c>
       <c r="H77" s="5" t="inlineStr">
         <is>
-          <t>6,77</t>
+          <t>6,80</t>
         </is>
       </c>
       <c r="I77" s="4" t="inlineStr">
         <is>
-          <t>70,633</t>
+          <t>70,652</t>
         </is>
       </c>
       <c r="J77" s="4" t="inlineStr">
@@ -9710,32 +9710,32 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>1,47839000</t>
+          <t>1,47241800</t>
         </is>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
-          <t>-0,003</t>
+          <t>-0,407</t>
         </is>
       </c>
       <c r="F78" s="7" t="inlineStr">
         <is>
-          <t>-1,57</t>
+          <t>-1,97</t>
         </is>
       </c>
       <c r="G78" s="3" t="inlineStr">
         <is>
-          <t>2,22</t>
+          <t>1,81</t>
         </is>
       </c>
       <c r="H78" s="3" t="inlineStr">
         <is>
-          <t>13,58</t>
+          <t>13,12</t>
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>191,689</t>
+          <t>190,914</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr">
@@ -9832,32 +9832,32 @@
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>1,79303600</t>
+          <t>1,78949700</t>
         </is>
       </c>
       <c r="E79" s="6" t="inlineStr">
         <is>
-          <t>-0,002</t>
+          <t>-0,199</t>
         </is>
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>0,70</t>
+          <t>0,50</t>
         </is>
       </c>
       <c r="G79" s="5" t="inlineStr">
         <is>
-          <t>1,50</t>
+          <t>1,30</t>
         </is>
       </c>
       <c r="H79" s="5" t="inlineStr">
         <is>
-          <t>10,87</t>
+          <t>10,65</t>
         </is>
       </c>
       <c r="I79" s="4" t="inlineStr">
         <is>
-          <t>176,188</t>
+          <t>175,840</t>
         </is>
       </c>
       <c r="J79" s="4" t="inlineStr">
@@ -10198,32 +10198,32 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>6,73078500</t>
+          <t>6,72459500</t>
         </is>
       </c>
       <c r="E82" s="7" t="inlineStr">
         <is>
-          <t>-0,004</t>
+          <t>-0,096</t>
         </is>
       </c>
       <c r="F82" s="7" t="inlineStr">
         <is>
-          <t>-1,57</t>
+          <t>-1,66</t>
         </is>
       </c>
       <c r="G82" s="3" t="inlineStr">
         <is>
-          <t>4,65</t>
+          <t>4,56</t>
         </is>
       </c>
       <c r="H82" s="3" t="inlineStr">
         <is>
-          <t>14,66</t>
+          <t>14,55</t>
         </is>
       </c>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t>127,299</t>
+          <t>127,182</t>
         </is>
       </c>
       <c r="J82" s="2" t="inlineStr">
@@ -10442,32 +10442,32 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>1,34407000</t>
+          <t>1,33970400</t>
         </is>
       </c>
       <c r="E84" s="7" t="inlineStr">
         <is>
-          <t>-0,002</t>
+          <t>-0,326</t>
         </is>
       </c>
       <c r="F84" s="3" t="inlineStr">
         <is>
-          <t>1,58</t>
+          <t>1,25</t>
         </is>
       </c>
       <c r="G84" s="3" t="inlineStr">
         <is>
-          <t>4,71</t>
+          <t>4,37</t>
         </is>
       </c>
       <c r="H84" s="3" t="inlineStr">
         <is>
-          <t>4,48</t>
+          <t>4,14</t>
         </is>
       </c>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t>13,116</t>
+          <t>13,074</t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr">
@@ -11780,32 +11780,32 @@
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
-          <t>1,23980500</t>
+          <t>1,22546800</t>
         </is>
       </c>
       <c r="E95" s="6" t="inlineStr">
         <is>
-          <t>-0,017</t>
+          <t>-1,174</t>
         </is>
       </c>
       <c r="F95" s="6" t="inlineStr">
         <is>
-          <t>-2,43</t>
+          <t>-3,56</t>
         </is>
       </c>
       <c r="G95" s="6" t="inlineStr">
         <is>
-          <t>-3,67</t>
+          <t>-4,78</t>
         </is>
       </c>
       <c r="H95" s="5" t="inlineStr">
         <is>
-          <t>5,15</t>
+          <t>3,94</t>
         </is>
       </c>
       <c r="I95" s="4" t="inlineStr">
         <is>
-          <t>280,349</t>
+          <t>277,107</t>
         </is>
       </c>
       <c r="J95" s="4" t="inlineStr">
@@ -13976,32 +13976,32 @@
       </c>
       <c r="D113" s="4" t="inlineStr">
         <is>
-          <t>977,98991400</t>
+          <t>969,32849400</t>
         </is>
       </c>
       <c r="E113" s="6" t="inlineStr">
         <is>
-          <t>-0,003</t>
+          <t>-0,888</t>
         </is>
       </c>
       <c r="F113" s="6" t="inlineStr">
         <is>
-          <t>-2,15</t>
+          <t>-3,01</t>
         </is>
       </c>
       <c r="G113" s="6" t="inlineStr">
         <is>
-          <t>-0,24</t>
+          <t>-1,12</t>
         </is>
       </c>
       <c r="H113" s="5" t="inlineStr">
         <is>
-          <t>14,75</t>
+          <t>13,73</t>
         </is>
       </c>
       <c r="I113" s="4" t="inlineStr">
         <is>
-          <t>7,944</t>
+          <t>7,874</t>
         </is>
       </c>
       <c r="J113" s="4" t="inlineStr">
@@ -14098,32 +14098,32 @@
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>1.464,51393600</t>
+          <t>1.450,47136800</t>
         </is>
       </c>
       <c r="E114" s="7" t="inlineStr">
         <is>
-          <t>-0,002</t>
+          <t>-0,961</t>
         </is>
       </c>
       <c r="F114" s="7" t="inlineStr">
         <is>
-          <t>-2,05</t>
+          <t>-2,99</t>
         </is>
       </c>
       <c r="G114" s="7" t="inlineStr">
         <is>
-          <t>-2,09</t>
+          <t>-3,03</t>
         </is>
       </c>
       <c r="H114" s="3" t="inlineStr">
         <is>
-          <t>9,29</t>
+          <t>8,24</t>
         </is>
       </c>
       <c r="I114" s="2" t="inlineStr">
         <is>
-          <t>21,110</t>
+          <t>20,907</t>
         </is>
       </c>
       <c r="J114" s="2" t="inlineStr">
@@ -19450,12 +19450,12 @@
       </c>
       <c r="L158" s="2" t="inlineStr">
         <is>
-          <t>05.164.356/0001-84</t>
+          <t>03.737.206/0001-97</t>
         </is>
       </c>
       <c r="M158" s="2" t="inlineStr">
         <is>
-          <t>5462</t>
+          <t>5404</t>
         </is>
       </c>
       <c r="N158" s="2" t="inlineStr">
@@ -19485,32 +19485,32 @@
       </c>
       <c r="S158" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5462.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5404.pdf</t>
         </is>
       </c>
       <c r="T158" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5462.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5404.pdf</t>
         </is>
       </c>
       <c r="U158" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5462.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5404.pdf</t>
         </is>
       </c>
       <c r="V158" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5462.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5404.pdf</t>
         </is>
       </c>
       <c r="W158" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5462.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5404.pdf</t>
         </is>
       </c>
       <c r="X158" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5462.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5404.pdf</t>
         </is>
       </c>
     </row>
@@ -20090,32 +20090,32 @@
       </c>
       <c r="D164" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E164" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F164" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G164" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H164" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1.530,12954000</t>
+        </is>
+      </c>
+      <c r="E164" s="7" t="inlineStr">
+        <is>
+          <t>-0,167</t>
+        </is>
+      </c>
+      <c r="F164" s="7" t="inlineStr">
+        <is>
+          <t>-1,35</t>
+        </is>
+      </c>
+      <c r="G164" s="3" t="inlineStr">
+        <is>
+          <t>3,08</t>
+        </is>
+      </c>
+      <c r="H164" s="3" t="inlineStr">
+        <is>
+          <t>11,03</t>
         </is>
       </c>
       <c r="I164" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>128,581</t>
         </is>
       </c>
       <c r="J164" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Dados atualizados via Robô: 15/06/2026 17:08
</commit_message>
<xml_diff>
--- a/dados_atuais.xlsx
+++ b/dados_atuais.xlsx
@@ -809,7 +809,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>408,242</t>
+          <t>405,891</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -904,7 +904,7 @@
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>6.675,758</t>
+          <t>6.599,761</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
@@ -1141,7 +1141,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>982,612</t>
+          <t>971,966</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -1618,7 +1618,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>119,869</t>
+          <t>119,868</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -1860,7 +1860,7 @@
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>96,756</t>
+          <t>96,673</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -1875,12 +1875,12 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>40.194.309/0001-84</t>
+          <t>40.194.314/0001-97</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>6532</t>
+          <t>6533</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
@@ -1890,27 +1890,27 @@
       </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
-          <t>0.7</t>
+          <t>0.55</t>
         </is>
       </c>
       <c r="P7" s="4" t="inlineStr">
         <is>
-          <t>0.01</t>
+          <t>10000.0</t>
         </is>
       </c>
       <c r="Q7" s="4" t="inlineStr">
         <is>
-          <t>0.01</t>
+          <t>100.0</t>
         </is>
       </c>
       <c r="R7" s="4" t="inlineStr">
         <is>
-          <t>0.01</t>
+          <t>100.0</t>
         </is>
       </c>
       <c r="S7" s="4" t="inlineStr">
         <is>
-          <t>0.01</t>
+          <t>1000.0</t>
         </is>
       </c>
       <c r="T7" s="4" t="inlineStr">
@@ -1950,7 +1950,7 @@
       </c>
       <c r="AA7" s="4" t="inlineStr">
         <is>
-          <t>GERAL</t>
+          <t>QUALIFICADO</t>
         </is>
       </c>
       <c r="AB7" s="4" t="inlineStr">
@@ -2006,48 +2006,52 @@
       </c>
       <c r="AM7" s="4" t="inlineStr">
         <is>
-          <t>CAIXA PLUS FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA CRÉDITO PRIVADO LONGO PRAZO - RESP LIMITADA</t>
-        </is>
-      </c>
-      <c r="AN7" s="4" t="inlineStr"/>
+          <t>CAIXA PLUS QUALIFICADO FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA CRÉDITO PRIVADO LP - RESP LIMITADA</t>
+        </is>
+      </c>
+      <c r="AN7" s="4" t="inlineStr">
+        <is>
+          <t>OBS: Este Fundo não está adaptado às normas vigentes para RPPS (Regimes Próprios de Previdência Social).</t>
+        </is>
+      </c>
       <c r="AO7" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_6532.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_6533.pdf</t>
         </is>
       </c>
       <c r="AP7" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_6532.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_6533.pdf</t>
         </is>
       </c>
       <c r="AQ7" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_6532.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_6533.pdf</t>
         </is>
       </c>
       <c r="AR7" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_6532.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_6533.pdf</t>
         </is>
       </c>
       <c r="AS7" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6532.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6533.pdf</t>
         </is>
       </c>
       <c r="AT7" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6532.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6533.pdf</t>
         </is>
       </c>
       <c r="AU7" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_6532.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_6533.pdf</t>
         </is>
       </c>
       <c r="AV7" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/caixa-asset/sumario-remuneracao/Documents/sumarios/6532-SUMARIO.pdf</t>
+          <t>https://www.caixa.gov.br/caixa-asset/sumario-remuneracao/Documents/sumarios/6533-SUMARIO.pdf</t>
         </is>
       </c>
       <c r="AW7" s="4" t="inlineStr"/>
@@ -2095,7 +2099,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>582,977</t>
+          <t>582,976</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -2569,7 +2573,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>1.665,658</t>
+          <t>1.665,645</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -3047,7 +3051,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>27,636</t>
+          <t>27,602</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -3062,12 +3066,12 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>03.191.874/0001-61</t>
+          <t>09.548.729/0001-71</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>5414</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -3077,27 +3081,27 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>0.3</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>100000.0</t>
+          <t>100.0</t>
         </is>
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>100.0</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="R12" s="2" t="inlineStr">
         <is>
-          <t>100.0</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="S12" s="2" t="inlineStr">
         <is>
-          <t>10000.0</t>
+          <t>10.0</t>
         </is>
       </c>
       <c r="T12" s="2" t="inlineStr">
@@ -3117,7 +3121,7 @@
       </c>
       <c r="W12" s="2" t="inlineStr">
         <is>
-          <t>IPCA+6%</t>
+          <t>NÃO SE APLICA</t>
         </is>
       </c>
       <c r="X12" s="2" t="inlineStr">
@@ -3167,12 +3171,12 @@
       </c>
       <c r="AG12" s="2" t="inlineStr">
         <is>
-          <t>["Institucional", "PJ Atacado"]</t>
+          <t>["Pessoa Física"]</t>
         </is>
       </c>
       <c r="AH12" s="2" t="inlineStr">
         <is>
-          <t>["Institucional", "PJ Atacado"]</t>
+          <t>["Pessoa Física"]</t>
         </is>
       </c>
       <c r="AI12" s="2" t="inlineStr">
@@ -3193,7 +3197,7 @@
       </c>
       <c r="AM12" s="2" t="inlineStr">
         <is>
-          <t>CAIXA PATRIMÔNIO ÍNDICE DE PREÇOS FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESP LIMITADA</t>
+          <t>CAIXA FOCO ÍNDICE DE PREÇOS FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESP LIMITADA</t>
         </is>
       </c>
       <c r="AN12" s="2" t="inlineStr">
@@ -3203,47 +3207,47 @@
       </c>
       <c r="AO12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_0046.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5414.pdf</t>
         </is>
       </c>
       <c r="AP12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_0046.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5414.pdf</t>
         </is>
       </c>
       <c r="AQ12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_0046.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5414.pdf</t>
         </is>
       </c>
       <c r="AR12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_46.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5414.pdf</t>
         </is>
       </c>
       <c r="AS12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_46.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5414.pdf</t>
         </is>
       </c>
       <c r="AT12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_46.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5414.pdf</t>
         </is>
       </c>
       <c r="AU12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_0046.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5414.pdf</t>
         </is>
       </c>
       <c r="AV12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/caixa-asset/sumario-remuneracao/Documents/sumarios/0046-SUMARIO.pdf</t>
+          <t>https://www.caixa.gov.br/caixa-asset/sumario-remuneracao/Documents/sumarios/5414-SUMARIO.pdf</t>
         </is>
       </c>
       <c r="AW12" s="2" t="inlineStr">
         <is>
-          <t>https://web.microsoftstream.com/video/140b7682-00df-491d-b451-73ae70a040fa?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
+          <t>https://web.microsoftstream.com/video/a5ab94de-1f04-4f00-87d2-ffa0c6babbaf?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
     </row>
@@ -3769,7 +3773,7 @@
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>78,480</t>
+          <t>78,270</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -4486,7 +4490,7 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>135,107</t>
+          <t>135,106</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -4729,7 +4733,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1.778,480</t>
+          <t>1.763,912</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -4960,7 +4964,7 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>2.192,110</t>
+          <t>2.192,107</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -5682,7 +5686,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>950,542</t>
+          <t>950,541</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -5896,32 +5900,32 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,11213849</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>-0,001</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>-0,20</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>3,10</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>205,303</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
@@ -6131,32 +6135,32 @@
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F25" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H25" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,24146100</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>-0,001</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>0,42</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>5,99</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>14,53</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>71,379</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -6387,7 +6391,7 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>175,519</t>
+          <t>175,488</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
@@ -6840,32 +6844,32 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,04048600</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>-0,001</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>0,42</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>6,11</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>21,972</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
@@ -7063,32 +7067,32 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H29" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,17181800</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>-0,001</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>0,56</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>5,52</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>13,98</t>
         </is>
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>66,553</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -7294,32 +7298,32 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,07566699</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>-0,001</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>0,60</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>4,09</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>305,785</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
@@ -7773,7 +7777,7 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>851,906</t>
+          <t>851,782</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
@@ -8012,7 +8016,7 @@
       </c>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>3.270,411</t>
+          <t>3.270,389</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -8478,7 +8482,7 @@
       </c>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>3.109,343</t>
+          <t>3.109,338</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -8713,7 +8717,7 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>123,284</t>
+          <t>123,161</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
@@ -8948,7 +8952,7 @@
       </c>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>586,365</t>
+          <t>586,364</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -9427,7 +9431,7 @@
       </c>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>391,367</t>
+          <t>391,366</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
@@ -9666,7 +9670,7 @@
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>2.369,327</t>
+          <t>2.369,324</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
@@ -9905,7 +9909,7 @@
       </c>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>545,808</t>
+          <t>545,807</t>
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr">
@@ -10145,7 +10149,7 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>15.579,370</t>
+          <t>15.579,204</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -10388,7 +10392,7 @@
       </c>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>1.391,015</t>
+          <t>1.391,014</t>
         </is>
       </c>
       <c r="J43" s="4" t="inlineStr">
@@ -10855,7 +10859,7 @@
       </c>
       <c r="I45" s="4" t="inlineStr">
         <is>
-          <t>163,978</t>
+          <t>163,975</t>
         </is>
       </c>
       <c r="J45" s="4" t="inlineStr">
@@ -11098,7 +11102,7 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>6.013,350</t>
+          <t>5.953,859</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
@@ -11335,7 +11339,7 @@
       </c>
       <c r="I47" s="4" t="inlineStr">
         <is>
-          <t>2.212,006</t>
+          <t>2.211,981</t>
         </is>
       </c>
       <c r="J47" s="4" t="inlineStr">
@@ -12061,7 +12065,7 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>15.996,953</t>
+          <t>15.996,852</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
@@ -12300,7 +12304,7 @@
       </c>
       <c r="I51" s="4" t="inlineStr">
         <is>
-          <t>9.484,560</t>
+          <t>9.484,514</t>
         </is>
       </c>
       <c r="J51" s="4" t="inlineStr">
@@ -12543,7 +12547,7 @@
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>21.165,250</t>
+          <t>21.165,088</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr">
@@ -12782,7 +12786,7 @@
       </c>
       <c r="I53" s="4" t="inlineStr">
         <is>
-          <t>13.583,436</t>
+          <t>13.583,393</t>
         </is>
       </c>
       <c r="J53" s="4" t="inlineStr">
@@ -13034,187 +13038,43 @@
           <t>https://www.caixa.gov.br/fundos-investimento/curto-prazo/fic-automatico-polis-rf-cp/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L54" s="2" t="inlineStr">
-        <is>
-          <t>39.594.941/0001-36</t>
-        </is>
-      </c>
-      <c r="M54" s="2" t="inlineStr">
-        <is>
-          <t>6520</t>
-        </is>
-      </c>
-      <c r="N54" s="2" t="inlineStr">
-        <is>
-          <t>Conservador</t>
-        </is>
-      </c>
-      <c r="O54" s="2" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
-      </c>
-      <c r="P54" s="2" t="inlineStr">
-        <is>
-          <t>10000.0</t>
-        </is>
-      </c>
-      <c r="Q54" s="2" t="inlineStr">
-        <is>
-          <t>100.0</t>
-        </is>
-      </c>
-      <c r="R54" s="2" t="inlineStr">
-        <is>
-          <t>100.0</t>
-        </is>
-      </c>
-      <c r="S54" s="2" t="inlineStr">
-        <is>
-          <t>1000.0</t>
-        </is>
-      </c>
-      <c r="T54" s="2" t="inlineStr">
-        <is>
-          <t>D+0 (du)</t>
-        </is>
-      </c>
-      <c r="U54" s="2" t="inlineStr">
-        <is>
-          <t>D+0 (du)</t>
-        </is>
-      </c>
-      <c r="V54" s="2" t="inlineStr">
-        <is>
-          <t>D+00 (du)</t>
-        </is>
-      </c>
-      <c r="W54" s="2" t="inlineStr">
-        <is>
-          <t>CDI</t>
-        </is>
-      </c>
-      <c r="X54" s="2" t="inlineStr">
-        <is>
-          <t>RF 100% TPF - Curto Prazo</t>
-        </is>
-      </c>
-      <c r="Y54" s="2" t="inlineStr">
-        <is>
-          <t>Aberto para captação</t>
-        </is>
-      </c>
-      <c r="Z54" s="2" t="inlineStr">
-        <is>
-          <t>CURTO PRAZO</t>
-        </is>
-      </c>
-      <c r="AA54" s="2" t="inlineStr">
-        <is>
-          <t>GERAL</t>
-        </is>
-      </c>
-      <c r="AB54" s="2" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="AC54" s="2" t="inlineStr">
-        <is>
-          <t>17h00</t>
-        </is>
-      </c>
-      <c r="AD54" s="2" t="inlineStr">
-        <is>
-          <t>Sim · Automatico · 100%</t>
-        </is>
-      </c>
-      <c r="AE54" s="2" t="inlineStr">
-        <is>
-          <t>AUTOMATICO</t>
-        </is>
-      </c>
-      <c r="AF54" s="2" t="inlineStr">
-        <is>
-          <t>100.0</t>
-        </is>
-      </c>
-      <c r="AG54" s="2" t="inlineStr">
-        <is>
-          <t>["Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private"]</t>
-        </is>
-      </c>
-      <c r="AH54" s="2" t="inlineStr">
-        <is>
-          <t>["Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private"]</t>
-        </is>
-      </c>
-      <c r="AI54" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="AJ54" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
+      <c r="L54" s="2" t="inlineStr"/>
+      <c r="M54" s="2" t="inlineStr"/>
+      <c r="N54" s="2" t="inlineStr"/>
+      <c r="O54" s="2" t="inlineStr"/>
+      <c r="P54" s="2" t="inlineStr"/>
+      <c r="Q54" s="2" t="inlineStr"/>
+      <c r="R54" s="2" t="inlineStr"/>
+      <c r="S54" s="2" t="inlineStr"/>
+      <c r="T54" s="2" t="inlineStr"/>
+      <c r="U54" s="2" t="inlineStr"/>
+      <c r="V54" s="2" t="inlineStr"/>
+      <c r="W54" s="2" t="inlineStr"/>
+      <c r="X54" s="2" t="inlineStr"/>
+      <c r="Y54" s="2" t="inlineStr"/>
+      <c r="Z54" s="2" t="inlineStr"/>
+      <c r="AA54" s="2" t="inlineStr"/>
+      <c r="AB54" s="2" t="inlineStr"/>
+      <c r="AC54" s="2" t="inlineStr"/>
+      <c r="AD54" s="2" t="inlineStr"/>
+      <c r="AE54" s="2" t="inlineStr"/>
+      <c r="AF54" s="2" t="inlineStr"/>
+      <c r="AG54" s="2" t="inlineStr"/>
+      <c r="AH54" s="2" t="inlineStr"/>
+      <c r="AI54" s="2" t="inlineStr"/>
+      <c r="AJ54" s="2" t="inlineStr"/>
       <c r="AK54" s="2" t="inlineStr"/>
-      <c r="AL54" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="AM54" s="2" t="inlineStr">
-        <is>
-          <t>CAIXA FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA CURTO PRAZO - RESPONSABILIDADE LIMITADA</t>
-        </is>
-      </c>
-      <c r="AN54" s="2" t="inlineStr">
-        <is>
-          <t>*Este Fundo não está adaptado às normas vigentes para RPPS (Regimes Próprios de Previdência Social).</t>
-        </is>
-      </c>
-      <c r="AO54" s="2" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_6520.pdf</t>
-        </is>
-      </c>
-      <c r="AP54" s="2" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_6520.pdf</t>
-        </is>
-      </c>
-      <c r="AQ54" s="2" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_6520.pdf</t>
-        </is>
-      </c>
-      <c r="AR54" s="2" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_6520.pdf</t>
-        </is>
-      </c>
-      <c r="AS54" s="2" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6520.pdf</t>
-        </is>
-      </c>
-      <c r="AT54" s="2" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6520.pdf</t>
-        </is>
-      </c>
-      <c r="AU54" s="2" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_6520.pdf</t>
-        </is>
-      </c>
-      <c r="AV54" s="2" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/caixa-asset/sumario-remuneracao/Documents/sumarios/6520-SUMARIO.pdf</t>
-        </is>
-      </c>
+      <c r="AL54" s="2" t="inlineStr"/>
+      <c r="AM54" s="2" t="inlineStr"/>
+      <c r="AN54" s="2" t="inlineStr"/>
+      <c r="AO54" s="2" t="inlineStr"/>
+      <c r="AP54" s="2" t="inlineStr"/>
+      <c r="AQ54" s="2" t="inlineStr"/>
+      <c r="AR54" s="2" t="inlineStr"/>
+      <c r="AS54" s="2" t="inlineStr"/>
+      <c r="AT54" s="2" t="inlineStr"/>
+      <c r="AU54" s="2" t="inlineStr"/>
+      <c r="AV54" s="2" t="inlineStr"/>
       <c r="AW54" s="2" t="inlineStr"/>
     </row>
     <row r="55">
@@ -13235,32 +13095,32 @@
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E55" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F55" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G55" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H55" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,41687500</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>0,049</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="inlineStr">
+        <is>
+          <t>0,44</t>
+        </is>
+      </c>
+      <c r="G55" s="5" t="inlineStr">
+        <is>
+          <t>5,82</t>
+        </is>
+      </c>
+      <c r="H55" s="5" t="inlineStr">
+        <is>
+          <t>14,26</t>
         </is>
       </c>
       <c r="I55" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>67,794</t>
         </is>
       </c>
       <c r="J55" s="4" t="inlineStr">
@@ -13466,32 +13326,32 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E56" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F56" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G56" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H56" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1.196,86800100</t>
+        </is>
+      </c>
+      <c r="E56" s="7" t="inlineStr">
+        <is>
+          <t>-0,002</t>
+        </is>
+      </c>
+      <c r="F56" s="7" t="inlineStr">
+        <is>
+          <t>-0,56</t>
+        </is>
+      </c>
+      <c r="G56" s="7" t="inlineStr">
+        <is>
+          <t>-4,61</t>
+        </is>
+      </c>
+      <c r="H56" s="3" t="inlineStr">
+        <is>
+          <t>0,02</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>36,489</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
@@ -13740,7 +13600,7 @@
       </c>
       <c r="I57" s="4" t="inlineStr">
         <is>
-          <t>323,482</t>
+          <t>540,035</t>
         </is>
       </c>
       <c r="J57" s="4" t="inlineStr">
@@ -13810,32 +13670,32 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E58" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F58" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G58" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H58" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1.628,04128700</t>
+        </is>
+      </c>
+      <c r="E58" s="7" t="inlineStr">
+        <is>
+          <t>-0,006</t>
+        </is>
+      </c>
+      <c r="F58" s="7" t="inlineStr">
+        <is>
+          <t>-0,55</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="inlineStr">
+        <is>
+          <t>3,89</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr">
+        <is>
+          <t>11,83</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>113,885</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
@@ -13850,12 +13710,12 @@
       </c>
       <c r="L58" s="2" t="inlineStr">
         <is>
-          <t>34.660.276/0001-18</t>
+          <t>34.660.333/0001-69</t>
         </is>
       </c>
       <c r="M58" s="2" t="inlineStr">
         <is>
-          <t>6439</t>
+          <t>6440</t>
         </is>
       </c>
       <c r="N58" s="2" t="inlineStr">
@@ -13940,23 +13800,27 @@
       </c>
       <c r="AD58" s="2" t="inlineStr">
         <is>
-          <t>Não se aplica</t>
+          <t>Sim · Automatico · 100%</t>
         </is>
       </c>
       <c r="AE58" s="2" t="inlineStr">
         <is>
-          <t>NÃO SE APLICA</t>
-        </is>
-      </c>
-      <c r="AF58" s="2" t="inlineStr"/>
+          <t>AUTOMATICO</t>
+        </is>
+      </c>
+      <c r="AF58" s="2" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
       <c r="AG58" s="2" t="inlineStr">
         <is>
-          <t>["GOV", "RPPS"]</t>
+          <t>["Pessoa Física", "Private"]</t>
         </is>
       </c>
       <c r="AH58" s="2" t="inlineStr">
         <is>
-          <t>["GOV", "RPPS"]</t>
+          <t>["Pessoa Física", "Private"]</t>
         </is>
       </c>
       <c r="AI58" s="2" t="inlineStr">
@@ -13977,48 +13841,48 @@
       </c>
       <c r="AM58" s="2" t="inlineStr">
         <is>
-          <t>CAIXA BRASIL ESTRATÉGIA LIVRE FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO MULTIMERCADO LONGO PRAZO - RESPONSABILIDADE</t>
+          <t>CAIXA ESTRATÉGIA LIVRE FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO MULTIMERCADO LONGO PRAZO - RESPONSABILIDADE LIMITA</t>
         </is>
       </c>
       <c r="AN58" s="2" t="inlineStr"/>
       <c r="AO58" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_6439.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_6440.pdf</t>
         </is>
       </c>
       <c r="AP58" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_6439.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_6440.pdf</t>
         </is>
       </c>
       <c r="AQ58" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_6439.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_6440.pdf</t>
         </is>
       </c>
       <c r="AR58" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_6439.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_6440.pdf</t>
         </is>
       </c>
       <c r="AS58" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6439.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6440.pdf</t>
         </is>
       </c>
       <c r="AT58" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6439.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6440.pdf</t>
         </is>
       </c>
       <c r="AU58" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_6439.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_6440.pdf</t>
         </is>
       </c>
       <c r="AV58" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/caixa-asset/sumario-remuneracao/Documents/sumarios/6439-SUMARIO.pdf</t>
+          <t>https://www.caixa.gov.br/caixa-asset/sumario-remuneracao/Documents/sumarios/6440-SUMARIO.pdf</t>
         </is>
       </c>
       <c r="AW58" s="2" t="inlineStr"/>
@@ -14503,32 +14367,32 @@
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E61" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F61" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G61" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H61" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,24946500</t>
+        </is>
+      </c>
+      <c r="E61" s="6" t="inlineStr">
+        <is>
+          <t>-0,005</t>
+        </is>
+      </c>
+      <c r="F61" s="6" t="inlineStr">
+        <is>
+          <t>-0,16</t>
+        </is>
+      </c>
+      <c r="G61" s="5" t="inlineStr">
+        <is>
+          <t>2,30</t>
+        </is>
+      </c>
+      <c r="H61" s="5" t="inlineStr">
+        <is>
+          <t>9,79</t>
         </is>
       </c>
       <c r="I61" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>6,293</t>
         </is>
       </c>
       <c r="J61" s="4" t="inlineStr">
@@ -15200,32 +15064,32 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E64" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F64" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G64" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H64" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,39551400</t>
+        </is>
+      </c>
+      <c r="E64" s="7" t="inlineStr">
+        <is>
+          <t>-0,004</t>
+        </is>
+      </c>
+      <c r="F64" s="7" t="inlineStr">
+        <is>
+          <t>-1,74</t>
+        </is>
+      </c>
+      <c r="G64" s="3" t="inlineStr">
+        <is>
+          <t>2,23</t>
+        </is>
+      </c>
+      <c r="H64" s="3" t="inlineStr">
+        <is>
+          <t>14,69</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11,570</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
@@ -15687,7 +15551,7 @@
       </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>3,729</t>
+          <t>3,705</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr">
@@ -15897,32 +15761,32 @@
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E67" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F67" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G67" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H67" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>5,31247165</t>
+        </is>
+      </c>
+      <c r="E67" s="6" t="inlineStr">
+        <is>
+          <t>-0,003</t>
+        </is>
+      </c>
+      <c r="F67" s="6" t="inlineStr">
+        <is>
+          <t>-0,45</t>
+        </is>
+      </c>
+      <c r="G67" s="5" t="inlineStr">
+        <is>
+          <t>3,53</t>
+        </is>
+      </c>
+      <c r="H67" s="5" t="inlineStr">
+        <is>
+          <t>11,68</t>
         </is>
       </c>
       <c r="I67" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>32,632</t>
         </is>
       </c>
       <c r="J67" s="4" t="inlineStr">
@@ -16161,7 +16025,7 @@
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>561,157</t>
+          <t>554,596</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr">
@@ -16375,32 +16239,32 @@
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E69" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F69" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G69" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H69" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>2,84200700</t>
+        </is>
+      </c>
+      <c r="E69" s="6" t="inlineStr">
+        <is>
+          <t>-0,013</t>
+        </is>
+      </c>
+      <c r="F69" s="6" t="inlineStr">
+        <is>
+          <t>-0,73</t>
+        </is>
+      </c>
+      <c r="G69" s="5" t="inlineStr">
+        <is>
+          <t>1,75</t>
+        </is>
+      </c>
+      <c r="H69" s="5" t="inlineStr">
+        <is>
+          <t>9,10</t>
         </is>
       </c>
       <c r="I69" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>73,553</t>
         </is>
       </c>
       <c r="J69" s="4" t="inlineStr">
@@ -16874,7 +16738,7 @@
       </c>
       <c r="I71" s="4" t="inlineStr">
         <is>
-          <t>2.342,414</t>
+          <t>2.341,499</t>
         </is>
       </c>
       <c r="J71" s="4" t="inlineStr">
@@ -17113,7 +16977,7 @@
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>21,645</t>
+          <t>21,644</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr">
@@ -17327,32 +17191,32 @@
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E73" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F73" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G73" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H73" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1.649,79185500</t>
+        </is>
+      </c>
+      <c r="E73" s="6" t="inlineStr">
+        <is>
+          <t>-0,003</t>
+        </is>
+      </c>
+      <c r="F73" s="6" t="inlineStr">
+        <is>
+          <t>-0,51</t>
+        </is>
+      </c>
+      <c r="G73" s="5" t="inlineStr">
+        <is>
+          <t>4,31</t>
+        </is>
+      </c>
+      <c r="H73" s="5" t="inlineStr">
+        <is>
+          <t>12,80</t>
         </is>
       </c>
       <c r="I73" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14,434</t>
         </is>
       </c>
       <c r="J73" s="4" t="inlineStr">
@@ -17554,32 +17418,32 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E74" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F74" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G74" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>0,45956255</t>
+        </is>
+      </c>
+      <c r="E74" s="7" t="inlineStr">
+        <is>
+          <t>-0,005</t>
+        </is>
+      </c>
+      <c r="F74" s="7" t="inlineStr">
+        <is>
+          <t>-12,77</t>
+        </is>
+      </c>
+      <c r="G74" s="7" t="inlineStr">
+        <is>
+          <t>-36,35</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3,631</t>
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr">
@@ -17796,32 +17660,32 @@
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E75" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F75" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G75" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H75" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>3,25662600</t>
+        </is>
+      </c>
+      <c r="E75" s="6" t="inlineStr">
+        <is>
+          <t>-0,005</t>
+        </is>
+      </c>
+      <c r="F75" s="6" t="inlineStr">
+        <is>
+          <t>-0,70</t>
+        </is>
+      </c>
+      <c r="G75" s="5" t="inlineStr">
+        <is>
+          <t>2,21</t>
+        </is>
+      </c>
+      <c r="H75" s="5" t="inlineStr">
+        <is>
+          <t>8,55</t>
         </is>
       </c>
       <c r="I75" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>155,108</t>
         </is>
       </c>
       <c r="J75" s="4" t="inlineStr">
@@ -17836,145 +17700,882 @@
       </c>
       <c r="L75" s="4" t="inlineStr">
         <is>
+          <t>14.239.659/0001-00</t>
+        </is>
+      </c>
+      <c r="M75" s="4" t="inlineStr">
+        <is>
+          <t>5475</t>
+        </is>
+      </c>
+      <c r="N75" s="4" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="O75" s="4" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+      <c r="P75" s="4" t="inlineStr">
+        <is>
+          <t>5000.0</t>
+        </is>
+      </c>
+      <c r="Q75" s="4" t="inlineStr">
+        <is>
+          <t>500.0</t>
+        </is>
+      </c>
+      <c r="R75" s="4" t="inlineStr">
+        <is>
+          <t>500.0</t>
+        </is>
+      </c>
+      <c r="S75" s="4" t="inlineStr">
+        <is>
+          <t>4000.0</t>
+        </is>
+      </c>
+      <c r="T75" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="U75" s="4" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="V75" s="4" t="inlineStr">
+        <is>
+          <t>D+03 (du)</t>
+        </is>
+      </c>
+      <c r="W75" s="4" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="X75" s="4" t="inlineStr">
+        <is>
+          <t>Capital Protegido</t>
+        </is>
+      </c>
+      <c r="Y75" s="4" t="inlineStr">
+        <is>
+          <t>Fechado para captação</t>
+        </is>
+      </c>
+      <c r="Z75" s="4" t="inlineStr">
+        <is>
+          <t>LONGO PRAZO</t>
+        </is>
+      </c>
+      <c r="AA75" s="4" t="inlineStr">
+        <is>
+          <t>GERAL</t>
+        </is>
+      </c>
+      <c r="AB75" s="4" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="AC75" s="4" t="inlineStr">
+        <is>
+          <t>17h00</t>
+        </is>
+      </c>
+      <c r="AD75" s="4" t="inlineStr">
+        <is>
+          <t>Sim · Automatico · 100%</t>
+        </is>
+      </c>
+      <c r="AE75" s="4" t="inlineStr">
+        <is>
+          <t>AUTOMATICO</t>
+        </is>
+      </c>
+      <c r="AF75" s="4" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
+      <c r="AG75" s="4" t="inlineStr">
+        <is>
+          <t>["GOV"]</t>
+        </is>
+      </c>
+      <c r="AH75" s="4" t="inlineStr">
+        <is>
+          <t>["GOV"]</t>
+        </is>
+      </c>
+      <c r="AI75" s="4" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AJ75" s="4" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="AK75" s="4" t="inlineStr">
+        <is>
+          <t>2027-10-01T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="AL75" s="4" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AM75" s="4" t="inlineStr">
+        <is>
+          <t>CAIXA CAPITAL PROTEGIDO IBOVESPA CÍCLICO I FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO MULTIMERCADO - RESPOSANBILIDAD</t>
+        </is>
+      </c>
+      <c r="AN75" s="4" t="inlineStr">
+        <is>
+          <t>Fundo com prazo de carência para aplicação e resgate, conforme Regulamento. Durante a carência, não é permitida a realização de aplicações ou resgates.
+Nova operação estruturada com inicio em 02/SET/2025 e termino em 01/OUT/2027. 
+Fundo Fechado a para aplicações a partir de 02/09/2025 (inclusive)</t>
+        </is>
+      </c>
+      <c r="AO75" s="4" t="inlineStr">
+        <is>
+          <t>http://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5475.pdf</t>
+        </is>
+      </c>
+      <c r="AP75" s="4" t="inlineStr">
+        <is>
+          <t>http://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5475.pdf</t>
+        </is>
+      </c>
+      <c r="AQ75" s="4" t="inlineStr">
+        <is>
+          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5475.pdf</t>
+        </is>
+      </c>
+      <c r="AR75" s="4" t="inlineStr">
+        <is>
+          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_5475.pdf</t>
+        </is>
+      </c>
+      <c r="AS75" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5475.pdf</t>
+        </is>
+      </c>
+      <c r="AT75" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5475.pdf</t>
+        </is>
+      </c>
+      <c r="AU75" s="4" t="inlineStr">
+        <is>
+          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5475.pdf</t>
+        </is>
+      </c>
+      <c r="AV75" s="4" t="inlineStr">
+        <is>
+          <t>http://www.caixa.gov.br/caixa-asset/sumario-remuneracao/Documents/sumarios/5475-SUMARIO.pdf</t>
+        </is>
+      </c>
+      <c r="AW75" s="4" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>MULTIMERCADO</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>CAIXA CAPITAL PROTEGIDO CÍCLICO III FIC FIF MM LP - RESP LTDA</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>10/01/2022</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>1,53082000</t>
+        </is>
+      </c>
+      <c r="E76" s="7" t="inlineStr">
+        <is>
+          <t>-0,004</t>
+        </is>
+      </c>
+      <c r="F76" s="7" t="inlineStr">
+        <is>
+          <t>-1,18</t>
+        </is>
+      </c>
+      <c r="G76" s="3" t="inlineStr">
+        <is>
+          <t>2,52</t>
+        </is>
+      </c>
+      <c r="H76" s="3" t="inlineStr">
+        <is>
+          <t>18,97</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="inlineStr">
+        <is>
+          <t>14,421</t>
+        </is>
+      </c>
+      <c r="J76" s="2" t="inlineStr">
+        <is>
+          <t>PF | PJ | RPPS</t>
+        </is>
+      </c>
+      <c r="K76" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-capital-protegido-ciclico-iii-multimercado-lp/Paginas/default.aspx</t>
+        </is>
+      </c>
+      <c r="L76" s="2" t="inlineStr">
+        <is>
+          <t>44.683.343/0001-73</t>
+        </is>
+      </c>
+      <c r="M76" s="2" t="inlineStr">
+        <is>
+          <t>6608</t>
+        </is>
+      </c>
+      <c r="N76" s="2" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="O76" s="2" t="inlineStr">
+        <is>
+          <t>0.9</t>
+        </is>
+      </c>
+      <c r="P76" s="2" t="inlineStr">
+        <is>
+          <t>5000.0</t>
+        </is>
+      </c>
+      <c r="Q76" s="2" t="inlineStr">
+        <is>
+          <t>500.0</t>
+        </is>
+      </c>
+      <c r="R76" s="2" t="inlineStr">
+        <is>
+          <t>500.0</t>
+        </is>
+      </c>
+      <c r="S76" s="2" t="inlineStr">
+        <is>
+          <t>4000.0</t>
+        </is>
+      </c>
+      <c r="T76" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="U76" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="V76" s="2" t="inlineStr">
+        <is>
+          <t>D+02 (du)</t>
+        </is>
+      </c>
+      <c r="W76" s="2" t="inlineStr">
+        <is>
+          <t>NÃO SE APLICA</t>
+        </is>
+      </c>
+      <c r="X76" s="2" t="inlineStr">
+        <is>
+          <t>Capital Protegido</t>
+        </is>
+      </c>
+      <c r="Y76" s="2" t="inlineStr">
+        <is>
+          <t>Fechado para captação</t>
+        </is>
+      </c>
+      <c r="Z76" s="2" t="inlineStr">
+        <is>
+          <t>LONGO PRAZO</t>
+        </is>
+      </c>
+      <c r="AA76" s="2" t="inlineStr">
+        <is>
+          <t>GERAL</t>
+        </is>
+      </c>
+      <c r="AB76" s="2" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="AC76" s="2" t="inlineStr">
+        <is>
+          <t>16h00</t>
+        </is>
+      </c>
+      <c r="AD76" s="2" t="inlineStr">
+        <is>
+          <t>Sim · Automatico · 100%</t>
+        </is>
+      </c>
+      <c r="AE76" s="2" t="inlineStr">
+        <is>
+          <t>AUTOMATICO</t>
+        </is>
+      </c>
+      <c r="AF76" s="2" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
+      <c r="AG76" s="2" t="inlineStr">
+        <is>
+          <t>["GOV", "Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private", "RPPS"]</t>
+        </is>
+      </c>
+      <c r="AH76" s="2" t="inlineStr">
+        <is>
+          <t>["GOV", "Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private", "RPPS"]</t>
+        </is>
+      </c>
+      <c r="AI76" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AJ76" s="2" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="AK76" s="2" t="inlineStr">
+        <is>
+          <t>2028-07-07T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="AL76" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AM76" s="2" t="inlineStr">
+        <is>
+          <t>CAIXA CAPITAL PROTEGIDO CÍCLICO III FIC DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO MULTIMERCADO LONGO PRAZO - RESP LIMITADA</t>
+        </is>
+      </c>
+      <c r="AN76" s="2" t="inlineStr">
+        <is>
+          <t>Fundo com prazo de carência para aplicação e resgate, conforme Regulamento. Durante a carência, não é permitida a realização de aplicações ou resgates.                                                                  Período de Captação 02/03/2026 à 24/04/2026
+Início da Operação Estruturada: 27/04/2026
+Fim da Operação Estruturada: 03/07/2028</t>
+        </is>
+      </c>
+      <c r="AO76" s="2" t="inlineStr">
+        <is>
+          <t>http://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_6608.pdf</t>
+        </is>
+      </c>
+      <c r="AP76" s="2" t="inlineStr">
+        <is>
+          <t>http://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_6608.pdf</t>
+        </is>
+      </c>
+      <c r="AQ76" s="2" t="inlineStr">
+        <is>
+          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_6608.pdf</t>
+        </is>
+      </c>
+      <c r="AR76" s="2" t="inlineStr">
+        <is>
+          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_6608.pdf</t>
+        </is>
+      </c>
+      <c r="AS76" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6608.pdf</t>
+        </is>
+      </c>
+      <c r="AT76" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6608.pdf</t>
+        </is>
+      </c>
+      <c r="AU76" s="2" t="inlineStr">
+        <is>
+          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_6608.pdf</t>
+        </is>
+      </c>
+      <c r="AV76" s="2" t="inlineStr">
+        <is>
+          <t>http://www.caixa.gov.br/caixa-asset/sumario-remuneracao/Documents/sumarios/6608-SUMARIO.pdf</t>
+        </is>
+      </c>
+      <c r="AW76" s="2" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="inlineStr">
+        <is>
+          <t>MULTIMERCADO</t>
+        </is>
+      </c>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>CAIXA FIC FIF CAPITAL PROTEGIDO CESTA AGRO MM</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t>04/07/2022</t>
+        </is>
+      </c>
+      <c r="D77" s="4" t="inlineStr">
+        <is>
+          <t>1,38037000</t>
+        </is>
+      </c>
+      <c r="E77" s="6" t="inlineStr">
+        <is>
+          <t>-0,003</t>
+        </is>
+      </c>
+      <c r="F77" s="5" t="inlineStr">
+        <is>
+          <t>0,47</t>
+        </is>
+      </c>
+      <c r="G77" s="5" t="inlineStr">
+        <is>
+          <t>1,78</t>
+        </is>
+      </c>
+      <c r="H77" s="5" t="inlineStr">
+        <is>
+          <t>6,77</t>
+        </is>
+      </c>
+      <c r="I77" s="4" t="inlineStr">
+        <is>
+          <t>70,737</t>
+        </is>
+      </c>
+      <c r="J77" s="4" t="inlineStr">
+        <is>
+          <t>GOV | PF | PJ | RPPS</t>
+        </is>
+      </c>
+      <c r="K77" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/caixa_fic_fim_cap_protegido_cesta_agro/Paginas/default.aspx</t>
+        </is>
+      </c>
+      <c r="L77" s="4" t="inlineStr">
+        <is>
+          <t>42.229.068/0001-97</t>
+        </is>
+      </c>
+      <c r="M77" s="4" t="inlineStr">
+        <is>
+          <t>6621</t>
+        </is>
+      </c>
+      <c r="N77" s="4" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="O77" s="4" t="inlineStr">
+        <is>
+          <t>0.9</t>
+        </is>
+      </c>
+      <c r="P77" s="4" t="inlineStr">
+        <is>
+          <t>5000.0</t>
+        </is>
+      </c>
+      <c r="Q77" s="4" t="inlineStr">
+        <is>
+          <t>500.0</t>
+        </is>
+      </c>
+      <c r="R77" s="4" t="inlineStr">
+        <is>
+          <t>500.0</t>
+        </is>
+      </c>
+      <c r="S77" s="4" t="inlineStr">
+        <is>
+          <t>4000.0</t>
+        </is>
+      </c>
+      <c r="T77" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="U77" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="V77" s="4" t="inlineStr">
+        <is>
+          <t>D+02 (du)</t>
+        </is>
+      </c>
+      <c r="W77" s="4" t="inlineStr">
+        <is>
+          <t>OUTROS</t>
+        </is>
+      </c>
+      <c r="X77" s="4" t="inlineStr">
+        <is>
+          <t>Capital Protegido</t>
+        </is>
+      </c>
+      <c r="Y77" s="4" t="inlineStr">
+        <is>
+          <t>Fechado para captação</t>
+        </is>
+      </c>
+      <c r="Z77" s="4" t="inlineStr">
+        <is>
+          <t>LONGO PRAZO</t>
+        </is>
+      </c>
+      <c r="AA77" s="4" t="inlineStr">
+        <is>
+          <t>GERAL</t>
+        </is>
+      </c>
+      <c r="AB77" s="4" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="AC77" s="4" t="inlineStr">
+        <is>
+          <t>16h00</t>
+        </is>
+      </c>
+      <c r="AD77" s="4" t="inlineStr">
+        <is>
+          <t>Sim · Automatico · 100%</t>
+        </is>
+      </c>
+      <c r="AE77" s="4" t="inlineStr">
+        <is>
+          <t>AUTOMATICO</t>
+        </is>
+      </c>
+      <c r="AF77" s="4" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
+      <c r="AG77" s="4" t="inlineStr">
+        <is>
+          <t>["GOV", "Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private", "RPPS"]</t>
+        </is>
+      </c>
+      <c r="AH77" s="4" t="inlineStr">
+        <is>
+          <t>["GOV", "Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private", "RPPS"]</t>
+        </is>
+      </c>
+      <c r="AI77" s="4" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AJ77" s="4" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="AK77" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-01T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="AL77" s="4" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AM77" s="4" t="inlineStr">
+        <is>
+          <t>CAIXA CAPITAL PROTEGIDO CESTA AGRO FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO MULTIMERCADO LONGO PRAZO - RESPONSABIL</t>
+        </is>
+      </c>
+      <c r="AN77" s="4" t="inlineStr">
+        <is>
+          <t>Fundo com prazo de carência para aplicação e resgate, conforme Regulamento. Durante a carência, não é permitida a realização de aplicações ou resgates.
+Nova Operação Estruturada:
+Dia 07/10/2024 -&gt; Reabertura para Resgates e Aplicações do fundo;
+Dia 25/10/2024 -&gt; Fechamento para Aplicações e Resgates
+Dia 29/10/2024 -&gt; Início da nova operação estruturada de Cesta Agro.</t>
+        </is>
+      </c>
+      <c r="AO77" s="4" t="inlineStr">
+        <is>
+          <t>http://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_6621.pdf</t>
+        </is>
+      </c>
+      <c r="AP77" s="4" t="inlineStr">
+        <is>
+          <t>http://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_6621.pdf</t>
+        </is>
+      </c>
+      <c r="AQ77" s="4" t="inlineStr">
+        <is>
+          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_6621.pdf</t>
+        </is>
+      </c>
+      <c r="AR77" s="4" t="inlineStr">
+        <is>
+          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_6621.pdf</t>
+        </is>
+      </c>
+      <c r="AS77" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6621.pdf</t>
+        </is>
+      </c>
+      <c r="AT77" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6621.pdf</t>
+        </is>
+      </c>
+      <c r="AU77" s="4" t="inlineStr">
+        <is>
+          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_6621.pdf</t>
+        </is>
+      </c>
+      <c r="AV77" s="4" t="inlineStr">
+        <is>
+          <t>http://www.caixa.gov.br/caixa-asset/sumario-remuneracao/Documents/sumarios/6621-SUMARIO.pdf</t>
+        </is>
+      </c>
+      <c r="AW77" s="4" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>MULTIMERCADO</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>CAIXA FIC FIM CAPITAL PROTEGIDO CICLICO II LP - RL</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>18/07/2022</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>1,47074800</t>
+        </is>
+      </c>
+      <c r="E78" s="7" t="inlineStr">
+        <is>
+          <t>-0,003</t>
+        </is>
+      </c>
+      <c r="F78" s="7" t="inlineStr">
+        <is>
+          <t>-2,08</t>
+        </is>
+      </c>
+      <c r="G78" s="3" t="inlineStr">
+        <is>
+          <t>1,70</t>
+        </is>
+      </c>
+      <c r="H78" s="3" t="inlineStr">
+        <is>
+          <t>13,23</t>
+        </is>
+      </c>
+      <c r="I78" s="2" t="inlineStr">
+        <is>
+          <t>190,698</t>
+        </is>
+      </c>
+      <c r="J78" s="2" t="inlineStr">
+        <is>
+          <t>GOV | PF | PJ | RPPS</t>
+        </is>
+      </c>
+      <c r="K78" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/caixa-fic-fim-cap-protegido-ciclico-ii</t>
+        </is>
+      </c>
+      <c r="L78" s="2" t="inlineStr">
+        <is>
           <t>45.443.651/0001-94</t>
         </is>
       </c>
-      <c r="M75" s="4" t="inlineStr">
+      <c r="M78" s="2" t="inlineStr">
         <is>
           <t>6623</t>
         </is>
       </c>
-      <c r="N75" s="4" t="inlineStr">
+      <c r="N78" s="2" t="inlineStr">
         <is>
           <t>Conservador</t>
         </is>
       </c>
-      <c r="O75" s="4" t="inlineStr">
+      <c r="O78" s="2" t="inlineStr">
         <is>
           <t>0.9</t>
         </is>
       </c>
-      <c r="P75" s="4" t="inlineStr">
+      <c r="P78" s="2" t="inlineStr">
         <is>
           <t>5000.0</t>
         </is>
       </c>
-      <c r="Q75" s="4" t="inlineStr">
+      <c r="Q78" s="2" t="inlineStr">
         <is>
           <t>500.0</t>
         </is>
       </c>
-      <c r="R75" s="4" t="inlineStr">
+      <c r="R78" s="2" t="inlineStr">
         <is>
           <t>500.0</t>
         </is>
       </c>
-      <c r="S75" s="4" t="inlineStr">
+      <c r="S78" s="2" t="inlineStr">
         <is>
           <t>4000.0</t>
         </is>
       </c>
-      <c r="T75" s="4" t="inlineStr">
+      <c r="T78" s="2" t="inlineStr">
         <is>
           <t>D+0 (du)</t>
         </is>
       </c>
-      <c r="U75" s="4" t="inlineStr">
+      <c r="U78" s="2" t="inlineStr">
         <is>
           <t>D+0 (du)</t>
         </is>
       </c>
-      <c r="V75" s="4" t="inlineStr">
+      <c r="V78" s="2" t="inlineStr">
         <is>
           <t>D+02 (du)</t>
         </is>
       </c>
-      <c r="W75" s="4" t="inlineStr">
+      <c r="W78" s="2" t="inlineStr">
         <is>
           <t>NÃO SE APLICA</t>
         </is>
       </c>
-      <c r="X75" s="4" t="inlineStr">
+      <c r="X78" s="2" t="inlineStr">
         <is>
           <t>Capital Protegido</t>
         </is>
       </c>
-      <c r="Y75" s="4" t="inlineStr">
+      <c r="Y78" s="2" t="inlineStr">
         <is>
           <t>Fechado para captação</t>
         </is>
       </c>
-      <c r="Z75" s="4" t="inlineStr">
+      <c r="Z78" s="2" t="inlineStr">
         <is>
           <t>LONGO PRAZO</t>
         </is>
       </c>
-      <c r="AA75" s="4" t="inlineStr">
+      <c r="AA78" s="2" t="inlineStr">
         <is>
           <t>GERAL</t>
         </is>
       </c>
-      <c r="AB75" s="4" t="inlineStr">
+      <c r="AB78" s="2" t="inlineStr">
         <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="AC75" s="4" t="inlineStr">
+      <c r="AC78" s="2" t="inlineStr">
         <is>
           <t>16h00</t>
         </is>
       </c>
-      <c r="AD75" s="4" t="inlineStr">
+      <c r="AD78" s="2" t="inlineStr">
         <is>
           <t>Sim · Automatico · 100%</t>
         </is>
       </c>
-      <c r="AE75" s="4" t="inlineStr">
+      <c r="AE78" s="2" t="inlineStr">
         <is>
           <t>AUTOMATICO</t>
         </is>
       </c>
-      <c r="AF75" s="4" t="inlineStr">
+      <c r="AF78" s="2" t="inlineStr">
         <is>
           <t>100.0</t>
         </is>
       </c>
-      <c r="AG75" s="4" t="inlineStr">
+      <c r="AG78" s="2" t="inlineStr">
         <is>
           <t>["GOV", "Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private", "RPPS"]</t>
         </is>
       </c>
-      <c r="AH75" s="4" t="inlineStr">
+      <c r="AH78" s="2" t="inlineStr">
         <is>
           <t>["GOV", "Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private", "RPPS"]</t>
         </is>
       </c>
-      <c r="AI75" s="4" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="AJ75" s="4" t="inlineStr">
+      <c r="AI78" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AJ78" s="2" t="inlineStr">
         <is>
           <t>Sim</t>
         </is>
       </c>
-      <c r="AK75" s="4" t="inlineStr">
+      <c r="AK78" s="2" t="inlineStr">
         <is>
           <t>2026-07-01T00:00:00Z</t>
         </is>
       </c>
-      <c r="AL75" s="4" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="AM75" s="4" t="inlineStr">
+      <c r="AL78" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AM78" s="2" t="inlineStr">
         <is>
           <t>CAIXA CAPITAL PROTEGIDO CICLICO II FIC DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO MULTIMERCADO LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
         </is>
       </c>
-      <c r="AN75" s="4" t="inlineStr">
+      <c r="AN78" s="2" t="inlineStr">
         <is>
           <t>Fundo com prazo de carência para aplicação e resgate, conforme Regulamento. Durante a carência, não é permitida a realização de aplicações ou resgates.
 Fechado para Aplicações e Resgates a partir de 26/08/2024 
@@ -17983,745 +18584,6 @@
 Fim da Operação Estruturada - 01/07/2026</t>
         </is>
       </c>
-      <c r="AO75" s="4" t="inlineStr">
-        <is>
-          <t>http://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_6623.pdf</t>
-        </is>
-      </c>
-      <c r="AP75" s="4" t="inlineStr">
-        <is>
-          <t>http://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_6623.pdf</t>
-        </is>
-      </c>
-      <c r="AQ75" s="4" t="inlineStr">
-        <is>
-          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_6623.pdf</t>
-        </is>
-      </c>
-      <c r="AR75" s="4" t="inlineStr">
-        <is>
-          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_6623.pdf</t>
-        </is>
-      </c>
-      <c r="AS75" s="4" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6623.pdf</t>
-        </is>
-      </c>
-      <c r="AT75" s="4" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6623.pdf</t>
-        </is>
-      </c>
-      <c r="AU75" s="4" t="inlineStr">
-        <is>
-          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_6623.pdf</t>
-        </is>
-      </c>
-      <c r="AV75" s="4" t="inlineStr">
-        <is>
-          <t>http://www.caixa.gov.br/caixa-asset/sumario-remuneracao/Documents/sumarios/6623-SUMARIO.pdf</t>
-        </is>
-      </c>
-      <c r="AW75" s="4" t="inlineStr"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="2" t="inlineStr">
-        <is>
-          <t>MULTIMERCADO</t>
-        </is>
-      </c>
-      <c r="B76" s="2" t="inlineStr">
-        <is>
-          <t>CAIXA CAPITAL PROTEGIDO CÍCLICO III FIC FIF MM LP - RESP LTDA</t>
-        </is>
-      </c>
-      <c r="C76" s="2" t="inlineStr">
-        <is>
-          <t>10/01/2022</t>
-        </is>
-      </c>
-      <c r="D76" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E76" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F76" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G76" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H76" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I76" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J76" s="2" t="inlineStr">
-        <is>
-          <t>PF | PJ | RPPS</t>
-        </is>
-      </c>
-      <c r="K76" s="2" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-capital-protegido-ciclico-iii-multimercado-lp/Paginas/default.aspx</t>
-        </is>
-      </c>
-      <c r="L76" s="2" t="inlineStr">
-        <is>
-          <t>44.683.343/0001-73</t>
-        </is>
-      </c>
-      <c r="M76" s="2" t="inlineStr">
-        <is>
-          <t>6608</t>
-        </is>
-      </c>
-      <c r="N76" s="2" t="inlineStr">
-        <is>
-          <t>Conservador</t>
-        </is>
-      </c>
-      <c r="O76" s="2" t="inlineStr">
-        <is>
-          <t>0.9</t>
-        </is>
-      </c>
-      <c r="P76" s="2" t="inlineStr">
-        <is>
-          <t>5000.0</t>
-        </is>
-      </c>
-      <c r="Q76" s="2" t="inlineStr">
-        <is>
-          <t>500.0</t>
-        </is>
-      </c>
-      <c r="R76" s="2" t="inlineStr">
-        <is>
-          <t>500.0</t>
-        </is>
-      </c>
-      <c r="S76" s="2" t="inlineStr">
-        <is>
-          <t>4000.0</t>
-        </is>
-      </c>
-      <c r="T76" s="2" t="inlineStr">
-        <is>
-          <t>D+0 (du)</t>
-        </is>
-      </c>
-      <c r="U76" s="2" t="inlineStr">
-        <is>
-          <t>D+0 (du)</t>
-        </is>
-      </c>
-      <c r="V76" s="2" t="inlineStr">
-        <is>
-          <t>D+02 (du)</t>
-        </is>
-      </c>
-      <c r="W76" s="2" t="inlineStr">
-        <is>
-          <t>NÃO SE APLICA</t>
-        </is>
-      </c>
-      <c r="X76" s="2" t="inlineStr">
-        <is>
-          <t>Capital Protegido</t>
-        </is>
-      </c>
-      <c r="Y76" s="2" t="inlineStr">
-        <is>
-          <t>Fechado para captação</t>
-        </is>
-      </c>
-      <c r="Z76" s="2" t="inlineStr">
-        <is>
-          <t>LONGO PRAZO</t>
-        </is>
-      </c>
-      <c r="AA76" s="2" t="inlineStr">
-        <is>
-          <t>GERAL</t>
-        </is>
-      </c>
-      <c r="AB76" s="2" t="inlineStr">
-        <is>
-          <t>16:00</t>
-        </is>
-      </c>
-      <c r="AC76" s="2" t="inlineStr">
-        <is>
-          <t>16h00</t>
-        </is>
-      </c>
-      <c r="AD76" s="2" t="inlineStr">
-        <is>
-          <t>Sim · Automatico · 100%</t>
-        </is>
-      </c>
-      <c r="AE76" s="2" t="inlineStr">
-        <is>
-          <t>AUTOMATICO</t>
-        </is>
-      </c>
-      <c r="AF76" s="2" t="inlineStr">
-        <is>
-          <t>100.0</t>
-        </is>
-      </c>
-      <c r="AG76" s="2" t="inlineStr">
-        <is>
-          <t>["GOV", "Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private", "RPPS"]</t>
-        </is>
-      </c>
-      <c r="AH76" s="2" t="inlineStr">
-        <is>
-          <t>["GOV", "Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private", "RPPS"]</t>
-        </is>
-      </c>
-      <c r="AI76" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="AJ76" s="2" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AK76" s="2" t="inlineStr">
-        <is>
-          <t>2028-07-07T00:00:00Z</t>
-        </is>
-      </c>
-      <c r="AL76" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="AM76" s="2" t="inlineStr">
-        <is>
-          <t>CAIXA CAPITAL PROTEGIDO CÍCLICO III FIC DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO MULTIMERCADO LONGO PRAZO - RESP LIMITADA</t>
-        </is>
-      </c>
-      <c r="AN76" s="2" t="inlineStr">
-        <is>
-          <t>Fundo com prazo de carência para aplicação e resgate, conforme Regulamento. Durante a carência, não é permitida a realização de aplicações ou resgates.                                                                  Período de Captação 02/03/2026 à 24/04/2026
-Início da Operação Estruturada: 27/04/2026
-Fim da Operação Estruturada: 03/07/2028</t>
-        </is>
-      </c>
-      <c r="AO76" s="2" t="inlineStr">
-        <is>
-          <t>http://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_6608.pdf</t>
-        </is>
-      </c>
-      <c r="AP76" s="2" t="inlineStr">
-        <is>
-          <t>http://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_6608.pdf</t>
-        </is>
-      </c>
-      <c r="AQ76" s="2" t="inlineStr">
-        <is>
-          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_6608.pdf</t>
-        </is>
-      </c>
-      <c r="AR76" s="2" t="inlineStr">
-        <is>
-          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_6608.pdf</t>
-        </is>
-      </c>
-      <c r="AS76" s="2" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6608.pdf</t>
-        </is>
-      </c>
-      <c r="AT76" s="2" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6608.pdf</t>
-        </is>
-      </c>
-      <c r="AU76" s="2" t="inlineStr">
-        <is>
-          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_6608.pdf</t>
-        </is>
-      </c>
-      <c r="AV76" s="2" t="inlineStr">
-        <is>
-          <t>http://www.caixa.gov.br/caixa-asset/sumario-remuneracao/Documents/sumarios/6608-SUMARIO.pdf</t>
-        </is>
-      </c>
-      <c r="AW76" s="2" t="inlineStr"/>
-    </row>
-    <row r="77">
-      <c r="A77" s="4" t="inlineStr">
-        <is>
-          <t>MULTIMERCADO</t>
-        </is>
-      </c>
-      <c r="B77" s="4" t="inlineStr">
-        <is>
-          <t>CAIXA FIC FIF CAPITAL PROTEGIDO CESTA AGRO MM</t>
-        </is>
-      </c>
-      <c r="C77" s="4" t="inlineStr">
-        <is>
-          <t>04/07/2022</t>
-        </is>
-      </c>
-      <c r="D77" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E77" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F77" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G77" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H77" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I77" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J77" s="4" t="inlineStr">
-        <is>
-          <t>GOV | PF | PJ | RPPS</t>
-        </is>
-      </c>
-      <c r="K77" s="4" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/caixa_fic_fim_cap_protegido_cesta_agro/Paginas/default.aspx</t>
-        </is>
-      </c>
-      <c r="L77" s="4" t="inlineStr">
-        <is>
-          <t>42.229.068/0001-97</t>
-        </is>
-      </c>
-      <c r="M77" s="4" t="inlineStr">
-        <is>
-          <t>6621</t>
-        </is>
-      </c>
-      <c r="N77" s="4" t="inlineStr">
-        <is>
-          <t>Conservador</t>
-        </is>
-      </c>
-      <c r="O77" s="4" t="inlineStr">
-        <is>
-          <t>0.9</t>
-        </is>
-      </c>
-      <c r="P77" s="4" t="inlineStr">
-        <is>
-          <t>5000.0</t>
-        </is>
-      </c>
-      <c r="Q77" s="4" t="inlineStr">
-        <is>
-          <t>500.0</t>
-        </is>
-      </c>
-      <c r="R77" s="4" t="inlineStr">
-        <is>
-          <t>500.0</t>
-        </is>
-      </c>
-      <c r="S77" s="4" t="inlineStr">
-        <is>
-          <t>4000.0</t>
-        </is>
-      </c>
-      <c r="T77" s="4" t="inlineStr">
-        <is>
-          <t>D+0 (du)</t>
-        </is>
-      </c>
-      <c r="U77" s="4" t="inlineStr">
-        <is>
-          <t>D+0 (du)</t>
-        </is>
-      </c>
-      <c r="V77" s="4" t="inlineStr">
-        <is>
-          <t>D+02 (du)</t>
-        </is>
-      </c>
-      <c r="W77" s="4" t="inlineStr">
-        <is>
-          <t>OUTROS</t>
-        </is>
-      </c>
-      <c r="X77" s="4" t="inlineStr">
-        <is>
-          <t>Capital Protegido</t>
-        </is>
-      </c>
-      <c r="Y77" s="4" t="inlineStr">
-        <is>
-          <t>Fechado para captação</t>
-        </is>
-      </c>
-      <c r="Z77" s="4" t="inlineStr">
-        <is>
-          <t>LONGO PRAZO</t>
-        </is>
-      </c>
-      <c r="AA77" s="4" t="inlineStr">
-        <is>
-          <t>GERAL</t>
-        </is>
-      </c>
-      <c r="AB77" s="4" t="inlineStr">
-        <is>
-          <t>16:00</t>
-        </is>
-      </c>
-      <c r="AC77" s="4" t="inlineStr">
-        <is>
-          <t>16h00</t>
-        </is>
-      </c>
-      <c r="AD77" s="4" t="inlineStr">
-        <is>
-          <t>Sim · Automatico · 100%</t>
-        </is>
-      </c>
-      <c r="AE77" s="4" t="inlineStr">
-        <is>
-          <t>AUTOMATICO</t>
-        </is>
-      </c>
-      <c r="AF77" s="4" t="inlineStr">
-        <is>
-          <t>100.0</t>
-        </is>
-      </c>
-      <c r="AG77" s="4" t="inlineStr">
-        <is>
-          <t>["GOV", "Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private", "RPPS"]</t>
-        </is>
-      </c>
-      <c r="AH77" s="4" t="inlineStr">
-        <is>
-          <t>["GOV", "Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private", "RPPS"]</t>
-        </is>
-      </c>
-      <c r="AI77" s="4" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="AJ77" s="4" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AK77" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-01T00:00:00Z</t>
-        </is>
-      </c>
-      <c r="AL77" s="4" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="AM77" s="4" t="inlineStr">
-        <is>
-          <t>CAIXA CAPITAL PROTEGIDO CESTA AGRO FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO MULTIMERCADO LONGO PRAZO - RESPONSABIL</t>
-        </is>
-      </c>
-      <c r="AN77" s="4" t="inlineStr">
-        <is>
-          <t>Fundo com prazo de carência para aplicação e resgate, conforme Regulamento. Durante a carência, não é permitida a realização de aplicações ou resgates.
-Nova Operação Estruturada:
-Dia 07/10/2024 -&gt; Reabertura para Resgates e Aplicações do fundo;
-Dia 25/10/2024 -&gt; Fechamento para Aplicações e Resgates
-Dia 29/10/2024 -&gt; Início da nova operação estruturada de Cesta Agro.</t>
-        </is>
-      </c>
-      <c r="AO77" s="4" t="inlineStr">
-        <is>
-          <t>http://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_6621.pdf</t>
-        </is>
-      </c>
-      <c r="AP77" s="4" t="inlineStr">
-        <is>
-          <t>http://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_6621.pdf</t>
-        </is>
-      </c>
-      <c r="AQ77" s="4" t="inlineStr">
-        <is>
-          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_6621.pdf</t>
-        </is>
-      </c>
-      <c r="AR77" s="4" t="inlineStr">
-        <is>
-          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_6621.pdf</t>
-        </is>
-      </c>
-      <c r="AS77" s="4" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6621.pdf</t>
-        </is>
-      </c>
-      <c r="AT77" s="4" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6621.pdf</t>
-        </is>
-      </c>
-      <c r="AU77" s="4" t="inlineStr">
-        <is>
-          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_6621.pdf</t>
-        </is>
-      </c>
-      <c r="AV77" s="4" t="inlineStr">
-        <is>
-          <t>http://www.caixa.gov.br/caixa-asset/sumario-remuneracao/Documents/sumarios/6621-SUMARIO.pdf</t>
-        </is>
-      </c>
-      <c r="AW77" s="4" t="inlineStr"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="2" t="inlineStr">
-        <is>
-          <t>MULTIMERCADO</t>
-        </is>
-      </c>
-      <c r="B78" s="2" t="inlineStr">
-        <is>
-          <t>CAIXA FIC FIM CAPITAL PROTEGIDO CICLICO II LP - RL</t>
-        </is>
-      </c>
-      <c r="C78" s="2" t="inlineStr">
-        <is>
-          <t>18/07/2022</t>
-        </is>
-      </c>
-      <c r="D78" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E78" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F78" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G78" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H78" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I78" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J78" s="2" t="inlineStr">
-        <is>
-          <t>GOV | PF | PJ | RPPS</t>
-        </is>
-      </c>
-      <c r="K78" s="2" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-capital-protegido-ciclico-ii-multimercado-lp/Paginas/default.aspx</t>
-        </is>
-      </c>
-      <c r="L78" s="2" t="inlineStr">
-        <is>
-          <t>45.443.651/0001-94</t>
-        </is>
-      </c>
-      <c r="M78" s="2" t="inlineStr">
-        <is>
-          <t>6623</t>
-        </is>
-      </c>
-      <c r="N78" s="2" t="inlineStr">
-        <is>
-          <t>Conservador</t>
-        </is>
-      </c>
-      <c r="O78" s="2" t="inlineStr">
-        <is>
-          <t>0.9</t>
-        </is>
-      </c>
-      <c r="P78" s="2" t="inlineStr">
-        <is>
-          <t>5000.0</t>
-        </is>
-      </c>
-      <c r="Q78" s="2" t="inlineStr">
-        <is>
-          <t>500.0</t>
-        </is>
-      </c>
-      <c r="R78" s="2" t="inlineStr">
-        <is>
-          <t>500.0</t>
-        </is>
-      </c>
-      <c r="S78" s="2" t="inlineStr">
-        <is>
-          <t>4000.0</t>
-        </is>
-      </c>
-      <c r="T78" s="2" t="inlineStr">
-        <is>
-          <t>D+0 (du)</t>
-        </is>
-      </c>
-      <c r="U78" s="2" t="inlineStr">
-        <is>
-          <t>D+0 (du)</t>
-        </is>
-      </c>
-      <c r="V78" s="2" t="inlineStr">
-        <is>
-          <t>D+02 (du)</t>
-        </is>
-      </c>
-      <c r="W78" s="2" t="inlineStr">
-        <is>
-          <t>NÃO SE APLICA</t>
-        </is>
-      </c>
-      <c r="X78" s="2" t="inlineStr">
-        <is>
-          <t>Capital Protegido</t>
-        </is>
-      </c>
-      <c r="Y78" s="2" t="inlineStr">
-        <is>
-          <t>Fechado para captação</t>
-        </is>
-      </c>
-      <c r="Z78" s="2" t="inlineStr">
-        <is>
-          <t>LONGO PRAZO</t>
-        </is>
-      </c>
-      <c r="AA78" s="2" t="inlineStr">
-        <is>
-          <t>GERAL</t>
-        </is>
-      </c>
-      <c r="AB78" s="2" t="inlineStr">
-        <is>
-          <t>16:00</t>
-        </is>
-      </c>
-      <c r="AC78" s="2" t="inlineStr">
-        <is>
-          <t>16h00</t>
-        </is>
-      </c>
-      <c r="AD78" s="2" t="inlineStr">
-        <is>
-          <t>Sim · Automatico · 100%</t>
-        </is>
-      </c>
-      <c r="AE78" s="2" t="inlineStr">
-        <is>
-          <t>AUTOMATICO</t>
-        </is>
-      </c>
-      <c r="AF78" s="2" t="inlineStr">
-        <is>
-          <t>100.0</t>
-        </is>
-      </c>
-      <c r="AG78" s="2" t="inlineStr">
-        <is>
-          <t>["GOV", "Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private", "RPPS"]</t>
-        </is>
-      </c>
-      <c r="AH78" s="2" t="inlineStr">
-        <is>
-          <t>["GOV", "Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private", "RPPS"]</t>
-        </is>
-      </c>
-      <c r="AI78" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="AJ78" s="2" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AK78" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-01T00:00:00Z</t>
-        </is>
-      </c>
-      <c r="AL78" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="AM78" s="2" t="inlineStr">
-        <is>
-          <t>CAIXA CAPITAL PROTEGIDO CICLICO II FIC DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO MULTIMERCADO LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
-        </is>
-      </c>
-      <c r="AN78" s="2" t="inlineStr">
-        <is>
-          <t>Fundo com prazo de carência para aplicação e resgate, conforme Regulamento. Durante a carência, não é permitida a realização de aplicações ou resgates.
-Fechado para Aplicações e Resgates a partir de 26/08/2024 
--------
-Início da Operação Estruturada - 27/08/2024
-Fim da Operação Estruturada - 01/07/2026</t>
-        </is>
-      </c>
       <c r="AO78" s="2" t="inlineStr">
         <is>
           <t>http://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_6623.pdf</t>
@@ -18782,32 +18644,32 @@
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E79" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F79" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G79" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H79" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,78558600</t>
+        </is>
+      </c>
+      <c r="E79" s="6" t="inlineStr">
+        <is>
+          <t>-0,002</t>
+        </is>
+      </c>
+      <c r="F79" s="5" t="inlineStr">
+        <is>
+          <t>0,28</t>
+        </is>
+      </c>
+      <c r="G79" s="5" t="inlineStr">
+        <is>
+          <t>1,07</t>
+        </is>
+      </c>
+      <c r="H79" s="5" t="inlineStr">
+        <is>
+          <t>10,23</t>
         </is>
       </c>
       <c r="I79" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>175,417</t>
         </is>
       </c>
       <c r="J79" s="4" t="inlineStr">
@@ -19042,7 +18904,7 @@
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>896,026</t>
+          <t>895,915</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr">
@@ -19281,7 +19143,7 @@
       </c>
       <c r="I81" s="4" t="inlineStr">
         <is>
-          <t>746,101</t>
+          <t>746,100</t>
         </is>
       </c>
       <c r="J81" s="4" t="inlineStr">
@@ -19491,32 +19353,32 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E82" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F82" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G82" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H82" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>6,77731300</t>
+        </is>
+      </c>
+      <c r="E82" s="7" t="inlineStr">
+        <is>
+          <t>-0,004</t>
+        </is>
+      </c>
+      <c r="F82" s="7" t="inlineStr">
+        <is>
+          <t>-0,89</t>
+        </is>
+      </c>
+      <c r="G82" s="3" t="inlineStr">
+        <is>
+          <t>5,37</t>
+        </is>
+      </c>
+      <c r="H82" s="3" t="inlineStr">
+        <is>
+          <t>15,35</t>
         </is>
       </c>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>127,999</t>
         </is>
       </c>
       <c r="J82" s="2" t="inlineStr">
@@ -19726,32 +19588,32 @@
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E83" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F83" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G83" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H83" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,43079100</t>
+        </is>
+      </c>
+      <c r="E83" s="6" t="inlineStr">
+        <is>
+          <t>-0,003</t>
+        </is>
+      </c>
+      <c r="F83" s="5" t="inlineStr">
+        <is>
+          <t>0,28</t>
+        </is>
+      </c>
+      <c r="G83" s="5" t="inlineStr">
+        <is>
+          <t>3,85</t>
+        </is>
+      </c>
+      <c r="H83" s="5" t="inlineStr">
+        <is>
+          <t>15,06</t>
         </is>
       </c>
       <c r="I83" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>283,344</t>
         </is>
       </c>
       <c r="J83" s="4" t="inlineStr">
@@ -19966,32 +19828,32 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E84" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F84" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G84" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H84" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,35003000</t>
+        </is>
+      </c>
+      <c r="E84" s="7" t="inlineStr">
+        <is>
+          <t>-0,001</t>
+        </is>
+      </c>
+      <c r="F84" s="3" t="inlineStr">
+        <is>
+          <t>2,03</t>
+        </is>
+      </c>
+      <c r="G84" s="3" t="inlineStr">
+        <is>
+          <t>5,18</t>
+        </is>
+      </c>
+      <c r="H84" s="3" t="inlineStr">
+        <is>
+          <t>5,12</t>
         </is>
       </c>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13,174</t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr">
@@ -20230,7 +20092,7 @@
       </c>
       <c r="I85" s="4" t="inlineStr">
         <is>
-          <t>95,784</t>
+          <t>95,734</t>
         </is>
       </c>
       <c r="J85" s="4" t="inlineStr">
@@ -20708,7 +20570,7 @@
       </c>
       <c r="I87" s="4" t="inlineStr">
         <is>
-          <t>13,069</t>
+          <t>13,064</t>
         </is>
       </c>
       <c r="J87" s="4" t="inlineStr">
@@ -20723,12 +20585,12 @@
       </c>
       <c r="L87" s="4" t="inlineStr">
         <is>
-          <t>15.154.410/0001-64</t>
+          <t>01.525.057/0001-77</t>
         </is>
       </c>
       <c r="M87" s="4" t="inlineStr">
         <is>
-          <t>5832</t>
+          <t>53</t>
         </is>
       </c>
       <c r="N87" s="4" t="inlineStr">
@@ -20738,7 +20600,7 @@
       </c>
       <c r="O87" s="4" t="inlineStr">
         <is>
-          <t>0.8</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="P87" s="4" t="inlineStr">
@@ -20801,7 +20663,11 @@
           <t>GERAL</t>
         </is>
       </c>
-      <c r="AB87" s="4" t="inlineStr"/>
+      <c r="AB87" s="4" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
       <c r="AC87" s="4" t="inlineStr">
         <is>
           <t>17h00</t>
@@ -20850,52 +20716,52 @@
       </c>
       <c r="AM87" s="4" t="inlineStr">
         <is>
-          <t>CAIXA E-FUNDO IBOVESPA FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO EM AÇÕES - RESPONSABILIDADE LIMITADA</t>
+          <t>CAIXA IBOVESPA FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO EM AÇÕES - RESPONSABILIDADE LIMITADA</t>
         </is>
       </c>
       <c r="AN87" s="4" t="inlineStr">
         <is>
-          <t>As movimentações neste Fundo são realizadas exclusivamente pelo Internet Banking. A contagem para conversão de cotas e pagamento do resgate é feita em dias úteis, conforme estabelecido no Regulamento do Fundo. Este Fundo não está adaptado às normas vigentes para RPPS (Regimes Próprios de Previdência Social).</t>
+          <t>A contagem para conversão de cotas e pagamento do resgate é feita em dias úteis, conforme estabelecido no Regulamento do Fundo.</t>
         </is>
       </c>
       <c r="AO87" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5832.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_0053.pdf</t>
         </is>
       </c>
       <c r="AP87" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5832.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_0053.pdf</t>
         </is>
       </c>
       <c r="AQ87" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5832.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_0053.pdf</t>
         </is>
       </c>
       <c r="AR87" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_5832.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_0053.pdf</t>
         </is>
       </c>
       <c r="AS87" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5832.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_53.pdf</t>
         </is>
       </c>
       <c r="AT87" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5832.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_53.pdf</t>
         </is>
       </c>
       <c r="AU87" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5832.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_0053.pdf</t>
         </is>
       </c>
       <c r="AV87" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/caixa-asset/sumario-remuneracao/Documents/sumarios/5832-SUMARIO.pdf</t>
+          <t>https://www.caixa.gov.br/caixa-asset/sumario-remuneracao/Documents/sumarios/0053-SUMARIO.pdf</t>
         </is>
       </c>
       <c r="AW87" s="4" t="inlineStr"/>
@@ -21171,7 +21037,7 @@
       </c>
       <c r="I89" s="4" t="inlineStr">
         <is>
-          <t>273,136</t>
+          <t>272,946</t>
         </is>
       </c>
       <c r="J89" s="4" t="inlineStr">
@@ -21410,7 +21276,7 @@
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>436,541</t>
+          <t>436,520</t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr">
@@ -21649,7 +21515,7 @@
       </c>
       <c r="I91" s="4" t="inlineStr">
         <is>
-          <t>55,778</t>
+          <t>55,755</t>
         </is>
       </c>
       <c r="J91" s="4" t="inlineStr">
@@ -22127,7 +21993,7 @@
       </c>
       <c r="I93" s="4" t="inlineStr">
         <is>
-          <t>76,204</t>
+          <t>76,177</t>
         </is>
       </c>
       <c r="J93" s="4" t="inlineStr">
@@ -22580,32 +22446,32 @@
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E95" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F95" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G95" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H95" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,24755100</t>
+        </is>
+      </c>
+      <c r="E95" s="6" t="inlineStr">
+        <is>
+          <t>-0,021</t>
+        </is>
+      </c>
+      <c r="F95" s="6" t="inlineStr">
+        <is>
+          <t>-1,82</t>
+        </is>
+      </c>
+      <c r="G95" s="6" t="inlineStr">
+        <is>
+          <t>-3,07</t>
+        </is>
+      </c>
+      <c r="H95" s="5" t="inlineStr">
+        <is>
+          <t>5,30</t>
         </is>
       </c>
       <c r="I95" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>282,085</t>
         </is>
       </c>
       <c r="J95" s="4" t="inlineStr">
@@ -22844,7 +22710,7 @@
       </c>
       <c r="I96" s="2" t="inlineStr">
         <is>
-          <t>111,700</t>
+          <t>111,654</t>
         </is>
       </c>
       <c r="J96" s="2" t="inlineStr">
@@ -23083,7 +22949,7 @@
       </c>
       <c r="I97" s="4" t="inlineStr">
         <is>
-          <t>124,715</t>
+          <t>124,658</t>
         </is>
       </c>
       <c r="J97" s="4" t="inlineStr">
@@ -23322,7 +23188,7 @@
       </c>
       <c r="I98" s="2" t="inlineStr">
         <is>
-          <t>48,402</t>
+          <t>48,392</t>
         </is>
       </c>
       <c r="J98" s="2" t="inlineStr">
@@ -23565,7 +23431,7 @@
       </c>
       <c r="I99" s="4" t="inlineStr">
         <is>
-          <t>117,088</t>
+          <t>116,758</t>
         </is>
       </c>
       <c r="J99" s="4" t="inlineStr">
@@ -23804,7 +23670,7 @@
       </c>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t>39,901</t>
+          <t>39,899</t>
         </is>
       </c>
       <c r="J100" s="2" t="inlineStr">
@@ -24043,7 +23909,7 @@
       </c>
       <c r="I101" s="4" t="inlineStr">
         <is>
-          <t>629,705</t>
+          <t>629,401</t>
         </is>
       </c>
       <c r="J101" s="4" t="inlineStr">
@@ -24282,7 +24148,7 @@
       </c>
       <c r="I102" s="2" t="inlineStr">
         <is>
-          <t>466,941</t>
+          <t>466,540</t>
         </is>
       </c>
       <c r="J102" s="2" t="inlineStr">
@@ -24764,7 +24630,7 @@
       </c>
       <c r="I104" s="2" t="inlineStr">
         <is>
-          <t>29,338</t>
+          <t>29,329</t>
         </is>
       </c>
       <c r="J104" s="2" t="inlineStr">
@@ -25003,7 +24869,7 @@
       </c>
       <c r="I105" s="4" t="inlineStr">
         <is>
-          <t>1,723</t>
+          <t>1,718</t>
         </is>
       </c>
       <c r="J105" s="4" t="inlineStr">
@@ -25465,7 +25331,7 @@
       </c>
       <c r="I107" s="4" t="inlineStr">
         <is>
-          <t>35,003</t>
+          <t>34,828</t>
         </is>
       </c>
       <c r="J107" s="4" t="inlineStr">
@@ -25704,7 +25570,7 @@
       </c>
       <c r="I108" s="2" t="inlineStr">
         <is>
-          <t>834,076</t>
+          <t>832,919</t>
         </is>
       </c>
       <c r="J108" s="2" t="inlineStr">
@@ -26652,7 +26518,7 @@
       </c>
       <c r="I112" s="2" t="inlineStr">
         <is>
-          <t>268,165</t>
+          <t>268,052</t>
         </is>
       </c>
       <c r="J112" s="2" t="inlineStr">
@@ -26870,32 +26736,32 @@
       </c>
       <c r="D113" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E113" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F113" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G113" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H113" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>986,43017800</t>
+        </is>
+      </c>
+      <c r="E113" s="6" t="inlineStr">
+        <is>
+          <t>-0,003</t>
+        </is>
+      </c>
+      <c r="F113" s="6" t="inlineStr">
+        <is>
+          <t>-1,30</t>
+        </is>
+      </c>
+      <c r="G113" s="5" t="inlineStr">
+        <is>
+          <t>0,61</t>
+        </is>
+      </c>
+      <c r="H113" s="5" t="inlineStr">
+        <is>
+          <t>15,27</t>
         </is>
       </c>
       <c r="I113" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>8,000</t>
         </is>
       </c>
       <c r="J113" s="4" t="inlineStr">
@@ -27109,32 +26975,32 @@
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E114" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F114" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G114" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H114" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1.483,47485600</t>
+        </is>
+      </c>
+      <c r="E114" s="7" t="inlineStr">
+        <is>
+          <t>-0,002</t>
+        </is>
+      </c>
+      <c r="F114" s="7" t="inlineStr">
+        <is>
+          <t>-0,78</t>
+        </is>
+      </c>
+      <c r="G114" s="7" t="inlineStr">
+        <is>
+          <t>-0,82</t>
+        </is>
+      </c>
+      <c r="H114" s="3" t="inlineStr">
+        <is>
+          <t>9,76</t>
         </is>
       </c>
       <c r="I114" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>21,383</t>
         </is>
       </c>
       <c r="J114" s="2" t="inlineStr">
@@ -27344,7 +27210,7 @@
       </c>
       <c r="D115" s="4" t="inlineStr">
         <is>
-          <t>167,07500900</t>
+          <t>167,07500868</t>
         </is>
       </c>
       <c r="E115" s="6" t="inlineStr">
@@ -27608,7 +27474,7 @@
       </c>
       <c r="I116" s="2" t="inlineStr">
         <is>
-          <t>4,925</t>
+          <t>4,919</t>
         </is>
       </c>
       <c r="J116" s="2" t="inlineStr">
@@ -27844,7 +27710,7 @@
       </c>
       <c r="I117" s="4" t="inlineStr">
         <is>
-          <t>1.596,589</t>
+          <t>1.596,064</t>
         </is>
       </c>
       <c r="J117" s="4" t="inlineStr">
@@ -28076,7 +27942,7 @@
       </c>
       <c r="I118" s="2" t="inlineStr">
         <is>
-          <t>674,368</t>
+          <t>674,266</t>
         </is>
       </c>
       <c r="J118" s="2" t="inlineStr">
@@ -28299,7 +28165,7 @@
       </c>
       <c r="I119" s="4" t="inlineStr">
         <is>
-          <t>746,566</t>
+          <t>746,473</t>
         </is>
       </c>
       <c r="J119" s="4" t="inlineStr">
@@ -28522,7 +28388,7 @@
       </c>
       <c r="I120" s="2" t="inlineStr">
         <is>
-          <t>111,660</t>
+          <t>111,578</t>
         </is>
       </c>
       <c r="J120" s="2" t="inlineStr">
@@ -28982,7 +28848,7 @@
       </c>
       <c r="I122" s="2" t="inlineStr">
         <is>
-          <t>581,621</t>
+          <t>581,297</t>
         </is>
       </c>
       <c r="J122" s="2" t="inlineStr">
@@ -29210,7 +29076,7 @@
       </c>
       <c r="I123" s="4" t="inlineStr">
         <is>
-          <t>448,559</t>
+          <t>448,447</t>
         </is>
       </c>
       <c r="J123" s="4" t="inlineStr">
@@ -29433,7 +29299,7 @@
       </c>
       <c r="I124" s="2" t="inlineStr">
         <is>
-          <t>667,305</t>
+          <t>666,123</t>
         </is>
       </c>
       <c r="J124" s="2" t="inlineStr">
@@ -29898,7 +29764,7 @@
       </c>
       <c r="I126" s="2" t="inlineStr">
         <is>
-          <t>273,172</t>
+          <t>255,689</t>
         </is>
       </c>
       <c r="J126" s="2" t="inlineStr">
@@ -30616,7 +30482,7 @@
       </c>
       <c r="I129" s="4" t="inlineStr">
         <is>
-          <t>19,404</t>
+          <t>19,403</t>
         </is>
       </c>
       <c r="J129" s="4" t="inlineStr">
@@ -30857,7 +30723,7 @@
       </c>
       <c r="I130" s="2" t="inlineStr">
         <is>
-          <t>94,279</t>
+          <t>94,276</t>
         </is>
       </c>
       <c r="J130" s="2" t="inlineStr">
@@ -31100,7 +30966,7 @@
       </c>
       <c r="I131" s="4" t="inlineStr">
         <is>
-          <t>8.116,732</t>
+          <t>7.983,447</t>
         </is>
       </c>
       <c r="J131" s="4" t="inlineStr">
@@ -31338,7 +31204,7 @@
       </c>
       <c r="I132" s="2" t="inlineStr">
         <is>
-          <t>16.099,200</t>
+          <t>16.099,143</t>
         </is>
       </c>
       <c r="J132" s="2" t="inlineStr">
@@ -31577,7 +31443,7 @@
       </c>
       <c r="I133" s="4" t="inlineStr">
         <is>
-          <t>3.007,320</t>
+          <t>3.007,317</t>
         </is>
       </c>
       <c r="J133" s="4" t="inlineStr">
@@ -31791,7 +31657,7 @@
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>1,55391800</t>
+          <t>1,55391842</t>
         </is>
       </c>
       <c r="E134" s="3" t="inlineStr">
@@ -32275,7 +32141,7 @@
       </c>
       <c r="I136" s="2" t="inlineStr">
         <is>
-          <t>3.962,335</t>
+          <t>3.962,334</t>
         </is>
       </c>
       <c r="J136" s="2" t="inlineStr">
@@ -32725,7 +32591,7 @@
       </c>
       <c r="I138" s="2" t="inlineStr">
         <is>
-          <t>13.781,689</t>
+          <t>13.547,600</t>
         </is>
       </c>
       <c r="J138" s="2" t="inlineStr">
@@ -32963,7 +32829,7 @@
       </c>
       <c r="I139" s="4" t="inlineStr">
         <is>
-          <t>13.293,626</t>
+          <t>13.293,188</t>
         </is>
       </c>
       <c r="J139" s="4" t="inlineStr">
@@ -33202,7 +33068,7 @@
       </c>
       <c r="I140" s="2" t="inlineStr">
         <is>
-          <t>3.515,620</t>
+          <t>3.515,607</t>
         </is>
       </c>
       <c r="J140" s="2" t="inlineStr">
@@ -33676,7 +33542,7 @@
       </c>
       <c r="I142" s="2" t="inlineStr">
         <is>
-          <t>32.821,865</t>
+          <t>32.798,152</t>
         </is>
       </c>
       <c r="J142" s="2" t="inlineStr">
@@ -33912,7 +33778,7 @@
       </c>
       <c r="I143" s="4" t="inlineStr">
         <is>
-          <t>2.831,498</t>
+          <t>2.798,318</t>
         </is>
       </c>
       <c r="J143" s="4" t="inlineStr">
@@ -34150,7 +34016,7 @@
       </c>
       <c r="I144" s="2" t="inlineStr">
         <is>
-          <t>16.487,897</t>
+          <t>16.648,650</t>
         </is>
       </c>
       <c r="J144" s="2" t="inlineStr">
@@ -35112,7 +34978,7 @@
       </c>
       <c r="I148" s="2" t="inlineStr">
         <is>
-          <t>460,633</t>
+          <t>459,420</t>
         </is>
       </c>
       <c r="J148" s="2" t="inlineStr">
@@ -35839,7 +35705,7 @@
       </c>
       <c r="I151" s="4" t="inlineStr">
         <is>
-          <t>1.730,392</t>
+          <t>1.730,370</t>
         </is>
       </c>
       <c r="J151" s="4" t="inlineStr">
@@ -37390,7 +37256,7 @@
       </c>
       <c r="I158" s="2" t="inlineStr">
         <is>
-          <t>13.113,026</t>
+          <t>13.113,024</t>
         </is>
       </c>
       <c r="J158" s="2" t="inlineStr">
@@ -37405,12 +37271,12 @@
       </c>
       <c r="L158" s="2" t="inlineStr">
         <is>
-          <t>05.164.356/0001-84</t>
+          <t>03.737.206/0001-97</t>
         </is>
       </c>
       <c r="M158" s="2" t="inlineStr">
         <is>
-          <t>5462</t>
+          <t>5404</t>
         </is>
       </c>
       <c r="N158" s="2" t="inlineStr">
@@ -37465,7 +37331,7 @@
       </c>
       <c r="X158" s="2" t="inlineStr">
         <is>
-          <t>RF 100% TPF - Longo Prazo</t>
+          <t>RF DI até 49% Crédito Privado</t>
         </is>
       </c>
       <c r="Y158" s="2" t="inlineStr">
@@ -37536,57 +37402,58 @@
       </c>
       <c r="AM158" s="2" t="inlineStr">
         <is>
-          <t>CAIXA BRASIL TÍTULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
+          <t>CAIXA BRASIL FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA REFERENCIADO DI LONGO PRAZO - RESP LIMITADA</t>
         </is>
       </c>
       <c r="AN158" s="2" t="inlineStr">
         <is>
-          <t>Para aplicação no fundo é necessário o cadastramento prévio de cotistas, conforme descrito no FI657. O procedimento de inclusão da conta deverá ser realizado sempre que houver qualquer aplicação, mesmo para os clientes que já realizaram o cadsatramento anteriormente.</t>
+          <t>1. Para aplicação por meio de conta operação 003, é necessário o cadastramento prévio de cotistas, conforme descrito no item Adesão, do FI612.
+2. O procedimento de inclusão da conta deverá ser realizado sempre que houver qualquer aplicação por meio de conta operação 003, mesmo para os clientes que já realizaram o cadastramento anteriormente.</t>
         </is>
       </c>
       <c r="AO158" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5462.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5404.pdf</t>
         </is>
       </c>
       <c r="AP158" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5462.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5404.pdf</t>
         </is>
       </c>
       <c r="AQ158" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5462.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5404.pdf</t>
         </is>
       </c>
       <c r="AR158" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5462.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5404.pdf</t>
         </is>
       </c>
       <c r="AS158" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5462.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5404.pdf</t>
         </is>
       </c>
       <c r="AT158" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5462.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5404.pdf</t>
         </is>
       </c>
       <c r="AU158" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5462.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5404.pdf</t>
         </is>
       </c>
       <c r="AV158" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/caixa-asset/sumario-remuneracao/Documents/sumarios/5462-SUMARIO.pdf</t>
+          <t>https://www.caixa.gov.br/caixa-asset/sumario-remuneracao/Documents/sumarios/5404-SUMARIO.pdf</t>
         </is>
       </c>
       <c r="AW158" s="2" t="inlineStr">
         <is>
-          <t>https://web.microsoftstream.com/video/91aaf70b-85c2-4cf1-b537-e42b3bd894ec?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
+          <t>https://web.microsoftstream.com/video/f88f1fc7-aac3-44df-a2a5-ce3ac05edfb3?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
     </row>
@@ -38107,7 +37974,7 @@
       </c>
       <c r="I161" s="4" t="inlineStr">
         <is>
-          <t>1.568,519</t>
+          <t>1.541,491</t>
         </is>
       </c>
       <c r="J161" s="4" t="inlineStr">
@@ -38344,7 +38211,7 @@
       </c>
       <c r="I162" s="2" t="inlineStr">
         <is>
-          <t>24.067,652</t>
+          <t>24.067,648</t>
         </is>
       </c>
       <c r="J162" s="2" t="inlineStr">
@@ -38910,7 +38777,7 @@
       </c>
       <c r="I165" s="4" t="inlineStr">
         <is>
-          <t>282,305</t>
+          <t>282,301</t>
         </is>
       </c>
       <c r="J165" s="4" t="inlineStr">
@@ -39363,7 +39230,7 @@
       </c>
       <c r="D167" s="4" t="inlineStr">
         <is>
-          <t>11,11490200</t>
+          <t>11,11490221</t>
         </is>
       </c>
       <c r="E167" s="6" t="inlineStr">
@@ -40076,7 +39943,7 @@
       </c>
       <c r="D170" s="2" t="inlineStr">
         <is>
-          <t>3,39992000</t>
+          <t>3,39991961</t>
         </is>
       </c>
       <c r="E170" s="7" t="inlineStr">
@@ -40307,7 +40174,7 @@
       </c>
       <c r="D171" s="4" t="inlineStr">
         <is>
-          <t>2,45068700</t>
+          <t>2,45068727</t>
         </is>
       </c>
       <c r="E171" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Dados atualizados via Robô: 15/06/2026 19:11
</commit_message>
<xml_diff>
--- a/dados_atuais.xlsx
+++ b/dados_atuais.xlsx
@@ -822,43 +822,185 @@
           <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fi-renda-fixa-simples-lp/</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" s="2" t="inlineStr"/>
-      <c r="N2" s="2" t="inlineStr"/>
-      <c r="O2" s="2" t="inlineStr"/>
-      <c r="P2" s="2" t="inlineStr"/>
-      <c r="Q2" s="2" t="inlineStr"/>
-      <c r="R2" s="2" t="inlineStr"/>
-      <c r="S2" s="2" t="inlineStr"/>
-      <c r="T2" s="2" t="inlineStr"/>
-      <c r="U2" s="2" t="inlineStr"/>
-      <c r="V2" s="2" t="inlineStr"/>
-      <c r="W2" s="2" t="inlineStr"/>
-      <c r="X2" s="2" t="inlineStr"/>
-      <c r="Y2" s="2" t="inlineStr"/>
-      <c r="Z2" s="2" t="inlineStr"/>
-      <c r="AA2" s="2" t="inlineStr"/>
-      <c r="AB2" s="2" t="inlineStr"/>
-      <c r="AC2" s="2" t="inlineStr"/>
-      <c r="AD2" s="2" t="inlineStr"/>
-      <c r="AE2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>22.791.329/0001-50</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>5980</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="S2" s="2" t="inlineStr">
+        <is>
+          <t>0.02</t>
+        </is>
+      </c>
+      <c r="T2" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="U2" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="V2" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
+      <c r="W2" s="2" t="inlineStr">
+        <is>
+          <t>SELIC</t>
+        </is>
+      </c>
+      <c r="X2" s="2" t="inlineStr">
+        <is>
+          <t>RF Simples até 49% Crédito Privado</t>
+        </is>
+      </c>
+      <c r="Y2" s="2" t="inlineStr">
+        <is>
+          <t>Aberto para captação</t>
+        </is>
+      </c>
+      <c r="Z2" s="2" t="inlineStr">
+        <is>
+          <t>LONGO PRAZO</t>
+        </is>
+      </c>
+      <c r="AA2" s="2" t="inlineStr">
+        <is>
+          <t>GERAL</t>
+        </is>
+      </c>
+      <c r="AB2" s="2" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="AC2" s="2" t="inlineStr">
+        <is>
+          <t>17h00</t>
+        </is>
+      </c>
+      <c r="AD2" s="2" t="inlineStr">
+        <is>
+          <t>Não se aplica</t>
+        </is>
+      </c>
+      <c r="AE2" s="2" t="inlineStr">
+        <is>
+          <t>NÃO SE APLICA</t>
+        </is>
+      </c>
       <c r="AF2" s="2" t="inlineStr"/>
-      <c r="AG2" s="2" t="inlineStr"/>
-      <c r="AH2" s="2" t="inlineStr"/>
-      <c r="AI2" s="2" t="inlineStr"/>
-      <c r="AJ2" s="2" t="inlineStr"/>
+      <c r="AG2" s="2" t="inlineStr">
+        <is>
+          <t>["Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private"]</t>
+        </is>
+      </c>
+      <c r="AH2" s="2" t="inlineStr">
+        <is>
+          <t>["Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private"]</t>
+        </is>
+      </c>
+      <c r="AI2" s="2" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="AJ2" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
       <c r="AK2" s="2" t="inlineStr"/>
-      <c r="AL2" s="2" t="inlineStr"/>
-      <c r="AM2" s="2" t="inlineStr"/>
-      <c r="AN2" s="2" t="inlineStr"/>
-      <c r="AO2" s="2" t="inlineStr"/>
-      <c r="AP2" s="2" t="inlineStr"/>
-      <c r="AQ2" s="2" t="inlineStr"/>
-      <c r="AR2" s="2" t="inlineStr"/>
-      <c r="AS2" s="2" t="inlineStr"/>
-      <c r="AT2" s="2" t="inlineStr"/>
-      <c r="AU2" s="2" t="inlineStr"/>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AL2" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AM2" s="2" t="inlineStr">
+        <is>
+          <t>CAIXA E-SIMPLES FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
+        </is>
+      </c>
+      <c r="AN2" s="2" t="inlineStr">
+        <is>
+          <t>Fundo com movimentação exclusiva pelo IBC/APP.
+OBS: O Fundo possui a funcionalidade de Resgate Automático em caso de adesão pelo cotista, o gerente deverá proceder à contratação no SIART. Para ativar a funcionalidade de Resgate Automático, acessar o SIART -&gt; Movimentação Automática -&gt; Marcar
+As regras da funcionalidade de Movimentação Automática estão descritas no MN TE099.</t>
+        </is>
+      </c>
+      <c r="AO2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5980.pdf</t>
+        </is>
+      </c>
+      <c r="AP2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5980.pdf</t>
+        </is>
+      </c>
+      <c r="AQ2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5980.pdf</t>
+        </is>
+      </c>
+      <c r="AR2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5980.pdf</t>
+        </is>
+      </c>
+      <c r="AS2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5980.pdf</t>
+        </is>
+      </c>
+      <c r="AT2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5980.pdf</t>
+        </is>
+      </c>
+      <c r="AU2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5980.pdf</t>
+        </is>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/caixa-asset/sumario-remuneracao/Documents/sumarios/5980-SUMARIO.pdf</t>
+        </is>
+      </c>
       <c r="AW2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
@@ -13613,44 +13755,192 @@
           <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fi-multimercado-rv30-longo-prazo</t>
         </is>
       </c>
-      <c r="L57" s="4" t="inlineStr"/>
-      <c r="M57" s="4" t="inlineStr"/>
-      <c r="N57" s="4" t="inlineStr"/>
-      <c r="O57" s="4" t="inlineStr"/>
-      <c r="P57" s="4" t="inlineStr"/>
-      <c r="Q57" s="4" t="inlineStr"/>
-      <c r="R57" s="4" t="inlineStr"/>
-      <c r="S57" s="4" t="inlineStr"/>
-      <c r="T57" s="4" t="inlineStr"/>
-      <c r="U57" s="4" t="inlineStr"/>
-      <c r="V57" s="4" t="inlineStr"/>
-      <c r="W57" s="4" t="inlineStr"/>
-      <c r="X57" s="4" t="inlineStr"/>
-      <c r="Y57" s="4" t="inlineStr"/>
-      <c r="Z57" s="4" t="inlineStr"/>
-      <c r="AA57" s="4" t="inlineStr"/>
-      <c r="AB57" s="4" t="inlineStr"/>
-      <c r="AC57" s="4" t="inlineStr"/>
-      <c r="AD57" s="4" t="inlineStr"/>
-      <c r="AE57" s="4" t="inlineStr"/>
-      <c r="AF57" s="4" t="inlineStr"/>
-      <c r="AG57" s="4" t="inlineStr"/>
-      <c r="AH57" s="4" t="inlineStr"/>
-      <c r="AI57" s="4" t="inlineStr"/>
-      <c r="AJ57" s="4" t="inlineStr"/>
+      <c r="L57" s="4" t="inlineStr">
+        <is>
+          <t>03.737.188/0001-43</t>
+        </is>
+      </c>
+      <c r="M57" s="4" t="inlineStr">
+        <is>
+          <t>82</t>
+        </is>
+      </c>
+      <c r="N57" s="4" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="O57" s="4" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="P57" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="Q57" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="R57" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="S57" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="T57" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="U57" s="4" t="inlineStr">
+        <is>
+          <t>D+1 (du)</t>
+        </is>
+      </c>
+      <c r="V57" s="4" t="inlineStr">
+        <is>
+          <t>D+03 (du)</t>
+        </is>
+      </c>
+      <c r="W57" s="4" t="inlineStr">
+        <is>
+          <t>70% CDI + 30% IBOV</t>
+        </is>
+      </c>
+      <c r="X57" s="4" t="inlineStr">
+        <is>
+          <t>Multimercado</t>
+        </is>
+      </c>
+      <c r="Y57" s="4" t="inlineStr">
+        <is>
+          <t>Aberto para captação</t>
+        </is>
+      </c>
+      <c r="Z57" s="4" t="inlineStr">
+        <is>
+          <t>LONGO PRAZO</t>
+        </is>
+      </c>
+      <c r="AA57" s="4" t="inlineStr">
+        <is>
+          <t>GERAL</t>
+        </is>
+      </c>
+      <c r="AB57" s="4" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="AC57" s="4" t="inlineStr">
+        <is>
+          <t>16h00</t>
+        </is>
+      </c>
+      <c r="AD57" s="4" t="inlineStr">
+        <is>
+          <t>Sim · Automatico · 100%</t>
+        </is>
+      </c>
+      <c r="AE57" s="4" t="inlineStr">
+        <is>
+          <t>AUTOMATICO</t>
+        </is>
+      </c>
+      <c r="AF57" s="4" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
+      <c r="AG57" s="4" t="inlineStr">
+        <is>
+          <t>["GOV", "Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private", "RPPS"]</t>
+        </is>
+      </c>
+      <c r="AH57" s="4" t="inlineStr">
+        <is>
+          <t>["GOV", "Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private", "RPPS"]</t>
+        </is>
+      </c>
+      <c r="AI57" s="4" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AJ57" s="4" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
       <c r="AK57" s="4" t="inlineStr"/>
-      <c r="AL57" s="4" t="inlineStr"/>
-      <c r="AM57" s="4" t="inlineStr"/>
-      <c r="AN57" s="4" t="inlineStr"/>
-      <c r="AO57" s="4" t="inlineStr"/>
-      <c r="AP57" s="4" t="inlineStr"/>
-      <c r="AQ57" s="4" t="inlineStr"/>
-      <c r="AR57" s="4" t="inlineStr"/>
-      <c r="AS57" s="4" t="inlineStr"/>
-      <c r="AT57" s="4" t="inlineStr"/>
-      <c r="AU57" s="4" t="inlineStr"/>
-      <c r="AV57" s="4" t="inlineStr"/>
-      <c r="AW57" s="4" t="inlineStr"/>
+      <c r="AL57" s="4" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AM57" s="4" t="inlineStr">
+        <is>
+          <t>CAIXA RV 30 FUNDO DE INVESTIMENTO FINANCEIRO MULTIMERCADO LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
+        </is>
+      </c>
+      <c r="AN57" s="4" t="inlineStr">
+        <is>
+          <t>A contagem para conversão de cotas e pagamento do resgate é feita em dias úteis, conforme estabelecido no Regulamento do Fundo. Este Fundo está adaptado às normas vigentes para RPPS (Regimes Próprios de Previdência Social).</t>
+        </is>
+      </c>
+      <c r="AO57" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_0082.pdf</t>
+        </is>
+      </c>
+      <c r="AP57" s="4" t="inlineStr">
+        <is>
+          <t>http://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_0082.pdf</t>
+        </is>
+      </c>
+      <c r="AQ57" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_0082.pdf</t>
+        </is>
+      </c>
+      <c r="AR57" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_0082.pdf</t>
+        </is>
+      </c>
+      <c r="AS57" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_82.pdf</t>
+        </is>
+      </c>
+      <c r="AT57" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_82.pdf</t>
+        </is>
+      </c>
+      <c r="AU57" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_0082.pdf</t>
+        </is>
+      </c>
+      <c r="AV57" s="4" t="inlineStr">
+        <is>
+          <t>http://www.caixa.gov.br/caixa-asset/sumario-remuneracao/Documents/sumarios/0082-SUMARIO.pdf</t>
+        </is>
+      </c>
+      <c r="AW57" s="4" t="inlineStr">
+        <is>
+          <t>https://web.microsoftstream.com/video/86aa0100-d5af-4db2-9f67-441255924e4e?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -17224,15 +17514,19 @@
           <t>PF</t>
         </is>
       </c>
-      <c r="K73" s="4" t="inlineStr"/>
+      <c r="K73" s="4" t="inlineStr">
+        <is>
+          <t>http://www.caixa.gov.br/fundos-investimento/multimercado/estrategia-livre-mm-lp/Paginas/default.aspx</t>
+        </is>
+      </c>
       <c r="L73" s="4" t="inlineStr">
         <is>
-          <t>35.536.472/0001-48</t>
+          <t>34.660.333/0001-69</t>
         </is>
       </c>
       <c r="M73" s="4" t="inlineStr">
         <is>
-          <t>6479</t>
+          <t>6440</t>
         </is>
       </c>
       <c r="N73" s="4" t="inlineStr">
@@ -17242,7 +17536,7 @@
       </c>
       <c r="O73" s="4" t="inlineStr">
         <is>
-          <t>0.6</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="P73" s="4" t="inlineStr">
@@ -17330,8 +17624,16 @@
           <t>100.0</t>
         </is>
       </c>
-      <c r="AG73" s="4" t="inlineStr"/>
-      <c r="AH73" s="4" t="inlineStr"/>
+      <c r="AG73" s="4" t="inlineStr">
+        <is>
+          <t>["Pessoa Física", "Private"]</t>
+        </is>
+      </c>
+      <c r="AH73" s="4" t="inlineStr">
+        <is>
+          <t>["Pessoa Física", "Private"]</t>
+        </is>
+      </c>
       <c r="AI73" s="4" t="inlineStr">
         <is>
           <t>Não</t>
@@ -17350,52 +17652,48 @@
       </c>
       <c r="AM73" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FUNCIONÁRIOS ESTRATÉGIA LIVRE FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO MULTIMERCADO LONGO PRAZO - RESPONSABI</t>
-        </is>
-      </c>
-      <c r="AN73" s="4" t="inlineStr">
-        <is>
-          <t>Fundo destinado a Funcionários e aposentados da Caixa Econômica Federal. Disponível para aplicação somente via conta corrente marcada como conta-salário empregado CAIXA.</t>
-        </is>
-      </c>
+          <t>CAIXA ESTRATÉGIA LIVRE FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO MULTIMERCADO LONGO PRAZO - RESPONSABILIDADE LIMITA</t>
+        </is>
+      </c>
+      <c r="AN73" s="4" t="inlineStr"/>
       <c r="AO73" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_6479.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_6440.pdf</t>
         </is>
       </c>
       <c r="AP73" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_6479.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_6440.pdf</t>
         </is>
       </c>
       <c r="AQ73" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_6479.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_6440.pdf</t>
         </is>
       </c>
       <c r="AR73" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_6479.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_6440.pdf</t>
         </is>
       </c>
       <c r="AS73" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6479.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6440.pdf</t>
         </is>
       </c>
       <c r="AT73" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6479.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6440.pdf</t>
         </is>
       </c>
       <c r="AU73" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_6479.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_6440.pdf</t>
         </is>
       </c>
       <c r="AV73" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/caixa-asset/sumario-remuneracao/Documents/sumarios/6479-SUMARIO.pdf</t>
+          <t>https://www.caixa.gov.br/caixa-asset/sumario-remuneracao/Documents/sumarios/6440-SUMARIO.pdf</t>
         </is>
       </c>
       <c r="AW73" s="4" t="inlineStr"/>

</xml_diff>

<commit_message>
Dados atualizados via Robô: 18/06/2026 02:27
</commit_message>
<xml_diff>
--- a/dados_atuais.xlsx
+++ b/dados_atuais.xlsx
@@ -2493,183 +2493,43 @@
           <t>https://www.caixa.gov.br/fundos-investimento/e-fundos/renda-fixa-longo-prazo</t>
         </is>
       </c>
-      <c r="L9" s="4" t="inlineStr">
-        <is>
-          <t>15.154.422/0001-99</t>
-        </is>
-      </c>
-      <c r="M9" s="4" t="inlineStr">
-        <is>
-          <t>5834</t>
-        </is>
-      </c>
-      <c r="N9" s="4" t="inlineStr">
-        <is>
-          <t>Moderado</t>
-        </is>
-      </c>
-      <c r="O9" s="4" t="inlineStr">
-        <is>
-          <t>0.7</t>
-        </is>
-      </c>
-      <c r="P9" s="4" t="inlineStr">
-        <is>
-          <t>0.01</t>
-        </is>
-      </c>
-      <c r="Q9" s="4" t="inlineStr">
-        <is>
-          <t>0.01</t>
-        </is>
-      </c>
-      <c r="R9" s="4" t="inlineStr">
-        <is>
-          <t>0.01</t>
-        </is>
-      </c>
-      <c r="S9" s="4" t="inlineStr">
-        <is>
-          <t>0.01</t>
-        </is>
-      </c>
-      <c r="T9" s="4" t="inlineStr">
-        <is>
-          <t>D+0 (du)</t>
-        </is>
-      </c>
-      <c r="U9" s="4" t="inlineStr">
-        <is>
-          <t>D+0 (du)</t>
-        </is>
-      </c>
-      <c r="V9" s="4" t="inlineStr">
-        <is>
-          <t>D+00 (du)</t>
-        </is>
-      </c>
-      <c r="W9" s="4" t="inlineStr">
-        <is>
-          <t>CDI</t>
-        </is>
-      </c>
-      <c r="X9" s="4" t="inlineStr">
-        <is>
-          <t>RF até 49% Crédito Privado</t>
-        </is>
-      </c>
-      <c r="Y9" s="4" t="inlineStr">
-        <is>
-          <t>Aberto para captação</t>
-        </is>
-      </c>
-      <c r="Z9" s="4" t="inlineStr">
-        <is>
-          <t>LONGO PRAZO</t>
-        </is>
-      </c>
-      <c r="AA9" s="4" t="inlineStr">
-        <is>
-          <t>GERAL</t>
-        </is>
-      </c>
+      <c r="L9" s="4" t="inlineStr"/>
+      <c r="M9" s="4" t="inlineStr"/>
+      <c r="N9" s="4" t="inlineStr"/>
+      <c r="O9" s="4" t="inlineStr"/>
+      <c r="P9" s="4" t="inlineStr"/>
+      <c r="Q9" s="4" t="inlineStr"/>
+      <c r="R9" s="4" t="inlineStr"/>
+      <c r="S9" s="4" t="inlineStr"/>
+      <c r="T9" s="4" t="inlineStr"/>
+      <c r="U9" s="4" t="inlineStr"/>
+      <c r="V9" s="4" t="inlineStr"/>
+      <c r="W9" s="4" t="inlineStr"/>
+      <c r="X9" s="4" t="inlineStr"/>
+      <c r="Y9" s="4" t="inlineStr"/>
+      <c r="Z9" s="4" t="inlineStr"/>
+      <c r="AA9" s="4" t="inlineStr"/>
       <c r="AB9" s="4" t="inlineStr"/>
-      <c r="AC9" s="4" t="inlineStr">
-        <is>
-          <t>17h00</t>
-        </is>
-      </c>
-      <c r="AD9" s="4" t="inlineStr">
-        <is>
-          <t>Sim · Automatico · 90%</t>
-        </is>
-      </c>
-      <c r="AE9" s="4" t="inlineStr">
-        <is>
-          <t>AUTOMATICO</t>
-        </is>
-      </c>
-      <c r="AF9" s="4" t="inlineStr">
-        <is>
-          <t>90.0</t>
-        </is>
-      </c>
-      <c r="AG9" s="4" t="inlineStr">
-        <is>
-          <t>["Pessoa Física", "PJ Varejo", "Private"]</t>
-        </is>
-      </c>
-      <c r="AH9" s="4" t="inlineStr">
-        <is>
-          <t>["Pessoa Física", "PJ Varejo", "Private"]</t>
-        </is>
-      </c>
-      <c r="AI9" s="4" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="AJ9" s="4" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
+      <c r="AC9" s="4" t="inlineStr"/>
+      <c r="AD9" s="4" t="inlineStr"/>
+      <c r="AE9" s="4" t="inlineStr"/>
+      <c r="AF9" s="4" t="inlineStr"/>
+      <c r="AG9" s="4" t="inlineStr"/>
+      <c r="AH9" s="4" t="inlineStr"/>
+      <c r="AI9" s="4" t="inlineStr"/>
+      <c r="AJ9" s="4" t="inlineStr"/>
       <c r="AK9" s="4" t="inlineStr"/>
-      <c r="AL9" s="4" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="AM9" s="4" t="inlineStr">
-        <is>
-          <t>CAIXA E-FUNDO FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
-        </is>
-      </c>
-      <c r="AN9" s="4" t="inlineStr">
-        <is>
-          <t>Este Fundo não está adaptado às normas vigentes para RPPS (Regimes Próprios de Previdência Social).As movimentações neste Fundo são realizadas exclusivamente pelo Internet Banking.</t>
-        </is>
-      </c>
-      <c r="AO9" s="4" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5834.pdf</t>
-        </is>
-      </c>
-      <c r="AP9" s="4" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5834.pdf</t>
-        </is>
-      </c>
-      <c r="AQ9" s="4" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5834.pdf</t>
-        </is>
-      </c>
-      <c r="AR9" s="4" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_5834.pdf</t>
-        </is>
-      </c>
-      <c r="AS9" s="4" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5834.pdf</t>
-        </is>
-      </c>
-      <c r="AT9" s="4" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5834.pdf</t>
-        </is>
-      </c>
-      <c r="AU9" s="4" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5834.pdf</t>
-        </is>
-      </c>
-      <c r="AV9" s="4" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/caixa-asset/sumario-remuneracao/Documents/sumarios/5834-SUMARIO.pdf</t>
-        </is>
-      </c>
+      <c r="AL9" s="4" t="inlineStr"/>
+      <c r="AM9" s="4" t="inlineStr"/>
+      <c r="AN9" s="4" t="inlineStr"/>
+      <c r="AO9" s="4" t="inlineStr"/>
+      <c r="AP9" s="4" t="inlineStr"/>
+      <c r="AQ9" s="4" t="inlineStr"/>
+      <c r="AR9" s="4" t="inlineStr"/>
+      <c r="AS9" s="4" t="inlineStr"/>
+      <c r="AT9" s="4" t="inlineStr"/>
+      <c r="AU9" s="4" t="inlineStr"/>
+      <c r="AV9" s="4" t="inlineStr"/>
       <c r="AW9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
@@ -6042,32 +5902,32 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>1,11451698</t>
+          <t>1,11391100</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>-0,001</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
+          <t>-0,055</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>-0,04</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>3,26</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t>0,00</t>
         </is>
       </c>
-      <c r="G24" s="3" t="inlineStr">
-        <is>
-          <t>3,32</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>205,640</t>
+          <t>205,529</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
@@ -6277,32 +6137,32 @@
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>1,24296800</t>
-        </is>
-      </c>
-      <c r="E25" s="6" t="inlineStr">
-        <is>
-          <t>-0,001</t>
+          <t>1,24367200</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>0,055</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>0,55</t>
+          <t>0,60</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>6,12</t>
+          <t>6,18</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr">
         <is>
-          <t>14,54</t>
+          <t>14,61</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>71,373</t>
+          <t>71,413</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -6986,22 +6846,22 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>1,04160500</t>
-        </is>
-      </c>
-      <c r="E28" s="7" t="inlineStr">
-        <is>
-          <t>-0,002</t>
+          <t>1,04234000</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>0,068</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>0,53</t>
+          <t>0,60</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>6,22</t>
+          <t>6,30</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -7011,7 +6871,7 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>22,003</t>
+          <t>22,019</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
@@ -7209,32 +7069,32 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>1,17312400</t>
-        </is>
-      </c>
-      <c r="E29" s="6" t="inlineStr">
-        <is>
-          <t>-0,001</t>
+          <t>1,17384200</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>0,059</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>0,68</t>
+          <t>0,74</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>5,64</t>
+          <t>5,70</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr">
         <is>
-          <t>13,98</t>
+          <t>14,05</t>
         </is>
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>66,320</t>
+          <t>66,360</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -7440,22 +7300,22 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>1,07838119</t>
-        </is>
-      </c>
-      <c r="E30" s="7" t="inlineStr">
-        <is>
-          <t>-0,001</t>
+          <t>1,07985700</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>0,135</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>0,85</t>
+          <t>0,99</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>4,36</t>
+          <t>4,50</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -7465,7 +7325,7 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>304,803</t>
+          <t>305,220</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
@@ -13209,187 +13069,43 @@
           <t>https://www.caixa.gov.br/fundos-investimento/curto-prazo/fic-automatico-polis-rf-cp/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="L54" s="2" t="inlineStr">
-        <is>
-          <t>39.594.941/0001-36</t>
-        </is>
-      </c>
-      <c r="M54" s="2" t="inlineStr">
-        <is>
-          <t>6520</t>
-        </is>
-      </c>
-      <c r="N54" s="2" t="inlineStr">
-        <is>
-          <t>Conservador</t>
-        </is>
-      </c>
-      <c r="O54" s="2" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
-      </c>
-      <c r="P54" s="2" t="inlineStr">
-        <is>
-          <t>10000.0</t>
-        </is>
-      </c>
-      <c r="Q54" s="2" t="inlineStr">
-        <is>
-          <t>100.0</t>
-        </is>
-      </c>
-      <c r="R54" s="2" t="inlineStr">
-        <is>
-          <t>100.0</t>
-        </is>
-      </c>
-      <c r="S54" s="2" t="inlineStr">
-        <is>
-          <t>1000.0</t>
-        </is>
-      </c>
-      <c r="T54" s="2" t="inlineStr">
-        <is>
-          <t>D+0 (du)</t>
-        </is>
-      </c>
-      <c r="U54" s="2" t="inlineStr">
-        <is>
-          <t>D+0 (du)</t>
-        </is>
-      </c>
-      <c r="V54" s="2" t="inlineStr">
-        <is>
-          <t>D+00 (du)</t>
-        </is>
-      </c>
-      <c r="W54" s="2" t="inlineStr">
-        <is>
-          <t>CDI</t>
-        </is>
-      </c>
-      <c r="X54" s="2" t="inlineStr">
-        <is>
-          <t>RF 100% TPF - Curto Prazo</t>
-        </is>
-      </c>
-      <c r="Y54" s="2" t="inlineStr">
-        <is>
-          <t>Aberto para captação</t>
-        </is>
-      </c>
-      <c r="Z54" s="2" t="inlineStr">
-        <is>
-          <t>CURTO PRAZO</t>
-        </is>
-      </c>
-      <c r="AA54" s="2" t="inlineStr">
-        <is>
-          <t>GERAL</t>
-        </is>
-      </c>
-      <c r="AB54" s="2" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="AC54" s="2" t="inlineStr">
-        <is>
-          <t>17h00</t>
-        </is>
-      </c>
-      <c r="AD54" s="2" t="inlineStr">
-        <is>
-          <t>Sim · Automatico · 100%</t>
-        </is>
-      </c>
-      <c r="AE54" s="2" t="inlineStr">
-        <is>
-          <t>AUTOMATICO</t>
-        </is>
-      </c>
-      <c r="AF54" s="2" t="inlineStr">
-        <is>
-          <t>100.0</t>
-        </is>
-      </c>
-      <c r="AG54" s="2" t="inlineStr">
-        <is>
-          <t>["Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private"]</t>
-        </is>
-      </c>
-      <c r="AH54" s="2" t="inlineStr">
-        <is>
-          <t>["Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private"]</t>
-        </is>
-      </c>
-      <c r="AI54" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="AJ54" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
+      <c r="L54" s="2" t="inlineStr"/>
+      <c r="M54" s="2" t="inlineStr"/>
+      <c r="N54" s="2" t="inlineStr"/>
+      <c r="O54" s="2" t="inlineStr"/>
+      <c r="P54" s="2" t="inlineStr"/>
+      <c r="Q54" s="2" t="inlineStr"/>
+      <c r="R54" s="2" t="inlineStr"/>
+      <c r="S54" s="2" t="inlineStr"/>
+      <c r="T54" s="2" t="inlineStr"/>
+      <c r="U54" s="2" t="inlineStr"/>
+      <c r="V54" s="2" t="inlineStr"/>
+      <c r="W54" s="2" t="inlineStr"/>
+      <c r="X54" s="2" t="inlineStr"/>
+      <c r="Y54" s="2" t="inlineStr"/>
+      <c r="Z54" s="2" t="inlineStr"/>
+      <c r="AA54" s="2" t="inlineStr"/>
+      <c r="AB54" s="2" t="inlineStr"/>
+      <c r="AC54" s="2" t="inlineStr"/>
+      <c r="AD54" s="2" t="inlineStr"/>
+      <c r="AE54" s="2" t="inlineStr"/>
+      <c r="AF54" s="2" t="inlineStr"/>
+      <c r="AG54" s="2" t="inlineStr"/>
+      <c r="AH54" s="2" t="inlineStr"/>
+      <c r="AI54" s="2" t="inlineStr"/>
+      <c r="AJ54" s="2" t="inlineStr"/>
       <c r="AK54" s="2" t="inlineStr"/>
-      <c r="AL54" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="AM54" s="2" t="inlineStr">
-        <is>
-          <t>CAIXA FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA CURTO PRAZO - RESPONSABILIDADE LIMITADA</t>
-        </is>
-      </c>
-      <c r="AN54" s="2" t="inlineStr">
-        <is>
-          <t>*Este Fundo não está adaptado às normas vigentes para RPPS (Regimes Próprios de Previdência Social).</t>
-        </is>
-      </c>
-      <c r="AO54" s="2" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_6520.pdf</t>
-        </is>
-      </c>
-      <c r="AP54" s="2" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_6520.pdf</t>
-        </is>
-      </c>
-      <c r="AQ54" s="2" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_6520.pdf</t>
-        </is>
-      </c>
-      <c r="AR54" s="2" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_6520.pdf</t>
-        </is>
-      </c>
-      <c r="AS54" s="2" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6520.pdf</t>
-        </is>
-      </c>
-      <c r="AT54" s="2" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6520.pdf</t>
-        </is>
-      </c>
-      <c r="AU54" s="2" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_6520.pdf</t>
-        </is>
-      </c>
-      <c r="AV54" s="2" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/caixa-asset/sumario-remuneracao/Documents/sumarios/6520-SUMARIO.pdf</t>
-        </is>
-      </c>
+      <c r="AL54" s="2" t="inlineStr"/>
+      <c r="AM54" s="2" t="inlineStr"/>
+      <c r="AN54" s="2" t="inlineStr"/>
+      <c r="AO54" s="2" t="inlineStr"/>
+      <c r="AP54" s="2" t="inlineStr"/>
+      <c r="AQ54" s="2" t="inlineStr"/>
+      <c r="AR54" s="2" t="inlineStr"/>
+      <c r="AS54" s="2" t="inlineStr"/>
+      <c r="AT54" s="2" t="inlineStr"/>
+      <c r="AU54" s="2" t="inlineStr"/>
+      <c r="AV54" s="2" t="inlineStr"/>
       <c r="AW54" s="2" t="inlineStr"/>
     </row>
     <row r="55">
@@ -13410,32 +13126,32 @@
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>1,41776500</t>
-        </is>
-      </c>
-      <c r="E55" s="6" t="inlineStr">
-        <is>
-          <t>-0,008</t>
+          <t>1,41959400</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>0,055</t>
         </is>
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>0,50</t>
+          <t>0,63</t>
         </is>
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
-          <t>5,89</t>
+          <t>6,03</t>
         </is>
       </c>
       <c r="H55" s="5" t="inlineStr">
         <is>
-          <t>14,22</t>
+          <t>14,37</t>
         </is>
       </c>
       <c r="I55" s="4" t="inlineStr">
         <is>
-          <t>67,836</t>
+          <t>67,924</t>
         </is>
       </c>
       <c r="J55" s="4" t="inlineStr">
@@ -13641,32 +13357,32 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>1.194,07335400</t>
-        </is>
-      </c>
-      <c r="E56" s="7" t="inlineStr">
-        <is>
-          <t>-0,002</t>
-        </is>
-      </c>
-      <c r="F56" s="7" t="inlineStr">
-        <is>
-          <t>-0,79</t>
+          <t>1.217,72962800</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>0,365</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>1,17</t>
         </is>
       </c>
       <c r="G56" s="7" t="inlineStr">
         <is>
-          <t>-4,83</t>
+          <t>-2,95</t>
         </is>
       </c>
       <c r="H56" s="3" t="inlineStr">
         <is>
-          <t>0,74</t>
+          <t>2,73</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>36,394</t>
+          <t>37,115</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
@@ -13915,7 +13631,7 @@
       </c>
       <c r="I57" s="4" t="inlineStr">
         <is>
-          <t>540,035</t>
+          <t>322,067</t>
         </is>
       </c>
       <c r="J57" s="4" t="inlineStr">
@@ -14133,32 +13849,32 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>1.633,53388100</t>
+          <t>1.629,90381800</t>
         </is>
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
-          <t>-0,006</t>
+          <t>-0,228</t>
         </is>
       </c>
       <c r="F58" s="7" t="inlineStr">
         <is>
-          <t>-0,22</t>
+          <t>-0,44</t>
         </is>
       </c>
       <c r="G58" s="3" t="inlineStr">
         <is>
-          <t>4,25</t>
+          <t>4,01</t>
         </is>
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>12,10</t>
+          <t>11,85</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>114,178</t>
+          <t>113,924</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
@@ -14830,32 +14546,32 @@
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>1,25247300</t>
-        </is>
-      </c>
-      <c r="E61" s="6" t="inlineStr">
-        <is>
-          <t>-0,005</t>
+          <t>1,25334900</t>
+        </is>
+      </c>
+      <c r="E61" s="5" t="inlineStr">
+        <is>
+          <t>0,064</t>
         </is>
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>0,07</t>
+          <t>0,14</t>
         </is>
       </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
-          <t>2,55</t>
+          <t>2,62</t>
         </is>
       </c>
       <c r="H61" s="5" t="inlineStr">
         <is>
-          <t>10,08</t>
+          <t>10,15</t>
         </is>
       </c>
       <c r="I61" s="4" t="inlineStr">
         <is>
-          <t>6,308</t>
+          <t>6,313</t>
         </is>
       </c>
       <c r="J61" s="4" t="inlineStr">
@@ -15527,32 +15243,32 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>1,40160000</t>
+          <t>1,39964100</t>
         </is>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>-0,004</t>
+          <t>-0,144</t>
         </is>
       </c>
       <c r="F64" s="7" t="inlineStr">
         <is>
-          <t>-1,32</t>
+          <t>-1,45</t>
         </is>
       </c>
       <c r="G64" s="3" t="inlineStr">
         <is>
-          <t>2,67</t>
+          <t>2,53</t>
         </is>
       </c>
       <c r="H64" s="3" t="inlineStr">
         <is>
-          <t>14,69</t>
+          <t>14,53</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>11,621</t>
+          <t>11,604</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
@@ -16224,32 +15940,32 @@
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>5,32743032</t>
+          <t>5,31853100</t>
         </is>
       </c>
       <c r="E67" s="6" t="inlineStr">
         <is>
-          <t>-0,003</t>
+          <t>-0,170</t>
         </is>
       </c>
       <c r="F67" s="6" t="inlineStr">
         <is>
-          <t>-0,17</t>
+          <t>-0,34</t>
         </is>
       </c>
       <c r="G67" s="5" t="inlineStr">
         <is>
-          <t>3,82</t>
+          <t>3,65</t>
         </is>
       </c>
       <c r="H67" s="5" t="inlineStr">
         <is>
-          <t>11,88</t>
+          <t>11,69</t>
         </is>
       </c>
       <c r="I67" s="4" t="inlineStr">
         <is>
-          <t>32,705</t>
+          <t>32,651</t>
         </is>
       </c>
       <c r="J67" s="4" t="inlineStr">
@@ -16702,32 +16418,32 @@
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>2,85853100</t>
+          <t>2,85529000</t>
         </is>
       </c>
       <c r="E69" s="6" t="inlineStr">
         <is>
-          <t>-0,004</t>
+          <t>-0,117</t>
         </is>
       </c>
       <c r="F69" s="6" t="inlineStr">
         <is>
-          <t>-0,16</t>
+          <t>-0,27</t>
         </is>
       </c>
       <c r="G69" s="5" t="inlineStr">
         <is>
-          <t>2,34</t>
+          <t>2,22</t>
         </is>
       </c>
       <c r="H69" s="5" t="inlineStr">
         <is>
-          <t>9,66</t>
+          <t>9,54</t>
         </is>
       </c>
       <c r="I69" s="4" t="inlineStr">
         <is>
-          <t>73,670</t>
+          <t>73,586</t>
         </is>
       </c>
       <c r="J69" s="4" t="inlineStr">
@@ -17654,32 +17370,32 @@
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>1.655,47601300</t>
+          <t>1.651,77540600</t>
         </is>
       </c>
       <c r="E73" s="6" t="inlineStr">
         <is>
-          <t>-0,003</t>
+          <t>-0,226</t>
         </is>
       </c>
       <c r="F73" s="6" t="inlineStr">
         <is>
-          <t>-0,17</t>
+          <t>-0,39</t>
         </is>
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>4,67</t>
+          <t>4,44</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
         <is>
-          <t>13,08</t>
+          <t>12,82</t>
         </is>
       </c>
       <c r="I73" s="4" t="inlineStr">
         <is>
-          <t>14,426</t>
+          <t>14,394</t>
         </is>
       </c>
       <c r="J73" s="4" t="inlineStr">
@@ -17889,22 +17605,22 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>0,48056572</t>
+          <t>0,47587800</t>
         </is>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>-0,005</t>
+          <t>-0,981</t>
         </is>
       </c>
       <c r="F74" s="7" t="inlineStr">
         <is>
-          <t>-8,79</t>
+          <t>-9,68</t>
         </is>
       </c>
       <c r="G74" s="7" t="inlineStr">
         <is>
-          <t>-33,44</t>
+          <t>-34,09</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
@@ -17914,7 +17630,7 @@
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>3,819</t>
+          <t>3,782</t>
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr">
@@ -18131,32 +17847,32 @@
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>3,26822500</t>
-        </is>
-      </c>
-      <c r="E75" s="6" t="inlineStr">
-        <is>
-          <t>-0,005</t>
+          <t>3,27155200</t>
+        </is>
+      </c>
+      <c r="E75" s="5" t="inlineStr">
+        <is>
+          <t>0,095</t>
         </is>
       </c>
       <c r="F75" s="6" t="inlineStr">
         <is>
-          <t>-0,35</t>
+          <t>-0,25</t>
         </is>
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2,57</t>
+          <t>2,68</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
         <is>
-          <t>7,79</t>
+          <t>7,89</t>
         </is>
       </c>
       <c r="I75" s="4" t="inlineStr">
         <is>
-          <t>155,660</t>
+          <t>155,819</t>
         </is>
       </c>
       <c r="J75" s="4" t="inlineStr">
@@ -18376,32 +18092,32 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>1,53915200</t>
+          <t>1,53744800</t>
         </is>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>-0,004</t>
+          <t>-0,115</t>
         </is>
       </c>
       <c r="F76" s="7" t="inlineStr">
         <is>
-          <t>-0,64</t>
+          <t>-0,75</t>
         </is>
       </c>
       <c r="G76" s="3" t="inlineStr">
         <is>
-          <t>3,08</t>
+          <t>2,96</t>
         </is>
       </c>
       <c r="H76" s="3" t="inlineStr">
         <is>
-          <t>18,86</t>
+          <t>18,73</t>
         </is>
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>14,500</t>
+          <t>14,484</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr">
@@ -18621,32 +18337,32 @@
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>1,37928700</t>
-        </is>
-      </c>
-      <c r="E77" s="6" t="inlineStr">
-        <is>
-          <t>-0,003</t>
+          <t>1,38258800</t>
+        </is>
+      </c>
+      <c r="E77" s="5" t="inlineStr">
+        <is>
+          <t>0,235</t>
         </is>
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>0,39</t>
+          <t>0,63</t>
         </is>
       </c>
       <c r="G77" s="5" t="inlineStr">
         <is>
-          <t>1,70</t>
+          <t>1,94</t>
         </is>
       </c>
       <c r="H77" s="5" t="inlineStr">
         <is>
-          <t>6,21</t>
+          <t>6,46</t>
         </is>
       </c>
       <c r="I77" s="4" t="inlineStr">
         <is>
-          <t>70,681</t>
+          <t>70,850</t>
         </is>
       </c>
       <c r="J77" s="4" t="inlineStr">
@@ -18868,32 +18584,32 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>1,47508600</t>
-        </is>
-      </c>
-      <c r="E78" s="7" t="inlineStr">
-        <is>
-          <t>-0,003</t>
+          <t>1,48188800</t>
+        </is>
+      </c>
+      <c r="E78" s="3" t="inlineStr">
+        <is>
+          <t>0,457</t>
         </is>
       </c>
       <c r="F78" s="7" t="inlineStr">
         <is>
-          <t>-1,79</t>
+          <t>-1,34</t>
         </is>
       </c>
       <c r="G78" s="3" t="inlineStr">
         <is>
-          <t>2,00</t>
+          <t>2,47</t>
         </is>
       </c>
       <c r="H78" s="3" t="inlineStr">
         <is>
-          <t>13,63</t>
+          <t>14,15</t>
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>191,260</t>
+          <t>192,142</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr">
@@ -19115,32 +18831,32 @@
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>1,78886200</t>
-        </is>
-      </c>
-      <c r="E79" s="6" t="inlineStr">
-        <is>
-          <t>-0,002</t>
+          <t>1,78973900</t>
+        </is>
+      </c>
+      <c r="E79" s="5" t="inlineStr">
+        <is>
+          <t>0,047</t>
         </is>
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>0,46</t>
+          <t>0,51</t>
         </is>
       </c>
       <c r="G79" s="5" t="inlineStr">
         <is>
-          <t>1,26</t>
+          <t>1,31</t>
         </is>
       </c>
       <c r="H79" s="5" t="inlineStr">
         <is>
-          <t>10,08</t>
+          <t>10,13</t>
         </is>
       </c>
       <c r="I79" s="4" t="inlineStr">
         <is>
-          <t>175,689</t>
+          <t>175,775</t>
         </is>
       </c>
       <c r="J79" s="4" t="inlineStr">
@@ -19824,32 +19540,32 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>6,83251800</t>
+          <t>6,82102000</t>
         </is>
       </c>
       <c r="E82" s="7" t="inlineStr">
         <is>
-          <t>-0,004</t>
+          <t>-0,172</t>
         </is>
       </c>
       <c r="F82" s="7" t="inlineStr">
         <is>
-          <t>-0,08</t>
+          <t>-0,25</t>
         </is>
       </c>
       <c r="G82" s="3" t="inlineStr">
         <is>
-          <t>6,23</t>
+          <t>6,05</t>
         </is>
       </c>
       <c r="H82" s="3" t="inlineStr">
         <is>
-          <t>16,13</t>
+          <t>15,93</t>
         </is>
       </c>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t>129,074</t>
+          <t>128,857</t>
         </is>
       </c>
       <c r="J82" s="2" t="inlineStr">
@@ -20299,32 +20015,32 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>1,36033300</t>
+          <t>1,35361800</t>
         </is>
       </c>
       <c r="E84" s="7" t="inlineStr">
         <is>
-          <t>-0,002</t>
+          <t>-0,495</t>
         </is>
       </c>
       <c r="F84" s="3" t="inlineStr">
         <is>
-          <t>2,81</t>
+          <t>2,31</t>
         </is>
       </c>
       <c r="G84" s="3" t="inlineStr">
         <is>
-          <t>5,98</t>
+          <t>5,46</t>
         </is>
       </c>
       <c r="H84" s="3" t="inlineStr">
         <is>
-          <t>5,83</t>
+          <t>5,31</t>
         </is>
       </c>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t>13,089</t>
+          <t>13,024</t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr">
@@ -22917,32 +22633,32 @@
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
-          <t>1,23795100</t>
+          <t>1,23155100</t>
         </is>
       </c>
       <c r="E95" s="6" t="inlineStr">
         <is>
-          <t>-0,026</t>
+          <t>-0,537</t>
         </is>
       </c>
       <c r="F95" s="6" t="inlineStr">
         <is>
-          <t>-2,57</t>
+          <t>-3,08</t>
         </is>
       </c>
       <c r="G95" s="6" t="inlineStr">
         <is>
-          <t>-3,81</t>
+          <t>-4,31</t>
         </is>
       </c>
       <c r="H95" s="5" t="inlineStr">
         <is>
-          <t>3,71</t>
+          <t>3,17</t>
         </is>
       </c>
       <c r="I95" s="4" t="inlineStr">
         <is>
-          <t>279,767</t>
+          <t>278,321</t>
         </is>
       </c>
       <c r="J95" s="4" t="inlineStr">
@@ -26765,12 +26481,12 @@
       </c>
       <c r="L111" s="4" t="inlineStr">
         <is>
-          <t>59.815.671/0001-53</t>
+          <t>30.068.049/0001-47</t>
         </is>
       </c>
       <c r="M111" s="4" t="inlineStr">
         <is>
-          <t>7971</t>
+          <t>6499</t>
         </is>
       </c>
       <c r="N111" s="4" t="inlineStr">
@@ -26805,7 +26521,7 @@
       </c>
       <c r="T111" s="4" t="inlineStr">
         <is>
-          <t>D+0 (du)</t>
+          <t>D+1 (du)</t>
         </is>
       </c>
       <c r="U111" s="4" t="inlineStr">
@@ -26820,7 +26536,7 @@
       </c>
       <c r="W111" s="4" t="inlineStr">
         <is>
-          <t>NÃO SE APLICA</t>
+          <t>IBOV</t>
         </is>
       </c>
       <c r="X111" s="4" t="inlineStr">
@@ -26830,7 +26546,7 @@
       </c>
       <c r="Y111" s="4" t="inlineStr">
         <is>
-          <t>Fechado para captação</t>
+          <t>Aberto para captação</t>
         </is>
       </c>
       <c r="Z111" s="4" t="inlineStr">
@@ -26855,23 +26571,27 @@
       </c>
       <c r="AD111" s="4" t="inlineStr">
         <is>
-          <t>Não se aplica</t>
+          <t>Sim · Automatico · 100%</t>
         </is>
       </c>
       <c r="AE111" s="4" t="inlineStr">
         <is>
-          <t>NÃO SE APLICA</t>
-        </is>
-      </c>
-      <c r="AF111" s="4" t="inlineStr"/>
+          <t>AUTOMATICO</t>
+        </is>
+      </c>
+      <c r="AF111" s="4" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
       <c r="AG111" s="4" t="inlineStr">
         <is>
-          <t>["GOV", "Pessoa Física", "PJ Atacado", "Private"]</t>
+          <t>["GOV", "Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private"]</t>
         </is>
       </c>
       <c r="AH111" s="4" t="inlineStr">
         <is>
-          <t>["GOV", "Pessoa Física", "PJ Atacado", "Private"]</t>
+          <t>["GOV", "Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private"]</t>
         </is>
       </c>
       <c r="AI111" s="4" t="inlineStr">
@@ -26886,7 +26606,7 @@
       </c>
       <c r="AK111" s="4" t="inlineStr">
         <is>
-          <t>2025-05-04T00:00:00Z</t>
+          <t>2021-06-13T00:00:00Z</t>
         </is>
       </c>
       <c r="AL111" s="4" t="inlineStr">
@@ -26896,52 +26616,52 @@
       </c>
       <c r="AM111" s="4" t="inlineStr">
         <is>
-          <t>CAIXA SEGURIDADE II FUNDO DE INVESTIMENTO FINANCEIRO AÇÕES - RESPONSABILIDADE LIMITADA</t>
+          <t>CAIXA SEGURIDADE FUNDO DE INVESTIMENTO FINANCEIRO EM AÇÕES - RESPONSABILIDADE LIMITADA</t>
         </is>
       </c>
       <c r="AN111" s="4" t="inlineStr">
         <is>
-          <t>Fundo ficará fechado para novas aplicações a partir do dia 13/05/2025 (inclusive).</t>
+          <t>Canal de distribuição: Rede CAIXA, IBC. A reserva inicial, no âmbito da OFERTA, será feita por meio do Home Broker CAIXA. Resgates: Lock up de 45 dias. Inicio dia 30/04/2021 - Termino 13/06/2021. Liberado resgate a partir do dia 14/06/2021 (segunda-feira).</t>
         </is>
       </c>
       <c r="AO111" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_7971.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_6499.pdf</t>
         </is>
       </c>
       <c r="AP111" s="4" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_7971.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_6499.pdf</t>
         </is>
       </c>
       <c r="AQ111" s="4" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_7971.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_6499.pdf</t>
         </is>
       </c>
       <c r="AR111" s="4" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_7971.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_6499.pdf</t>
         </is>
       </c>
       <c r="AS111" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_7971.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6499.pdf</t>
         </is>
       </c>
       <c r="AT111" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_7971.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6499.pdf</t>
         </is>
       </c>
       <c r="AU111" s="4" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_7971.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_6499.pdf</t>
         </is>
       </c>
       <c r="AV111" s="4" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/caixa-asset/sumario-remuneracao/Documents/sumarios/7971-SUMARIO.pdf</t>
+          <t>https://www.caixa.gov.br/caixa-asset/sumario-remuneracao/Documents/sumarios/6499-SUMARIO.pdf</t>
         </is>
       </c>
       <c r="AW111" s="4" t="inlineStr"/>
@@ -27207,32 +26927,32 @@
       </c>
       <c r="D113" s="4" t="inlineStr">
         <is>
-          <t>980,80098800</t>
+          <t>976,60273900</t>
         </is>
       </c>
       <c r="E113" s="6" t="inlineStr">
         <is>
-          <t>-0,003</t>
+          <t>-0,431</t>
         </is>
       </c>
       <c r="F113" s="6" t="inlineStr">
         <is>
-          <t>-1,87</t>
-        </is>
-      </c>
-      <c r="G113" s="5" t="inlineStr">
-        <is>
-          <t>0,04</t>
+          <t>-2,29</t>
+        </is>
+      </c>
+      <c r="G113" s="6" t="inlineStr">
+        <is>
+          <t>-0,38</t>
         </is>
       </c>
       <c r="H113" s="5" t="inlineStr">
         <is>
-          <t>13,75</t>
+          <t>13,26</t>
         </is>
       </c>
       <c r="I113" s="4" t="inlineStr">
         <is>
-          <t>7,954</t>
+          <t>7,920</t>
         </is>
       </c>
       <c r="J113" s="4" t="inlineStr">
@@ -27446,32 +27166,32 @@
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>1.466,80464200</t>
+          <t>1.458,80592500</t>
         </is>
       </c>
       <c r="E114" s="7" t="inlineStr">
         <is>
-          <t>-0,002</t>
+          <t>-0,548</t>
         </is>
       </c>
       <c r="F114" s="7" t="inlineStr">
         <is>
-          <t>-1,90</t>
+          <t>-2,43</t>
         </is>
       </c>
       <c r="G114" s="7" t="inlineStr">
         <is>
-          <t>-1,93</t>
+          <t>-2,47</t>
         </is>
       </c>
       <c r="H114" s="3" t="inlineStr">
         <is>
-          <t>7,50</t>
+          <t>6,91</t>
         </is>
       </c>
       <c r="I114" s="2" t="inlineStr">
         <is>
-          <t>21,142</t>
+          <t>21,027</t>
         </is>
       </c>
       <c r="J114" s="2" t="inlineStr">
@@ -27681,7 +27401,7 @@
       </c>
       <c r="D115" s="4" t="inlineStr">
         <is>
-          <t>165,64717459</t>
+          <t>165,64717500</t>
         </is>
       </c>
       <c r="E115" s="6" t="inlineStr">
@@ -29329,17 +29049,17 @@
       </c>
       <c r="K122" s="2" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/fundos-investimento/mutuos-privatizacao/fmp-fgts-petrobas-2</t>
+          <t>https://www.caixa.gov.br/fundos-investimento/mutuos-privatizacao/fmp-fgts-petrobas-4</t>
         </is>
       </c>
       <c r="L122" s="2" t="inlineStr">
         <is>
-          <t>03.915.910/0001-92</t>
+          <t>03.555.959/0001-81</t>
         </is>
       </c>
       <c r="M122" s="2" t="inlineStr">
         <is>
-          <t>5202</t>
+          <t>5204</t>
         </is>
       </c>
       <c r="N122" s="2" t="inlineStr">
@@ -29349,29 +29069,29 @@
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>0.95</t>
         </is>
       </c>
       <c r="P122" s="2" t="inlineStr">
         <is>
+          <t>300.0</t>
+        </is>
+      </c>
+      <c r="Q122" s="2" t="inlineStr">
+        <is>
           <t>0.01</t>
         </is>
       </c>
-      <c r="Q122" s="2" t="inlineStr">
+      <c r="R122" s="2" t="inlineStr">
         <is>
           <t>0.01</t>
         </is>
       </c>
-      <c r="R122" s="2" t="inlineStr">
+      <c r="S122" s="2" t="inlineStr">
         <is>
           <t>0.01</t>
         </is>
       </c>
-      <c r="S122" s="2" t="inlineStr">
-        <is>
-          <t>0.01</t>
-        </is>
-      </c>
       <c r="T122" s="2" t="inlineStr">
         <is>
           <t>D+0 (du)</t>
@@ -29399,7 +29119,7 @@
       </c>
       <c r="Y122" s="2" t="inlineStr">
         <is>
-          <t>Aberto para captação</t>
+          <t>Fechado para captação</t>
         </is>
       </c>
       <c r="Z122" s="2" t="inlineStr">
@@ -29412,11 +29132,7 @@
           <t>GERAL</t>
         </is>
       </c>
-      <c r="AB122" s="2" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
+      <c r="AB122" s="2" t="inlineStr"/>
       <c r="AC122" s="2" t="inlineStr">
         <is>
           <t>17h00</t>
@@ -29453,53 +29169,52 @@
       </c>
       <c r="AM122" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FUNDO MÚTUO DE PRIVATIZAÇÃO - FGTS - PETROBRAS II - RESPONSABILIDADE LIMITADA</t>
+          <t>CAIXA FUNDO MÚTUO DE PRIVATIZAÇÃO - FGTS - PETROBRAS IV - RESPONSABILIDADE LIMITADA</t>
         </is>
       </c>
       <c r="AN122" s="2" t="inlineStr">
         <is>
-          <t>O fundo encontra-se aberto para receber recursos provenientes de outros Fundos FMP-FGTS.
-Prazo de carência: 6 meses para transferência total ou parcial do investimento no FUNDO para outro FMP- FGTS ou para um Clube de Investimento – FGTS, ou 12 meses para retorno à(s) conta(s) vinculada(s) do investidor junto ao FGTS.</t>
+          <t>FUNDO FECHADO.</t>
         </is>
       </c>
       <c r="AO122" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5202.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5204.pdf</t>
         </is>
       </c>
       <c r="AP122" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5202.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5204.pdf</t>
         </is>
       </c>
       <c r="AQ122" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5202.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5204.pdf</t>
         </is>
       </c>
       <c r="AR122" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5202.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5204.pdf</t>
         </is>
       </c>
       <c r="AS122" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5202.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5204.pdf</t>
         </is>
       </c>
       <c r="AT122" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5202.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5204.pdf</t>
         </is>
       </c>
       <c r="AU122" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5202.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5204.pdf</t>
         </is>
       </c>
       <c r="AV122" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/caixa-asset/sumario-remuneracao/Documents/sumarios/5202-SUMARIO.pdf</t>
+          <t>https://www.caixa.gov.br/caixa-asset/sumario-remuneracao/Documents/sumarios/5204-SUMARIO.pdf</t>
         </is>
       </c>
       <c r="AW122" s="2" t="inlineStr"/>
@@ -29997,7 +29712,7 @@
       </c>
       <c r="I125" s="4" t="inlineStr">
         <is>
-          <t>58,108</t>
+          <t>59,525</t>
         </is>
       </c>
       <c r="J125" s="4" t="inlineStr">
@@ -30732,12 +30447,12 @@
       </c>
       <c r="L128" s="2" t="inlineStr">
         <is>
-          <t>09.181.268/0001-41</t>
+          <t>09.548.725/0001-93</t>
         </is>
       </c>
       <c r="M128" s="2" t="inlineStr">
         <is>
-          <t>5080</t>
+          <t>5132</t>
         </is>
       </c>
       <c r="N128" s="2" t="inlineStr">
@@ -30747,12 +30462,12 @@
       </c>
       <c r="O128" s="2" t="inlineStr">
         <is>
-          <t>0.35</t>
+          <t>0.07</t>
         </is>
       </c>
       <c r="P128" s="2" t="inlineStr">
         <is>
-          <t>1000.0</t>
+          <t>10000000.0</t>
         </is>
       </c>
       <c r="Q128" s="2" t="inlineStr">
@@ -30767,7 +30482,7 @@
       </c>
       <c r="S128" s="2" t="inlineStr">
         <is>
-          <t>100.0</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="T128" s="2" t="inlineStr">
@@ -30807,7 +30522,7 @@
       </c>
       <c r="AA128" s="2" t="inlineStr">
         <is>
-          <t>GERAL</t>
+          <t>QUALIFICADO</t>
         </is>
       </c>
       <c r="AB128" s="2" t="inlineStr">
@@ -30855,7 +30570,7 @@
       </c>
       <c r="AM128" s="2" t="inlineStr">
         <is>
-          <t>CAIXA SAÚDE SUPLEMENTAR - ANS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
+          <t>CAIXA SAUDE SUPLEMENTAR - ANS II FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
         </is>
       </c>
       <c r="AN128" s="2" t="inlineStr">
@@ -30870,42 +30585,42 @@
       </c>
       <c r="AO128" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5080.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5132.pdf</t>
         </is>
       </c>
       <c r="AP128" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5080.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5132.pdf</t>
         </is>
       </c>
       <c r="AQ128" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5080.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5132.pdf</t>
         </is>
       </c>
       <c r="AR128" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5080.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5132.pdf</t>
         </is>
       </c>
       <c r="AS128" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5080.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5132.pdf</t>
         </is>
       </c>
       <c r="AT128" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5080.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5132.pdf</t>
         </is>
       </c>
       <c r="AU128" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5080.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5132.pdf</t>
         </is>
       </c>
       <c r="AV128" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/caixa-asset/sumario-remuneracao/Documents/sumarios/5080-SUMARIO.pdf</t>
+          <t>https://www.caixa.gov.br/caixa-asset/sumario-remuneracao/Documents/sumarios/5132-SUMARIO.pdf</t>
         </is>
       </c>
       <c r="AW128" s="2" t="inlineStr"/>
@@ -32136,7 +31851,7 @@
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>1,55554369</t>
+          <t>1,55554400</t>
         </is>
       </c>
       <c r="E134" s="3" t="inlineStr">
@@ -39007,32 +38722,32 @@
       </c>
       <c r="D164" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E164" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F164" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G164" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H164" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1.544,39933900</t>
+        </is>
+      </c>
+      <c r="E164" s="7" t="inlineStr">
+        <is>
+          <t>-0,228</t>
+        </is>
+      </c>
+      <c r="F164" s="7" t="inlineStr">
+        <is>
+          <t>-0,43</t>
+        </is>
+      </c>
+      <c r="G164" s="3" t="inlineStr">
+        <is>
+          <t>4,04</t>
+        </is>
+      </c>
+      <c r="H164" s="3" t="inlineStr">
+        <is>
+          <t>11,88</t>
         </is>
       </c>
       <c r="I164" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>129,780</t>
         </is>
       </c>
       <c r="J164" s="2" t="inlineStr">
@@ -39712,7 +39427,7 @@
       </c>
       <c r="D167" s="4" t="inlineStr">
         <is>
-          <t>11,29707516</t>
+          <t>11,29707500</t>
         </is>
       </c>
       <c r="E167" s="6" t="inlineStr">
@@ -40425,7 +40140,7 @@
       </c>
       <c r="D170" s="2" t="inlineStr">
         <is>
-          <t>3,37140494</t>
+          <t>3,37140500</t>
         </is>
       </c>
       <c r="E170" s="7" t="inlineStr">
@@ -40656,7 +40371,7 @@
       </c>
       <c r="D171" s="4" t="inlineStr">
         <is>
-          <t>2,43492074</t>
+          <t>2,43492100</t>
         </is>
       </c>
       <c r="E171" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Dados atualizados via Robô: 24/06/2026 15:52
</commit_message>
<xml_diff>
--- a/dados_atuais.xlsx
+++ b/dados_atuais.xlsx
@@ -3208,12 +3208,12 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>03.218.183/0001-04</t>
+          <t>03.191.874/0001-61</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>46</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -3223,27 +3223,27 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>0.3</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>0.01</t>
+          <t>100000.0</t>
         </is>
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>0.01</t>
+          <t>100.0</t>
         </is>
       </c>
       <c r="R12" s="2" t="inlineStr">
         <is>
-          <t>0.01</t>
+          <t>100.0</t>
         </is>
       </c>
       <c r="S12" s="2" t="inlineStr">
         <is>
-          <t>0.01</t>
+          <t>10000.0</t>
         </is>
       </c>
       <c r="T12" s="2" t="inlineStr">
@@ -3313,12 +3313,12 @@
       </c>
       <c r="AG12" s="2" t="inlineStr">
         <is>
-          <t>["Pessoa Física"]</t>
+          <t>["Institucional", "PJ Atacado"]</t>
         </is>
       </c>
       <c r="AH12" s="2" t="inlineStr">
         <is>
-          <t>["Pessoa Física"]</t>
+          <t>["Institucional", "PJ Atacado"]</t>
         </is>
       </c>
       <c r="AI12" s="2" t="inlineStr">
@@ -3339,7 +3339,7 @@
       </c>
       <c r="AM12" s="2" t="inlineStr">
         <is>
-          <t>CAIXA CAPITAL ÍNDICE DE PREÇOS FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESP LIMITADA</t>
+          <t>CAIXA PATRIMÔNIO ÍNDICE DE PREÇOS FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESP LIMITADA</t>
         </is>
       </c>
       <c r="AN12" s="2" t="inlineStr">
@@ -3349,47 +3349,47 @@
       </c>
       <c r="AO12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_0087.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_0046.pdf</t>
         </is>
       </c>
       <c r="AP12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_0087.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_0046.pdf</t>
         </is>
       </c>
       <c r="AQ12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_0087.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_0046.pdf</t>
         </is>
       </c>
       <c r="AR12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_87.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_46.pdf</t>
         </is>
       </c>
       <c r="AS12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_87.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_46.pdf</t>
         </is>
       </c>
       <c r="AT12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_87.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_46.pdf</t>
         </is>
       </c>
       <c r="AU12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_0087.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_0046.pdf</t>
         </is>
       </c>
       <c r="AV12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/caixa-asset/sumario-remuneracao/Documents/sumarios/0087-SUMARIO.pdf</t>
+          <t>https://www.caixa.gov.br/caixa-asset/sumario-remuneracao/Documents/sumarios/0046-SUMARIO.pdf</t>
         </is>
       </c>
       <c r="AW12" s="2" t="inlineStr">
         <is>
-          <t>https://web.microsoftstream.com/video/32d65536-1de1-4f2f-a9b8-0fbb0d9347fc?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
+          <t>https://web.microsoftstream.com/video/140b7682-00df-491d-b451-73ae70a040fa?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
     </row>
@@ -37780,12 +37780,12 @@
       </c>
       <c r="L158" s="2" t="inlineStr">
         <is>
-          <t>03.737.206/0001-97</t>
+          <t>05.164.356/0001-84</t>
         </is>
       </c>
       <c r="M158" s="2" t="inlineStr">
         <is>
-          <t>5404</t>
+          <t>5462</t>
         </is>
       </c>
       <c r="N158" s="2" t="inlineStr">
@@ -37840,7 +37840,7 @@
       </c>
       <c r="X158" s="2" t="inlineStr">
         <is>
-          <t>RF DI até 49% Crédito Privado</t>
+          <t>RF 100% TPF - Longo Prazo</t>
         </is>
       </c>
       <c r="Y158" s="2" t="inlineStr">
@@ -37911,58 +37911,57 @@
       </c>
       <c r="AM158" s="2" t="inlineStr">
         <is>
-          <t>CAIXA BRASIL FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA REFERENCIADO DI LONGO PRAZO - RESP LIMITADA</t>
+          <t>CAIXA BRASIL TÍTULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
         </is>
       </c>
       <c r="AN158" s="2" t="inlineStr">
         <is>
-          <t>1. Para aplicação por meio de conta operação 003, é necessário o cadastramento prévio de cotistas, conforme descrito no item Adesão, do FI612.
-2. O procedimento de inclusão da conta deverá ser realizado sempre que houver qualquer aplicação por meio de conta operação 003, mesmo para os clientes que já realizaram o cadastramento anteriormente.</t>
+          <t>Para aplicação no fundo é necessário o cadastramento prévio de cotistas, conforme descrito no FI657. O procedimento de inclusão da conta deverá ser realizado sempre que houver qualquer aplicação, mesmo para os clientes que já realizaram o cadsatramento anteriormente.</t>
         </is>
       </c>
       <c r="AO158" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5404.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5462.pdf</t>
         </is>
       </c>
       <c r="AP158" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5404.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5462.pdf</t>
         </is>
       </c>
       <c r="AQ158" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5404.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5462.pdf</t>
         </is>
       </c>
       <c r="AR158" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5404.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5462.pdf</t>
         </is>
       </c>
       <c r="AS158" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5404.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5462.pdf</t>
         </is>
       </c>
       <c r="AT158" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5404.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5462.pdf</t>
         </is>
       </c>
       <c r="AU158" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5404.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5462.pdf</t>
         </is>
       </c>
       <c r="AV158" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/caixa-asset/sumario-remuneracao/Documents/sumarios/5404-SUMARIO.pdf</t>
+          <t>https://www.caixa.gov.br/caixa-asset/sumario-remuneracao/Documents/sumarios/5462-SUMARIO.pdf</t>
         </is>
       </c>
       <c r="AW158" s="2" t="inlineStr">
         <is>
-          <t>https://web.microsoftstream.com/video/f88f1fc7-aac3-44df-a2a5-ce3ac05edfb3?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
+          <t>https://web.microsoftstream.com/video/91aaf70b-85c2-4cf1-b537-e42b3bd894ec?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dados atualizados via Robô: 07/07/2026 16:12
</commit_message>
<xml_diff>
--- a/dados_atuais.xlsx
+++ b/dados_atuais.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW172"/>
+  <dimension ref="A1:BB172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -517,6 +517,11 @@
     <col width="15" customWidth="1" min="47" max="47"/>
     <col width="15" customWidth="1" min="48" max="48"/>
     <col width="15" customWidth="1" min="49" max="49"/>
+    <col width="15" customWidth="1" min="50" max="50"/>
+    <col width="15" customWidth="1" min="51" max="51"/>
+    <col width="15" customWidth="1" min="52" max="52"/>
+    <col width="15" customWidth="1" min="53" max="53"/>
+    <col width="15" customWidth="1" min="54" max="54"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -763,6 +768,31 @@
       <c r="AW1" s="1" t="inlineStr">
         <is>
           <t>doc_raio_x</t>
+        </is>
+      </c>
+      <c r="AX1" s="1" t="inlineStr">
+        <is>
+          <t>Data Base Consulta</t>
+        </is>
+      </c>
+      <c r="AY1" s="1" t="inlineStr">
+        <is>
+          <t>Data Rentabilidade Ref</t>
+        </is>
+      </c>
+      <c r="AZ1" s="1" t="inlineStr">
+        <is>
+          <t>Fallback Rentabilidade</t>
+        </is>
+      </c>
+      <c r="BA1" s="1" t="inlineStr">
+        <is>
+          <t>Dias Úteis Fallback</t>
+        </is>
+      </c>
+      <c r="BB1" s="1" t="inlineStr">
+        <is>
+          <t>Alerta Rentabilidade Defasada</t>
         </is>
       </c>
     </row>
@@ -1000,6 +1030,11 @@
       </c>
       <c r="AV2" s="2" t="inlineStr"/>
       <c r="AW2" s="2" t="inlineStr"/>
+      <c r="AX2" s="2" t="inlineStr"/>
+      <c r="AY2" s="2" t="inlineStr"/>
+      <c r="AZ2" s="2" t="inlineStr"/>
+      <c r="BA2" s="2" t="inlineStr"/>
+      <c r="BB2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -1235,6 +1270,11 @@
       </c>
       <c r="AV3" s="4" t="inlineStr"/>
       <c r="AW3" s="4" t="inlineStr"/>
+      <c r="AX3" s="4" t="inlineStr"/>
+      <c r="AY3" s="4" t="inlineStr"/>
+      <c r="AZ3" s="4" t="inlineStr"/>
+      <c r="BA3" s="4" t="inlineStr"/>
+      <c r="BB3" s="4" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1469,6 +1509,11 @@
       </c>
       <c r="AV4" s="2" t="inlineStr"/>
       <c r="AW4" s="2" t="inlineStr"/>
+      <c r="AX4" s="2" t="inlineStr"/>
+      <c r="AY4" s="2" t="inlineStr"/>
+      <c r="AZ4" s="2" t="inlineStr"/>
+      <c r="BA4" s="2" t="inlineStr"/>
+      <c r="BB4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -1704,6 +1749,11 @@
       </c>
       <c r="AV5" s="4" t="inlineStr"/>
       <c r="AW5" s="4" t="inlineStr"/>
+      <c r="AX5" s="4" t="inlineStr"/>
+      <c r="AY5" s="4" t="inlineStr"/>
+      <c r="AZ5" s="4" t="inlineStr"/>
+      <c r="BA5" s="4" t="inlineStr"/>
+      <c r="BB5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1942,6 +1992,11 @@
       </c>
       <c r="AV6" s="2" t="inlineStr"/>
       <c r="AW6" s="2" t="inlineStr"/>
+      <c r="AX6" s="2" t="inlineStr"/>
+      <c r="AY6" s="2" t="inlineStr"/>
+      <c r="AZ6" s="2" t="inlineStr"/>
+      <c r="BA6" s="2" t="inlineStr"/>
+      <c r="BB6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -2173,6 +2228,11 @@
       </c>
       <c r="AV7" s="4" t="inlineStr"/>
       <c r="AW7" s="4" t="inlineStr"/>
+      <c r="AX7" s="4" t="inlineStr"/>
+      <c r="AY7" s="4" t="inlineStr"/>
+      <c r="AZ7" s="4" t="inlineStr"/>
+      <c r="BA7" s="4" t="inlineStr"/>
+      <c r="BB7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2408,6 +2468,11 @@
       </c>
       <c r="AV8" s="2" t="inlineStr"/>
       <c r="AW8" s="2" t="inlineStr"/>
+      <c r="AX8" s="2" t="inlineStr"/>
+      <c r="AY8" s="2" t="inlineStr"/>
+      <c r="AZ8" s="2" t="inlineStr"/>
+      <c r="BA8" s="2" t="inlineStr"/>
+      <c r="BB8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -2639,6 +2704,11 @@
       </c>
       <c r="AV9" s="4" t="inlineStr"/>
       <c r="AW9" s="4" t="inlineStr"/>
+      <c r="AX9" s="4" t="inlineStr"/>
+      <c r="AY9" s="4" t="inlineStr"/>
+      <c r="AZ9" s="4" t="inlineStr"/>
+      <c r="BA9" s="4" t="inlineStr"/>
+      <c r="BB9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2870,6 +2940,11 @@
       </c>
       <c r="AV10" s="2" t="inlineStr"/>
       <c r="AW10" s="2" t="inlineStr"/>
+      <c r="AX10" s="2" t="inlineStr"/>
+      <c r="AY10" s="2" t="inlineStr"/>
+      <c r="AZ10" s="2" t="inlineStr"/>
+      <c r="BA10" s="2" t="inlineStr"/>
+      <c r="BB10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -3109,6 +3184,11 @@
           <t>https://web.microsoftstream.com/video/cec16660-0485-4e14-9a79-ff7c9fd2158f?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
+      <c r="AX11" s="4" t="inlineStr"/>
+      <c r="AY11" s="4" t="inlineStr"/>
+      <c r="AZ11" s="4" t="inlineStr"/>
+      <c r="BA11" s="4" t="inlineStr"/>
+      <c r="BB11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -3348,6 +3428,11 @@
           <t>https://web.microsoftstream.com/video/140b7682-00df-491d-b451-73ae70a040fa?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
+      <c r="AX12" s="2" t="inlineStr"/>
+      <c r="AY12" s="2" t="inlineStr"/>
+      <c r="AZ12" s="2" t="inlineStr"/>
+      <c r="BA12" s="2" t="inlineStr"/>
+      <c r="BB12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -3584,6 +3669,11 @@
       </c>
       <c r="AV13" s="4" t="inlineStr"/>
       <c r="AW13" s="4" t="inlineStr"/>
+      <c r="AX13" s="4" t="inlineStr"/>
+      <c r="AY13" s="4" t="inlineStr"/>
+      <c r="AZ13" s="4" t="inlineStr"/>
+      <c r="BA13" s="4" t="inlineStr"/>
+      <c r="BB13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -3819,6 +3909,11 @@
       </c>
       <c r="AV14" s="2" t="inlineStr"/>
       <c r="AW14" s="2" t="inlineStr"/>
+      <c r="AX14" s="2" t="inlineStr"/>
+      <c r="AY14" s="2" t="inlineStr"/>
+      <c r="AZ14" s="2" t="inlineStr"/>
+      <c r="BA14" s="2" t="inlineStr"/>
+      <c r="BB14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -4058,6 +4153,11 @@
           <t>https://web.microsoftstream.com/video/a5ab94de-1f04-4f00-87d2-ffa0c6babbaf?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
+      <c r="AX15" s="4" t="inlineStr"/>
+      <c r="AY15" s="4" t="inlineStr"/>
+      <c r="AZ15" s="4" t="inlineStr"/>
+      <c r="BA15" s="4" t="inlineStr"/>
+      <c r="BB15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -4293,6 +4393,11 @@
       </c>
       <c r="AV16" s="2" t="inlineStr"/>
       <c r="AW16" s="2" t="inlineStr"/>
+      <c r="AX16" s="2" t="inlineStr"/>
+      <c r="AY16" s="2" t="inlineStr"/>
+      <c r="AZ16" s="2" t="inlineStr"/>
+      <c r="BA16" s="2" t="inlineStr"/>
+      <c r="BB16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -4524,6 +4629,11 @@
       </c>
       <c r="AV17" s="4" t="inlineStr"/>
       <c r="AW17" s="4" t="inlineStr"/>
+      <c r="AX17" s="4" t="inlineStr"/>
+      <c r="AY17" s="4" t="inlineStr"/>
+      <c r="AZ17" s="4" t="inlineStr"/>
+      <c r="BA17" s="4" t="inlineStr"/>
+      <c r="BB17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -4763,6 +4873,11 @@
           <t>https://web.microsoftstream.com/video/2fc898a1-d287-4c38-9f3a-9efa66e9bf47?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
+      <c r="AX18" s="2" t="inlineStr"/>
+      <c r="AY18" s="2" t="inlineStr"/>
+      <c r="AZ18" s="2" t="inlineStr"/>
+      <c r="BA18" s="2" t="inlineStr"/>
+      <c r="BB18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -4992,6 +5107,11 @@
       </c>
       <c r="AV19" s="4" t="inlineStr"/>
       <c r="AW19" s="4" t="inlineStr"/>
+      <c r="AX19" s="4" t="inlineStr"/>
+      <c r="AY19" s="4" t="inlineStr"/>
+      <c r="AZ19" s="4" t="inlineStr"/>
+      <c r="BA19" s="4" t="inlineStr"/>
+      <c r="BB19" s="4" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -5227,6 +5347,11 @@
       </c>
       <c r="AV20" s="2" t="inlineStr"/>
       <c r="AW20" s="2" t="inlineStr"/>
+      <c r="AX20" s="2" t="inlineStr"/>
+      <c r="AY20" s="2" t="inlineStr"/>
+      <c r="AZ20" s="2" t="inlineStr"/>
+      <c r="BA20" s="2" t="inlineStr"/>
+      <c r="BB20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -5467,6 +5592,11 @@
       </c>
       <c r="AV21" s="4" t="inlineStr"/>
       <c r="AW21" s="4" t="inlineStr"/>
+      <c r="AX21" s="4" t="inlineStr"/>
+      <c r="AY21" s="4" t="inlineStr"/>
+      <c r="AZ21" s="4" t="inlineStr"/>
+      <c r="BA21" s="4" t="inlineStr"/>
+      <c r="BB21" s="4" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -5702,6 +5832,11 @@
       </c>
       <c r="AV22" s="2" t="inlineStr"/>
       <c r="AW22" s="2" t="inlineStr"/>
+      <c r="AX22" s="2" t="inlineStr"/>
+      <c r="AY22" s="2" t="inlineStr"/>
+      <c r="AZ22" s="2" t="inlineStr"/>
+      <c r="BA22" s="2" t="inlineStr"/>
+      <c r="BB22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -5937,6 +6072,11 @@
       </c>
       <c r="AV23" s="4" t="inlineStr"/>
       <c r="AW23" s="4" t="inlineStr"/>
+      <c r="AX23" s="4" t="inlineStr"/>
+      <c r="AY23" s="4" t="inlineStr"/>
+      <c r="AZ23" s="4" t="inlineStr"/>
+      <c r="BA23" s="4" t="inlineStr"/>
+      <c r="BB23" s="4" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -6168,6 +6308,11 @@
       </c>
       <c r="AV24" s="2" t="inlineStr"/>
       <c r="AW24" s="2" t="inlineStr"/>
+      <c r="AX24" s="2" t="inlineStr"/>
+      <c r="AY24" s="2" t="inlineStr"/>
+      <c r="AZ24" s="2" t="inlineStr"/>
+      <c r="BA24" s="2" t="inlineStr"/>
+      <c r="BB24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -6403,6 +6548,11 @@
       </c>
       <c r="AV25" s="4" t="inlineStr"/>
       <c r="AW25" s="4" t="inlineStr"/>
+      <c r="AX25" s="4" t="inlineStr"/>
+      <c r="AY25" s="4" t="inlineStr"/>
+      <c r="AZ25" s="4" t="inlineStr"/>
+      <c r="BA25" s="4" t="inlineStr"/>
+      <c r="BB25" s="4" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -6638,6 +6788,11 @@
       </c>
       <c r="AV26" s="2" t="inlineStr"/>
       <c r="AW26" s="2" t="inlineStr"/>
+      <c r="AX26" s="2" t="inlineStr"/>
+      <c r="AY26" s="2" t="inlineStr"/>
+      <c r="AZ26" s="2" t="inlineStr"/>
+      <c r="BA26" s="2" t="inlineStr"/>
+      <c r="BB26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -6873,6 +7028,11 @@
       </c>
       <c r="AV27" s="4" t="inlineStr"/>
       <c r="AW27" s="4" t="inlineStr"/>
+      <c r="AX27" s="4" t="inlineStr"/>
+      <c r="AY27" s="4" t="inlineStr"/>
+      <c r="AZ27" s="4" t="inlineStr"/>
+      <c r="BA27" s="4" t="inlineStr"/>
+      <c r="BB27" s="4" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -7096,6 +7256,11 @@
       </c>
       <c r="AV28" s="2" t="inlineStr"/>
       <c r="AW28" s="2" t="inlineStr"/>
+      <c r="AX28" s="2" t="inlineStr"/>
+      <c r="AY28" s="2" t="inlineStr"/>
+      <c r="AZ28" s="2" t="inlineStr"/>
+      <c r="BA28" s="2" t="inlineStr"/>
+      <c r="BB28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -7323,6 +7488,11 @@
           <t>https://caixa.sharepoint.com/:v:/t/O365GRP-GEICO/EeFPVsuRvYtKt6bMstsCLiUBtcBOAe5vK4jLZ_DjXA4drg?e=XxU8cb</t>
         </is>
       </c>
+      <c r="AX29" s="4" t="inlineStr"/>
+      <c r="AY29" s="4" t="inlineStr"/>
+      <c r="AZ29" s="4" t="inlineStr"/>
+      <c r="BA29" s="4" t="inlineStr"/>
+      <c r="BB29" s="4" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -7550,6 +7720,11 @@
       </c>
       <c r="AV30" s="2" t="inlineStr"/>
       <c r="AW30" s="2" t="inlineStr"/>
+      <c r="AX30" s="2" t="inlineStr"/>
+      <c r="AY30" s="2" t="inlineStr"/>
+      <c r="AZ30" s="2" t="inlineStr"/>
+      <c r="BA30" s="2" t="inlineStr"/>
+      <c r="BB30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -7773,6 +7948,11 @@
       </c>
       <c r="AV31" s="4" t="inlineStr"/>
       <c r="AW31" s="4" t="inlineStr"/>
+      <c r="AX31" s="4" t="inlineStr"/>
+      <c r="AY31" s="4" t="inlineStr"/>
+      <c r="AZ31" s="4" t="inlineStr"/>
+      <c r="BA31" s="4" t="inlineStr"/>
+      <c r="BB31" s="4" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -8008,6 +8188,11 @@
       </c>
       <c r="AV32" s="2" t="inlineStr"/>
       <c r="AW32" s="2" t="inlineStr"/>
+      <c r="AX32" s="2" t="inlineStr"/>
+      <c r="AY32" s="2" t="inlineStr"/>
+      <c r="AZ32" s="2" t="inlineStr"/>
+      <c r="BA32" s="2" t="inlineStr"/>
+      <c r="BB32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -8243,6 +8428,11 @@
       </c>
       <c r="AV33" s="4" t="inlineStr"/>
       <c r="AW33" s="4" t="inlineStr"/>
+      <c r="AX33" s="4" t="inlineStr"/>
+      <c r="AY33" s="4" t="inlineStr"/>
+      <c r="AZ33" s="4" t="inlineStr"/>
+      <c r="BA33" s="4" t="inlineStr"/>
+      <c r="BB33" s="4" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -8466,6 +8656,11 @@
       </c>
       <c r="AV34" s="2" t="inlineStr"/>
       <c r="AW34" s="2" t="inlineStr"/>
+      <c r="AX34" s="2" t="inlineStr"/>
+      <c r="AY34" s="2" t="inlineStr"/>
+      <c r="AZ34" s="2" t="inlineStr"/>
+      <c r="BA34" s="2" t="inlineStr"/>
+      <c r="BB34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -8697,6 +8892,11 @@
       </c>
       <c r="AV35" s="4" t="inlineStr"/>
       <c r="AW35" s="4" t="inlineStr"/>
+      <c r="AX35" s="4" t="inlineStr"/>
+      <c r="AY35" s="4" t="inlineStr"/>
+      <c r="AZ35" s="4" t="inlineStr"/>
+      <c r="BA35" s="4" t="inlineStr"/>
+      <c r="BB35" s="4" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -8928,6 +9128,11 @@
       </c>
       <c r="AV36" s="2" t="inlineStr"/>
       <c r="AW36" s="2" t="inlineStr"/>
+      <c r="AX36" s="2" t="inlineStr"/>
+      <c r="AY36" s="2" t="inlineStr"/>
+      <c r="AZ36" s="2" t="inlineStr"/>
+      <c r="BA36" s="2" t="inlineStr"/>
+      <c r="BB36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -9163,6 +9368,11 @@
       </c>
       <c r="AV37" s="4" t="inlineStr"/>
       <c r="AW37" s="4" t="inlineStr"/>
+      <c r="AX37" s="4" t="inlineStr"/>
+      <c r="AY37" s="4" t="inlineStr"/>
+      <c r="AZ37" s="4" t="inlineStr"/>
+      <c r="BA37" s="4" t="inlineStr"/>
+      <c r="BB37" s="4" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -9399,6 +9609,11 @@
       </c>
       <c r="AV38" s="2" t="inlineStr"/>
       <c r="AW38" s="2" t="inlineStr"/>
+      <c r="AX38" s="2" t="inlineStr"/>
+      <c r="AY38" s="2" t="inlineStr"/>
+      <c r="AZ38" s="2" t="inlineStr"/>
+      <c r="BA38" s="2" t="inlineStr"/>
+      <c r="BB38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
@@ -9634,6 +9849,11 @@
       </c>
       <c r="AV39" s="4" t="inlineStr"/>
       <c r="AW39" s="4" t="inlineStr"/>
+      <c r="AX39" s="4" t="inlineStr"/>
+      <c r="AY39" s="4" t="inlineStr"/>
+      <c r="AZ39" s="4" t="inlineStr"/>
+      <c r="BA39" s="4" t="inlineStr"/>
+      <c r="BB39" s="4" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -9869,6 +10089,11 @@
       </c>
       <c r="AV40" s="2" t="inlineStr"/>
       <c r="AW40" s="2" t="inlineStr"/>
+      <c r="AX40" s="2" t="inlineStr"/>
+      <c r="AY40" s="2" t="inlineStr"/>
+      <c r="AZ40" s="2" t="inlineStr"/>
+      <c r="BA40" s="2" t="inlineStr"/>
+      <c r="BB40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
@@ -10105,6 +10330,11 @@
       </c>
       <c r="AV41" s="4" t="inlineStr"/>
       <c r="AW41" s="4" t="inlineStr"/>
+      <c r="AX41" s="4" t="inlineStr"/>
+      <c r="AY41" s="4" t="inlineStr"/>
+      <c r="AZ41" s="4" t="inlineStr"/>
+      <c r="BA41" s="4" t="inlineStr"/>
+      <c r="BB41" s="4" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -10344,6 +10574,11 @@
           <t>https://web.microsoftstream.com/video/1689d147-ff5e-41df-9e77-e9270bae338b?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
+      <c r="AX42" s="2" t="inlineStr"/>
+      <c r="AY42" s="2" t="inlineStr"/>
+      <c r="AZ42" s="2" t="inlineStr"/>
+      <c r="BA42" s="2" t="inlineStr"/>
+      <c r="BB42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
@@ -10580,6 +10815,11 @@
       </c>
       <c r="AV43" s="4" t="inlineStr"/>
       <c r="AW43" s="4" t="inlineStr"/>
+      <c r="AX43" s="4" t="inlineStr"/>
+      <c r="AY43" s="4" t="inlineStr"/>
+      <c r="AZ43" s="4" t="inlineStr"/>
+      <c r="BA43" s="4" t="inlineStr"/>
+      <c r="BB43" s="4" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -10807,6 +11047,11 @@
       </c>
       <c r="AV44" s="2" t="inlineStr"/>
       <c r="AW44" s="2" t="inlineStr"/>
+      <c r="AX44" s="2" t="inlineStr"/>
+      <c r="AY44" s="2" t="inlineStr"/>
+      <c r="AZ44" s="2" t="inlineStr"/>
+      <c r="BA44" s="2" t="inlineStr"/>
+      <c r="BB44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
@@ -11046,6 +11291,11 @@
           <t>https://web.microsoftstream.com/video/f0b7478a-7800-4df0-8a43-0113c5248eec?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
+      <c r="AX45" s="4" t="inlineStr"/>
+      <c r="AY45" s="4" t="inlineStr"/>
+      <c r="AZ45" s="4" t="inlineStr"/>
+      <c r="BA45" s="4" t="inlineStr"/>
+      <c r="BB45" s="4" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -11281,6 +11531,11 @@
       </c>
       <c r="AV46" s="2" t="inlineStr"/>
       <c r="AW46" s="2" t="inlineStr"/>
+      <c r="AX46" s="2" t="inlineStr"/>
+      <c r="AY46" s="2" t="inlineStr"/>
+      <c r="AZ46" s="2" t="inlineStr"/>
+      <c r="BA46" s="2" t="inlineStr"/>
+      <c r="BB46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
@@ -11520,6 +11775,11 @@
           <t>https://web.microsoftstream.com/video/5f6afa60-a43f-403c-8879-e04a2d36c5fa?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
+      <c r="AX47" s="4" t="inlineStr"/>
+      <c r="AY47" s="4" t="inlineStr"/>
+      <c r="AZ47" s="4" t="inlineStr"/>
+      <c r="BA47" s="4" t="inlineStr"/>
+      <c r="BB47" s="4" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -11755,6 +12015,11 @@
       </c>
       <c r="AV48" s="2" t="inlineStr"/>
       <c r="AW48" s="2" t="inlineStr"/>
+      <c r="AX48" s="2" t="inlineStr"/>
+      <c r="AY48" s="2" t="inlineStr"/>
+      <c r="AZ48" s="2" t="inlineStr"/>
+      <c r="BA48" s="2" t="inlineStr"/>
+      <c r="BB48" s="2" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
@@ -11995,6 +12260,11 @@
           <t>https://web.microsoftstream.com/video/ee622bf6-774a-41bd-afd8-1775b6b730b9?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
+      <c r="AX49" s="4" t="inlineStr"/>
+      <c r="AY49" s="4" t="inlineStr"/>
+      <c r="AZ49" s="4" t="inlineStr"/>
+      <c r="BA49" s="4" t="inlineStr"/>
+      <c r="BB49" s="4" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -12230,6 +12500,11 @@
           <t>https://web.microsoftstream.com/video/4be15710-4acb-4afd-a959-c6ed0d090cac?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
+      <c r="AX50" s="2" t="inlineStr"/>
+      <c r="AY50" s="2" t="inlineStr"/>
+      <c r="AZ50" s="2" t="inlineStr"/>
+      <c r="BA50" s="2" t="inlineStr"/>
+      <c r="BB50" s="2" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
@@ -12469,6 +12744,11 @@
           <t>https://web.microsoftstream.com/video/3cd97374-bb4b-4204-bdef-48cfa0e370c8?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
+      <c r="AX51" s="4" t="inlineStr"/>
+      <c r="AY51" s="4" t="inlineStr"/>
+      <c r="AZ51" s="4" t="inlineStr"/>
+      <c r="BA51" s="4" t="inlineStr"/>
+      <c r="BB51" s="4" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -12704,6 +12984,11 @@
           <t>https://web.microsoftstream.com/video/6fd51e32-7197-4736-ab0d-031b75c372fd?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
+      <c r="AX52" s="2" t="inlineStr"/>
+      <c r="AY52" s="2" t="inlineStr"/>
+      <c r="AZ52" s="2" t="inlineStr"/>
+      <c r="BA52" s="2" t="inlineStr"/>
+      <c r="BB52" s="2" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
@@ -12939,6 +13224,11 @@
           <t>https://web.microsoftstream.com/video/5f0c9eff-f752-448b-8f0a-3e2fff710aa9?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
+      <c r="AX53" s="4" t="inlineStr"/>
+      <c r="AY53" s="4" t="inlineStr"/>
+      <c r="AZ53" s="4" t="inlineStr"/>
+      <c r="BA53" s="4" t="inlineStr"/>
+      <c r="BB53" s="4" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -13174,6 +13464,11 @@
       </c>
       <c r="AV54" s="2" t="inlineStr"/>
       <c r="AW54" s="2" t="inlineStr"/>
+      <c r="AX54" s="2" t="inlineStr"/>
+      <c r="AY54" s="2" t="inlineStr"/>
+      <c r="AZ54" s="2" t="inlineStr"/>
+      <c r="BA54" s="2" t="inlineStr"/>
+      <c r="BB54" s="2" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
@@ -13401,6 +13696,11 @@
       </c>
       <c r="AV55" s="4" t="inlineStr"/>
       <c r="AW55" s="4" t="inlineStr"/>
+      <c r="AX55" s="4" t="inlineStr"/>
+      <c r="AY55" s="4" t="inlineStr"/>
+      <c r="AZ55" s="4" t="inlineStr"/>
+      <c r="BA55" s="4" t="inlineStr"/>
+      <c r="BB55" s="4" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -13646,6 +13946,11 @@
           <t>https://web.microsoftstream.com/video/ca76c442-41bd-4e49-bf93-7c88dfc75f01?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
+      <c r="AX56" s="2" t="inlineStr"/>
+      <c r="AY56" s="2" t="inlineStr"/>
+      <c r="AZ56" s="2" t="inlineStr"/>
+      <c r="BA56" s="2" t="inlineStr"/>
+      <c r="BB56" s="2" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
@@ -13885,6 +14190,11 @@
           <t>https://web.microsoftstream.com/video/86aa0100-d5af-4db2-9f67-441255924e4e?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
+      <c r="AX57" s="4" t="inlineStr"/>
+      <c r="AY57" s="4" t="inlineStr"/>
+      <c r="AZ57" s="4" t="inlineStr"/>
+      <c r="BA57" s="4" t="inlineStr"/>
+      <c r="BB57" s="4" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -14116,6 +14426,11 @@
       </c>
       <c r="AV58" s="2" t="inlineStr"/>
       <c r="AW58" s="2" t="inlineStr"/>
+      <c r="AX58" s="2" t="inlineStr"/>
+      <c r="AY58" s="2" t="inlineStr"/>
+      <c r="AZ58" s="2" t="inlineStr"/>
+      <c r="BA58" s="2" t="inlineStr"/>
+      <c r="BB58" s="2" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
@@ -14347,6 +14662,11 @@
       </c>
       <c r="AV59" s="4" t="inlineStr"/>
       <c r="AW59" s="4" t="inlineStr"/>
+      <c r="AX59" s="4" t="inlineStr"/>
+      <c r="AY59" s="4" t="inlineStr"/>
+      <c r="AZ59" s="4" t="inlineStr"/>
+      <c r="BA59" s="4" t="inlineStr"/>
+      <c r="BB59" s="4" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -14574,6 +14894,11 @@
       </c>
       <c r="AV60" s="2" t="inlineStr"/>
       <c r="AW60" s="2" t="inlineStr"/>
+      <c r="AX60" s="2" t="inlineStr"/>
+      <c r="AY60" s="2" t="inlineStr"/>
+      <c r="AZ60" s="2" t="inlineStr"/>
+      <c r="BA60" s="2" t="inlineStr"/>
+      <c r="BB60" s="2" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
@@ -14805,6 +15130,11 @@
       </c>
       <c r="AV61" s="4" t="inlineStr"/>
       <c r="AW61" s="4" t="inlineStr"/>
+      <c r="AX61" s="4" t="inlineStr"/>
+      <c r="AY61" s="4" t="inlineStr"/>
+      <c r="AZ61" s="4" t="inlineStr"/>
+      <c r="BA61" s="4" t="inlineStr"/>
+      <c r="BB61" s="4" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -15036,6 +15366,11 @@
       </c>
       <c r="AV62" s="2" t="inlineStr"/>
       <c r="AW62" s="2" t="inlineStr"/>
+      <c r="AX62" s="2" t="inlineStr"/>
+      <c r="AY62" s="2" t="inlineStr"/>
+      <c r="AZ62" s="2" t="inlineStr"/>
+      <c r="BA62" s="2" t="inlineStr"/>
+      <c r="BB62" s="2" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
@@ -15263,6 +15598,11 @@
       </c>
       <c r="AV63" s="4" t="inlineStr"/>
       <c r="AW63" s="4" t="inlineStr"/>
+      <c r="AX63" s="4" t="inlineStr"/>
+      <c r="AY63" s="4" t="inlineStr"/>
+      <c r="AZ63" s="4" t="inlineStr"/>
+      <c r="BA63" s="4" t="inlineStr"/>
+      <c r="BB63" s="4" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -15494,6 +15834,11 @@
       </c>
       <c r="AV64" s="2" t="inlineStr"/>
       <c r="AW64" s="2" t="inlineStr"/>
+      <c r="AX64" s="2" t="inlineStr"/>
+      <c r="AY64" s="2" t="inlineStr"/>
+      <c r="AZ64" s="2" t="inlineStr"/>
+      <c r="BA64" s="2" t="inlineStr"/>
+      <c r="BB64" s="2" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
@@ -15721,6 +16066,11 @@
       </c>
       <c r="AV65" s="4" t="inlineStr"/>
       <c r="AW65" s="4" t="inlineStr"/>
+      <c r="AX65" s="4" t="inlineStr"/>
+      <c r="AY65" s="4" t="inlineStr"/>
+      <c r="AZ65" s="4" t="inlineStr"/>
+      <c r="BA65" s="4" t="inlineStr"/>
+      <c r="BB65" s="4" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -15952,6 +16302,11 @@
       </c>
       <c r="AV66" s="2" t="inlineStr"/>
       <c r="AW66" s="2" t="inlineStr"/>
+      <c r="AX66" s="2" t="inlineStr"/>
+      <c r="AY66" s="2" t="inlineStr"/>
+      <c r="AZ66" s="2" t="inlineStr"/>
+      <c r="BA66" s="2" t="inlineStr"/>
+      <c r="BB66" s="2" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
@@ -16187,6 +16542,11 @@
       </c>
       <c r="AV67" s="4" t="inlineStr"/>
       <c r="AW67" s="4" t="inlineStr"/>
+      <c r="AX67" s="4" t="inlineStr"/>
+      <c r="AY67" s="4" t="inlineStr"/>
+      <c r="AZ67" s="4" t="inlineStr"/>
+      <c r="BA67" s="4" t="inlineStr"/>
+      <c r="BB67" s="4" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -16422,6 +16782,11 @@
       </c>
       <c r="AV68" s="2" t="inlineStr"/>
       <c r="AW68" s="2" t="inlineStr"/>
+      <c r="AX68" s="2" t="inlineStr"/>
+      <c r="AY68" s="2" t="inlineStr"/>
+      <c r="AZ68" s="2" t="inlineStr"/>
+      <c r="BA68" s="2" t="inlineStr"/>
+      <c r="BB68" s="2" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
@@ -16653,6 +17018,11 @@
       </c>
       <c r="AV69" s="4" t="inlineStr"/>
       <c r="AW69" s="4" t="inlineStr"/>
+      <c r="AX69" s="4" t="inlineStr"/>
+      <c r="AY69" s="4" t="inlineStr"/>
+      <c r="AZ69" s="4" t="inlineStr"/>
+      <c r="BA69" s="4" t="inlineStr"/>
+      <c r="BB69" s="4" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -16888,6 +17258,11 @@
       </c>
       <c r="AV70" s="2" t="inlineStr"/>
       <c r="AW70" s="2" t="inlineStr"/>
+      <c r="AX70" s="2" t="inlineStr"/>
+      <c r="AY70" s="2" t="inlineStr"/>
+      <c r="AZ70" s="2" t="inlineStr"/>
+      <c r="BA70" s="2" t="inlineStr"/>
+      <c r="BB70" s="2" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
@@ -17123,6 +17498,11 @@
           <t>https://web.microsoftstream.com/video/7ad96d1d-faee-497b-9eb5-c3093ebf417d?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
+      <c r="AX71" s="4" t="inlineStr"/>
+      <c r="AY71" s="4" t="inlineStr"/>
+      <c r="AZ71" s="4" t="inlineStr"/>
+      <c r="BA71" s="4" t="inlineStr"/>
+      <c r="BB71" s="4" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -17358,6 +17738,11 @@
       </c>
       <c r="AV72" s="2" t="inlineStr"/>
       <c r="AW72" s="2" t="inlineStr"/>
+      <c r="AX72" s="2" t="inlineStr"/>
+      <c r="AY72" s="2" t="inlineStr"/>
+      <c r="AZ72" s="2" t="inlineStr"/>
+      <c r="BA72" s="2" t="inlineStr"/>
+      <c r="BB72" s="2" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
@@ -17581,6 +17966,11 @@
       </c>
       <c r="AV73" s="4" t="inlineStr"/>
       <c r="AW73" s="4" t="inlineStr"/>
+      <c r="AX73" s="4" t="inlineStr"/>
+      <c r="AY73" s="4" t="inlineStr"/>
+      <c r="AZ73" s="4" t="inlineStr"/>
+      <c r="BA73" s="4" t="inlineStr"/>
+      <c r="BB73" s="4" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -17823,6 +18213,11 @@
       </c>
       <c r="AV74" s="2" t="inlineStr"/>
       <c r="AW74" s="2" t="inlineStr"/>
+      <c r="AX74" s="2" t="inlineStr"/>
+      <c r="AY74" s="2" t="inlineStr"/>
+      <c r="AZ74" s="2" t="inlineStr"/>
+      <c r="BA74" s="2" t="inlineStr"/>
+      <c r="BB74" s="2" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
@@ -18064,6 +18459,11 @@
       </c>
       <c r="AV75" s="4" t="inlineStr"/>
       <c r="AW75" s="4" t="inlineStr"/>
+      <c r="AX75" s="4" t="inlineStr"/>
+      <c r="AY75" s="4" t="inlineStr"/>
+      <c r="AZ75" s="4" t="inlineStr"/>
+      <c r="BA75" s="4" t="inlineStr"/>
+      <c r="BB75" s="4" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -18305,6 +18705,11 @@
       </c>
       <c r="AV76" s="2" t="inlineStr"/>
       <c r="AW76" s="2" t="inlineStr"/>
+      <c r="AX76" s="2" t="inlineStr"/>
+      <c r="AY76" s="2" t="inlineStr"/>
+      <c r="AZ76" s="2" t="inlineStr"/>
+      <c r="BA76" s="2" t="inlineStr"/>
+      <c r="BB76" s="2" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
@@ -18548,6 +18953,11 @@
       </c>
       <c r="AV77" s="4" t="inlineStr"/>
       <c r="AW77" s="4" t="inlineStr"/>
+      <c r="AX77" s="4" t="inlineStr"/>
+      <c r="AY77" s="4" t="inlineStr"/>
+      <c r="AZ77" s="4" t="inlineStr"/>
+      <c r="BA77" s="4" t="inlineStr"/>
+      <c r="BB77" s="4" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -18602,7 +19012,7 @@
       </c>
       <c r="K78" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-capital-protegido-ciclico-ii-multimercado-lp/Paginas/default.aspx</t>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/caixa-fic-fim-cap-protegido-ciclico-ii</t>
         </is>
       </c>
       <c r="L78" s="2" t="inlineStr">
@@ -18791,6 +19201,11 @@
       </c>
       <c r="AV78" s="2" t="inlineStr"/>
       <c r="AW78" s="2" t="inlineStr"/>
+      <c r="AX78" s="2" t="inlineStr"/>
+      <c r="AY78" s="2" t="inlineStr"/>
+      <c r="AZ78" s="2" t="inlineStr"/>
+      <c r="BA78" s="2" t="inlineStr"/>
+      <c r="BB78" s="2" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
@@ -19022,6 +19437,11 @@
       </c>
       <c r="AV79" s="4" t="inlineStr"/>
       <c r="AW79" s="4" t="inlineStr"/>
+      <c r="AX79" s="4" t="inlineStr"/>
+      <c r="AY79" s="4" t="inlineStr"/>
+      <c r="AZ79" s="4" t="inlineStr"/>
+      <c r="BA79" s="4" t="inlineStr"/>
+      <c r="BB79" s="4" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -19257,6 +19677,11 @@
           <t>https://web.microsoftstream.com/video/2cbfedbd-9ece-40fb-9cc2-7d866c3c427e?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
+      <c r="AX80" s="2" t="inlineStr"/>
+      <c r="AY80" s="2" t="inlineStr"/>
+      <c r="AZ80" s="2" t="inlineStr"/>
+      <c r="BA80" s="2" t="inlineStr"/>
+      <c r="BB80" s="2" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
@@ -19488,6 +19913,11 @@
       </c>
       <c r="AV81" s="4" t="inlineStr"/>
       <c r="AW81" s="4" t="inlineStr"/>
+      <c r="AX81" s="4" t="inlineStr"/>
+      <c r="AY81" s="4" t="inlineStr"/>
+      <c r="AZ81" s="4" t="inlineStr"/>
+      <c r="BA81" s="4" t="inlineStr"/>
+      <c r="BB81" s="4" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -19719,6 +20149,11 @@
       </c>
       <c r="AV82" s="2" t="inlineStr"/>
       <c r="AW82" s="2" t="inlineStr"/>
+      <c r="AX82" s="2" t="inlineStr"/>
+      <c r="AY82" s="2" t="inlineStr"/>
+      <c r="AZ82" s="2" t="inlineStr"/>
+      <c r="BA82" s="2" t="inlineStr"/>
+      <c r="BB82" s="2" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
@@ -19955,6 +20390,11 @@
       </c>
       <c r="AV83" s="4" t="inlineStr"/>
       <c r="AW83" s="4" t="inlineStr"/>
+      <c r="AX83" s="4" t="inlineStr"/>
+      <c r="AY83" s="4" t="inlineStr"/>
+      <c r="AZ83" s="4" t="inlineStr"/>
+      <c r="BA83" s="4" t="inlineStr"/>
+      <c r="BB83" s="4" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -20190,6 +20630,11 @@
       </c>
       <c r="AV84" s="2" t="inlineStr"/>
       <c r="AW84" s="2" t="inlineStr"/>
+      <c r="AX84" s="2" t="inlineStr"/>
+      <c r="AY84" s="2" t="inlineStr"/>
+      <c r="AZ84" s="2" t="inlineStr"/>
+      <c r="BA84" s="2" t="inlineStr"/>
+      <c r="BB84" s="2" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
@@ -20425,6 +20870,11 @@
       </c>
       <c r="AV85" s="4" t="inlineStr"/>
       <c r="AW85" s="4" t="inlineStr"/>
+      <c r="AX85" s="4" t="inlineStr"/>
+      <c r="AY85" s="4" t="inlineStr"/>
+      <c r="AZ85" s="4" t="inlineStr"/>
+      <c r="BA85" s="4" t="inlineStr"/>
+      <c r="BB85" s="4" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -20660,6 +21110,11 @@
       </c>
       <c r="AV86" s="2" t="inlineStr"/>
       <c r="AW86" s="2" t="inlineStr"/>
+      <c r="AX86" s="2" t="inlineStr"/>
+      <c r="AY86" s="2" t="inlineStr"/>
+      <c r="AZ86" s="2" t="inlineStr"/>
+      <c r="BA86" s="2" t="inlineStr"/>
+      <c r="BB86" s="2" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
@@ -20895,6 +21350,11 @@
       </c>
       <c r="AV87" s="4" t="inlineStr"/>
       <c r="AW87" s="4" t="inlineStr"/>
+      <c r="AX87" s="4" t="inlineStr"/>
+      <c r="AY87" s="4" t="inlineStr"/>
+      <c r="AZ87" s="4" t="inlineStr"/>
+      <c r="BA87" s="4" t="inlineStr"/>
+      <c r="BB87" s="4" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -21119,6 +21579,11 @@
       </c>
       <c r="AV88" s="2" t="inlineStr"/>
       <c r="AW88" s="2" t="inlineStr"/>
+      <c r="AX88" s="2" t="inlineStr"/>
+      <c r="AY88" s="2" t="inlineStr"/>
+      <c r="AZ88" s="2" t="inlineStr"/>
+      <c r="BA88" s="2" t="inlineStr"/>
+      <c r="BB88" s="2" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
@@ -21354,6 +21819,11 @@
       </c>
       <c r="AV89" s="4" t="inlineStr"/>
       <c r="AW89" s="4" t="inlineStr"/>
+      <c r="AX89" s="4" t="inlineStr"/>
+      <c r="AY89" s="4" t="inlineStr"/>
+      <c r="AZ89" s="4" t="inlineStr"/>
+      <c r="BA89" s="4" t="inlineStr"/>
+      <c r="BB89" s="4" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -21589,6 +22059,11 @@
       </c>
       <c r="AV90" s="2" t="inlineStr"/>
       <c r="AW90" s="2" t="inlineStr"/>
+      <c r="AX90" s="2" t="inlineStr"/>
+      <c r="AY90" s="2" t="inlineStr"/>
+      <c r="AZ90" s="2" t="inlineStr"/>
+      <c r="BA90" s="2" t="inlineStr"/>
+      <c r="BB90" s="2" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
@@ -21824,6 +22299,11 @@
       </c>
       <c r="AV91" s="4" t="inlineStr"/>
       <c r="AW91" s="4" t="inlineStr"/>
+      <c r="AX91" s="4" t="inlineStr"/>
+      <c r="AY91" s="4" t="inlineStr"/>
+      <c r="AZ91" s="4" t="inlineStr"/>
+      <c r="BA91" s="4" t="inlineStr"/>
+      <c r="BB91" s="4" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -22059,6 +22539,11 @@
       </c>
       <c r="AV92" s="2" t="inlineStr"/>
       <c r="AW92" s="2" t="inlineStr"/>
+      <c r="AX92" s="2" t="inlineStr"/>
+      <c r="AY92" s="2" t="inlineStr"/>
+      <c r="AZ92" s="2" t="inlineStr"/>
+      <c r="BA92" s="2" t="inlineStr"/>
+      <c r="BB92" s="2" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
@@ -22294,6 +22779,11 @@
       </c>
       <c r="AV93" s="4" t="inlineStr"/>
       <c r="AW93" s="4" t="inlineStr"/>
+      <c r="AX93" s="4" t="inlineStr"/>
+      <c r="AY93" s="4" t="inlineStr"/>
+      <c r="AZ93" s="4" t="inlineStr"/>
+      <c r="BA93" s="4" t="inlineStr"/>
+      <c r="BB93" s="4" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -22529,6 +23019,11 @@
       </c>
       <c r="AV94" s="2" t="inlineStr"/>
       <c r="AW94" s="2" t="inlineStr"/>
+      <c r="AX94" s="2" t="inlineStr"/>
+      <c r="AY94" s="2" t="inlineStr"/>
+      <c r="AZ94" s="2" t="inlineStr"/>
+      <c r="BA94" s="2" t="inlineStr"/>
+      <c r="BB94" s="2" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
@@ -22764,6 +23259,11 @@
       </c>
       <c r="AV95" s="4" t="inlineStr"/>
       <c r="AW95" s="4" t="inlineStr"/>
+      <c r="AX95" s="4" t="inlineStr"/>
+      <c r="AY95" s="4" t="inlineStr"/>
+      <c r="AZ95" s="4" t="inlineStr"/>
+      <c r="BA95" s="4" t="inlineStr"/>
+      <c r="BB95" s="4" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -22999,6 +23499,11 @@
       </c>
       <c r="AV96" s="2" t="inlineStr"/>
       <c r="AW96" s="2" t="inlineStr"/>
+      <c r="AX96" s="2" t="inlineStr"/>
+      <c r="AY96" s="2" t="inlineStr"/>
+      <c r="AZ96" s="2" t="inlineStr"/>
+      <c r="BA96" s="2" t="inlineStr"/>
+      <c r="BB96" s="2" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
@@ -23234,6 +23739,11 @@
       </c>
       <c r="AV97" s="4" t="inlineStr"/>
       <c r="AW97" s="4" t="inlineStr"/>
+      <c r="AX97" s="4" t="inlineStr"/>
+      <c r="AY97" s="4" t="inlineStr"/>
+      <c r="AZ97" s="4" t="inlineStr"/>
+      <c r="BA97" s="4" t="inlineStr"/>
+      <c r="BB97" s="4" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -23473,6 +23983,11 @@
           <t>https://web.microsoftstream.com/video/c97500d6-f87e-4c24-a7f6-50fa0a703f14?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
+      <c r="AX98" s="2" t="inlineStr"/>
+      <c r="AY98" s="2" t="inlineStr"/>
+      <c r="AZ98" s="2" t="inlineStr"/>
+      <c r="BA98" s="2" t="inlineStr"/>
+      <c r="BB98" s="2" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
@@ -23708,6 +24223,11 @@
       </c>
       <c r="AV99" s="4" t="inlineStr"/>
       <c r="AW99" s="4" t="inlineStr"/>
+      <c r="AX99" s="4" t="inlineStr"/>
+      <c r="AY99" s="4" t="inlineStr"/>
+      <c r="AZ99" s="4" t="inlineStr"/>
+      <c r="BA99" s="4" t="inlineStr"/>
+      <c r="BB99" s="4" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -23943,6 +24463,11 @@
       </c>
       <c r="AV100" s="2" t="inlineStr"/>
       <c r="AW100" s="2" t="inlineStr"/>
+      <c r="AX100" s="2" t="inlineStr"/>
+      <c r="AY100" s="2" t="inlineStr"/>
+      <c r="AZ100" s="2" t="inlineStr"/>
+      <c r="BA100" s="2" t="inlineStr"/>
+      <c r="BB100" s="2" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
@@ -24178,6 +24703,11 @@
       </c>
       <c r="AV101" s="4" t="inlineStr"/>
       <c r="AW101" s="4" t="inlineStr"/>
+      <c r="AX101" s="4" t="inlineStr"/>
+      <c r="AY101" s="4" t="inlineStr"/>
+      <c r="AZ101" s="4" t="inlineStr"/>
+      <c r="BA101" s="4" t="inlineStr"/>
+      <c r="BB101" s="4" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -24417,6 +24947,11 @@
       </c>
       <c r="AV102" s="2" t="inlineStr"/>
       <c r="AW102" s="2" t="inlineStr"/>
+      <c r="AX102" s="2" t="inlineStr"/>
+      <c r="AY102" s="2" t="inlineStr"/>
+      <c r="AZ102" s="2" t="inlineStr"/>
+      <c r="BA102" s="2" t="inlineStr"/>
+      <c r="BB102" s="2" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
@@ -24652,6 +25187,11 @@
       </c>
       <c r="AV103" s="4" t="inlineStr"/>
       <c r="AW103" s="4" t="inlineStr"/>
+      <c r="AX103" s="4" t="inlineStr"/>
+      <c r="AY103" s="4" t="inlineStr"/>
+      <c r="AZ103" s="4" t="inlineStr"/>
+      <c r="BA103" s="4" t="inlineStr"/>
+      <c r="BB103" s="4" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -24887,6 +25427,11 @@
       </c>
       <c r="AV104" s="2" t="inlineStr"/>
       <c r="AW104" s="2" t="inlineStr"/>
+      <c r="AX104" s="2" t="inlineStr"/>
+      <c r="AY104" s="2" t="inlineStr"/>
+      <c r="AZ104" s="2" t="inlineStr"/>
+      <c r="BA104" s="2" t="inlineStr"/>
+      <c r="BB104" s="2" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
@@ -25114,6 +25659,11 @@
       </c>
       <c r="AV105" s="4" t="inlineStr"/>
       <c r="AW105" s="4" t="inlineStr"/>
+      <c r="AX105" s="4" t="inlineStr"/>
+      <c r="AY105" s="4" t="inlineStr"/>
+      <c r="AZ105" s="4" t="inlineStr"/>
+      <c r="BA105" s="4" t="inlineStr"/>
+      <c r="BB105" s="4" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -25341,6 +25891,11 @@
       </c>
       <c r="AV106" s="2" t="inlineStr"/>
       <c r="AW106" s="2" t="inlineStr"/>
+      <c r="AX106" s="2" t="inlineStr"/>
+      <c r="AY106" s="2" t="inlineStr"/>
+      <c r="AZ106" s="2" t="inlineStr"/>
+      <c r="BA106" s="2" t="inlineStr"/>
+      <c r="BB106" s="2" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="4" t="inlineStr">
@@ -25576,6 +26131,11 @@
       </c>
       <c r="AV107" s="4" t="inlineStr"/>
       <c r="AW107" s="4" t="inlineStr"/>
+      <c r="AX107" s="4" t="inlineStr"/>
+      <c r="AY107" s="4" t="inlineStr"/>
+      <c r="AZ107" s="4" t="inlineStr"/>
+      <c r="BA107" s="4" t="inlineStr"/>
+      <c r="BB107" s="4" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -25811,6 +26371,11 @@
       </c>
       <c r="AV108" s="2" t="inlineStr"/>
       <c r="AW108" s="2" t="inlineStr"/>
+      <c r="AX108" s="2" t="inlineStr"/>
+      <c r="AY108" s="2" t="inlineStr"/>
+      <c r="AZ108" s="2" t="inlineStr"/>
+      <c r="BA108" s="2" t="inlineStr"/>
+      <c r="BB108" s="2" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="4" t="inlineStr">
@@ -26042,6 +26607,11 @@
       </c>
       <c r="AV109" s="4" t="inlineStr"/>
       <c r="AW109" s="4" t="inlineStr"/>
+      <c r="AX109" s="4" t="inlineStr"/>
+      <c r="AY109" s="4" t="inlineStr"/>
+      <c r="AZ109" s="4" t="inlineStr"/>
+      <c r="BA109" s="4" t="inlineStr"/>
+      <c r="BB109" s="4" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -26273,6 +26843,11 @@
       </c>
       <c r="AV110" s="2" t="inlineStr"/>
       <c r="AW110" s="2" t="inlineStr"/>
+      <c r="AX110" s="2" t="inlineStr"/>
+      <c r="AY110" s="2" t="inlineStr"/>
+      <c r="AZ110" s="2" t="inlineStr"/>
+      <c r="BA110" s="2" t="inlineStr"/>
+      <c r="BB110" s="2" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="4" t="inlineStr">
@@ -26508,6 +27083,11 @@
       </c>
       <c r="AV111" s="4" t="inlineStr"/>
       <c r="AW111" s="4" t="inlineStr"/>
+      <c r="AX111" s="4" t="inlineStr"/>
+      <c r="AY111" s="4" t="inlineStr"/>
+      <c r="AZ111" s="4" t="inlineStr"/>
+      <c r="BA111" s="4" t="inlineStr"/>
+      <c r="BB111" s="4" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -26747,6 +27327,11 @@
       </c>
       <c r="AV112" s="2" t="inlineStr"/>
       <c r="AW112" s="2" t="inlineStr"/>
+      <c r="AX112" s="2" t="inlineStr"/>
+      <c r="AY112" s="2" t="inlineStr"/>
+      <c r="AZ112" s="2" t="inlineStr"/>
+      <c r="BA112" s="2" t="inlineStr"/>
+      <c r="BB112" s="2" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="4" t="inlineStr">
@@ -26982,6 +27567,11 @@
       </c>
       <c r="AV113" s="4" t="inlineStr"/>
       <c r="AW113" s="4" t="inlineStr"/>
+      <c r="AX113" s="4" t="inlineStr"/>
+      <c r="AY113" s="4" t="inlineStr"/>
+      <c r="AZ113" s="4" t="inlineStr"/>
+      <c r="BA113" s="4" t="inlineStr"/>
+      <c r="BB113" s="4" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -27213,6 +27803,11 @@
       </c>
       <c r="AV114" s="2" t="inlineStr"/>
       <c r="AW114" s="2" t="inlineStr"/>
+      <c r="AX114" s="2" t="inlineStr"/>
+      <c r="AY114" s="2" t="inlineStr"/>
+      <c r="AZ114" s="2" t="inlineStr"/>
+      <c r="BA114" s="2" t="inlineStr"/>
+      <c r="BB114" s="2" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="4" t="inlineStr">
@@ -27448,6 +28043,11 @@
       </c>
       <c r="AV115" s="4" t="inlineStr"/>
       <c r="AW115" s="4" t="inlineStr"/>
+      <c r="AX115" s="4" t="inlineStr"/>
+      <c r="AY115" s="4" t="inlineStr"/>
+      <c r="AZ115" s="4" t="inlineStr"/>
+      <c r="BA115" s="4" t="inlineStr"/>
+      <c r="BB115" s="4" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -27680,6 +28280,11 @@
       </c>
       <c r="AV116" s="2" t="inlineStr"/>
       <c r="AW116" s="2" t="inlineStr"/>
+      <c r="AX116" s="2" t="inlineStr"/>
+      <c r="AY116" s="2" t="inlineStr"/>
+      <c r="AZ116" s="2" t="inlineStr"/>
+      <c r="BA116" s="2" t="inlineStr"/>
+      <c r="BB116" s="2" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="4" t="inlineStr">
@@ -27908,6 +28513,11 @@
       </c>
       <c r="AV117" s="4" t="inlineStr"/>
       <c r="AW117" s="4" t="inlineStr"/>
+      <c r="AX117" s="4" t="inlineStr"/>
+      <c r="AY117" s="4" t="inlineStr"/>
+      <c r="AZ117" s="4" t="inlineStr"/>
+      <c r="BA117" s="4" t="inlineStr"/>
+      <c r="BB117" s="4" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -28127,6 +28737,11 @@
       </c>
       <c r="AV118" s="2" t="inlineStr"/>
       <c r="AW118" s="2" t="inlineStr"/>
+      <c r="AX118" s="2" t="inlineStr"/>
+      <c r="AY118" s="2" t="inlineStr"/>
+      <c r="AZ118" s="2" t="inlineStr"/>
+      <c r="BA118" s="2" t="inlineStr"/>
+      <c r="BB118" s="2" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="4" t="inlineStr">
@@ -28346,6 +28961,11 @@
       </c>
       <c r="AV119" s="4" t="inlineStr"/>
       <c r="AW119" s="4" t="inlineStr"/>
+      <c r="AX119" s="4" t="inlineStr"/>
+      <c r="AY119" s="4" t="inlineStr"/>
+      <c r="AZ119" s="4" t="inlineStr"/>
+      <c r="BA119" s="4" t="inlineStr"/>
+      <c r="BB119" s="4" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -28574,6 +29194,11 @@
           <t>https://web.microsoftstream.com/video/462482fb-026d-4ac5-8d29-95b943fd4e67?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
+      <c r="AX120" s="2" t="inlineStr"/>
+      <c r="AY120" s="2" t="inlineStr"/>
+      <c r="AZ120" s="2" t="inlineStr"/>
+      <c r="BA120" s="2" t="inlineStr"/>
+      <c r="BB120" s="2" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="4" t="inlineStr">
@@ -28798,6 +29423,11 @@
       </c>
       <c r="AV121" s="4" t="inlineStr"/>
       <c r="AW121" s="4" t="inlineStr"/>
+      <c r="AX121" s="4" t="inlineStr"/>
+      <c r="AY121" s="4" t="inlineStr"/>
+      <c r="AZ121" s="4" t="inlineStr"/>
+      <c r="BA121" s="4" t="inlineStr"/>
+      <c r="BB121" s="4" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -29022,6 +29652,11 @@
       </c>
       <c r="AV122" s="2" t="inlineStr"/>
       <c r="AW122" s="2" t="inlineStr"/>
+      <c r="AX122" s="2" t="inlineStr"/>
+      <c r="AY122" s="2" t="inlineStr"/>
+      <c r="AZ122" s="2" t="inlineStr"/>
+      <c r="BA122" s="2" t="inlineStr"/>
+      <c r="BB122" s="2" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="4" t="inlineStr">
@@ -29241,6 +29876,11 @@
       </c>
       <c r="AV123" s="4" t="inlineStr"/>
       <c r="AW123" s="4" t="inlineStr"/>
+      <c r="AX123" s="4" t="inlineStr"/>
+      <c r="AY123" s="4" t="inlineStr"/>
+      <c r="AZ123" s="4" t="inlineStr"/>
+      <c r="BA123" s="4" t="inlineStr"/>
+      <c r="BB123" s="4" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -29464,6 +30104,11 @@
       </c>
       <c r="AV124" s="2" t="inlineStr"/>
       <c r="AW124" s="2" t="inlineStr"/>
+      <c r="AX124" s="2" t="inlineStr"/>
+      <c r="AY124" s="2" t="inlineStr"/>
+      <c r="AZ124" s="2" t="inlineStr"/>
+      <c r="BA124" s="2" t="inlineStr"/>
+      <c r="BB124" s="2" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" s="4" t="inlineStr">
@@ -29700,6 +30345,11 @@
       </c>
       <c r="AV125" s="4" t="inlineStr"/>
       <c r="AW125" s="4" t="inlineStr"/>
+      <c r="AX125" s="4" t="inlineStr"/>
+      <c r="AY125" s="4" t="inlineStr"/>
+      <c r="AZ125" s="4" t="inlineStr"/>
+      <c r="BA125" s="4" t="inlineStr"/>
+      <c r="BB125" s="4" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -29940,6 +30590,11 @@
       </c>
       <c r="AV126" s="2" t="inlineStr"/>
       <c r="AW126" s="2" t="inlineStr"/>
+      <c r="AX126" s="2" t="inlineStr"/>
+      <c r="AY126" s="2" t="inlineStr"/>
+      <c r="AZ126" s="2" t="inlineStr"/>
+      <c r="BA126" s="2" t="inlineStr"/>
+      <c r="BB126" s="2" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" s="4" t="inlineStr">
@@ -30176,6 +30831,11 @@
       </c>
       <c r="AV127" s="4" t="inlineStr"/>
       <c r="AW127" s="4" t="inlineStr"/>
+      <c r="AX127" s="4" t="inlineStr"/>
+      <c r="AY127" s="4" t="inlineStr"/>
+      <c r="AZ127" s="4" t="inlineStr"/>
+      <c r="BA127" s="4" t="inlineStr"/>
+      <c r="BB127" s="4" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -30408,6 +31068,11 @@
       </c>
       <c r="AV128" s="2" t="inlineStr"/>
       <c r="AW128" s="2" t="inlineStr"/>
+      <c r="AX128" s="2" t="inlineStr"/>
+      <c r="AY128" s="2" t="inlineStr"/>
+      <c r="AZ128" s="2" t="inlineStr"/>
+      <c r="BA128" s="2" t="inlineStr"/>
+      <c r="BB128" s="2" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="4" t="inlineStr">
@@ -30645,6 +31310,11 @@
       </c>
       <c r="AV129" s="4" t="inlineStr"/>
       <c r="AW129" s="4" t="inlineStr"/>
+      <c r="AX129" s="4" t="inlineStr"/>
+      <c r="AY129" s="4" t="inlineStr"/>
+      <c r="AZ129" s="4" t="inlineStr"/>
+      <c r="BA129" s="4" t="inlineStr"/>
+      <c r="BB129" s="4" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -30884,6 +31554,11 @@
           <t>https://web.microsoftstream.com/video/140b7682-00df-491d-b451-73ae70a040fa?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
+      <c r="AX130" s="2" t="inlineStr"/>
+      <c r="AY130" s="2" t="inlineStr"/>
+      <c r="AZ130" s="2" t="inlineStr"/>
+      <c r="BA130" s="2" t="inlineStr"/>
+      <c r="BB130" s="2" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="4" t="inlineStr">
@@ -31120,6 +31795,11 @@
       </c>
       <c r="AV131" s="4" t="inlineStr"/>
       <c r="AW131" s="4" t="inlineStr"/>
+      <c r="AX131" s="4" t="inlineStr"/>
+      <c r="AY131" s="4" t="inlineStr"/>
+      <c r="AZ131" s="4" t="inlineStr"/>
+      <c r="BA131" s="4" t="inlineStr"/>
+      <c r="BB131" s="4" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -31355,6 +32035,11 @@
           <t>https://web.microsoftstream.com/video/513ae285-b3cb-42e6-a51a-984face9af08?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
+      <c r="AX132" s="2" t="inlineStr"/>
+      <c r="AY132" s="2" t="inlineStr"/>
+      <c r="AZ132" s="2" t="inlineStr"/>
+      <c r="BA132" s="2" t="inlineStr"/>
+      <c r="BB132" s="2" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" s="4" t="inlineStr">
@@ -31590,6 +32275,11 @@
           <t>https://web.microsoftstream.com/video/edcf6e85-7c1c-4dd4-9cc1-599dd69841dc?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
+      <c r="AX133" s="4" t="inlineStr"/>
+      <c r="AY133" s="4" t="inlineStr"/>
+      <c r="AZ133" s="4" t="inlineStr"/>
+      <c r="BA133" s="4" t="inlineStr"/>
+      <c r="BB133" s="4" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -31809,6 +32499,11 @@
       </c>
       <c r="AV134" s="2" t="inlineStr"/>
       <c r="AW134" s="2" t="inlineStr"/>
+      <c r="AX134" s="2" t="inlineStr"/>
+      <c r="AY134" s="2" t="inlineStr"/>
+      <c r="AZ134" s="2" t="inlineStr"/>
+      <c r="BA134" s="2" t="inlineStr"/>
+      <c r="BB134" s="2" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="4" t="inlineStr">
@@ -32041,6 +32736,11 @@
       </c>
       <c r="AV135" s="4" t="inlineStr"/>
       <c r="AW135" s="4" t="inlineStr"/>
+      <c r="AX135" s="4" t="inlineStr"/>
+      <c r="AY135" s="4" t="inlineStr"/>
+      <c r="AZ135" s="4" t="inlineStr"/>
+      <c r="BA135" s="4" t="inlineStr"/>
+      <c r="BB135" s="4" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -32264,6 +32964,11 @@
       </c>
       <c r="AV136" s="2" t="inlineStr"/>
       <c r="AW136" s="2" t="inlineStr"/>
+      <c r="AX136" s="2" t="inlineStr"/>
+      <c r="AY136" s="2" t="inlineStr"/>
+      <c r="AZ136" s="2" t="inlineStr"/>
+      <c r="BA136" s="2" t="inlineStr"/>
+      <c r="BB136" s="2" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="4" t="inlineStr">
@@ -32483,6 +33188,11 @@
       </c>
       <c r="AV137" s="4" t="inlineStr"/>
       <c r="AW137" s="4" t="inlineStr"/>
+      <c r="AX137" s="4" t="inlineStr"/>
+      <c r="AY137" s="4" t="inlineStr"/>
+      <c r="AZ137" s="4" t="inlineStr"/>
+      <c r="BA137" s="4" t="inlineStr"/>
+      <c r="BB137" s="4" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -32719,6 +33429,11 @@
       </c>
       <c r="AV138" s="2" t="inlineStr"/>
       <c r="AW138" s="2" t="inlineStr"/>
+      <c r="AX138" s="2" t="inlineStr"/>
+      <c r="AY138" s="2" t="inlineStr"/>
+      <c r="AZ138" s="2" t="inlineStr"/>
+      <c r="BA138" s="2" t="inlineStr"/>
+      <c r="BB138" s="2" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" s="4" t="inlineStr">
@@ -32954,6 +33669,11 @@
           <t>https://web.microsoftstream.com/video/6e74c0e2-b2c6-4bd6-9b53-5982d3f1b8e1?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
+      <c r="AX139" s="4" t="inlineStr"/>
+      <c r="AY139" s="4" t="inlineStr"/>
+      <c r="AZ139" s="4" t="inlineStr"/>
+      <c r="BA139" s="4" t="inlineStr"/>
+      <c r="BB139" s="4" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -33185,6 +33905,11 @@
       </c>
       <c r="AV140" s="2" t="inlineStr"/>
       <c r="AW140" s="2" t="inlineStr"/>
+      <c r="AX140" s="2" t="inlineStr"/>
+      <c r="AY140" s="2" t="inlineStr"/>
+      <c r="AZ140" s="2" t="inlineStr"/>
+      <c r="BA140" s="2" t="inlineStr"/>
+      <c r="BB140" s="2" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" s="4" t="inlineStr">
@@ -33420,6 +34145,11 @@
           <t>https://web.microsoftstream.com/video/b2ec8a38-dced-4be0-9b7d-e8ceaec2a86e?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
+      <c r="AX141" s="4" t="inlineStr"/>
+      <c r="AY141" s="4" t="inlineStr"/>
+      <c r="AZ141" s="4" t="inlineStr"/>
+      <c r="BA141" s="4" t="inlineStr"/>
+      <c r="BB141" s="4" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -33654,6 +34384,11 @@
       </c>
       <c r="AV142" s="2" t="inlineStr"/>
       <c r="AW142" s="2" t="inlineStr"/>
+      <c r="AX142" s="2" t="inlineStr"/>
+      <c r="AY142" s="2" t="inlineStr"/>
+      <c r="AZ142" s="2" t="inlineStr"/>
+      <c r="BA142" s="2" t="inlineStr"/>
+      <c r="BB142" s="2" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" s="4" t="inlineStr">
@@ -33888,6 +34623,11 @@
       </c>
       <c r="AV143" s="4" t="inlineStr"/>
       <c r="AW143" s="4" t="inlineStr"/>
+      <c r="AX143" s="4" t="inlineStr"/>
+      <c r="AY143" s="4" t="inlineStr"/>
+      <c r="AZ143" s="4" t="inlineStr"/>
+      <c r="BA143" s="4" t="inlineStr"/>
+      <c r="BB143" s="4" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -34124,6 +34864,11 @@
       </c>
       <c r="AV144" s="2" t="inlineStr"/>
       <c r="AW144" s="2" t="inlineStr"/>
+      <c r="AX144" s="2" t="inlineStr"/>
+      <c r="AY144" s="2" t="inlineStr"/>
+      <c r="AZ144" s="2" t="inlineStr"/>
+      <c r="BA144" s="2" t="inlineStr"/>
+      <c r="BB144" s="2" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" s="4" t="inlineStr">
@@ -34363,6 +35108,11 @@
           <t>https://web.microsoftstream.com/video/40583c46-21c1-4547-8443-856ee5a2beb3?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
+      <c r="AX145" s="4" t="inlineStr"/>
+      <c r="AY145" s="4" t="inlineStr"/>
+      <c r="AZ145" s="4" t="inlineStr"/>
+      <c r="BA145" s="4" t="inlineStr"/>
+      <c r="BB145" s="4" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -34603,6 +35353,11 @@
           <t>https://web.microsoftstream.com/video/95da0d56-cc06-4781-a262-9d91a3e9b48d?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
+      <c r="AX146" s="2" t="inlineStr"/>
+      <c r="AY146" s="2" t="inlineStr"/>
+      <c r="AZ146" s="2" t="inlineStr"/>
+      <c r="BA146" s="2" t="inlineStr"/>
+      <c r="BB146" s="2" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" s="4" t="inlineStr">
@@ -34834,6 +35589,11 @@
       </c>
       <c r="AV147" s="4" t="inlineStr"/>
       <c r="AW147" s="4" t="inlineStr"/>
+      <c r="AX147" s="4" t="inlineStr"/>
+      <c r="AY147" s="4" t="inlineStr"/>
+      <c r="AZ147" s="4" t="inlineStr"/>
+      <c r="BA147" s="4" t="inlineStr"/>
+      <c r="BB147" s="4" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -35069,6 +35829,11 @@
       </c>
       <c r="AV148" s="2" t="inlineStr"/>
       <c r="AW148" s="2" t="inlineStr"/>
+      <c r="AX148" s="2" t="inlineStr"/>
+      <c r="AY148" s="2" t="inlineStr"/>
+      <c r="AZ148" s="2" t="inlineStr"/>
+      <c r="BA148" s="2" t="inlineStr"/>
+      <c r="BB148" s="2" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" s="4" t="inlineStr">
@@ -35311,6 +36076,11 @@
           <t>https://web.microsoftstream.com/video/e092ed57-1ff7-4570-9897-57fc78b1a0c8?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
+      <c r="AX149" s="4" t="inlineStr"/>
+      <c r="AY149" s="4" t="inlineStr"/>
+      <c r="AZ149" s="4" t="inlineStr"/>
+      <c r="BA149" s="4" t="inlineStr"/>
+      <c r="BB149" s="4" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -35549,6 +36319,11 @@
       </c>
       <c r="AV150" s="2" t="inlineStr"/>
       <c r="AW150" s="2" t="inlineStr"/>
+      <c r="AX150" s="2" t="inlineStr"/>
+      <c r="AY150" s="2" t="inlineStr"/>
+      <c r="AZ150" s="2" t="inlineStr"/>
+      <c r="BA150" s="2" t="inlineStr"/>
+      <c r="BB150" s="2" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" s="4" t="inlineStr">
@@ -35791,6 +36566,11 @@
           <t>https://web.microsoftstream.com/video/e092ed57-1ff7-4570-9897-57fc78b1a0c8?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
+      <c r="AX151" s="4" t="inlineStr"/>
+      <c r="AY151" s="4" t="inlineStr"/>
+      <c r="AZ151" s="4" t="inlineStr"/>
+      <c r="BA151" s="4" t="inlineStr"/>
+      <c r="BB151" s="4" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -36022,6 +36802,11 @@
       </c>
       <c r="AV152" s="2" t="inlineStr"/>
       <c r="AW152" s="2" t="inlineStr"/>
+      <c r="AX152" s="2" t="inlineStr"/>
+      <c r="AY152" s="2" t="inlineStr"/>
+      <c r="AZ152" s="2" t="inlineStr"/>
+      <c r="BA152" s="2" t="inlineStr"/>
+      <c r="BB152" s="2" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" s="4" t="inlineStr">
@@ -36253,6 +37038,11 @@
       </c>
       <c r="AV153" s="4" t="inlineStr"/>
       <c r="AW153" s="4" t="inlineStr"/>
+      <c r="AX153" s="4" t="inlineStr"/>
+      <c r="AY153" s="4" t="inlineStr"/>
+      <c r="AZ153" s="4" t="inlineStr"/>
+      <c r="BA153" s="4" t="inlineStr"/>
+      <c r="BB153" s="4" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -36490,6 +37280,11 @@
       </c>
       <c r="AV154" s="2" t="inlineStr"/>
       <c r="AW154" s="2" t="inlineStr"/>
+      <c r="AX154" s="2" t="inlineStr"/>
+      <c r="AY154" s="2" t="inlineStr"/>
+      <c r="AZ154" s="2" t="inlineStr"/>
+      <c r="BA154" s="2" t="inlineStr"/>
+      <c r="BB154" s="2" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" s="4" t="inlineStr">
@@ -36585,6 +37380,11 @@
       <c r="AU155" s="4" t="inlineStr"/>
       <c r="AV155" s="4" t="inlineStr"/>
       <c r="AW155" s="4" t="inlineStr"/>
+      <c r="AX155" s="4" t="inlineStr"/>
+      <c r="AY155" s="4" t="inlineStr"/>
+      <c r="AZ155" s="4" t="inlineStr"/>
+      <c r="BA155" s="4" t="inlineStr"/>
+      <c r="BB155" s="4" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -36816,6 +37616,11 @@
       </c>
       <c r="AV156" s="2" t="inlineStr"/>
       <c r="AW156" s="2" t="inlineStr"/>
+      <c r="AX156" s="2" t="inlineStr"/>
+      <c r="AY156" s="2" t="inlineStr"/>
+      <c r="AZ156" s="2" t="inlineStr"/>
+      <c r="BA156" s="2" t="inlineStr"/>
+      <c r="BB156" s="2" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" s="4" t="inlineStr">
@@ -37058,6 +37863,11 @@
           <t>https://web.microsoftstream.com/video/e092ed57-1ff7-4570-9897-57fc78b1a0c8?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
+      <c r="AX157" s="4" t="inlineStr"/>
+      <c r="AY157" s="4" t="inlineStr"/>
+      <c r="AZ157" s="4" t="inlineStr"/>
+      <c r="BA157" s="4" t="inlineStr"/>
+      <c r="BB157" s="4" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -37297,6 +38107,11 @@
           <t>https://web.microsoftstream.com/video/91aaf70b-85c2-4cf1-b537-e42b3bd894ec?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
+      <c r="AX158" s="2" t="inlineStr"/>
+      <c r="AY158" s="2" t="inlineStr"/>
+      <c r="AZ158" s="2" t="inlineStr"/>
+      <c r="BA158" s="2" t="inlineStr"/>
+      <c r="BB158" s="2" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" s="4" t="inlineStr">
@@ -37532,6 +38347,11 @@
       </c>
       <c r="AV159" s="4" t="inlineStr"/>
       <c r="AW159" s="4" t="inlineStr"/>
+      <c r="AX159" s="4" t="inlineStr"/>
+      <c r="AY159" s="4" t="inlineStr"/>
+      <c r="AZ159" s="4" t="inlineStr"/>
+      <c r="BA159" s="4" t="inlineStr"/>
+      <c r="BB159" s="4" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -37763,6 +38583,11 @@
       </c>
       <c r="AV160" s="2" t="inlineStr"/>
       <c r="AW160" s="2" t="inlineStr"/>
+      <c r="AX160" s="2" t="inlineStr"/>
+      <c r="AY160" s="2" t="inlineStr"/>
+      <c r="AZ160" s="2" t="inlineStr"/>
+      <c r="BA160" s="2" t="inlineStr"/>
+      <c r="BB160" s="2" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" s="4" t="inlineStr">
@@ -37996,6 +38821,11 @@
       </c>
       <c r="AV161" s="4" t="inlineStr"/>
       <c r="AW161" s="4" t="inlineStr"/>
+      <c r="AX161" s="4" t="inlineStr"/>
+      <c r="AY161" s="4" t="inlineStr"/>
+      <c r="AZ161" s="4" t="inlineStr"/>
+      <c r="BA161" s="4" t="inlineStr"/>
+      <c r="BB161" s="4" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -38091,6 +38921,11 @@
       <c r="AU162" s="2" t="inlineStr"/>
       <c r="AV162" s="2" t="inlineStr"/>
       <c r="AW162" s="2" t="inlineStr"/>
+      <c r="AX162" s="2" t="inlineStr"/>
+      <c r="AY162" s="2" t="inlineStr"/>
+      <c r="AZ162" s="2" t="inlineStr"/>
+      <c r="BA162" s="2" t="inlineStr"/>
+      <c r="BB162" s="2" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" s="4" t="inlineStr">
@@ -38327,6 +39162,11 @@
       </c>
       <c r="AV163" s="4" t="inlineStr"/>
       <c r="AW163" s="4" t="inlineStr"/>
+      <c r="AX163" s="4" t="inlineStr"/>
+      <c r="AY163" s="4" t="inlineStr"/>
+      <c r="AZ163" s="4" t="inlineStr"/>
+      <c r="BA163" s="4" t="inlineStr"/>
+      <c r="BB163" s="4" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -38554,6 +39394,11 @@
       </c>
       <c r="AV164" s="2" t="inlineStr"/>
       <c r="AW164" s="2" t="inlineStr"/>
+      <c r="AX164" s="2" t="inlineStr"/>
+      <c r="AY164" s="2" t="inlineStr"/>
+      <c r="AZ164" s="2" t="inlineStr"/>
+      <c r="BA164" s="2" t="inlineStr"/>
+      <c r="BB164" s="2" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" s="4" t="inlineStr">
@@ -38785,6 +39630,11 @@
       </c>
       <c r="AV165" s="4" t="inlineStr"/>
       <c r="AW165" s="4" t="inlineStr"/>
+      <c r="AX165" s="4" t="inlineStr"/>
+      <c r="AY165" s="4" t="inlineStr"/>
+      <c r="AZ165" s="4" t="inlineStr"/>
+      <c r="BA165" s="4" t="inlineStr"/>
+      <c r="BB165" s="4" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
@@ -39020,6 +39870,11 @@
       </c>
       <c r="AV166" s="2" t="inlineStr"/>
       <c r="AW166" s="2" t="inlineStr"/>
+      <c r="AX166" s="2" t="inlineStr"/>
+      <c r="AY166" s="2" t="inlineStr"/>
+      <c r="AZ166" s="2" t="inlineStr"/>
+      <c r="BA166" s="2" t="inlineStr"/>
+      <c r="BB166" s="2" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" s="4" t="inlineStr">
@@ -39255,6 +40110,11 @@
           <t>https://web.microsoftstream.com/video/d81cd129-394e-4fda-99cf-dd88633d940f?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
+      <c r="AX167" s="4" t="inlineStr"/>
+      <c r="AY167" s="4" t="inlineStr"/>
+      <c r="AZ167" s="4" t="inlineStr"/>
+      <c r="BA167" s="4" t="inlineStr"/>
+      <c r="BB167" s="4" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
@@ -39486,6 +40346,11 @@
       </c>
       <c r="AV168" s="2" t="inlineStr"/>
       <c r="AW168" s="2" t="inlineStr"/>
+      <c r="AX168" s="2" t="inlineStr"/>
+      <c r="AY168" s="2" t="inlineStr"/>
+      <c r="AZ168" s="2" t="inlineStr"/>
+      <c r="BA168" s="2" t="inlineStr"/>
+      <c r="BB168" s="2" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" s="4" t="inlineStr">
@@ -39721,6 +40586,11 @@
       </c>
       <c r="AV169" s="4" t="inlineStr"/>
       <c r="AW169" s="4" t="inlineStr"/>
+      <c r="AX169" s="4" t="inlineStr"/>
+      <c r="AY169" s="4" t="inlineStr"/>
+      <c r="AZ169" s="4" t="inlineStr"/>
+      <c r="BA169" s="4" t="inlineStr"/>
+      <c r="BB169" s="4" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
@@ -39948,6 +40818,11 @@
       </c>
       <c r="AV170" s="2" t="inlineStr"/>
       <c r="AW170" s="2" t="inlineStr"/>
+      <c r="AX170" s="2" t="inlineStr"/>
+      <c r="AY170" s="2" t="inlineStr"/>
+      <c r="AZ170" s="2" t="inlineStr"/>
+      <c r="BA170" s="2" t="inlineStr"/>
+      <c r="BB170" s="2" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" s="4" t="inlineStr">
@@ -40175,6 +41050,11 @@
       </c>
       <c r="AV171" s="4" t="inlineStr"/>
       <c r="AW171" s="4" t="inlineStr"/>
+      <c r="AX171" s="4" t="inlineStr"/>
+      <c r="AY171" s="4" t="inlineStr"/>
+      <c r="AZ171" s="4" t="inlineStr"/>
+      <c r="BA171" s="4" t="inlineStr"/>
+      <c r="BB171" s="4" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
@@ -40402,6 +41282,11 @@
       </c>
       <c r="AV172" s="2" t="inlineStr"/>
       <c r="AW172" s="2" t="inlineStr"/>
+      <c r="AX172" s="2" t="inlineStr"/>
+      <c r="AY172" s="2" t="inlineStr"/>
+      <c r="AZ172" s="2" t="inlineStr"/>
+      <c r="BA172" s="2" t="inlineStr"/>
+      <c r="BB172" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Dados atualizados via Robô: 08/07/2026 15:52
</commit_message>
<xml_diff>
--- a/dados_atuais.xlsx
+++ b/dados_atuais.xlsx
@@ -2695,42 +2695,178 @@
           <t>https://www.caixa.gov.br/fundos-investimento/e-fundos/renda-fixa-longo-prazo</t>
         </is>
       </c>
-      <c r="Q9" s="4" t="inlineStr"/>
-      <c r="R9" s="4" t="inlineStr"/>
-      <c r="S9" s="4" t="inlineStr"/>
-      <c r="T9" s="4" t="inlineStr"/>
-      <c r="U9" s="4" t="inlineStr"/>
-      <c r="V9" s="4" t="inlineStr"/>
-      <c r="W9" s="4" t="inlineStr"/>
-      <c r="X9" s="4" t="inlineStr"/>
-      <c r="Y9" s="4" t="inlineStr"/>
-      <c r="Z9" s="4" t="inlineStr"/>
-      <c r="AA9" s="4" t="inlineStr"/>
-      <c r="AB9" s="4" t="inlineStr"/>
-      <c r="AC9" s="4" t="inlineStr"/>
-      <c r="AD9" s="4" t="inlineStr"/>
-      <c r="AE9" s="4" t="inlineStr"/>
-      <c r="AF9" s="4" t="inlineStr"/>
+      <c r="Q9" s="4" t="inlineStr">
+        <is>
+          <t>15.154.422/0001-99</t>
+        </is>
+      </c>
+      <c r="R9" s="4" t="inlineStr">
+        <is>
+          <t>5834</t>
+        </is>
+      </c>
+      <c r="S9" s="4" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="T9" s="4" t="inlineStr">
+        <is>
+          <t>0.7</t>
+        </is>
+      </c>
+      <c r="U9" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="V9" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="W9" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="X9" s="4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="Y9" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Z9" s="4" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="AA9" s="4" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
+      <c r="AB9" s="4" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="AC9" s="4" t="inlineStr">
+        <is>
+          <t>RF até 49% Crédito Privado</t>
+        </is>
+      </c>
+      <c r="AD9" s="4" t="inlineStr">
+        <is>
+          <t>Aberto para captação</t>
+        </is>
+      </c>
+      <c r="AE9" s="4" t="inlineStr">
+        <is>
+          <t>LONGO PRAZO</t>
+        </is>
+      </c>
+      <c r="AF9" s="4" t="inlineStr">
+        <is>
+          <t>GERAL</t>
+        </is>
+      </c>
       <c r="AG9" s="4" t="inlineStr"/>
-      <c r="AH9" s="4" t="inlineStr"/>
-      <c r="AI9" s="4" t="inlineStr"/>
-      <c r="AJ9" s="4" t="inlineStr"/>
-      <c r="AK9" s="4" t="inlineStr"/>
-      <c r="AL9" s="4" t="inlineStr"/>
-      <c r="AM9" s="4" t="inlineStr"/>
-      <c r="AN9" s="4" t="inlineStr"/>
-      <c r="AO9" s="4" t="inlineStr"/>
+      <c r="AH9" s="4" t="inlineStr">
+        <is>
+          <t>17h00</t>
+        </is>
+      </c>
+      <c r="AI9" s="4" t="inlineStr">
+        <is>
+          <t>Sim · Automatico · 90%</t>
+        </is>
+      </c>
+      <c r="AJ9" s="4" t="inlineStr">
+        <is>
+          <t>AUTOMATICO</t>
+        </is>
+      </c>
+      <c r="AK9" s="4" t="inlineStr">
+        <is>
+          <t>90.0</t>
+        </is>
+      </c>
+      <c r="AL9" s="4" t="inlineStr">
+        <is>
+          <t>["Pessoa Física", "PJ Varejo", "Private"]</t>
+        </is>
+      </c>
+      <c r="AM9" s="4" t="inlineStr">
+        <is>
+          <t>["Pessoa Física", "PJ Varejo", "Private"]</t>
+        </is>
+      </c>
+      <c r="AN9" s="4" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AO9" s="4" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
       <c r="AP9" s="4" t="inlineStr"/>
-      <c r="AQ9" s="4" t="inlineStr"/>
-      <c r="AR9" s="4" t="inlineStr"/>
-      <c r="AS9" s="4" t="inlineStr"/>
-      <c r="AT9" s="4" t="inlineStr"/>
-      <c r="AU9" s="4" t="inlineStr"/>
-      <c r="AV9" s="4" t="inlineStr"/>
-      <c r="AW9" s="4" t="inlineStr"/>
-      <c r="AX9" s="4" t="inlineStr"/>
-      <c r="AY9" s="4" t="inlineStr"/>
-      <c r="AZ9" s="4" t="inlineStr"/>
+      <c r="AQ9" s="4" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AR9" s="4" t="inlineStr">
+        <is>
+          <t>CAIXA E-FUNDO FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
+        </is>
+      </c>
+      <c r="AS9" s="4" t="inlineStr">
+        <is>
+          <t>Este Fundo não está adaptado às normas vigentes para RPPS (Regimes Próprios de Previdência Social).As movimentações neste Fundo são realizadas exclusivamente pelo Internet Banking.</t>
+        </is>
+      </c>
+      <c r="AT9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5834.pdf</t>
+        </is>
+      </c>
+      <c r="AU9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5834.pdf</t>
+        </is>
+      </c>
+      <c r="AV9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5834.pdf</t>
+        </is>
+      </c>
+      <c r="AW9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_5834.pdf</t>
+        </is>
+      </c>
+      <c r="AX9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5834.pdf</t>
+        </is>
+      </c>
+      <c r="AY9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5834.pdf</t>
+        </is>
+      </c>
+      <c r="AZ9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5834.pdf</t>
+        </is>
+      </c>
       <c r="BA9" s="4" t="inlineStr"/>
       <c r="BB9" s="4" t="inlineStr"/>
     </row>
@@ -14215,42 +14351,182 @@
           <t>https://www.caixa.gov.br/fundos-investimento/curto-prazo/fic-automatico-polis-rf-cp/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="Q54" s="2" t="inlineStr"/>
-      <c r="R54" s="2" t="inlineStr"/>
-      <c r="S54" s="2" t="inlineStr"/>
-      <c r="T54" s="2" t="inlineStr"/>
-      <c r="U54" s="2" t="inlineStr"/>
-      <c r="V54" s="2" t="inlineStr"/>
-      <c r="W54" s="2" t="inlineStr"/>
-      <c r="X54" s="2" t="inlineStr"/>
-      <c r="Y54" s="2" t="inlineStr"/>
-      <c r="Z54" s="2" t="inlineStr"/>
-      <c r="AA54" s="2" t="inlineStr"/>
-      <c r="AB54" s="2" t="inlineStr"/>
-      <c r="AC54" s="2" t="inlineStr"/>
-      <c r="AD54" s="2" t="inlineStr"/>
-      <c r="AE54" s="2" t="inlineStr"/>
-      <c r="AF54" s="2" t="inlineStr"/>
-      <c r="AG54" s="2" t="inlineStr"/>
-      <c r="AH54" s="2" t="inlineStr"/>
-      <c r="AI54" s="2" t="inlineStr"/>
-      <c r="AJ54" s="2" t="inlineStr"/>
-      <c r="AK54" s="2" t="inlineStr"/>
-      <c r="AL54" s="2" t="inlineStr"/>
-      <c r="AM54" s="2" t="inlineStr"/>
-      <c r="AN54" s="2" t="inlineStr"/>
-      <c r="AO54" s="2" t="inlineStr"/>
+      <c r="Q54" s="2" t="inlineStr">
+        <is>
+          <t>39.594.941/0001-36</t>
+        </is>
+      </c>
+      <c r="R54" s="2" t="inlineStr">
+        <is>
+          <t>6520</t>
+        </is>
+      </c>
+      <c r="S54" s="2" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="T54" s="2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="U54" s="2" t="inlineStr">
+        <is>
+          <t>10000.0</t>
+        </is>
+      </c>
+      <c r="V54" s="2" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
+      <c r="W54" s="2" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
+      <c r="X54" s="2" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="Y54" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Z54" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="AA54" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
+      <c r="AB54" s="2" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="AC54" s="2" t="inlineStr">
+        <is>
+          <t>RF 100% TPF - Curto Prazo</t>
+        </is>
+      </c>
+      <c r="AD54" s="2" t="inlineStr">
+        <is>
+          <t>Aberto para captação</t>
+        </is>
+      </c>
+      <c r="AE54" s="2" t="inlineStr">
+        <is>
+          <t>CURTO PRAZO</t>
+        </is>
+      </c>
+      <c r="AF54" s="2" t="inlineStr">
+        <is>
+          <t>GERAL</t>
+        </is>
+      </c>
+      <c r="AG54" s="2" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="AH54" s="2" t="inlineStr">
+        <is>
+          <t>17h00</t>
+        </is>
+      </c>
+      <c r="AI54" s="2" t="inlineStr">
+        <is>
+          <t>Sim · Automatico · 100%</t>
+        </is>
+      </c>
+      <c r="AJ54" s="2" t="inlineStr">
+        <is>
+          <t>AUTOMATICO</t>
+        </is>
+      </c>
+      <c r="AK54" s="2" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
+      <c r="AL54" s="2" t="inlineStr">
+        <is>
+          <t>["Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private"]</t>
+        </is>
+      </c>
+      <c r="AM54" s="2" t="inlineStr">
+        <is>
+          <t>["Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private"]</t>
+        </is>
+      </c>
+      <c r="AN54" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AO54" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
       <c r="AP54" s="2" t="inlineStr"/>
-      <c r="AQ54" s="2" t="inlineStr"/>
-      <c r="AR54" s="2" t="inlineStr"/>
-      <c r="AS54" s="2" t="inlineStr"/>
-      <c r="AT54" s="2" t="inlineStr"/>
-      <c r="AU54" s="2" t="inlineStr"/>
-      <c r="AV54" s="2" t="inlineStr"/>
-      <c r="AW54" s="2" t="inlineStr"/>
-      <c r="AX54" s="2" t="inlineStr"/>
-      <c r="AY54" s="2" t="inlineStr"/>
-      <c r="AZ54" s="2" t="inlineStr"/>
+      <c r="AQ54" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AR54" s="2" t="inlineStr">
+        <is>
+          <t>CAIXA FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA CURTO PRAZO - RESPONSABILIDADE LIMITADA</t>
+        </is>
+      </c>
+      <c r="AS54" s="2" t="inlineStr">
+        <is>
+          <t>*Este Fundo não está adaptado às normas vigentes para RPPS (Regimes Próprios de Previdência Social).</t>
+        </is>
+      </c>
+      <c r="AT54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_6520.pdf</t>
+        </is>
+      </c>
+      <c r="AU54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_6520.pdf</t>
+        </is>
+      </c>
+      <c r="AV54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_6520.pdf</t>
+        </is>
+      </c>
+      <c r="AW54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_6520.pdf</t>
+        </is>
+      </c>
+      <c r="AX54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6520.pdf</t>
+        </is>
+      </c>
+      <c r="AY54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6520.pdf</t>
+        </is>
+      </c>
+      <c r="AZ54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_6520.pdf</t>
+        </is>
+      </c>
       <c r="BA54" s="2" t="inlineStr"/>
       <c r="BB54" s="2" t="inlineStr"/>
     </row>
@@ -28836,12 +29112,12 @@
       </c>
       <c r="Q111" s="4" t="inlineStr">
         <is>
-          <t>30.068.049/0001-47</t>
+          <t>59.815.671/0001-53</t>
         </is>
       </c>
       <c r="R111" s="4" t="inlineStr">
         <is>
-          <t>6499</t>
+          <t>7971</t>
         </is>
       </c>
       <c r="S111" s="4" t="inlineStr">
@@ -28876,14 +29152,14 @@
       </c>
       <c r="Y111" s="4" t="inlineStr">
         <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Z111" s="4" t="inlineStr">
+        <is>
           <t>D+1 (du)</t>
         </is>
       </c>
-      <c r="Z111" s="4" t="inlineStr">
-        <is>
-          <t>D+1 (du)</t>
-        </is>
-      </c>
       <c r="AA111" s="4" t="inlineStr">
         <is>
           <t>D+03 (du)</t>
@@ -28891,7 +29167,7 @@
       </c>
       <c r="AB111" s="4" t="inlineStr">
         <is>
-          <t>IBOV</t>
+          <t>NÃO SE APLICA</t>
         </is>
       </c>
       <c r="AC111" s="4" t="inlineStr">
@@ -28901,7 +29177,7 @@
       </c>
       <c r="AD111" s="4" t="inlineStr">
         <is>
-          <t>Aberto para captação</t>
+          <t>Fechado para captação</t>
         </is>
       </c>
       <c r="AE111" s="4" t="inlineStr">
@@ -28926,27 +29202,23 @@
       </c>
       <c r="AI111" s="4" t="inlineStr">
         <is>
-          <t>Sim · Automatico · 100%</t>
+          <t>Não se aplica</t>
         </is>
       </c>
       <c r="AJ111" s="4" t="inlineStr">
         <is>
-          <t>AUTOMATICO</t>
-        </is>
-      </c>
-      <c r="AK111" s="4" t="inlineStr">
-        <is>
-          <t>100.0</t>
-        </is>
-      </c>
+          <t>NÃO SE APLICA</t>
+        </is>
+      </c>
+      <c r="AK111" s="4" t="inlineStr"/>
       <c r="AL111" s="4" t="inlineStr">
         <is>
-          <t>["GOV", "Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private"]</t>
+          <t>["GOV", "Pessoa Física", "PJ Atacado", "Private"]</t>
         </is>
       </c>
       <c r="AM111" s="4" t="inlineStr">
         <is>
-          <t>["GOV", "Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private"]</t>
+          <t>["GOV", "Pessoa Física", "PJ Atacado", "Private"]</t>
         </is>
       </c>
       <c r="AN111" s="4" t="inlineStr">
@@ -28961,7 +29233,7 @@
       </c>
       <c r="AP111" s="4" t="inlineStr">
         <is>
-          <t>2021-06-13T00:00:00Z</t>
+          <t>2025-05-04T00:00:00Z</t>
         </is>
       </c>
       <c r="AQ111" s="4" t="inlineStr">
@@ -28971,47 +29243,47 @@
       </c>
       <c r="AR111" s="4" t="inlineStr">
         <is>
-          <t>CAIXA SEGURIDADE FUNDO DE INVESTIMENTO FINANCEIRO EM AÇÕES - RESPONSABILIDADE LIMITADA</t>
+          <t>CAIXA SEGURIDADE II FUNDO DE INVESTIMENTO FINANCEIRO AÇÕES - RESPONSABILIDADE LIMITADA</t>
         </is>
       </c>
       <c r="AS111" s="4" t="inlineStr">
         <is>
-          <t>Canal de distribuição: Rede CAIXA, IBC. A reserva inicial, no âmbito da OFERTA, será feita por meio do Home Broker CAIXA. Resgates: Lock up de 45 dias. Inicio dia 30/04/2021 - Termino 13/06/2021. Liberado resgate a partir do dia 14/06/2021 (segunda-feira).</t>
+          <t>Fundo ficará fechado para novas aplicações a partir do dia 13/05/2025 (inclusive).</t>
         </is>
       </c>
       <c r="AT111" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_6499.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_7971.pdf</t>
         </is>
       </c>
       <c r="AU111" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_6499.pdf</t>
+          <t>http://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_7971.pdf</t>
         </is>
       </c>
       <c r="AV111" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_6499.pdf</t>
+          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_7971.pdf</t>
         </is>
       </c>
       <c r="AW111" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_6499.pdf</t>
+          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_7971.pdf</t>
         </is>
       </c>
       <c r="AX111" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6499.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_7971.pdf</t>
         </is>
       </c>
       <c r="AY111" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6499.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_7971.pdf</t>
         </is>
       </c>
       <c r="AZ111" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_6499.pdf</t>
+          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_7971.pdf</t>
         </is>
       </c>
       <c r="BA111" s="4" t="inlineStr"/>
@@ -30645,17 +30917,17 @@
       </c>
       <c r="P118" s="2" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/fundos-investimento/mutuos-privatizacao/fmp-fgts-petrobas-2</t>
+          <t>https://www.caixa.gov.br/fundos-investimento/mutuos-privatizacao/fmp-fgts-petrobas-4</t>
         </is>
       </c>
       <c r="Q118" s="2" t="inlineStr">
         <is>
-          <t>03.915.910/0001-92</t>
+          <t>03.555.959/0001-81</t>
         </is>
       </c>
       <c r="R118" s="2" t="inlineStr">
         <is>
-          <t>5202</t>
+          <t>5204</t>
         </is>
       </c>
       <c r="S118" s="2" t="inlineStr">
@@ -30665,29 +30937,29 @@
       </c>
       <c r="T118" s="2" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>0.95</t>
         </is>
       </c>
       <c r="U118" s="2" t="inlineStr">
         <is>
+          <t>300.0</t>
+        </is>
+      </c>
+      <c r="V118" s="2" t="inlineStr">
+        <is>
           <t>0.01</t>
         </is>
       </c>
-      <c r="V118" s="2" t="inlineStr">
+      <c r="W118" s="2" t="inlineStr">
         <is>
           <t>0.01</t>
         </is>
       </c>
-      <c r="W118" s="2" t="inlineStr">
+      <c r="X118" s="2" t="inlineStr">
         <is>
           <t>0.01</t>
         </is>
       </c>
-      <c r="X118" s="2" t="inlineStr">
-        <is>
-          <t>0.01</t>
-        </is>
-      </c>
       <c r="Y118" s="2" t="inlineStr">
         <is>
           <t>D+0 (du)</t>
@@ -30715,7 +30987,7 @@
       </c>
       <c r="AD118" s="2" t="inlineStr">
         <is>
-          <t>Aberto para captação</t>
+          <t>Fechado para captação</t>
         </is>
       </c>
       <c r="AE118" s="2" t="inlineStr">
@@ -30728,11 +31000,7 @@
           <t>GERAL</t>
         </is>
       </c>
-      <c r="AG118" s="2" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
+      <c r="AG118" s="2" t="inlineStr"/>
       <c r="AH118" s="2" t="inlineStr">
         <is>
           <t>17h00</t>
@@ -30769,48 +31037,47 @@
       </c>
       <c r="AR118" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FUNDO MÚTUO DE PRIVATIZAÇÃO - FGTS - PETROBRAS II - RESPONSABILIDADE LIMITADA</t>
+          <t>CAIXA FUNDO MÚTUO DE PRIVATIZAÇÃO - FGTS - PETROBRAS IV - RESPONSABILIDADE LIMITADA</t>
         </is>
       </c>
       <c r="AS118" s="2" t="inlineStr">
         <is>
-          <t>O fundo encontra-se aberto para receber recursos provenientes de outros Fundos FMP-FGTS.
-Prazo de carência: 6 meses para transferência total ou parcial do investimento no FUNDO para outro FMP- FGTS ou para um Clube de Investimento – FGTS, ou 12 meses para retorno à(s) conta(s) vinculada(s) do investidor junto ao FGTS.</t>
+          <t>FUNDO FECHADO.</t>
         </is>
       </c>
       <c r="AT118" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5202.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5204.pdf</t>
         </is>
       </c>
       <c r="AU118" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5202.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5204.pdf</t>
         </is>
       </c>
       <c r="AV118" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5202.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5204.pdf</t>
         </is>
       </c>
       <c r="AW118" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5202.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5204.pdf</t>
         </is>
       </c>
       <c r="AX118" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5202.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5204.pdf</t>
         </is>
       </c>
       <c r="AY118" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5202.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5204.pdf</t>
         </is>
       </c>
       <c r="AZ118" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5202.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5204.pdf</t>
         </is>
       </c>
       <c r="BA118" s="2" t="inlineStr"/>
@@ -34981,12 +35248,12 @@
       </c>
       <c r="Q135" s="4" t="inlineStr">
         <is>
-          <t>09.181.268/0001-41</t>
+          <t>09.548.725/0001-93</t>
         </is>
       </c>
       <c r="R135" s="4" t="inlineStr">
         <is>
-          <t>5080</t>
+          <t>5132</t>
         </is>
       </c>
       <c r="S135" s="4" t="inlineStr">
@@ -34996,12 +35263,12 @@
       </c>
       <c r="T135" s="4" t="inlineStr">
         <is>
-          <t>0.35</t>
+          <t>0.07</t>
         </is>
       </c>
       <c r="U135" s="4" t="inlineStr">
         <is>
-          <t>1000.0</t>
+          <t>10000000.0</t>
         </is>
       </c>
       <c r="V135" s="4" t="inlineStr">
@@ -35016,7 +35283,7 @@
       </c>
       <c r="X135" s="4" t="inlineStr">
         <is>
-          <t>100.0</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="Y135" s="4" t="inlineStr">
@@ -35056,7 +35323,7 @@
       </c>
       <c r="AF135" s="4" t="inlineStr">
         <is>
-          <t>GERAL</t>
+          <t>QUALIFICADO</t>
         </is>
       </c>
       <c r="AG135" s="4" t="inlineStr">
@@ -35104,7 +35371,7 @@
       </c>
       <c r="AR135" s="4" t="inlineStr">
         <is>
-          <t>CAIXA SAÚDE SUPLEMENTAR - ANS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
+          <t>CAIXA SAUDE SUPLEMENTAR - ANS II FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
         </is>
       </c>
       <c r="AS135" s="4" t="inlineStr">
@@ -35119,37 +35386,37 @@
       </c>
       <c r="AT135" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5080.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5132.pdf</t>
         </is>
       </c>
       <c r="AU135" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5080.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5132.pdf</t>
         </is>
       </c>
       <c r="AV135" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5080.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5132.pdf</t>
         </is>
       </c>
       <c r="AW135" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5080.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5132.pdf</t>
         </is>
       </c>
       <c r="AX135" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5080.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5132.pdf</t>
         </is>
       </c>
       <c r="AY135" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5080.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5132.pdf</t>
         </is>
       </c>
       <c r="AZ135" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5080.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5132.pdf</t>
         </is>
       </c>
       <c r="BA135" s="4" t="inlineStr"/>

</xml_diff>

<commit_message>
Dados atualizados via Robô: 10/07/2026 00:38
</commit_message>
<xml_diff>
--- a/dados_atuais.xlsx
+++ b/dados_atuais.xlsx
@@ -3473,12 +3473,12 @@
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>03.191.874/0001-61</t>
+          <t>03.218.183/0001-04</t>
         </is>
       </c>
       <c r="R12" s="2" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>87</t>
         </is>
       </c>
       <c r="S12" s="2" t="inlineStr">
@@ -3488,27 +3488,27 @@
       </c>
       <c r="T12" s="2" t="inlineStr">
         <is>
-          <t>0.3</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="U12" s="2" t="inlineStr">
         <is>
-          <t>100000.0</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="V12" s="2" t="inlineStr">
         <is>
-          <t>100.0</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="W12" s="2" t="inlineStr">
         <is>
-          <t>100.0</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="X12" s="2" t="inlineStr">
         <is>
-          <t>10000.0</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="Y12" s="2" t="inlineStr">
@@ -3578,12 +3578,12 @@
       </c>
       <c r="AL12" s="2" t="inlineStr">
         <is>
-          <t>["Institucional", "PJ Atacado"]</t>
+          <t>["Pessoa Física"]</t>
         </is>
       </c>
       <c r="AM12" s="2" t="inlineStr">
         <is>
-          <t>["Institucional", "PJ Atacado"]</t>
+          <t>["Pessoa Física"]</t>
         </is>
       </c>
       <c r="AN12" s="2" t="inlineStr">
@@ -3604,7 +3604,7 @@
       </c>
       <c r="AR12" s="2" t="inlineStr">
         <is>
-          <t>CAIXA PATRIMÔNIO ÍNDICE DE PREÇOS FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESP LIMITADA</t>
+          <t>CAIXA CAPITAL ÍNDICE DE PREÇOS FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESP LIMITADA</t>
         </is>
       </c>
       <c r="AS12" s="2" t="inlineStr">
@@ -3614,43 +3614,43 @@
       </c>
       <c r="AT12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_0046.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_0087.pdf</t>
         </is>
       </c>
       <c r="AU12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_0046.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_0087.pdf</t>
         </is>
       </c>
       <c r="AV12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_0046.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_0087.pdf</t>
         </is>
       </c>
       <c r="AW12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_46.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_87.pdf</t>
         </is>
       </c>
       <c r="AX12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_46.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_87.pdf</t>
         </is>
       </c>
       <c r="AY12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_46.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_87.pdf</t>
         </is>
       </c>
       <c r="AZ12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_0046.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_0087.pdf</t>
         </is>
       </c>
       <c r="BA12" s="2" t="inlineStr"/>
       <c r="BB12" s="2" t="inlineStr">
         <is>
-          <t>https://web.microsoftstream.com/video/140b7682-00df-491d-b451-73ae70a040fa?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
+          <t>https://web.microsoftstream.com/video/32d65536-1de1-4f2f-a9b8-0fbb0d9347fc?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
     </row>
@@ -11063,12 +11063,12 @@
       </c>
       <c r="AL41" s="4" t="inlineStr">
         <is>
-          <t>["Private"]</t>
+          <t>["PJ Varejo", "Private"]</t>
         </is>
       </c>
       <c r="AM41" s="4" t="inlineStr">
         <is>
-          <t>["Private"]</t>
+          <t>["PJ Varejo", "Private"]</t>
         </is>
       </c>
       <c r="AN41" s="4" t="inlineStr">
@@ -16725,9 +16725,9 @@
           <t>1,41518700</t>
         </is>
       </c>
-      <c r="E64" s="7" t="inlineStr">
-        <is>
-          <t>-0,012</t>
+      <c r="E64" s="3" t="inlineStr">
+        <is>
+          <t>0,674</t>
         </is>
       </c>
       <c r="F64" s="7" t="inlineStr">
@@ -18009,9 +18009,9 @@
           <t>2,87074400</t>
         </is>
       </c>
-      <c r="E69" s="6" t="inlineStr">
-        <is>
-          <t>-0,155</t>
+      <c r="E69" s="5" t="inlineStr">
+        <is>
+          <t>0,067</t>
         </is>
       </c>
       <c r="F69" s="6" t="inlineStr">
@@ -24768,7 +24768,7 @@
       </c>
       <c r="E95" s="6" t="inlineStr">
         <is>
-          <t>-0,676</t>
+          <t>-0,015</t>
         </is>
       </c>
       <c r="F95" s="6" t="inlineStr">
@@ -34449,12 +34449,12 @@
       </c>
       <c r="AL132" s="2" t="inlineStr">
         <is>
-          <t>["Institucional", "PJ Atacado", "PJ Varejo"]</t>
+          <t>["Institucional", "PJ Atacado"]</t>
         </is>
       </c>
       <c r="AM132" s="2" t="inlineStr">
         <is>
-          <t>["Institucional", "PJ Atacado", "PJ Varejo"]</t>
+          <t>["Institucional", "PJ Atacado"]</t>
         </is>
       </c>
       <c r="AN132" s="2" t="inlineStr">
@@ -36138,7 +36138,7 @@
       </c>
       <c r="U139" s="4" t="inlineStr">
         <is>
-          <t>3000000.0</t>
+          <t>1000000.0</t>
         </is>
       </c>
       <c r="V139" s="4" t="inlineStr">
@@ -36153,7 +36153,7 @@
       </c>
       <c r="X139" s="4" t="inlineStr">
         <is>
-          <t>300000.0</t>
+          <t>100000.0</t>
         </is>
       </c>
       <c r="Y139" s="4" t="inlineStr">
@@ -36223,12 +36223,12 @@
       </c>
       <c r="AL139" s="4" t="inlineStr">
         <is>
-          <t>["Institucional", "PJ Atacado", "PJ Varejo"]</t>
+          <t>["Institucional", "PJ Atacado"]</t>
         </is>
       </c>
       <c r="AM139" s="4" t="inlineStr">
         <is>
-          <t>["Institucional", "PJ Atacado", "PJ Varejo"]</t>
+          <t>["Institucional", "PJ Atacado"]</t>
         </is>
       </c>
       <c r="AN139" s="4" t="inlineStr">
@@ -36252,7 +36252,17 @@
           <t>CAIXA TOPÁZIO CORPORATIVO FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA REFERENCIADO DI LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
         </is>
       </c>
-      <c r="AS139" s="4" t="inlineStr"/>
+      <c r="AS139" s="4" t="inlineStr">
+        <is>
+          <t>Campanha "Campanha Caixa Asset Lidera RPPS" de 06/07/2026 a 31/08/2026
+Redução de Tickets
+Aplicação Inicial:
+De: R$ 3.000.000,00 para R$ 1.000.000,00
+Saldo Mínimo: 
+De: R$ 300.000,00 para R$ 100.000,00
+OBS: Após a Campanha, voltam os parâmetros originais. Saldo abaixo do mínimo pode impedir resgates parciais (somente total).</t>
+        </is>
+      </c>
       <c r="AT139" s="4" t="inlineStr">
         <is>
           <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5189.pdf</t>
@@ -40932,12 +40942,12 @@
       </c>
       <c r="Q158" s="2" t="inlineStr">
         <is>
-          <t>05.164.356/0001-84</t>
+          <t>03.737.206/0001-97</t>
         </is>
       </c>
       <c r="R158" s="2" t="inlineStr">
         <is>
-          <t>5462</t>
+          <t>5404</t>
         </is>
       </c>
       <c r="S158" s="2" t="inlineStr">
@@ -40992,7 +41002,7 @@
       </c>
       <c r="AC158" s="2" t="inlineStr">
         <is>
-          <t>RF 100% TPF - Longo Prazo</t>
+          <t>RF DI até 49% Crédito Privado</t>
         </is>
       </c>
       <c r="AD158" s="2" t="inlineStr">
@@ -41063,53 +41073,54 @@
       </c>
       <c r="AR158" s="2" t="inlineStr">
         <is>
-          <t>CAIXA BRASIL TÍTULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
+          <t>CAIXA BRASIL FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA REFERENCIADO DI LONGO PRAZO - RESP LIMITADA</t>
         </is>
       </c>
       <c r="AS158" s="2" t="inlineStr">
         <is>
-          <t>Para aplicação no fundo é necessário o cadastramento prévio de cotistas, conforme descrito no FI657. O procedimento de inclusão da conta deverá ser realizado sempre que houver qualquer aplicação, mesmo para os clientes que já realizaram o cadsatramento anteriormente.</t>
+          <t>1. Para aplicação por meio de conta operação 003, é necessário o cadastramento prévio de cotistas, conforme descrito no item Adesão, do FI612.
+2. O procedimento de inclusão da conta deverá ser realizado sempre que houver qualquer aplicação por meio de conta operação 003, mesmo para os clientes que já realizaram o cadastramento anteriormente.</t>
         </is>
       </c>
       <c r="AT158" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5462.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5404.pdf</t>
         </is>
       </c>
       <c r="AU158" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5462.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5404.pdf</t>
         </is>
       </c>
       <c r="AV158" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5462.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5404.pdf</t>
         </is>
       </c>
       <c r="AW158" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5462.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5404.pdf</t>
         </is>
       </c>
       <c r="AX158" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5462.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5404.pdf</t>
         </is>
       </c>
       <c r="AY158" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5462.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5404.pdf</t>
         </is>
       </c>
       <c r="AZ158" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5462.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5404.pdf</t>
         </is>
       </c>
       <c r="BA158" s="2" t="inlineStr"/>
       <c r="BB158" s="2" t="inlineStr">
         <is>
-          <t>https://web.microsoftstream.com/video/91aaf70b-85c2-4cf1-b537-e42b3bd894ec?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
+          <t>https://web.microsoftstream.com/video/f88f1fc7-aac3-44df-a2a5-ce3ac05edfb3?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dados atualizados via Robô: 10/07/2026 15:53
</commit_message>
<xml_diff>
--- a/dados_atuais.xlsx
+++ b/dados_atuais.xlsx
@@ -14351,42 +14351,182 @@
           <t>https://www.caixa.gov.br/fundos-investimento/curto-prazo/fic-automatico-polis-rf-cp/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="Q54" s="2" t="inlineStr"/>
-      <c r="R54" s="2" t="inlineStr"/>
-      <c r="S54" s="2" t="inlineStr"/>
-      <c r="T54" s="2" t="inlineStr"/>
-      <c r="U54" s="2" t="inlineStr"/>
-      <c r="V54" s="2" t="inlineStr"/>
-      <c r="W54" s="2" t="inlineStr"/>
-      <c r="X54" s="2" t="inlineStr"/>
-      <c r="Y54" s="2" t="inlineStr"/>
-      <c r="Z54" s="2" t="inlineStr"/>
-      <c r="AA54" s="2" t="inlineStr"/>
-      <c r="AB54" s="2" t="inlineStr"/>
-      <c r="AC54" s="2" t="inlineStr"/>
-      <c r="AD54" s="2" t="inlineStr"/>
-      <c r="AE54" s="2" t="inlineStr"/>
-      <c r="AF54" s="2" t="inlineStr"/>
-      <c r="AG54" s="2" t="inlineStr"/>
-      <c r="AH54" s="2" t="inlineStr"/>
-      <c r="AI54" s="2" t="inlineStr"/>
-      <c r="AJ54" s="2" t="inlineStr"/>
-      <c r="AK54" s="2" t="inlineStr"/>
-      <c r="AL54" s="2" t="inlineStr"/>
-      <c r="AM54" s="2" t="inlineStr"/>
-      <c r="AN54" s="2" t="inlineStr"/>
-      <c r="AO54" s="2" t="inlineStr"/>
+      <c r="Q54" s="2" t="inlineStr">
+        <is>
+          <t>39.594.941/0001-36</t>
+        </is>
+      </c>
+      <c r="R54" s="2" t="inlineStr">
+        <is>
+          <t>6520</t>
+        </is>
+      </c>
+      <c r="S54" s="2" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="T54" s="2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="U54" s="2" t="inlineStr">
+        <is>
+          <t>10000.0</t>
+        </is>
+      </c>
+      <c r="V54" s="2" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
+      <c r="W54" s="2" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
+      <c r="X54" s="2" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="Y54" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Z54" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="AA54" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
+      <c r="AB54" s="2" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="AC54" s="2" t="inlineStr">
+        <is>
+          <t>RF 100% TPF - Curto Prazo</t>
+        </is>
+      </c>
+      <c r="AD54" s="2" t="inlineStr">
+        <is>
+          <t>Aberto para captação</t>
+        </is>
+      </c>
+      <c r="AE54" s="2" t="inlineStr">
+        <is>
+          <t>CURTO PRAZO</t>
+        </is>
+      </c>
+      <c r="AF54" s="2" t="inlineStr">
+        <is>
+          <t>GERAL</t>
+        </is>
+      </c>
+      <c r="AG54" s="2" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="AH54" s="2" t="inlineStr">
+        <is>
+          <t>17h00</t>
+        </is>
+      </c>
+      <c r="AI54" s="2" t="inlineStr">
+        <is>
+          <t>Sim · Automatico · 100%</t>
+        </is>
+      </c>
+      <c r="AJ54" s="2" t="inlineStr">
+        <is>
+          <t>AUTOMATICO</t>
+        </is>
+      </c>
+      <c r="AK54" s="2" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
+      <c r="AL54" s="2" t="inlineStr">
+        <is>
+          <t>["Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private"]</t>
+        </is>
+      </c>
+      <c r="AM54" s="2" t="inlineStr">
+        <is>
+          <t>["Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private"]</t>
+        </is>
+      </c>
+      <c r="AN54" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AO54" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
       <c r="AP54" s="2" t="inlineStr"/>
-      <c r="AQ54" s="2" t="inlineStr"/>
-      <c r="AR54" s="2" t="inlineStr"/>
-      <c r="AS54" s="2" t="inlineStr"/>
-      <c r="AT54" s="2" t="inlineStr"/>
-      <c r="AU54" s="2" t="inlineStr"/>
-      <c r="AV54" s="2" t="inlineStr"/>
-      <c r="AW54" s="2" t="inlineStr"/>
-      <c r="AX54" s="2" t="inlineStr"/>
-      <c r="AY54" s="2" t="inlineStr"/>
-      <c r="AZ54" s="2" t="inlineStr"/>
+      <c r="AQ54" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AR54" s="2" t="inlineStr">
+        <is>
+          <t>CAIXA FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA CURTO PRAZO - RESPONSABILIDADE LIMITADA</t>
+        </is>
+      </c>
+      <c r="AS54" s="2" t="inlineStr">
+        <is>
+          <t>*Este Fundo não está adaptado às normas vigentes para RPPS (Regimes Próprios de Previdência Social).</t>
+        </is>
+      </c>
+      <c r="AT54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_6520.pdf</t>
+        </is>
+      </c>
+      <c r="AU54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_6520.pdf</t>
+        </is>
+      </c>
+      <c r="AV54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_6520.pdf</t>
+        </is>
+      </c>
+      <c r="AW54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_6520.pdf</t>
+        </is>
+      </c>
+      <c r="AX54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6520.pdf</t>
+        </is>
+      </c>
+      <c r="AY54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6520.pdf</t>
+        </is>
+      </c>
+      <c r="AZ54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_6520.pdf</t>
+        </is>
+      </c>
       <c r="BA54" s="2" t="inlineStr"/>
       <c r="BB54" s="2" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Dados atualizados via Robô: 14/07/2026 15:15
</commit_message>
<xml_diff>
--- a/dados_atuais.xlsx
+++ b/dados_atuais.xlsx
@@ -7129,7 +7129,7 @@
       </c>
       <c r="U26" s="2" t="inlineStr">
         <is>
-          <t>20000.0</t>
+          <t>10000.0</t>
         </is>
       </c>
       <c r="V26" s="2" t="inlineStr">
@@ -7893,7 +7893,7 @@
       </c>
       <c r="U29" s="4" t="inlineStr">
         <is>
-          <t>20000.0</t>
+          <t>10000.0</t>
         </is>
       </c>
       <c r="V29" s="4" t="inlineStr">
@@ -8153,7 +8153,7 @@
       </c>
       <c r="U30" s="2" t="inlineStr">
         <is>
-          <t>100000.0</t>
+          <t>10000.0</t>
         </is>
       </c>
       <c r="V30" s="2" t="inlineStr">
@@ -8168,7 +8168,7 @@
       </c>
       <c r="X30" s="2" t="inlineStr">
         <is>
-          <t>10000.0</t>
+          <t>1000.0</t>
         </is>
       </c>
       <c r="Y30" s="2" t="inlineStr">
@@ -8917,7 +8917,7 @@
       </c>
       <c r="U33" s="4" t="inlineStr">
         <is>
-          <t>100000.0</t>
+          <t>10000.0</t>
         </is>
       </c>
       <c r="V33" s="4" t="inlineStr">
@@ -8932,7 +8932,7 @@
       </c>
       <c r="X33" s="4" t="inlineStr">
         <is>
-          <t>10000.0</t>
+          <t>1000.0</t>
         </is>
       </c>
       <c r="Y33" s="4" t="inlineStr">
@@ -9437,7 +9437,7 @@
       </c>
       <c r="U35" s="4" t="inlineStr">
         <is>
-          <t>200000.0</t>
+          <t>10000.0</t>
         </is>
       </c>
       <c r="V35" s="4" t="inlineStr">
@@ -9452,7 +9452,7 @@
       </c>
       <c r="X35" s="4" t="inlineStr">
         <is>
-          <t>20000.0</t>
+          <t>1000.0</t>
         </is>
       </c>
       <c r="Y35" s="4" t="inlineStr">
@@ -11239,7 +11239,7 @@
       </c>
       <c r="U42" s="2" t="inlineStr">
         <is>
-          <t>200000.0</t>
+          <t>100000.0</t>
         </is>
       </c>
       <c r="V42" s="2" t="inlineStr">
@@ -11254,7 +11254,7 @@
       </c>
       <c r="X42" s="2" t="inlineStr">
         <is>
-          <t>20000.0</t>
+          <t>10000.0</t>
         </is>
       </c>
       <c r="Y42" s="2" t="inlineStr">
@@ -12280,7 +12280,7 @@
       </c>
       <c r="U46" s="2" t="inlineStr">
         <is>
-          <t>1000.0</t>
+          <t>100.0</t>
         </is>
       </c>
       <c r="V46" s="2" t="inlineStr">
@@ -12295,7 +12295,7 @@
       </c>
       <c r="X46" s="2" t="inlineStr">
         <is>
-          <t>100.0</t>
+          <t>10.0</t>
         </is>
       </c>
       <c r="Y46" s="2" t="inlineStr">
@@ -13064,7 +13064,7 @@
       </c>
       <c r="U49" s="4" t="inlineStr">
         <is>
-          <t>1000000.0</t>
+          <t>10000.0</t>
         </is>
       </c>
       <c r="V49" s="4" t="inlineStr">
@@ -13079,7 +13079,7 @@
       </c>
       <c r="X49" s="4" t="inlineStr">
         <is>
-          <t>100000.0</t>
+          <t>1000.0</t>
         </is>
       </c>
       <c r="Y49" s="4" t="inlineStr">
@@ -13849,7 +13849,7 @@
       </c>
       <c r="U52" s="2" t="inlineStr">
         <is>
-          <t>300000.0</t>
+          <t>100000.0</t>
         </is>
       </c>
       <c r="V52" s="2" t="inlineStr">
@@ -13864,7 +13864,7 @@
       </c>
       <c r="X52" s="2" t="inlineStr">
         <is>
-          <t>30000.0</t>
+          <t>10000.0</t>
         </is>
       </c>
       <c r="Y52" s="2" t="inlineStr">
@@ -14351,42 +14351,182 @@
           <t>https://www.caixa.gov.br/fundos-investimento/curto-prazo/fic-automatico-polis-rf-cp/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="Q54" s="2" t="inlineStr"/>
-      <c r="R54" s="2" t="inlineStr"/>
-      <c r="S54" s="2" t="inlineStr"/>
-      <c r="T54" s="2" t="inlineStr"/>
-      <c r="U54" s="2" t="inlineStr"/>
-      <c r="V54" s="2" t="inlineStr"/>
-      <c r="W54" s="2" t="inlineStr"/>
-      <c r="X54" s="2" t="inlineStr"/>
-      <c r="Y54" s="2" t="inlineStr"/>
-      <c r="Z54" s="2" t="inlineStr"/>
-      <c r="AA54" s="2" t="inlineStr"/>
-      <c r="AB54" s="2" t="inlineStr"/>
-      <c r="AC54" s="2" t="inlineStr"/>
-      <c r="AD54" s="2" t="inlineStr"/>
-      <c r="AE54" s="2" t="inlineStr"/>
-      <c r="AF54" s="2" t="inlineStr"/>
-      <c r="AG54" s="2" t="inlineStr"/>
-      <c r="AH54" s="2" t="inlineStr"/>
-      <c r="AI54" s="2" t="inlineStr"/>
-      <c r="AJ54" s="2" t="inlineStr"/>
-      <c r="AK54" s="2" t="inlineStr"/>
-      <c r="AL54" s="2" t="inlineStr"/>
-      <c r="AM54" s="2" t="inlineStr"/>
-      <c r="AN54" s="2" t="inlineStr"/>
-      <c r="AO54" s="2" t="inlineStr"/>
+      <c r="Q54" s="2" t="inlineStr">
+        <is>
+          <t>39.594.941/0001-36</t>
+        </is>
+      </c>
+      <c r="R54" s="2" t="inlineStr">
+        <is>
+          <t>6520</t>
+        </is>
+      </c>
+      <c r="S54" s="2" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="T54" s="2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="U54" s="2" t="inlineStr">
+        <is>
+          <t>10000.0</t>
+        </is>
+      </c>
+      <c r="V54" s="2" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
+      <c r="W54" s="2" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
+      <c r="X54" s="2" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="Y54" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Z54" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="AA54" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
+      <c r="AB54" s="2" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="AC54" s="2" t="inlineStr">
+        <is>
+          <t>RF 100% TPF - Curto Prazo</t>
+        </is>
+      </c>
+      <c r="AD54" s="2" t="inlineStr">
+        <is>
+          <t>Aberto para captação</t>
+        </is>
+      </c>
+      <c r="AE54" s="2" t="inlineStr">
+        <is>
+          <t>CURTO PRAZO</t>
+        </is>
+      </c>
+      <c r="AF54" s="2" t="inlineStr">
+        <is>
+          <t>GERAL</t>
+        </is>
+      </c>
+      <c r="AG54" s="2" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="AH54" s="2" t="inlineStr">
+        <is>
+          <t>17h00</t>
+        </is>
+      </c>
+      <c r="AI54" s="2" t="inlineStr">
+        <is>
+          <t>Sim · Automatico · 100%</t>
+        </is>
+      </c>
+      <c r="AJ54" s="2" t="inlineStr">
+        <is>
+          <t>AUTOMATICO</t>
+        </is>
+      </c>
+      <c r="AK54" s="2" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
+      <c r="AL54" s="2" t="inlineStr">
+        <is>
+          <t>["Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private"]</t>
+        </is>
+      </c>
+      <c r="AM54" s="2" t="inlineStr">
+        <is>
+          <t>["Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private"]</t>
+        </is>
+      </c>
+      <c r="AN54" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AO54" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
       <c r="AP54" s="2" t="inlineStr"/>
-      <c r="AQ54" s="2" t="inlineStr"/>
-      <c r="AR54" s="2" t="inlineStr"/>
-      <c r="AS54" s="2" t="inlineStr"/>
-      <c r="AT54" s="2" t="inlineStr"/>
-      <c r="AU54" s="2" t="inlineStr"/>
-      <c r="AV54" s="2" t="inlineStr"/>
-      <c r="AW54" s="2" t="inlineStr"/>
-      <c r="AX54" s="2" t="inlineStr"/>
-      <c r="AY54" s="2" t="inlineStr"/>
-      <c r="AZ54" s="2" t="inlineStr"/>
+      <c r="AQ54" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AR54" s="2" t="inlineStr">
+        <is>
+          <t>CAIXA FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA CURTO PRAZO - RESPONSABILIDADE LIMITADA</t>
+        </is>
+      </c>
+      <c r="AS54" s="2" t="inlineStr">
+        <is>
+          <t>*Este Fundo não está adaptado às normas vigentes para RPPS (Regimes Próprios de Previdência Social).</t>
+        </is>
+      </c>
+      <c r="AT54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_6520.pdf</t>
+        </is>
+      </c>
+      <c r="AU54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_6520.pdf</t>
+        </is>
+      </c>
+      <c r="AV54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_6520.pdf</t>
+        </is>
+      </c>
+      <c r="AW54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_6520.pdf</t>
+        </is>
+      </c>
+      <c r="AX54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6520.pdf</t>
+        </is>
+      </c>
+      <c r="AY54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6520.pdf</t>
+        </is>
+      </c>
+      <c r="AZ54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_6520.pdf</t>
+        </is>
+      </c>
       <c r="BA54" s="2" t="inlineStr"/>
       <c r="BB54" s="2" t="inlineStr"/>
     </row>
@@ -19375,7 +19515,7 @@
       </c>
       <c r="U74" s="2" t="inlineStr">
         <is>
-          <t>10000.0</t>
+          <t>1000.0</t>
         </is>
       </c>
       <c r="V74" s="2" t="inlineStr">
@@ -19390,7 +19530,7 @@
       </c>
       <c r="X74" s="2" t="inlineStr">
         <is>
-          <t>1000.0</t>
+          <t>100.0</t>
         </is>
       </c>
       <c r="Y74" s="2" t="inlineStr">
@@ -19902,7 +20042,7 @@
       </c>
       <c r="U76" s="2" t="inlineStr">
         <is>
-          <t>10000.0</t>
+          <t>1000.0</t>
         </is>
       </c>
       <c r="V76" s="2" t="inlineStr">
@@ -19917,7 +20057,7 @@
       </c>
       <c r="X76" s="2" t="inlineStr">
         <is>
-          <t>1000.0</t>
+          <t>100.0</t>
         </is>
       </c>
       <c r="Y76" s="2" t="inlineStr">
@@ -42614,12 +42754,12 @@
       </c>
       <c r="Q165" s="4" t="inlineStr">
         <is>
-          <t>13.058.816/0001-18</t>
+          <t>15.154.236/0001-50</t>
         </is>
       </c>
       <c r="R165" s="4" t="inlineStr">
         <is>
-          <t>5445</t>
+          <t>5842</t>
         </is>
       </c>
       <c r="S165" s="4" t="inlineStr">
@@ -42679,7 +42819,7 @@
       </c>
       <c r="AD165" s="4" t="inlineStr">
         <is>
-          <t>Aberto para captação</t>
+          <t>Fechado para captação</t>
         </is>
       </c>
       <c r="AE165" s="4" t="inlineStr">
@@ -42745,43 +42885,47 @@
       </c>
       <c r="AR165" s="4" t="inlineStr">
         <is>
-          <t>CAIXA BRASIL INDEXA IBOVESPA FUNDO DE INVESTIMENTO FINANCEIRO EM AÇÕES - RESPONSABILIDADE LIMITADA</t>
-        </is>
-      </c>
-      <c r="AS165" s="4" t="inlineStr"/>
+          <t>CAIXA BRASIL ETF IBOVESPA FUNDO DE INVESTIMENTO FINANCEIRO EM AÇÕES - RESPONSABILIDADE LIMITADA</t>
+        </is>
+      </c>
+      <c r="AS165" s="4" t="inlineStr">
+        <is>
+          <t>Fundo fechado para novas aplicações, a novos investidores e cotistas atuais a partir de 03/04/2023 (inclusive)</t>
+        </is>
+      </c>
       <c r="AT165" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5445.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5842.pdf</t>
         </is>
       </c>
       <c r="AU165" s="4" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5445.pdf</t>
+          <t>http://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5842.pdf</t>
         </is>
       </c>
       <c r="AV165" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5445.pdf</t>
+          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5842.pdf</t>
         </is>
       </c>
       <c r="AW165" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_5445.pdf</t>
+          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_5842.pdf</t>
         </is>
       </c>
       <c r="AX165" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5445.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5842.pdf</t>
         </is>
       </c>
       <c r="AY165" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5445.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5842.pdf</t>
         </is>
       </c>
       <c r="AZ165" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5445.pdf</t>
+          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5842.pdf</t>
         </is>
       </c>
       <c r="BA165" s="4" t="inlineStr"/>

</xml_diff>

<commit_message>
Dados atualizados via Robô: 17/07/2026 14:55
</commit_message>
<xml_diff>
--- a/dados_atuais.xlsx
+++ b/dados_atuais.xlsx
@@ -3473,12 +3473,12 @@
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>03.218.183/0001-04</t>
+          <t>03.191.874/0001-61</t>
         </is>
       </c>
       <c r="R12" s="2" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>46</t>
         </is>
       </c>
       <c r="S12" s="2" t="inlineStr">
@@ -3488,27 +3488,27 @@
       </c>
       <c r="T12" s="2" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>0.3</t>
         </is>
       </c>
       <c r="U12" s="2" t="inlineStr">
         <is>
-          <t>0.01</t>
+          <t>100000.0</t>
         </is>
       </c>
       <c r="V12" s="2" t="inlineStr">
         <is>
-          <t>0.01</t>
+          <t>100.0</t>
         </is>
       </c>
       <c r="W12" s="2" t="inlineStr">
         <is>
-          <t>0.01</t>
+          <t>100.0</t>
         </is>
       </c>
       <c r="X12" s="2" t="inlineStr">
         <is>
-          <t>0.01</t>
+          <t>10000.0</t>
         </is>
       </c>
       <c r="Y12" s="2" t="inlineStr">
@@ -3578,12 +3578,12 @@
       </c>
       <c r="AL12" s="2" t="inlineStr">
         <is>
-          <t>["Pessoa Física"]</t>
+          <t>["Institucional", "PJ Atacado"]</t>
         </is>
       </c>
       <c r="AM12" s="2" t="inlineStr">
         <is>
-          <t>["Pessoa Física"]</t>
+          <t>["Institucional", "PJ Atacado"]</t>
         </is>
       </c>
       <c r="AN12" s="2" t="inlineStr">
@@ -3604,7 +3604,7 @@
       </c>
       <c r="AR12" s="2" t="inlineStr">
         <is>
-          <t>CAIXA CAPITAL ÍNDICE DE PREÇOS FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESP LIMITADA</t>
+          <t>CAIXA PATRIMÔNIO ÍNDICE DE PREÇOS FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESP LIMITADA</t>
         </is>
       </c>
       <c r="AS12" s="2" t="inlineStr">
@@ -3614,43 +3614,43 @@
       </c>
       <c r="AT12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_0087.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_0046.pdf</t>
         </is>
       </c>
       <c r="AU12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_0087.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_0046.pdf</t>
         </is>
       </c>
       <c r="AV12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_0087.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_0046.pdf</t>
         </is>
       </c>
       <c r="AW12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_87.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_46.pdf</t>
         </is>
       </c>
       <c r="AX12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_87.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_46.pdf</t>
         </is>
       </c>
       <c r="AY12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_87.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_46.pdf</t>
         </is>
       </c>
       <c r="AZ12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_0087.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_0046.pdf</t>
         </is>
       </c>
       <c r="BA12" s="2" t="inlineStr"/>
       <c r="BB12" s="2" t="inlineStr">
         <is>
-          <t>https://web.microsoftstream.com/video/32d65536-1de1-4f2f-a9b8-0fbb0d9347fc?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
+          <t>https://web.microsoftstream.com/video/140b7682-00df-491d-b451-73ae70a040fa?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
     </row>
@@ -42771,12 +42771,12 @@
       </c>
       <c r="Q165" s="4" t="inlineStr">
         <is>
-          <t>15.154.236/0001-50</t>
+          <t>13.058.816/0001-18</t>
         </is>
       </c>
       <c r="R165" s="4" t="inlineStr">
         <is>
-          <t>5842</t>
+          <t>5445</t>
         </is>
       </c>
       <c r="S165" s="4" t="inlineStr">
@@ -42836,7 +42836,7 @@
       </c>
       <c r="AD165" s="4" t="inlineStr">
         <is>
-          <t>Fechado para captação</t>
+          <t>Aberto para captação</t>
         </is>
       </c>
       <c r="AE165" s="4" t="inlineStr">
@@ -42902,47 +42902,43 @@
       </c>
       <c r="AR165" s="4" t="inlineStr">
         <is>
-          <t>CAIXA BRASIL ETF IBOVESPA FUNDO DE INVESTIMENTO FINANCEIRO EM AÇÕES - RESPONSABILIDADE LIMITADA</t>
-        </is>
-      </c>
-      <c r="AS165" s="4" t="inlineStr">
-        <is>
-          <t>Fundo fechado para novas aplicações, a novos investidores e cotistas atuais a partir de 03/04/2023 (inclusive)</t>
-        </is>
-      </c>
+          <t>CAIXA BRASIL INDEXA IBOVESPA FUNDO DE INVESTIMENTO FINANCEIRO EM AÇÕES - RESPONSABILIDADE LIMITADA</t>
+        </is>
+      </c>
+      <c r="AS165" s="4" t="inlineStr"/>
       <c r="AT165" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5842.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5445.pdf</t>
         </is>
       </c>
       <c r="AU165" s="4" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5842.pdf</t>
+          <t>http://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5445.pdf</t>
         </is>
       </c>
       <c r="AV165" s="4" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5842.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5445.pdf</t>
         </is>
       </c>
       <c r="AW165" s="4" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_5842.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_5445.pdf</t>
         </is>
       </c>
       <c r="AX165" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5842.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5445.pdf</t>
         </is>
       </c>
       <c r="AY165" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5842.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5445.pdf</t>
         </is>
       </c>
       <c r="AZ165" s="4" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5842.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5445.pdf</t>
         </is>
       </c>
       <c r="BA165" s="4" t="inlineStr"/>

</xml_diff>

<commit_message>
Dados atualizados via Robô: 20/07/2026 15:23
</commit_message>
<xml_diff>
--- a/dados_atuais.xlsx
+++ b/dados_atuais.xlsx
@@ -39665,12 +39665,12 @@
       </c>
       <c r="Q152" s="2" t="inlineStr">
         <is>
-          <t>10.740.658/0001-93</t>
+          <t>11.060.913/0001-10</t>
         </is>
       </c>
       <c r="R152" s="2" t="inlineStr">
         <is>
-          <t>5184</t>
+          <t>5187</t>
         </is>
       </c>
       <c r="S152" s="2" t="inlineStr">
@@ -39720,7 +39720,7 @@
       </c>
       <c r="AB152" s="2" t="inlineStr">
         <is>
-          <t>IMA-B TOTAL</t>
+          <t>IMA-B 5</t>
         </is>
       </c>
       <c r="AC152" s="2" t="inlineStr">
@@ -39796,49 +39796,43 @@
       </c>
       <c r="AR152" s="2" t="inlineStr">
         <is>
-          <t>CAIXA BRASIL IMA-B TÍTULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
-        </is>
-      </c>
-      <c r="AS152" s="2" t="inlineStr">
-        <is>
-          <t>1. O Fundo tem como parâmetro de rentabilidade o Índice de Mercado ANBIMA série B (IMA-B).
-2. Para aplicação por meio de conta operação 1292, é necessário o cadastramento prévio de cotistas, conforme descrito no item Adesão, do FI612.
-3. O procedimento de inclusão da conta deverá ser realizado sempre que houver qualquer aplicação por meio de conta operação 1292, mesmo para os clientes que já realizaram o cadastramento anteriormente.</t>
-        </is>
-      </c>
+          <t>CAIXA BRASIL IMA-B 5 TÍTULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
+        </is>
+      </c>
+      <c r="AS152" s="2" t="inlineStr"/>
       <c r="AT152" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5184.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5187.pdf</t>
         </is>
       </c>
       <c r="AU152" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5184.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5187.pdf</t>
         </is>
       </c>
       <c r="AV152" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5184.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5187.pdf</t>
         </is>
       </c>
       <c r="AW152" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5184.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5187.pdf</t>
         </is>
       </c>
       <c r="AX152" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5184.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5187.pdf</t>
         </is>
       </c>
       <c r="AY152" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5184.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5187.pdf</t>
         </is>
       </c>
       <c r="AZ152" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5184.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5187.pdf</t>
         </is>
       </c>
       <c r="BA152" s="2" t="inlineStr"/>
@@ -39927,12 +39921,12 @@
       </c>
       <c r="Q153" s="4" t="inlineStr">
         <is>
-          <t>10.740.658/0001-93</t>
+          <t>11.060.913/0001-10</t>
         </is>
       </c>
       <c r="R153" s="4" t="inlineStr">
         <is>
-          <t>5184</t>
+          <t>5187</t>
         </is>
       </c>
       <c r="S153" s="4" t="inlineStr">
@@ -39982,7 +39976,7 @@
       </c>
       <c r="AB153" s="4" t="inlineStr">
         <is>
-          <t>IMA-B TOTAL</t>
+          <t>IMA-B 5</t>
         </is>
       </c>
       <c r="AC153" s="4" t="inlineStr">
@@ -40058,49 +40052,43 @@
       </c>
       <c r="AR153" s="4" t="inlineStr">
         <is>
-          <t>CAIXA BRASIL IMA-B TÍTULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
-        </is>
-      </c>
-      <c r="AS153" s="4" t="inlineStr">
-        <is>
-          <t>1. O Fundo tem como parâmetro de rentabilidade o Índice de Mercado ANBIMA série B (IMA-B).
-2. Para aplicação por meio de conta operação 1292, é necessário o cadastramento prévio de cotistas, conforme descrito no item Adesão, do FI612.
-3. O procedimento de inclusão da conta deverá ser realizado sempre que houver qualquer aplicação por meio de conta operação 1292, mesmo para os clientes que já realizaram o cadastramento anteriormente.</t>
-        </is>
-      </c>
+          <t>CAIXA BRASIL IMA-B 5 TÍTULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
+        </is>
+      </c>
+      <c r="AS153" s="4" t="inlineStr"/>
       <c r="AT153" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5184.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5187.pdf</t>
         </is>
       </c>
       <c r="AU153" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5184.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5187.pdf</t>
         </is>
       </c>
       <c r="AV153" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5184.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5187.pdf</t>
         </is>
       </c>
       <c r="AW153" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5184.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5187.pdf</t>
         </is>
       </c>
       <c r="AX153" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5184.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5187.pdf</t>
         </is>
       </c>
       <c r="AY153" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5184.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5187.pdf</t>
         </is>
       </c>
       <c r="AZ153" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5184.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5187.pdf</t>
         </is>
       </c>
       <c r="BA153" s="4" t="inlineStr"/>
@@ -40571,12 +40559,12 @@
       </c>
       <c r="Q156" s="2" t="inlineStr">
         <is>
-          <t>10.740.658/0001-93</t>
+          <t>11.060.913/0001-10</t>
         </is>
       </c>
       <c r="R156" s="2" t="inlineStr">
         <is>
-          <t>5184</t>
+          <t>5187</t>
         </is>
       </c>
       <c r="S156" s="2" t="inlineStr">
@@ -40626,7 +40614,7 @@
       </c>
       <c r="AB156" s="2" t="inlineStr">
         <is>
-          <t>IMA-B TOTAL</t>
+          <t>IMA-B 5</t>
         </is>
       </c>
       <c r="AC156" s="2" t="inlineStr">
@@ -40702,49 +40690,43 @@
       </c>
       <c r="AR156" s="2" t="inlineStr">
         <is>
-          <t>CAIXA BRASIL IMA-B TÍTULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
-        </is>
-      </c>
-      <c r="AS156" s="2" t="inlineStr">
-        <is>
-          <t>1. O Fundo tem como parâmetro de rentabilidade o Índice de Mercado ANBIMA série B (IMA-B).
-2. Para aplicação por meio de conta operação 1292, é necessário o cadastramento prévio de cotistas, conforme descrito no item Adesão, do FI612.
-3. O procedimento de inclusão da conta deverá ser realizado sempre que houver qualquer aplicação por meio de conta operação 1292, mesmo para os clientes que já realizaram o cadastramento anteriormente.</t>
-        </is>
-      </c>
+          <t>CAIXA BRASIL IMA-B 5 TÍTULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
+        </is>
+      </c>
+      <c r="AS156" s="2" t="inlineStr"/>
       <c r="AT156" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5184.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5187.pdf</t>
         </is>
       </c>
       <c r="AU156" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5184.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5187.pdf</t>
         </is>
       </c>
       <c r="AV156" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5184.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5187.pdf</t>
         </is>
       </c>
       <c r="AW156" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5184.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5187.pdf</t>
         </is>
       </c>
       <c r="AX156" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5184.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5187.pdf</t>
         </is>
       </c>
       <c r="AY156" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5184.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5187.pdf</t>
         </is>
       </c>
       <c r="AZ156" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5184.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5187.pdf</t>
         </is>
       </c>
       <c r="BA156" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Dados atualizados via Robô: 24/07/2026 15:18
</commit_message>
<xml_diff>
--- a/dados_atuais.xlsx
+++ b/dados_atuais.xlsx
@@ -14343,42 +14343,182 @@
           <t>https://www.caixa.gov.br/fundos-investimento/curto-prazo/fic-automatico-polis-rf-cp/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="Q54" s="2" t="inlineStr"/>
-      <c r="R54" s="2" t="inlineStr"/>
-      <c r="S54" s="2" t="inlineStr"/>
-      <c r="T54" s="2" t="inlineStr"/>
-      <c r="U54" s="2" t="inlineStr"/>
-      <c r="V54" s="2" t="inlineStr"/>
-      <c r="W54" s="2" t="inlineStr"/>
-      <c r="X54" s="2" t="inlineStr"/>
-      <c r="Y54" s="2" t="inlineStr"/>
-      <c r="Z54" s="2" t="inlineStr"/>
-      <c r="AA54" s="2" t="inlineStr"/>
-      <c r="AB54" s="2" t="inlineStr"/>
-      <c r="AC54" s="2" t="inlineStr"/>
-      <c r="AD54" s="2" t="inlineStr"/>
-      <c r="AE54" s="2" t="inlineStr"/>
-      <c r="AF54" s="2" t="inlineStr"/>
-      <c r="AG54" s="2" t="inlineStr"/>
-      <c r="AH54" s="2" t="inlineStr"/>
-      <c r="AI54" s="2" t="inlineStr"/>
-      <c r="AJ54" s="2" t="inlineStr"/>
-      <c r="AK54" s="2" t="inlineStr"/>
-      <c r="AL54" s="2" t="inlineStr"/>
-      <c r="AM54" s="2" t="inlineStr"/>
-      <c r="AN54" s="2" t="inlineStr"/>
-      <c r="AO54" s="2" t="inlineStr"/>
+      <c r="Q54" s="2" t="inlineStr">
+        <is>
+          <t>39.594.941/0001-36</t>
+        </is>
+      </c>
+      <c r="R54" s="2" t="inlineStr">
+        <is>
+          <t>6520</t>
+        </is>
+      </c>
+      <c r="S54" s="2" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="T54" s="2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="U54" s="2" t="inlineStr">
+        <is>
+          <t>10000.0</t>
+        </is>
+      </c>
+      <c r="V54" s="2" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
+      <c r="W54" s="2" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
+      <c r="X54" s="2" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="Y54" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="Z54" s="2" t="inlineStr">
+        <is>
+          <t>D+0 (du)</t>
+        </is>
+      </c>
+      <c r="AA54" s="2" t="inlineStr">
+        <is>
+          <t>D+00 (du)</t>
+        </is>
+      </c>
+      <c r="AB54" s="2" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="AC54" s="2" t="inlineStr">
+        <is>
+          <t>RF 100% TPF - Curto Prazo</t>
+        </is>
+      </c>
+      <c r="AD54" s="2" t="inlineStr">
+        <is>
+          <t>Aberto para captação</t>
+        </is>
+      </c>
+      <c r="AE54" s="2" t="inlineStr">
+        <is>
+          <t>CURTO PRAZO</t>
+        </is>
+      </c>
+      <c r="AF54" s="2" t="inlineStr">
+        <is>
+          <t>GERAL</t>
+        </is>
+      </c>
+      <c r="AG54" s="2" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="AH54" s="2" t="inlineStr">
+        <is>
+          <t>17h00</t>
+        </is>
+      </c>
+      <c r="AI54" s="2" t="inlineStr">
+        <is>
+          <t>Sim · Automatico · 100%</t>
+        </is>
+      </c>
+      <c r="AJ54" s="2" t="inlineStr">
+        <is>
+          <t>AUTOMATICO</t>
+        </is>
+      </c>
+      <c r="AK54" s="2" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
+      <c r="AL54" s="2" t="inlineStr">
+        <is>
+          <t>["Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private"]</t>
+        </is>
+      </c>
+      <c r="AM54" s="2" t="inlineStr">
+        <is>
+          <t>["Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private"]</t>
+        </is>
+      </c>
+      <c r="AN54" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AO54" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
       <c r="AP54" s="2" t="inlineStr"/>
-      <c r="AQ54" s="2" t="inlineStr"/>
-      <c r="AR54" s="2" t="inlineStr"/>
-      <c r="AS54" s="2" t="inlineStr"/>
-      <c r="AT54" s="2" t="inlineStr"/>
-      <c r="AU54" s="2" t="inlineStr"/>
-      <c r="AV54" s="2" t="inlineStr"/>
-      <c r="AW54" s="2" t="inlineStr"/>
-      <c r="AX54" s="2" t="inlineStr"/>
-      <c r="AY54" s="2" t="inlineStr"/>
-      <c r="AZ54" s="2" t="inlineStr"/>
+      <c r="AQ54" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AR54" s="2" t="inlineStr">
+        <is>
+          <t>CAIXA FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA CURTO PRAZO - RESPONSABILIDADE LIMITADA</t>
+        </is>
+      </c>
+      <c r="AS54" s="2" t="inlineStr">
+        <is>
+          <t>*Este Fundo não está adaptado às normas vigentes para RPPS (Regimes Próprios de Previdência Social).</t>
+        </is>
+      </c>
+      <c r="AT54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_6520.pdf</t>
+        </is>
+      </c>
+      <c r="AU54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_6520.pdf</t>
+        </is>
+      </c>
+      <c r="AV54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_6520.pdf</t>
+        </is>
+      </c>
+      <c r="AW54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_6520.pdf</t>
+        </is>
+      </c>
+      <c r="AX54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6520.pdf</t>
+        </is>
+      </c>
+      <c r="AY54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6520.pdf</t>
+        </is>
+      </c>
+      <c r="AZ54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_6520.pdf</t>
+        </is>
+      </c>
       <c r="BA54" s="2" t="inlineStr"/>
       <c r="BB54" s="2" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Dados atualizados via Robô [fundos]: 15/08/2026 03:10
</commit_message>
<xml_diff>
--- a/dados_atuais.xlsx
+++ b/dados_atuais.xlsx
@@ -839,7 +839,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>404,524</t>
+          <t>402,198</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -1099,7 +1099,7 @@
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>6.683,634</t>
+          <t>6.633,409</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
@@ -1359,7 +1359,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>781,891</t>
+          <t>776,130</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -1618,7 +1618,7 @@
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>122,505</t>
+          <t>122,504</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
@@ -1881,7 +1881,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>1.701,047</t>
+          <t>1.701,033</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -2137,7 +2137,7 @@
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>96,853</t>
+          <t>96,792</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -2645,7 +2645,7 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>64,441</t>
+          <t>64,440</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -2683,178 +2683,42 @@
           <t>https://www.caixa.gov.br/fundos-investimento/e-fundos/renda-fixa-longo-prazo</t>
         </is>
       </c>
-      <c r="Q9" s="4" t="inlineStr">
-        <is>
-          <t>15.154.422/0001-99</t>
-        </is>
-      </c>
-      <c r="R9" s="4" t="inlineStr">
-        <is>
-          <t>5834</t>
-        </is>
-      </c>
-      <c r="S9" s="4" t="inlineStr">
-        <is>
-          <t>Moderado</t>
-        </is>
-      </c>
-      <c r="T9" s="4" t="inlineStr">
-        <is>
-          <t>0.7</t>
-        </is>
-      </c>
-      <c r="U9" s="4" t="inlineStr">
-        <is>
-          <t>0.01</t>
-        </is>
-      </c>
-      <c r="V9" s="4" t="inlineStr">
-        <is>
-          <t>0.01</t>
-        </is>
-      </c>
-      <c r="W9" s="4" t="inlineStr">
-        <is>
-          <t>0.01</t>
-        </is>
-      </c>
-      <c r="X9" s="4" t="inlineStr">
-        <is>
-          <t>0.01</t>
-        </is>
-      </c>
-      <c r="Y9" s="4" t="inlineStr">
-        <is>
-          <t>D+0 (du)</t>
-        </is>
-      </c>
-      <c r="Z9" s="4" t="inlineStr">
-        <is>
-          <t>D+0 (du)</t>
-        </is>
-      </c>
-      <c r="AA9" s="4" t="inlineStr">
-        <is>
-          <t>D+00 (du)</t>
-        </is>
-      </c>
-      <c r="AB9" s="4" t="inlineStr">
-        <is>
-          <t>CDI</t>
-        </is>
-      </c>
-      <c r="AC9" s="4" t="inlineStr">
-        <is>
-          <t>RF até 49% Crédito Privado</t>
-        </is>
-      </c>
-      <c r="AD9" s="4" t="inlineStr">
-        <is>
-          <t>Aberto para captação</t>
-        </is>
-      </c>
-      <c r="AE9" s="4" t="inlineStr">
-        <is>
-          <t>LONGO PRAZO</t>
-        </is>
-      </c>
-      <c r="AF9" s="4" t="inlineStr">
-        <is>
-          <t>GERAL</t>
-        </is>
-      </c>
+      <c r="Q9" s="4" t="inlineStr"/>
+      <c r="R9" s="4" t="inlineStr"/>
+      <c r="S9" s="4" t="inlineStr"/>
+      <c r="T9" s="4" t="inlineStr"/>
+      <c r="U9" s="4" t="inlineStr"/>
+      <c r="V9" s="4" t="inlineStr"/>
+      <c r="W9" s="4" t="inlineStr"/>
+      <c r="X9" s="4" t="inlineStr"/>
+      <c r="Y9" s="4" t="inlineStr"/>
+      <c r="Z9" s="4" t="inlineStr"/>
+      <c r="AA9" s="4" t="inlineStr"/>
+      <c r="AB9" s="4" t="inlineStr"/>
+      <c r="AC9" s="4" t="inlineStr"/>
+      <c r="AD9" s="4" t="inlineStr"/>
+      <c r="AE9" s="4" t="inlineStr"/>
+      <c r="AF9" s="4" t="inlineStr"/>
       <c r="AG9" s="4" t="inlineStr"/>
-      <c r="AH9" s="4" t="inlineStr">
-        <is>
-          <t>17h00</t>
-        </is>
-      </c>
-      <c r="AI9" s="4" t="inlineStr">
-        <is>
-          <t>Sim · Automatico · 90%</t>
-        </is>
-      </c>
-      <c r="AJ9" s="4" t="inlineStr">
-        <is>
-          <t>AUTOMATICO</t>
-        </is>
-      </c>
-      <c r="AK9" s="4" t="inlineStr">
-        <is>
-          <t>90.0</t>
-        </is>
-      </c>
-      <c r="AL9" s="4" t="inlineStr">
-        <is>
-          <t>["Pessoa Física", "PJ Varejo", "Private"]</t>
-        </is>
-      </c>
-      <c r="AM9" s="4" t="inlineStr">
-        <is>
-          <t>["Pessoa Física", "PJ Varejo", "Private"]</t>
-        </is>
-      </c>
-      <c r="AN9" s="4" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="AO9" s="4" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
+      <c r="AH9" s="4" t="inlineStr"/>
+      <c r="AI9" s="4" t="inlineStr"/>
+      <c r="AJ9" s="4" t="inlineStr"/>
+      <c r="AK9" s="4" t="inlineStr"/>
+      <c r="AL9" s="4" t="inlineStr"/>
+      <c r="AM9" s="4" t="inlineStr"/>
+      <c r="AN9" s="4" t="inlineStr"/>
+      <c r="AO9" s="4" t="inlineStr"/>
       <c r="AP9" s="4" t="inlineStr"/>
-      <c r="AQ9" s="4" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="AR9" s="4" t="inlineStr">
-        <is>
-          <t>CAIXA E-FUNDO FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
-        </is>
-      </c>
-      <c r="AS9" s="4" t="inlineStr">
-        <is>
-          <t>Este Fundo não está adaptado às normas vigentes para RPPS (Regimes Próprios de Previdência Social).As movimentações neste Fundo são realizadas exclusivamente pelo Internet Banking.</t>
-        </is>
-      </c>
-      <c r="AT9" s="4" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5834.pdf</t>
-        </is>
-      </c>
-      <c r="AU9" s="4" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5834.pdf</t>
-        </is>
-      </c>
-      <c r="AV9" s="4" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5834.pdf</t>
-        </is>
-      </c>
-      <c r="AW9" s="4" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_5834.pdf</t>
-        </is>
-      </c>
-      <c r="AX9" s="4" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5834.pdf</t>
-        </is>
-      </c>
-      <c r="AY9" s="4" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5834.pdf</t>
-        </is>
-      </c>
-      <c r="AZ9" s="4" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5834.pdf</t>
-        </is>
-      </c>
+      <c r="AQ9" s="4" t="inlineStr"/>
+      <c r="AR9" s="4" t="inlineStr"/>
+      <c r="AS9" s="4" t="inlineStr"/>
+      <c r="AT9" s="4" t="inlineStr"/>
+      <c r="AU9" s="4" t="inlineStr"/>
+      <c r="AV9" s="4" t="inlineStr"/>
+      <c r="AW9" s="4" t="inlineStr"/>
+      <c r="AX9" s="4" t="inlineStr"/>
+      <c r="AY9" s="4" t="inlineStr"/>
+      <c r="AZ9" s="4" t="inlineStr"/>
       <c r="BA9" s="4" t="inlineStr"/>
       <c r="BB9" s="4" t="inlineStr"/>
     </row>
@@ -2901,7 +2765,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>587,269</t>
+          <t>587,268</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -3161,7 +3025,7 @@
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>12,177</t>
+          <t>12,176</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -3421,7 +3285,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>27,791</t>
+          <t>27,776</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -3949,7 +3813,7 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>41,232</t>
+          <t>41,231</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -4730,7 +4594,7 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>77,122</t>
+          <t>76,972</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -5250,7 +5114,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>129,240</t>
+          <t>129,239</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -6039,7 +5903,7 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>1.808,192</t>
+          <t>1.796,673</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -6293,7 +6157,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>2.231,563</t>
+          <t>2.231,559</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -6553,7 +6417,7 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>967,731</t>
+          <t>967,729</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
@@ -6813,7 +6677,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>2.420,604</t>
+          <t>2.420,591</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -7321,7 +7185,7 @@
       </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>181,135</t>
+          <t>181,127</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -7581,7 +7445,7 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>3.399,259</t>
+          <t>3.399,219</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
@@ -7816,32 +7680,32 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H29" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,27233900</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>0,046</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>0,49</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>8,63</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>14,58</t>
         </is>
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>73,362</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -8076,32 +7940,32 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,13610700</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>-0,013</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>0,66</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>5,32</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>9,28</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>199,704</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
@@ -8332,32 +8196,32 @@
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G31" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H31" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,20209000</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>0,039</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>0,50</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t>8,25</t>
+        </is>
+      </c>
+      <c r="H31" s="5" t="inlineStr">
+        <is>
+          <t>14,10</t>
         </is>
       </c>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>64,934</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -8584,32 +8448,32 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G32" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,10368400</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>0,054</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>0,38</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>6,81</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>306,104</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
@@ -8861,7 +8725,7 @@
       </c>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>451,016</t>
+          <t>451,014</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -9617,32 +9481,32 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F36" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G36" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,06550200</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>0,047</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>0,48</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>8,66</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>22,208</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
@@ -9890,7 +9754,7 @@
       </c>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>853,551</t>
+          <t>853,399</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -10398,7 +10262,7 @@
       </c>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>3.125,809</t>
+          <t>3.125,798</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
@@ -10654,7 +10518,7 @@
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>658,890</t>
+          <t>658,884</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
@@ -10914,7 +10778,7 @@
       </c>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>120,697</t>
+          <t>120,443</t>
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr">
@@ -11170,7 +11034,7 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>122,332</t>
+          <t>122,331</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -11431,7 +11295,7 @@
       </c>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>16.389,045</t>
+          <t>16.388,823</t>
         </is>
       </c>
       <c r="J43" s="4" t="inlineStr">
@@ -11695,7 +11559,7 @@
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>1.498,135</t>
+          <t>1.498,134</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
@@ -12472,7 +12336,7 @@
       </c>
       <c r="I47" s="4" t="inlineStr">
         <is>
-          <t>2.286,952</t>
+          <t>2.286,911</t>
         </is>
       </c>
       <c r="J47" s="4" t="inlineStr">
@@ -12736,7 +12600,7 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>6.118,667</t>
+          <t>6.074,985</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
@@ -12996,7 +12860,7 @@
       </c>
       <c r="I49" s="4" t="inlineStr">
         <is>
-          <t>69,440</t>
+          <t>69,436</t>
         </is>
       </c>
       <c r="J49" s="4" t="inlineStr">
@@ -13256,7 +13120,7 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>14.015,569</t>
+          <t>14.015,456</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
@@ -13516,7 +13380,7 @@
       </c>
       <c r="I51" s="4" t="inlineStr">
         <is>
-          <t>826,865</t>
+          <t>826,864</t>
         </is>
       </c>
       <c r="J51" s="4" t="inlineStr">
@@ -13781,7 +13645,7 @@
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>16.870,811</t>
+          <t>16.870,646</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr">
@@ -14041,7 +13905,7 @@
       </c>
       <c r="I53" s="4" t="inlineStr">
         <is>
-          <t>22.760,188</t>
+          <t>22.759,995</t>
         </is>
       </c>
       <c r="J53" s="4" t="inlineStr">
@@ -14301,7 +14165,7 @@
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>9.573,659</t>
+          <t>9.573,613</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr">
@@ -14603,182 +14467,42 @@
           <t>https://www.caixa.gov.br/fundos-investimento/curto-prazo/fic-automatico-polis-rf-cp/Paginas/default.aspx</t>
         </is>
       </c>
-      <c r="Q55" s="4" t="inlineStr">
-        <is>
-          <t>39.594.941/0001-36</t>
-        </is>
-      </c>
-      <c r="R55" s="4" t="inlineStr">
-        <is>
-          <t>6520</t>
-        </is>
-      </c>
-      <c r="S55" s="4" t="inlineStr">
-        <is>
-          <t>Conservador</t>
-        </is>
-      </c>
-      <c r="T55" s="4" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
-      </c>
-      <c r="U55" s="4" t="inlineStr">
-        <is>
-          <t>10000.0</t>
-        </is>
-      </c>
-      <c r="V55" s="4" t="inlineStr">
-        <is>
-          <t>100.0</t>
-        </is>
-      </c>
-      <c r="W55" s="4" t="inlineStr">
-        <is>
-          <t>100.0</t>
-        </is>
-      </c>
-      <c r="X55" s="4" t="inlineStr">
-        <is>
-          <t>1000.0</t>
-        </is>
-      </c>
-      <c r="Y55" s="4" t="inlineStr">
-        <is>
-          <t>D+0 (du)</t>
-        </is>
-      </c>
-      <c r="Z55" s="4" t="inlineStr">
-        <is>
-          <t>D+0 (du)</t>
-        </is>
-      </c>
-      <c r="AA55" s="4" t="inlineStr">
-        <is>
-          <t>D+00 (du)</t>
-        </is>
-      </c>
-      <c r="AB55" s="4" t="inlineStr">
-        <is>
-          <t>CDI</t>
-        </is>
-      </c>
-      <c r="AC55" s="4" t="inlineStr">
-        <is>
-          <t>RF 100% TPF - Curto Prazo</t>
-        </is>
-      </c>
-      <c r="AD55" s="4" t="inlineStr">
-        <is>
-          <t>Aberto para captação</t>
-        </is>
-      </c>
-      <c r="AE55" s="4" t="inlineStr">
-        <is>
-          <t>CURTO PRAZO</t>
-        </is>
-      </c>
-      <c r="AF55" s="4" t="inlineStr">
-        <is>
-          <t>GERAL</t>
-        </is>
-      </c>
-      <c r="AG55" s="4" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="AH55" s="4" t="inlineStr">
-        <is>
-          <t>17h00</t>
-        </is>
-      </c>
-      <c r="AI55" s="4" t="inlineStr">
-        <is>
-          <t>Sim · Automatico · 100%</t>
-        </is>
-      </c>
-      <c r="AJ55" s="4" t="inlineStr">
-        <is>
-          <t>AUTOMATICO</t>
-        </is>
-      </c>
-      <c r="AK55" s="4" t="inlineStr">
-        <is>
-          <t>100.0</t>
-        </is>
-      </c>
-      <c r="AL55" s="4" t="inlineStr">
-        <is>
-          <t>["Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private"]</t>
-        </is>
-      </c>
-      <c r="AM55" s="4" t="inlineStr">
-        <is>
-          <t>["Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private"]</t>
-        </is>
-      </c>
-      <c r="AN55" s="4" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="AO55" s="4" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
+      <c r="Q55" s="4" t="inlineStr"/>
+      <c r="R55" s="4" t="inlineStr"/>
+      <c r="S55" s="4" t="inlineStr"/>
+      <c r="T55" s="4" t="inlineStr"/>
+      <c r="U55" s="4" t="inlineStr"/>
+      <c r="V55" s="4" t="inlineStr"/>
+      <c r="W55" s="4" t="inlineStr"/>
+      <c r="X55" s="4" t="inlineStr"/>
+      <c r="Y55" s="4" t="inlineStr"/>
+      <c r="Z55" s="4" t="inlineStr"/>
+      <c r="AA55" s="4" t="inlineStr"/>
+      <c r="AB55" s="4" t="inlineStr"/>
+      <c r="AC55" s="4" t="inlineStr"/>
+      <c r="AD55" s="4" t="inlineStr"/>
+      <c r="AE55" s="4" t="inlineStr"/>
+      <c r="AF55" s="4" t="inlineStr"/>
+      <c r="AG55" s="4" t="inlineStr"/>
+      <c r="AH55" s="4" t="inlineStr"/>
+      <c r="AI55" s="4" t="inlineStr"/>
+      <c r="AJ55" s="4" t="inlineStr"/>
+      <c r="AK55" s="4" t="inlineStr"/>
+      <c r="AL55" s="4" t="inlineStr"/>
+      <c r="AM55" s="4" t="inlineStr"/>
+      <c r="AN55" s="4" t="inlineStr"/>
+      <c r="AO55" s="4" t="inlineStr"/>
       <c r="AP55" s="4" t="inlineStr"/>
-      <c r="AQ55" s="4" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="AR55" s="4" t="inlineStr">
-        <is>
-          <t>CAIXA FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA CURTO PRAZO - RESPONSABILIDADE LIMITADA</t>
-        </is>
-      </c>
-      <c r="AS55" s="4" t="inlineStr">
-        <is>
-          <t>*Este Fundo não está adaptado às normas vigentes para RPPS (Regimes Próprios de Previdência Social).</t>
-        </is>
-      </c>
-      <c r="AT55" s="4" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_6520.pdf</t>
-        </is>
-      </c>
-      <c r="AU55" s="4" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_6520.pdf</t>
-        </is>
-      </c>
-      <c r="AV55" s="4" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_6520.pdf</t>
-        </is>
-      </c>
-      <c r="AW55" s="4" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_6520.pdf</t>
-        </is>
-      </c>
-      <c r="AX55" s="4" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6520.pdf</t>
-        </is>
-      </c>
-      <c r="AY55" s="4" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6520.pdf</t>
-        </is>
-      </c>
-      <c r="AZ55" s="4" t="inlineStr">
-        <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_6520.pdf</t>
-        </is>
-      </c>
+      <c r="AQ55" s="4" t="inlineStr"/>
+      <c r="AR55" s="4" t="inlineStr"/>
+      <c r="AS55" s="4" t="inlineStr"/>
+      <c r="AT55" s="4" t="inlineStr"/>
+      <c r="AU55" s="4" t="inlineStr"/>
+      <c r="AV55" s="4" t="inlineStr"/>
+      <c r="AW55" s="4" t="inlineStr"/>
+      <c r="AX55" s="4" t="inlineStr"/>
+      <c r="AY55" s="4" t="inlineStr"/>
+      <c r="AZ55" s="4" t="inlineStr"/>
       <c r="BA55" s="4" t="inlineStr"/>
       <c r="BB55" s="4" t="inlineStr"/>
     </row>
@@ -14800,32 +14524,32 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E56" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F56" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G56" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H56" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,45238300</t>
+        </is>
+      </c>
+      <c r="E56" s="7" t="inlineStr">
+        <is>
+          <t>-0,010</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>0,44</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr">
+        <is>
+          <t>8,47</t>
+        </is>
+      </c>
+      <c r="H56" s="3" t="inlineStr">
+        <is>
+          <t>14,37</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>65,035</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
@@ -15077,7 +14801,7 @@
       </c>
       <c r="I57" s="4" t="inlineStr">
         <is>
-          <t>322,695</t>
+          <t>540,035</t>
         </is>
       </c>
       <c r="J57" s="4" t="inlineStr">
@@ -15316,32 +15040,32 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E58" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F58" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G58" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H58" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1.667,85353700</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>0,097</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>0,16</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="inlineStr">
+        <is>
+          <t>6,44</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr">
+        <is>
+          <t>12,06</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>113,126</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
@@ -15597,7 +15321,7 @@
       </c>
       <c r="I59" s="4" t="inlineStr">
         <is>
-          <t>14,680</t>
+          <t>14,678</t>
         </is>
       </c>
       <c r="J59" s="4" t="inlineStr">
@@ -16080,32 +15804,32 @@
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E61" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F61" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G61" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H61" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,26991800</t>
+        </is>
+      </c>
+      <c r="E61" s="5" t="inlineStr">
+        <is>
+          <t>0,491</t>
+        </is>
+      </c>
+      <c r="F61" s="5" t="inlineStr">
+        <is>
+          <t>0,26</t>
+        </is>
+      </c>
+      <c r="G61" s="5" t="inlineStr">
+        <is>
+          <t>3,97</t>
+        </is>
+      </c>
+      <c r="H61" s="5" t="inlineStr">
+        <is>
+          <t>9,79</t>
         </is>
       </c>
       <c r="I61" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>5,273</t>
         </is>
       </c>
       <c r="J61" s="4" t="inlineStr">
@@ -16844,32 +16568,32 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E64" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F64" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G64" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H64" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,35897000</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="inlineStr">
+        <is>
+          <t>0,188</t>
+        </is>
+      </c>
+      <c r="F64" s="7" t="inlineStr">
+        <is>
+          <t>-1,92</t>
+        </is>
+      </c>
+      <c r="G64" s="7" t="inlineStr">
+        <is>
+          <t>-0,44</t>
+        </is>
+      </c>
+      <c r="H64" s="3" t="inlineStr">
+        <is>
+          <t>9,67</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10,904</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
@@ -17377,7 +17101,7 @@
       </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>3,137</t>
+          <t>3,131</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr">
@@ -17608,32 +17332,32 @@
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E67" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F67" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G67" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H67" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>5,44766800</t>
+        </is>
+      </c>
+      <c r="E67" s="5" t="inlineStr">
+        <is>
+          <t>0,078</t>
+        </is>
+      </c>
+      <c r="F67" s="5" t="inlineStr">
+        <is>
+          <t>0,08</t>
+        </is>
+      </c>
+      <c r="G67" s="5" t="inlineStr">
+        <is>
+          <t>6,16</t>
+        </is>
+      </c>
+      <c r="H67" s="5" t="inlineStr">
+        <is>
+          <t>11,93</t>
         </is>
       </c>
       <c r="I67" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>32,483</t>
         </is>
       </c>
       <c r="J67" s="4" t="inlineStr">
@@ -17868,32 +17592,32 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E68" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F68" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G68" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H68" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1.285,56920200</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="inlineStr">
+        <is>
+          <t>0,909</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
+          <t>5,10</t>
+        </is>
+      </c>
+      <c r="G68" s="3" t="inlineStr">
+        <is>
+          <t>2,45</t>
+        </is>
+      </c>
+      <c r="H68" s="3" t="inlineStr">
+        <is>
+          <t>6,56</t>
         </is>
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>38,949</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr">
@@ -18163,7 +17887,7 @@
       </c>
       <c r="I69" s="4" t="inlineStr">
         <is>
-          <t>543,136</t>
+          <t>542,423</t>
         </is>
       </c>
       <c r="J69" s="4" t="inlineStr">
@@ -18398,32 +18122,32 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E70" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F70" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G70" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H70" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>2,88588000</t>
+        </is>
+      </c>
+      <c r="E70" s="3" t="inlineStr">
+        <is>
+          <t>0,130</t>
+        </is>
+      </c>
+      <c r="F70" s="3" t="inlineStr">
+        <is>
+          <t>0,86</t>
+        </is>
+      </c>
+      <c r="G70" s="3" t="inlineStr">
+        <is>
+          <t>3,32</t>
+        </is>
+      </c>
+      <c r="H70" s="3" t="inlineStr">
+        <is>
+          <t>8,49</t>
         </is>
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>70,724</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
@@ -18679,7 +18403,7 @@
       </c>
       <c r="I71" s="4" t="inlineStr">
         <is>
-          <t>30,712</t>
+          <t>30,705</t>
         </is>
       </c>
       <c r="J71" s="4" t="inlineStr">
@@ -18939,7 +18663,7 @@
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>2.488,904</t>
+          <t>2.488,760</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr">
@@ -19434,32 +19158,32 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E74" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F74" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G74" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H74" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1.692,44442300</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="inlineStr">
+        <is>
+          <t>0,100</t>
+        </is>
+      </c>
+      <c r="F74" s="3" t="inlineStr">
+        <is>
+          <t>0,19</t>
+        </is>
+      </c>
+      <c r="G74" s="3" t="inlineStr">
+        <is>
+          <t>7,01</t>
+        </is>
+      </c>
+      <c r="H74" s="3" t="inlineStr">
+        <is>
+          <t>13,03</t>
         </is>
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14,181</t>
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr">
@@ -19715,7 +19439,7 @@
       </c>
       <c r="I75" s="4" t="inlineStr">
         <is>
-          <t>901,878</t>
+          <t>900,912</t>
         </is>
       </c>
       <c r="J75" s="4" t="inlineStr">
@@ -19950,32 +19674,32 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E76" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F76" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G76" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>0,46633000</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="inlineStr">
+        <is>
+          <t>0,369</t>
+        </is>
+      </c>
+      <c r="F76" s="3" t="inlineStr">
+        <is>
+          <t>2,28</t>
+        </is>
+      </c>
+      <c r="G76" s="7" t="inlineStr">
+        <is>
+          <t>-35,41</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3,728</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr">
@@ -20242,7 +19966,7 @@
       </c>
       <c r="I77" s="4" t="inlineStr">
         <is>
-          <t>720,066</t>
+          <t>720,065</t>
         </is>
       </c>
       <c r="J77" s="4" t="inlineStr">
@@ -20473,32 +20197,32 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E78" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F78" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G78" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H78" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,42004300</t>
+        </is>
+      </c>
+      <c r="E78" s="3" t="inlineStr">
+        <is>
+          <t>0,278</t>
+        </is>
+      </c>
+      <c r="F78" s="7" t="inlineStr">
+        <is>
+          <t>-0,09</t>
+        </is>
+      </c>
+      <c r="G78" s="3" t="inlineStr">
+        <is>
+          <t>4,71</t>
+        </is>
+      </c>
+      <c r="H78" s="3" t="inlineStr">
+        <is>
+          <t>9,03</t>
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>72,770</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr">
@@ -20741,32 +20465,32 @@
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E79" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F79" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G79" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H79" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,51502500</t>
+        </is>
+      </c>
+      <c r="E79" s="5" t="inlineStr">
+        <is>
+          <t>0,048</t>
+        </is>
+      </c>
+      <c r="F79" s="5" t="inlineStr">
+        <is>
+          <t>0,43</t>
+        </is>
+      </c>
+      <c r="G79" s="5" t="inlineStr">
+        <is>
+          <t>4,76</t>
+        </is>
+      </c>
+      <c r="H79" s="5" t="inlineStr">
+        <is>
+          <t>11,75</t>
         </is>
       </c>
       <c r="I79" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>196,439</t>
         </is>
       </c>
       <c r="J79" s="4" t="inlineStr">
@@ -20801,7 +20525,7 @@
       </c>
       <c r="P79" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-capital-protegido-ciclico-ii-multimercado-lp/Paginas/default.aspx</t>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/caixa-fic-fim-cap-protegido-ciclico-ii</t>
         </is>
       </c>
       <c r="Q79" s="4" t="inlineStr">
@@ -21009,32 +20733,32 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E80" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F80" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G80" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H80" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>3,38602300</t>
+        </is>
+      </c>
+      <c r="E80" s="7" t="inlineStr">
+        <is>
+          <t>-1,319</t>
+        </is>
+      </c>
+      <c r="F80" s="3" t="inlineStr">
+        <is>
+          <t>0,47</t>
+        </is>
+      </c>
+      <c r="G80" s="3" t="inlineStr">
+        <is>
+          <t>6,27</t>
+        </is>
+      </c>
+      <c r="H80" s="3" t="inlineStr">
+        <is>
+          <t>9,85</t>
         </is>
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>161,271</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr">
@@ -21275,32 +20999,32 @@
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E81" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F81" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G81" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H81" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,58148300</t>
+        </is>
+      </c>
+      <c r="E81" s="6" t="inlineStr">
+        <is>
+          <t>-0,042</t>
+        </is>
+      </c>
+      <c r="F81" s="5" t="inlineStr">
+        <is>
+          <t>0,32</t>
+        </is>
+      </c>
+      <c r="G81" s="5" t="inlineStr">
+        <is>
+          <t>5,91</t>
+        </is>
+      </c>
+      <c r="H81" s="5" t="inlineStr">
+        <is>
+          <t>22,91</t>
         </is>
       </c>
       <c r="I81" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14,899</t>
         </is>
       </c>
       <c r="J81" s="4" t="inlineStr">
@@ -21541,32 +21265,32 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E82" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F82" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G82" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H82" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>6,85423500</t>
+        </is>
+      </c>
+      <c r="E82" s="7" t="inlineStr">
+        <is>
+          <t>-0,142</t>
+        </is>
+      </c>
+      <c r="F82" s="7" t="inlineStr">
+        <is>
+          <t>-0,02</t>
+        </is>
+      </c>
+      <c r="G82" s="3" t="inlineStr">
+        <is>
+          <t>6,57</t>
+        </is>
+      </c>
+      <c r="H82" s="3" t="inlineStr">
+        <is>
+          <t>13,69</t>
         </is>
       </c>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>125,638</t>
         </is>
       </c>
       <c r="J82" s="2" t="inlineStr">
@@ -21797,32 +21521,32 @@
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E83" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F83" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G83" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H83" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,83393300</t>
+        </is>
+      </c>
+      <c r="E83" s="5" t="inlineStr">
+        <is>
+          <t>0,429</t>
+        </is>
+      </c>
+      <c r="F83" s="5" t="inlineStr">
+        <is>
+          <t>1,69</t>
+        </is>
+      </c>
+      <c r="G83" s="5" t="inlineStr">
+        <is>
+          <t>3,81</t>
+        </is>
+      </c>
+      <c r="H83" s="5" t="inlineStr">
+        <is>
+          <t>10,03</t>
         </is>
       </c>
       <c r="I83" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>171,397</t>
         </is>
       </c>
       <c r="J83" s="4" t="inlineStr">
@@ -22053,32 +21777,32 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E84" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F84" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G84" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H84" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,44881800</t>
+        </is>
+      </c>
+      <c r="E84" s="7" t="inlineStr">
+        <is>
+          <t>-0,003</t>
+        </is>
+      </c>
+      <c r="F84" s="3" t="inlineStr">
+        <is>
+          <t>0,94</t>
+        </is>
+      </c>
+      <c r="G84" s="3" t="inlineStr">
+        <is>
+          <t>5,16</t>
+        </is>
+      </c>
+      <c r="H84" s="3" t="inlineStr">
+        <is>
+          <t>12,27</t>
         </is>
       </c>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>280,761</t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr">
@@ -22314,32 +22038,32 @@
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E85" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F85" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G85" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H85" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,44083500</t>
+        </is>
+      </c>
+      <c r="E85" s="5" t="inlineStr">
+        <is>
+          <t>0,556</t>
+        </is>
+      </c>
+      <c r="F85" s="5" t="inlineStr">
+        <is>
+          <t>4,37</t>
+        </is>
+      </c>
+      <c r="G85" s="5" t="inlineStr">
+        <is>
+          <t>12,25</t>
+        </is>
+      </c>
+      <c r="H85" s="5" t="inlineStr">
+        <is>
+          <t>11,08</t>
         </is>
       </c>
       <c r="I85" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12,966</t>
         </is>
       </c>
       <c r="J85" s="4" t="inlineStr">
@@ -22599,7 +22323,7 @@
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>97,612</t>
+          <t>97,589</t>
         </is>
       </c>
       <c r="J86" s="2" t="inlineStr">
@@ -22859,7 +22583,7 @@
       </c>
       <c r="I87" s="4" t="inlineStr">
         <is>
-          <t>311,288</t>
+          <t>311,248</t>
         </is>
       </c>
       <c r="J87" s="4" t="inlineStr">
@@ -23635,7 +23359,7 @@
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>8,722</t>
+          <t>8,700</t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr">
@@ -23884,7 +23608,7 @@
       </c>
       <c r="I91" s="4" t="inlineStr">
         <is>
-          <t>282,392</t>
+          <t>282,280</t>
         </is>
       </c>
       <c r="J91" s="4" t="inlineStr">
@@ -24144,7 +23868,7 @@
       </c>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>394,628</t>
+          <t>394,610</t>
         </is>
       </c>
       <c r="J92" s="2" t="inlineStr">
@@ -24404,7 +24128,7 @@
       </c>
       <c r="I93" s="4" t="inlineStr">
         <is>
-          <t>49,963</t>
+          <t>49,962</t>
         </is>
       </c>
       <c r="J93" s="4" t="inlineStr">
@@ -25184,7 +24908,7 @@
       </c>
       <c r="I96" s="2" t="inlineStr">
         <is>
-          <t>82,823</t>
+          <t>82,822</t>
         </is>
       </c>
       <c r="J96" s="2" t="inlineStr">
@@ -25419,32 +25143,32 @@
       </c>
       <c r="D97" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E97" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F97" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G97" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H97" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,19984400</t>
+        </is>
+      </c>
+      <c r="E97" s="5" t="inlineStr">
+        <is>
+          <t>0,551</t>
+        </is>
+      </c>
+      <c r="F97" s="6" t="inlineStr">
+        <is>
+          <t>-5,70</t>
+        </is>
+      </c>
+      <c r="G97" s="6" t="inlineStr">
+        <is>
+          <t>-6,77</t>
+        </is>
+      </c>
+      <c r="H97" s="5" t="inlineStr">
+        <is>
+          <t>4,53</t>
         </is>
       </c>
       <c r="I97" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>267,798</t>
         </is>
       </c>
       <c r="J97" s="4" t="inlineStr">
@@ -25704,7 +25428,7 @@
       </c>
       <c r="I98" s="2" t="inlineStr">
         <is>
-          <t>100,267</t>
+          <t>100,228</t>
         </is>
       </c>
       <c r="J98" s="2" t="inlineStr">
@@ -25964,7 +25688,7 @@
       </c>
       <c r="I99" s="4" t="inlineStr">
         <is>
-          <t>111,507</t>
+          <t>111,494</t>
         </is>
       </c>
       <c r="J99" s="4" t="inlineStr">
@@ -26224,7 +25948,7 @@
       </c>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t>44,814</t>
+          <t>44,813</t>
         </is>
       </c>
       <c r="J100" s="2" t="inlineStr">
@@ -26488,7 +26212,7 @@
       </c>
       <c r="I101" s="4" t="inlineStr">
         <is>
-          <t>116,754</t>
+          <t>116,729</t>
         </is>
       </c>
       <c r="J101" s="4" t="inlineStr">
@@ -26748,7 +26472,7 @@
       </c>
       <c r="I102" s="2" t="inlineStr">
         <is>
-          <t>36,930</t>
+          <t>36,920</t>
         </is>
       </c>
       <c r="J102" s="2" t="inlineStr">
@@ -27008,7 +26732,7 @@
       </c>
       <c r="I103" s="4" t="inlineStr">
         <is>
-          <t>592,117</t>
+          <t>591,346</t>
         </is>
       </c>
       <c r="J103" s="4" t="inlineStr">
@@ -27268,7 +26992,7 @@
       </c>
       <c r="I104" s="2" t="inlineStr">
         <is>
-          <t>449,259</t>
+          <t>448,247</t>
         </is>
       </c>
       <c r="J104" s="2" t="inlineStr">
@@ -27532,7 +27256,7 @@
       </c>
       <c r="I105" s="4" t="inlineStr">
         <is>
-          <t>22,435</t>
+          <t>22,399</t>
         </is>
       </c>
       <c r="J105" s="4" t="inlineStr">
@@ -27792,7 +27516,7 @@
       </c>
       <c r="I106" s="2" t="inlineStr">
         <is>
-          <t>28,865</t>
+          <t>28,863</t>
         </is>
       </c>
       <c r="J106" s="2" t="inlineStr">
@@ -28052,7 +27776,7 @@
       </c>
       <c r="I107" s="4" t="inlineStr">
         <is>
-          <t>1,648</t>
+          <t>1,643</t>
         </is>
       </c>
       <c r="J107" s="4" t="inlineStr">
@@ -28556,7 +28280,7 @@
       </c>
       <c r="I109" s="4" t="inlineStr">
         <is>
-          <t>33,203</t>
+          <t>31,761</t>
         </is>
       </c>
       <c r="J109" s="4" t="inlineStr">
@@ -28816,7 +28540,7 @@
       </c>
       <c r="I110" s="2" t="inlineStr">
         <is>
-          <t>825,124</t>
+          <t>825,033</t>
         </is>
       </c>
       <c r="J110" s="2" t="inlineStr">
@@ -29492,12 +29216,12 @@
       </c>
       <c r="Q113" s="4" t="inlineStr">
         <is>
-          <t>59.815.671/0001-53</t>
+          <t>30.068.049/0001-47</t>
         </is>
       </c>
       <c r="R113" s="4" t="inlineStr">
         <is>
-          <t>7971</t>
+          <t>6499</t>
         </is>
       </c>
       <c r="S113" s="4" t="inlineStr">
@@ -29532,7 +29256,7 @@
       </c>
       <c r="Y113" s="4" t="inlineStr">
         <is>
-          <t>D+0 (du)</t>
+          <t>D+1 (du)</t>
         </is>
       </c>
       <c r="Z113" s="4" t="inlineStr">
@@ -29547,7 +29271,7 @@
       </c>
       <c r="AB113" s="4" t="inlineStr">
         <is>
-          <t>NÃO SE APLICA</t>
+          <t>IBOV</t>
         </is>
       </c>
       <c r="AC113" s="4" t="inlineStr">
@@ -29557,7 +29281,7 @@
       </c>
       <c r="AD113" s="4" t="inlineStr">
         <is>
-          <t>Fechado para captação</t>
+          <t>Aberto para captação</t>
         </is>
       </c>
       <c r="AE113" s="4" t="inlineStr">
@@ -29582,23 +29306,27 @@
       </c>
       <c r="AI113" s="4" t="inlineStr">
         <is>
-          <t>Não se aplica</t>
+          <t>Sim · Automatico · 100%</t>
         </is>
       </c>
       <c r="AJ113" s="4" t="inlineStr">
         <is>
-          <t>NÃO SE APLICA</t>
-        </is>
-      </c>
-      <c r="AK113" s="4" t="inlineStr"/>
+          <t>AUTOMATICO</t>
+        </is>
+      </c>
+      <c r="AK113" s="4" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
       <c r="AL113" s="4" t="inlineStr">
         <is>
-          <t>["GOV", "Pessoa Física", "PJ Atacado", "Private"]</t>
+          <t>["GOV", "Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private"]</t>
         </is>
       </c>
       <c r="AM113" s="4" t="inlineStr">
         <is>
-          <t>["GOV", "Pessoa Física", "PJ Atacado", "Private"]</t>
+          <t>["GOV", "Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private"]</t>
         </is>
       </c>
       <c r="AN113" s="4" t="inlineStr">
@@ -29613,7 +29341,7 @@
       </c>
       <c r="AP113" s="4" t="inlineStr">
         <is>
-          <t>2025-05-04T00:00:00Z</t>
+          <t>2021-06-13T00:00:00Z</t>
         </is>
       </c>
       <c r="AQ113" s="4" t="inlineStr">
@@ -29623,47 +29351,47 @@
       </c>
       <c r="AR113" s="4" t="inlineStr">
         <is>
-          <t>CAIXA SEGURIDADE II FUNDO DE INVESTIMENTO FINANCEIRO AÇÕES - RESPONSABILIDADE LIMITADA</t>
+          <t>CAIXA SEGURIDADE FUNDO DE INVESTIMENTO FINANCEIRO EM AÇÕES - RESPONSABILIDADE LIMITADA</t>
         </is>
       </c>
       <c r="AS113" s="4" t="inlineStr">
         <is>
-          <t>Fundo ficará fechado para novas aplicações a partir do dia 13/05/2025 (inclusive).</t>
+          <t>Canal de distribuição: Rede CAIXA, IBC. A reserva inicial, no âmbito da OFERTA, será feita por meio do Home Broker CAIXA. Resgates: Lock up de 45 dias. Inicio dia 30/04/2021 - Termino 13/06/2021. Liberado resgate a partir do dia 14/06/2021 (segunda-feira).</t>
         </is>
       </c>
       <c r="AT113" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_7971.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_6499.pdf</t>
         </is>
       </c>
       <c r="AU113" s="4" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_7971.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_6499.pdf</t>
         </is>
       </c>
       <c r="AV113" s="4" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_7971.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_6499.pdf</t>
         </is>
       </c>
       <c r="AW113" s="4" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_7971.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_6499.pdf</t>
         </is>
       </c>
       <c r="AX113" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_7971.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6499.pdf</t>
         </is>
       </c>
       <c r="AY113" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_7971.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6499.pdf</t>
         </is>
       </c>
       <c r="AZ113" s="4" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_7971.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_6499.pdf</t>
         </is>
       </c>
       <c r="BA113" s="4" t="inlineStr"/>
@@ -29712,7 +29440,7 @@
       </c>
       <c r="I114" s="2" t="inlineStr">
         <is>
-          <t>253,736</t>
+          <t>253,097</t>
         </is>
       </c>
       <c r="J114" s="2" t="inlineStr">
@@ -29951,32 +29679,32 @@
       </c>
       <c r="D115" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E115" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F115" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G115" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H115" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>960,87813200</t>
+        </is>
+      </c>
+      <c r="E115" s="5" t="inlineStr">
+        <is>
+          <t>0,167</t>
+        </is>
+      </c>
+      <c r="F115" s="6" t="inlineStr">
+        <is>
+          <t>-4,75</t>
+        </is>
+      </c>
+      <c r="G115" s="6" t="inlineStr">
+        <is>
+          <t>-1,98</t>
+        </is>
+      </c>
+      <c r="H115" s="5" t="inlineStr">
+        <is>
+          <t>12,20</t>
         </is>
       </c>
       <c r="I115" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>7,705</t>
         </is>
       </c>
       <c r="J115" s="4" t="inlineStr">
@@ -30071,32 +29799,32 @@
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E116" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F116" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G116" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H116" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1.410,04317100</t>
+        </is>
+      </c>
+      <c r="E116" s="3" t="inlineStr">
+        <is>
+          <t>0,285</t>
+        </is>
+      </c>
+      <c r="F116" s="7" t="inlineStr">
+        <is>
+          <t>-6,20</t>
+        </is>
+      </c>
+      <c r="G116" s="7" t="inlineStr">
+        <is>
+          <t>-5,73</t>
+        </is>
+      </c>
+      <c r="H116" s="3" t="inlineStr">
+        <is>
+          <t>6,23</t>
         </is>
       </c>
       <c r="I116" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>20,273</t>
         </is>
       </c>
       <c r="J116" s="2" t="inlineStr">
@@ -30327,7 +30055,7 @@
       </c>
       <c r="D117" s="4" t="inlineStr">
         <is>
-          <t>163,43781900</t>
+          <t>163,43781872</t>
         </is>
       </c>
       <c r="E117" s="6" t="inlineStr">
@@ -30869,7 +30597,7 @@
       </c>
       <c r="I119" s="4" t="inlineStr">
         <is>
-          <t>1.510,717</t>
+          <t>1.510,410</t>
         </is>
       </c>
       <c r="J119" s="4" t="inlineStr">
@@ -31122,7 +30850,7 @@
       </c>
       <c r="I120" s="2" t="inlineStr">
         <is>
-          <t>668,664</t>
+          <t>668,626</t>
         </is>
       </c>
       <c r="J120" s="2" t="inlineStr">
@@ -31157,17 +30885,17 @@
       </c>
       <c r="P120" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/fundos-investimento/mutuos-privatizacao/fmp-fgts-petrobas-4</t>
+          <t>http://www.caixa.gov.br/fundos-investimento/mutuos-privatizacao/fmp-fgts-petrobas-2</t>
         </is>
       </c>
       <c r="Q120" s="2" t="inlineStr">
         <is>
-          <t>03.555.959/0001-81</t>
+          <t>03.915.910/0001-92</t>
         </is>
       </c>
       <c r="R120" s="2" t="inlineStr">
         <is>
-          <t>5204</t>
+          <t>5202</t>
         </is>
       </c>
       <c r="S120" s="2" t="inlineStr">
@@ -31177,12 +30905,12 @@
       </c>
       <c r="T120" s="2" t="inlineStr">
         <is>
-          <t>0.95</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="U120" s="2" t="inlineStr">
         <is>
-          <t>300.0</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="V120" s="2" t="inlineStr">
@@ -31227,7 +30955,7 @@
       </c>
       <c r="AD120" s="2" t="inlineStr">
         <is>
-          <t>Fechado para captação</t>
+          <t>Aberto para captação</t>
         </is>
       </c>
       <c r="AE120" s="2" t="inlineStr">
@@ -31240,7 +30968,11 @@
           <t>GERAL</t>
         </is>
       </c>
-      <c r="AG120" s="2" t="inlineStr"/>
+      <c r="AG120" s="2" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
       <c r="AH120" s="2" t="inlineStr">
         <is>
           <t>17h00</t>
@@ -31277,47 +31009,48 @@
       </c>
       <c r="AR120" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FUNDO MÚTUO DE PRIVATIZAÇÃO - FGTS - PETROBRAS IV - RESPONSABILIDADE LIMITADA</t>
+          <t>CAIXA FUNDO MÚTUO DE PRIVATIZAÇÃO - FGTS - PETROBRAS II - RESPONSABILIDADE LIMITADA</t>
         </is>
       </c>
       <c r="AS120" s="2" t="inlineStr">
         <is>
-          <t>FUNDO FECHADO.</t>
+          <t>O fundo encontra-se aberto para receber recursos provenientes de outros Fundos FMP-FGTS.
+Prazo de carência: 6 meses para transferência total ou parcial do investimento no FUNDO para outro FMP- FGTS ou para um Clube de Investimento – FGTS, ou 12 meses para retorno à(s) conta(s) vinculada(s) do investidor junto ao FGTS.</t>
         </is>
       </c>
       <c r="AT120" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5204.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5202.pdf</t>
         </is>
       </c>
       <c r="AU120" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5204.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5202.pdf</t>
         </is>
       </c>
       <c r="AV120" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5204.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5202.pdf</t>
         </is>
       </c>
       <c r="AW120" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5204.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5202.pdf</t>
         </is>
       </c>
       <c r="AX120" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5204.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5202.pdf</t>
         </is>
       </c>
       <c r="AY120" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5204.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5202.pdf</t>
         </is>
       </c>
       <c r="AZ120" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5204.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5202.pdf</t>
         </is>
       </c>
       <c r="BA120" s="2" t="inlineStr"/>
@@ -31366,7 +31099,7 @@
       </c>
       <c r="I121" s="4" t="inlineStr">
         <is>
-          <t>684,500</t>
+          <t>684,108</t>
         </is>
       </c>
       <c r="J121" s="4" t="inlineStr">
@@ -31610,7 +31343,7 @@
       </c>
       <c r="I122" s="2" t="inlineStr">
         <is>
-          <t>101,910</t>
+          <t>101,897</t>
         </is>
       </c>
       <c r="J122" s="2" t="inlineStr">
@@ -32112,7 +31845,7 @@
       </c>
       <c r="I124" s="2" t="inlineStr">
         <is>
-          <t>576,446</t>
+          <t>576,096</t>
         </is>
       </c>
       <c r="J124" s="2" t="inlineStr">
@@ -32361,7 +32094,7 @@
       </c>
       <c r="I125" s="4" t="inlineStr">
         <is>
-          <t>412,415</t>
+          <t>412,108</t>
         </is>
       </c>
       <c r="J125" s="4" t="inlineStr">
@@ -32605,7 +32338,7 @@
       </c>
       <c r="I126" s="2" t="inlineStr">
         <is>
-          <t>659,147</t>
+          <t>656,957</t>
         </is>
       </c>
       <c r="J126" s="2" t="inlineStr">
@@ -33114,7 +32847,7 @@
       </c>
       <c r="I128" s="2" t="inlineStr">
         <is>
-          <t>215,680</t>
+          <t>203,239</t>
         </is>
       </c>
       <c r="J128" s="2" t="inlineStr">
@@ -34423,7 +34156,7 @@
       </c>
       <c r="I133" s="4" t="inlineStr">
         <is>
-          <t>8.152,897</t>
+          <t>8.002,241</t>
         </is>
       </c>
       <c r="J133" s="4" t="inlineStr">
@@ -34684,7 +34417,7 @@
       </c>
       <c r="I134" s="2" t="inlineStr">
         <is>
-          <t>2.962,433</t>
+          <t>2.962,428</t>
         </is>
       </c>
       <c r="J134" s="2" t="inlineStr">
@@ -34944,7 +34677,7 @@
       </c>
       <c r="I135" s="4" t="inlineStr">
         <is>
-          <t>16.933,787</t>
+          <t>16.933,521</t>
         </is>
       </c>
       <c r="J135" s="4" t="inlineStr">
@@ -35179,7 +34912,7 @@
       </c>
       <c r="D136" s="2" t="inlineStr">
         <is>
-          <t>1,59001300</t>
+          <t>1,59001321</t>
         </is>
       </c>
       <c r="E136" s="3" t="inlineStr">
@@ -35488,12 +35221,12 @@
       </c>
       <c r="Q137" s="4" t="inlineStr">
         <is>
-          <t>09.548.725/0001-93</t>
+          <t>09.181.268/0001-41</t>
         </is>
       </c>
       <c r="R137" s="4" t="inlineStr">
         <is>
-          <t>5132</t>
+          <t>5080</t>
         </is>
       </c>
       <c r="S137" s="4" t="inlineStr">
@@ -35503,12 +35236,12 @@
       </c>
       <c r="T137" s="4" t="inlineStr">
         <is>
-          <t>0.07</t>
+          <t>0.35</t>
         </is>
       </c>
       <c r="U137" s="4" t="inlineStr">
         <is>
-          <t>10000000.0</t>
+          <t>1000.0</t>
         </is>
       </c>
       <c r="V137" s="4" t="inlineStr">
@@ -35523,7 +35256,7 @@
       </c>
       <c r="X137" s="4" t="inlineStr">
         <is>
-          <t>0.01</t>
+          <t>100.0</t>
         </is>
       </c>
       <c r="Y137" s="4" t="inlineStr">
@@ -35563,7 +35296,7 @@
       </c>
       <c r="AF137" s="4" t="inlineStr">
         <is>
-          <t>QUALIFICADO</t>
+          <t>GERAL</t>
         </is>
       </c>
       <c r="AG137" s="4" t="inlineStr">
@@ -35611,7 +35344,7 @@
       </c>
       <c r="AR137" s="4" t="inlineStr">
         <is>
-          <t>CAIXA SAUDE SUPLEMENTAR - ANS II FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
+          <t>CAIXA SAÚDE SUPLEMENTAR - ANS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
         </is>
       </c>
       <c r="AS137" s="4" t="inlineStr">
@@ -35626,37 +35359,37 @@
       </c>
       <c r="AT137" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5132.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5080.pdf</t>
         </is>
       </c>
       <c r="AU137" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5132.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5080.pdf</t>
         </is>
       </c>
       <c r="AV137" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5132.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5080.pdf</t>
         </is>
       </c>
       <c r="AW137" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5132.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5080.pdf</t>
         </is>
       </c>
       <c r="AX137" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5132.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5080.pdf</t>
         </is>
       </c>
       <c r="AY137" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5132.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5080.pdf</t>
         </is>
       </c>
       <c r="AZ137" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5132.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5080.pdf</t>
         </is>
       </c>
       <c r="BA137" s="4" t="inlineStr"/>
@@ -36449,7 +36182,7 @@
       </c>
       <c r="I141" s="4" t="inlineStr">
         <is>
-          <t>14.308,284</t>
+          <t>14.121,874</t>
         </is>
       </c>
       <c r="J141" s="4" t="inlineStr">
@@ -36710,7 +36443,7 @@
       </c>
       <c r="I142" s="2" t="inlineStr">
         <is>
-          <t>3.539,273</t>
+          <t>3.539,226</t>
         </is>
       </c>
       <c r="J142" s="2" t="inlineStr">
@@ -36966,7 +36699,7 @@
       </c>
       <c r="I143" s="4" t="inlineStr">
         <is>
-          <t>14.228,696</t>
+          <t>14.228,469</t>
         </is>
       </c>
       <c r="J143" s="4" t="inlineStr">
@@ -37461,42 +37194,42 @@
       </c>
       <c r="B145" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF PRÁTICO RF CURTO PRAZO RESP LTDA</t>
+          <t>CAIXA FIC FIF AUTOMATICO POLIS RF CURTO PRAZO RESP LTDA</t>
         </is>
       </c>
       <c r="C145" s="4" t="inlineStr">
         <is>
-          <t>02/10/1995</t>
+          <t>13/06/2023</t>
         </is>
       </c>
       <c r="D145" s="4" t="inlineStr">
         <is>
-          <t>9,62018100</t>
+          <t>1,33601300</t>
         </is>
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t>0,044</t>
+          <t>0,041</t>
         </is>
       </c>
       <c r="F145" s="5" t="inlineStr">
         <is>
-          <t>0,40</t>
+          <t>0,37</t>
         </is>
       </c>
       <c r="G145" s="5" t="inlineStr">
         <is>
-          <t>7,47</t>
+          <t>6,95</t>
         </is>
       </c>
       <c r="H145" s="5" t="inlineStr">
         <is>
-          <t>12,55</t>
+          <t>11,66</t>
         </is>
       </c>
       <c r="I145" s="4" t="inlineStr">
         <is>
-          <t>2.774,955</t>
+          <t>33.397,540</t>
         </is>
       </c>
       <c r="J145" s="4" t="inlineStr">
@@ -37526,22 +37259,22 @@
       </c>
       <c r="O145" s="4" t="inlineStr">
         <is>
-          <t>GOV | TODOS</t>
+          <t>GOV</t>
         </is>
       </c>
       <c r="P145" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/fundos-investimento/curto-prazo/fic-pratico-curto-prazo</t>
+          <t>https://www.caixa.gov.br/fundos-investimento/curto-prazo/fic-automatico-polis-rf-cp/Paginas/default.aspx</t>
         </is>
       </c>
       <c r="Q145" s="4" t="inlineStr">
         <is>
-          <t>00.834.074/0001-23</t>
+          <t>50.803.936/0001-29</t>
         </is>
       </c>
       <c r="R145" s="4" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>7869</t>
         </is>
       </c>
       <c r="S145" s="4" t="inlineStr">
@@ -37591,7 +37324,7 @@
       </c>
       <c r="AB145" s="4" t="inlineStr">
         <is>
-          <t>CDI</t>
+          <t>NÃO SE APLICA</t>
         </is>
       </c>
       <c r="AC145" s="4" t="inlineStr">
@@ -37601,7 +37334,7 @@
       </c>
       <c r="AD145" s="4" t="inlineStr">
         <is>
-          <t>Fechado para captação</t>
+          <t>Aberto para captação</t>
         </is>
       </c>
       <c r="AE145" s="4" t="inlineStr">
@@ -37663,12 +37396,12 @@
       </c>
       <c r="AR145" s="4" t="inlineStr">
         <is>
-          <t>CAIXA PRÁTICO FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA CURTO PRAZO - RESPONSABILIDADE LIMITADA</t>
+          <t>CAIXA AUTOMÁTICO POLIS FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA CURTO PRAZO - RESPONSABILIDADE LIMITADA</t>
         </is>
       </c>
       <c r="AS145" s="4" t="inlineStr">
         <is>
-          <t>Movimentações: O FUNDO oferece mecanismo resgate automático.
+          <t>Movimentações: O FUNDO oferece mecanismo de aplicação e resgate automáticos, exigindo a manutenção de um saldo em caixa adequado para suportar movimentações ocorridas após o fechamento do mercado.
 Para ativar a funcionalidade de Resgate Automático, acessar o SIART -&gt; Movimentação Automática -&gt; Marcar
 As regras da funcionalidade de Movimentação Automática estão descritas no MN TE099.
 **Esse fundo não possui adiantamento de resgate, os resgates efetuados ficarão disponíveis no processamento noturno.</t>
@@ -37676,37 +37409,37 @@
       </c>
       <c r="AT145" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_0055.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_7869.pdf</t>
         </is>
       </c>
       <c r="AU145" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_0055.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_7869.pdf</t>
         </is>
       </c>
       <c r="AV145" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_0055.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_7869.pdf</t>
         </is>
       </c>
       <c r="AW145" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_0055.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_7869.pdf</t>
         </is>
       </c>
       <c r="AX145" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_55.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_7869.pdf</t>
         </is>
       </c>
       <c r="AY145" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_55.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_7869.pdf</t>
         </is>
       </c>
       <c r="AZ145" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_0055.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_7869.pdf</t>
         </is>
       </c>
       <c r="BA145" s="4" t="inlineStr"/>
@@ -37720,42 +37453,42 @@
       </c>
       <c r="B146" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF AUTOMATICO POLIS RF CURTO PRAZO RESP LTDA</t>
+          <t>CAIXA FIC FIF PRÁTICO RF CURTO PRAZO RESP LTDA</t>
         </is>
       </c>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>13/06/2023</t>
+          <t>02/10/1995</t>
         </is>
       </c>
       <c r="D146" s="2" t="inlineStr">
         <is>
-          <t>1,33601300</t>
+          <t>9,62018100</t>
         </is>
       </c>
       <c r="E146" s="3" t="inlineStr">
         <is>
-          <t>0,041</t>
+          <t>0,044</t>
         </is>
       </c>
       <c r="F146" s="3" t="inlineStr">
         <is>
-          <t>0,37</t>
+          <t>0,40</t>
         </is>
       </c>
       <c r="G146" s="3" t="inlineStr">
         <is>
-          <t>6,95</t>
+          <t>7,47</t>
         </is>
       </c>
       <c r="H146" s="3" t="inlineStr">
         <is>
-          <t>11,66</t>
+          <t>12,55</t>
         </is>
       </c>
       <c r="I146" s="2" t="inlineStr">
         <is>
-          <t>33.538,459</t>
+          <t>2.746,101</t>
         </is>
       </c>
       <c r="J146" s="2" t="inlineStr">
@@ -37785,22 +37518,22 @@
       </c>
       <c r="O146" s="2" t="inlineStr">
         <is>
-          <t>GOV</t>
+          <t>GOV | TODOS</t>
         </is>
       </c>
       <c r="P146" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/fundos-investimento/curto-prazo/fic-automatico-polis-rf-cp/Paginas/default.aspx</t>
+          <t>https://www.caixa.gov.br/fundos-investimento/curto-prazo/fic-pratico-curto-prazo</t>
         </is>
       </c>
       <c r="Q146" s="2" t="inlineStr">
         <is>
-          <t>50.803.936/0001-29</t>
+          <t>00.834.074/0001-23</t>
         </is>
       </c>
       <c r="R146" s="2" t="inlineStr">
         <is>
-          <t>7869</t>
+          <t>55</t>
         </is>
       </c>
       <c r="S146" s="2" t="inlineStr">
@@ -37850,7 +37583,7 @@
       </c>
       <c r="AB146" s="2" t="inlineStr">
         <is>
-          <t>NÃO SE APLICA</t>
+          <t>CDI</t>
         </is>
       </c>
       <c r="AC146" s="2" t="inlineStr">
@@ -37860,7 +37593,7 @@
       </c>
       <c r="AD146" s="2" t="inlineStr">
         <is>
-          <t>Aberto para captação</t>
+          <t>Fechado para captação</t>
         </is>
       </c>
       <c r="AE146" s="2" t="inlineStr">
@@ -37922,12 +37655,12 @@
       </c>
       <c r="AR146" s="2" t="inlineStr">
         <is>
-          <t>CAIXA AUTOMÁTICO POLIS FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA CURTO PRAZO - RESPONSABILIDADE LIMITADA</t>
+          <t>CAIXA PRÁTICO FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA CURTO PRAZO - RESPONSABILIDADE LIMITADA</t>
         </is>
       </c>
       <c r="AS146" s="2" t="inlineStr">
         <is>
-          <t>Movimentações: O FUNDO oferece mecanismo de aplicação e resgate automáticos, exigindo a manutenção de um saldo em caixa adequado para suportar movimentações ocorridas após o fechamento do mercado.
+          <t>Movimentações: O FUNDO oferece mecanismo resgate automático.
 Para ativar a funcionalidade de Resgate Automático, acessar o SIART -&gt; Movimentação Automática -&gt; Marcar
 As regras da funcionalidade de Movimentação Automática estão descritas no MN TE099.
 **Esse fundo não possui adiantamento de resgate, os resgates efetuados ficarão disponíveis no processamento noturno.</t>
@@ -37935,37 +37668,37 @@
       </c>
       <c r="AT146" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_7869.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_0055.pdf</t>
         </is>
       </c>
       <c r="AU146" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_7869.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_0055.pdf</t>
         </is>
       </c>
       <c r="AV146" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_7869.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_0055.pdf</t>
         </is>
       </c>
       <c r="AW146" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_7869.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_0055.pdf</t>
         </is>
       </c>
       <c r="AX146" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_7869.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_55.pdf</t>
         </is>
       </c>
       <c r="AY146" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_7869.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_55.pdf</t>
         </is>
       </c>
       <c r="AZ146" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_7869.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_0055.pdf</t>
         </is>
       </c>
       <c r="BA146" s="2" t="inlineStr"/>
@@ -38014,7 +37747,7 @@
       </c>
       <c r="I147" s="4" t="inlineStr">
         <is>
-          <t>18.263,230</t>
+          <t>18.209,658</t>
         </is>
       </c>
       <c r="J147" s="4" t="inlineStr">
@@ -38275,7 +38008,7 @@
       </c>
       <c r="I148" s="2" t="inlineStr">
         <is>
-          <t>8.801,697</t>
+          <t>8.801,665</t>
         </is>
       </c>
       <c r="J148" s="2" t="inlineStr">
@@ -40373,7 +40106,7 @@
       </c>
       <c r="I156" s="2" t="inlineStr">
         <is>
-          <t>5.627,158</t>
+          <t>5.627,150</t>
         </is>
       </c>
       <c r="J156" s="2" t="inlineStr">
@@ -40629,7 +40362,7 @@
       </c>
       <c r="I157" s="4" t="inlineStr">
         <is>
-          <t>473,372</t>
+          <t>473,371</t>
         </is>
       </c>
       <c r="J157" s="4" t="inlineStr">
@@ -42314,7 +42047,7 @@
       </c>
       <c r="I164" s="2" t="inlineStr">
         <is>
-          <t>1.457,736</t>
+          <t>1.554,406</t>
         </is>
       </c>
       <c r="J164" s="2" t="inlineStr">
@@ -42928,32 +42661,32 @@
       </c>
       <c r="D167" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E167" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F167" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G167" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H167" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1.580,38341700</t>
+        </is>
+      </c>
+      <c r="E167" s="5" t="inlineStr">
+        <is>
+          <t>0,097</t>
+        </is>
+      </c>
+      <c r="F167" s="5" t="inlineStr">
+        <is>
+          <t>0,16</t>
+        </is>
+      </c>
+      <c r="G167" s="5" t="inlineStr">
+        <is>
+          <t>6,47</t>
+        </is>
+      </c>
+      <c r="H167" s="5" t="inlineStr">
+        <is>
+          <t>12,08</t>
         </is>
       </c>
       <c r="I167" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>130,783</t>
         </is>
       </c>
       <c r="J167" s="4" t="inlineStr">
@@ -43696,7 +43429,7 @@
       </c>
       <c r="D170" s="2" t="inlineStr">
         <is>
-          <t>11,97181100</t>
+          <t>11,97181068</t>
         </is>
       </c>
       <c r="E170" s="3" t="inlineStr">
@@ -44472,7 +44205,7 @@
       </c>
       <c r="D173" s="4" t="inlineStr">
         <is>
-          <t>3,32040800</t>
+          <t>3,32040837</t>
         </is>
       </c>
       <c r="E173" s="5" t="inlineStr">
@@ -44724,7 +44457,7 @@
       </c>
       <c r="D174" s="2" t="inlineStr">
         <is>
-          <t>2,37151400</t>
+          <t>2,37151405</t>
         </is>
       </c>
       <c r="E174" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Dados atualizados via Robô: 18/08/2026 14:34
</commit_message>
<xml_diff>
--- a/dados_atuais.xlsx
+++ b/dados_atuais.xlsx
@@ -2428,7 +2428,7 @@
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/debentures-incentivadas/caixa-smart-infraestrutura-debincentivadas-</t>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/debentures-incentivadas/caixa-smart-infraestrutura-debincentivadas-cdi-rf-cred-priv-lp-subclasse-varejo/Paginas/default.aspx</t>
         </is>
       </c>
       <c r="Q8" s="2" t="inlineStr">
@@ -20801,7 +20801,7 @@
       </c>
       <c r="P79" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-capital-protegido-ciclico-ii-multimercado-lp/Paginas/default.aspx</t>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/caixa-fic-fim-cap-protegido-ciclico-ii</t>
         </is>
       </c>
       <c r="Q79" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Dados atualizados via Robô: 19/08/2026 14:23
</commit_message>
<xml_diff>
--- a/dados_atuais.xlsx
+++ b/dados_atuais.xlsx
@@ -2498,7 +2498,7 @@
       </c>
       <c r="AD8" s="2" t="inlineStr">
         <is>
-          <t>Fechado para captação</t>
+          <t>Aberto para captação</t>
         </is>
       </c>
       <c r="AE8" s="2" t="inlineStr">
@@ -33293,7 +33293,7 @@
 PG - Estatal Corporativo;
 PP - Estatal Corporativo Ultra
 Movimentações: O FUNDO oferece mecanismo de aplicação e resgate automáticos, exigindo a manutenção de um saldo em caixa adequado para suportar movimentações ocorridas após o fechamento do mercado.
-Para ativar a funcionalidade de Resgate Automático, acessar o SIART -&gt; Movimentação Automática -&gt; Marcar
+Para ativar a funcionalidade de Aplicação e Resgate Automático, acessar o SIART -&gt; Movimentação Automática -&gt; Marcar
 As regras da funcionalidade de Movimentação Automática estão descritas no MN TE099.
 **Esse fundo não possui adiantamento de resgate, os resgates efetuados ficarão disponíveis no processamento noturno.</t>
         </is>
@@ -40157,12 +40157,12 @@
       </c>
       <c r="Q155" s="4" t="inlineStr">
         <is>
-          <t>11.060.913/0001-10</t>
+          <t>10.740.658/0001-93</t>
         </is>
       </c>
       <c r="R155" s="4" t="inlineStr">
         <is>
-          <t>5187</t>
+          <t>5184</t>
         </is>
       </c>
       <c r="S155" s="4" t="inlineStr">
@@ -40212,7 +40212,7 @@
       </c>
       <c r="AB155" s="4" t="inlineStr">
         <is>
-          <t>IMA-B 5</t>
+          <t>IMA-B TOTAL</t>
         </is>
       </c>
       <c r="AC155" s="4" t="inlineStr">
@@ -40288,43 +40288,49 @@
       </c>
       <c r="AR155" s="4" t="inlineStr">
         <is>
-          <t>CAIXA BRASIL IMA-B 5 TÍTULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
-        </is>
-      </c>
-      <c r="AS155" s="4" t="inlineStr"/>
+          <t>CAIXA BRASIL IMA-B TÍTULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
+        </is>
+      </c>
+      <c r="AS155" s="4" t="inlineStr">
+        <is>
+          <t>1. O Fundo tem como parâmetro de rentabilidade o Índice de Mercado ANBIMA série B (IMA-B).
+2. Para aplicação por meio de conta operação 1292, é necessário o cadastramento prévio de cotistas, conforme descrito no item Adesão, do FI612.
+3. O procedimento de inclusão da conta deverá ser realizado sempre que houver qualquer aplicação por meio de conta operação 1292, mesmo para os clientes que já realizaram o cadastramento anteriormente.</t>
+        </is>
+      </c>
       <c r="AT155" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5187.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5184.pdf</t>
         </is>
       </c>
       <c r="AU155" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5187.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5184.pdf</t>
         </is>
       </c>
       <c r="AV155" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5187.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5184.pdf</t>
         </is>
       </c>
       <c r="AW155" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5187.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5184.pdf</t>
         </is>
       </c>
       <c r="AX155" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5187.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5184.pdf</t>
         </is>
       </c>
       <c r="AY155" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5187.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5184.pdf</t>
         </is>
       </c>
       <c r="AZ155" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5187.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5184.pdf</t>
         </is>
       </c>
       <c r="BA155" s="4" t="inlineStr"/>
@@ -40413,12 +40419,12 @@
       </c>
       <c r="Q156" s="2" t="inlineStr">
         <is>
-          <t>11.060.913/0001-10</t>
+          <t>10.740.658/0001-93</t>
         </is>
       </c>
       <c r="R156" s="2" t="inlineStr">
         <is>
-          <t>5187</t>
+          <t>5184</t>
         </is>
       </c>
       <c r="S156" s="2" t="inlineStr">
@@ -40468,7 +40474,7 @@
       </c>
       <c r="AB156" s="2" t="inlineStr">
         <is>
-          <t>IMA-B 5</t>
+          <t>IMA-B TOTAL</t>
         </is>
       </c>
       <c r="AC156" s="2" t="inlineStr">
@@ -40544,43 +40550,49 @@
       </c>
       <c r="AR156" s="2" t="inlineStr">
         <is>
-          <t>CAIXA BRASIL IMA-B 5 TÍTULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
-        </is>
-      </c>
-      <c r="AS156" s="2" t="inlineStr"/>
+          <t>CAIXA BRASIL IMA-B TÍTULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
+        </is>
+      </c>
+      <c r="AS156" s="2" t="inlineStr">
+        <is>
+          <t>1. O Fundo tem como parâmetro de rentabilidade o Índice de Mercado ANBIMA série B (IMA-B).
+2. Para aplicação por meio de conta operação 1292, é necessário o cadastramento prévio de cotistas, conforme descrito no item Adesão, do FI612.
+3. O procedimento de inclusão da conta deverá ser realizado sempre que houver qualquer aplicação por meio de conta operação 1292, mesmo para os clientes que já realizaram o cadastramento anteriormente.</t>
+        </is>
+      </c>
       <c r="AT156" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5187.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5184.pdf</t>
         </is>
       </c>
       <c r="AU156" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5187.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5184.pdf</t>
         </is>
       </c>
       <c r="AV156" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5187.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5184.pdf</t>
         </is>
       </c>
       <c r="AW156" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5187.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5184.pdf</t>
         </is>
       </c>
       <c r="AX156" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5187.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5184.pdf</t>
         </is>
       </c>
       <c r="AY156" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5187.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5184.pdf</t>
         </is>
       </c>
       <c r="AZ156" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5187.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5184.pdf</t>
         </is>
       </c>
       <c r="BA156" s="2" t="inlineStr"/>
@@ -41051,12 +41063,12 @@
       </c>
       <c r="Q159" s="4" t="inlineStr">
         <is>
-          <t>11.060.913/0001-10</t>
+          <t>10.740.658/0001-93</t>
         </is>
       </c>
       <c r="R159" s="4" t="inlineStr">
         <is>
-          <t>5187</t>
+          <t>5184</t>
         </is>
       </c>
       <c r="S159" s="4" t="inlineStr">
@@ -41106,7 +41118,7 @@
       </c>
       <c r="AB159" s="4" t="inlineStr">
         <is>
-          <t>IMA-B 5</t>
+          <t>IMA-B TOTAL</t>
         </is>
       </c>
       <c r="AC159" s="4" t="inlineStr">
@@ -41182,43 +41194,49 @@
       </c>
       <c r="AR159" s="4" t="inlineStr">
         <is>
-          <t>CAIXA BRASIL IMA-B 5 TÍTULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
-        </is>
-      </c>
-      <c r="AS159" s="4" t="inlineStr"/>
+          <t>CAIXA BRASIL IMA-B TÍTULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
+        </is>
+      </c>
+      <c r="AS159" s="4" t="inlineStr">
+        <is>
+          <t>1. O Fundo tem como parâmetro de rentabilidade o Índice de Mercado ANBIMA série B (IMA-B).
+2. Para aplicação por meio de conta operação 1292, é necessário o cadastramento prévio de cotistas, conforme descrito no item Adesão, do FI612.
+3. O procedimento de inclusão da conta deverá ser realizado sempre que houver qualquer aplicação por meio de conta operação 1292, mesmo para os clientes que já realizaram o cadastramento anteriormente.</t>
+        </is>
+      </c>
       <c r="AT159" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5187.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5184.pdf</t>
         </is>
       </c>
       <c r="AU159" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5187.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5184.pdf</t>
         </is>
       </c>
       <c r="AV159" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5187.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5184.pdf</t>
         </is>
       </c>
       <c r="AW159" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5187.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5184.pdf</t>
         </is>
       </c>
       <c r="AX159" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5187.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5184.pdf</t>
         </is>
       </c>
       <c r="AY159" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5187.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5184.pdf</t>
         </is>
       </c>
       <c r="AZ159" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5187.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5184.pdf</t>
         </is>
       </c>
       <c r="BA159" s="4" t="inlineStr"/>

</xml_diff>

<commit_message>
Dados atualizados via Robô: 02/09/2026 14:28
</commit_message>
<xml_diff>
--- a/dados_atuais.xlsx
+++ b/dados_atuais.xlsx
@@ -3318,12 +3318,12 @@
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>03.218.183/0001-04</t>
+          <t>09.548.729/0001-71</t>
         </is>
       </c>
       <c r="R12" s="2" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>5414</t>
         </is>
       </c>
       <c r="S12" s="2" t="inlineStr">
@@ -3333,27 +3333,27 @@
       </c>
       <c r="T12" s="2" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="U12" s="2" t="inlineStr">
         <is>
+          <t>100.0</t>
+        </is>
+      </c>
+      <c r="V12" s="2" t="inlineStr">
+        <is>
           <t>0.01</t>
         </is>
       </c>
-      <c r="V12" s="2" t="inlineStr">
+      <c r="W12" s="2" t="inlineStr">
         <is>
           <t>0.01</t>
         </is>
       </c>
-      <c r="W12" s="2" t="inlineStr">
-        <is>
-          <t>0.01</t>
-        </is>
-      </c>
       <c r="X12" s="2" t="inlineStr">
         <is>
-          <t>0.01</t>
+          <t>10.0</t>
         </is>
       </c>
       <c r="Y12" s="2" t="inlineStr">
@@ -3373,7 +3373,7 @@
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
-          <t>IPCA+6%</t>
+          <t>NÃO SE APLICA</t>
         </is>
       </c>
       <c r="AC12" s="2" t="inlineStr">
@@ -3449,7 +3449,7 @@
       </c>
       <c r="AR12" s="2" t="inlineStr">
         <is>
-          <t>CAIXA CAPITAL ÍNDICE DE PREÇOS FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESP LIMITADA</t>
+          <t>CAIXA FOCO ÍNDICE DE PREÇOS FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESP LIMITADA</t>
         </is>
       </c>
       <c r="AS12" s="2" t="inlineStr">
@@ -3459,43 +3459,43 @@
       </c>
       <c r="AT12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_0087.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5414.pdf</t>
         </is>
       </c>
       <c r="AU12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_0087.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5414.pdf</t>
         </is>
       </c>
       <c r="AV12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_0087.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5414.pdf</t>
         </is>
       </c>
       <c r="AW12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_87.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5414.pdf</t>
         </is>
       </c>
       <c r="AX12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_87.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5414.pdf</t>
         </is>
       </c>
       <c r="AY12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_87.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5414.pdf</t>
         </is>
       </c>
       <c r="AZ12" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_0087.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5414.pdf</t>
         </is>
       </c>
       <c r="BA12" s="2" t="inlineStr"/>
       <c r="BB12" s="2" t="inlineStr">
         <is>
-          <t>https://web.microsoftstream.com/video/32d65536-1de1-4f2f-a9b8-0fbb0d9347fc?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
+          <t>https://web.microsoftstream.com/video/a5ab94de-1f04-4f00-87d2-ffa0c6babbaf?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
     </row>
@@ -6969,12 +6969,12 @@
       </c>
       <c r="Q26" s="2" t="inlineStr">
         <is>
-          <t>10.646.888/0001-98</t>
+          <t>58.113.332/0001-62</t>
         </is>
       </c>
       <c r="R26" s="2" t="inlineStr">
         <is>
-          <t>5156</t>
+          <t>7931</t>
         </is>
       </c>
       <c r="S26" s="2" t="inlineStr">
@@ -6984,7 +6984,7 @@
       </c>
       <c r="T26" s="2" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>0.3</t>
         </is>
       </c>
       <c r="U26" s="2" t="inlineStr">
@@ -7014,22 +7014,22 @@
       </c>
       <c r="Z26" s="2" t="inlineStr">
         <is>
-          <t>D+0 (du)</t>
+          <t>D+13 (du)</t>
         </is>
       </c>
       <c r="AA26" s="2" t="inlineStr">
         <is>
-          <t>D+00 (du)</t>
+          <t>D+15 (du)</t>
         </is>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
-          <t>CDI</t>
+          <t>NÃO SE APLICA</t>
         </is>
       </c>
       <c r="AC26" s="2" t="inlineStr">
         <is>
-          <t>RF Crédito Privado sem Risco Mercado</t>
+          <t>RF Crédito Privado permite Risco Mercado</t>
         </is>
       </c>
       <c r="AD26" s="2" t="inlineStr">
@@ -7049,37 +7049,33 @@
       </c>
       <c r="AG26" s="2" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="AH26" s="2" t="inlineStr">
         <is>
-          <t>17h00</t>
+          <t>13h00</t>
         </is>
       </c>
       <c r="AI26" s="2" t="inlineStr">
         <is>
-          <t>Sim · Automatico · 90%</t>
+          <t>Não se aplica</t>
         </is>
       </c>
       <c r="AJ26" s="2" t="inlineStr">
         <is>
-          <t>AUTOMATICO</t>
-        </is>
-      </c>
-      <c r="AK26" s="2" t="inlineStr">
-        <is>
-          <t>90.0</t>
-        </is>
-      </c>
+          <t>NÃO SE APLICA</t>
+        </is>
+      </c>
+      <c r="AK26" s="2" t="inlineStr"/>
       <c r="AL26" s="2" t="inlineStr">
         <is>
-          <t>["Pessoa Física", "PJ Varejo", "Private"]</t>
+          <t>["GOV", "Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private", "RPPS"]</t>
         </is>
       </c>
       <c r="AM26" s="2" t="inlineStr">
         <is>
-          <t>["Pessoa Física", "PJ Varejo", "Private"]</t>
+          <t>["GOV", "Institucional", "Pessoa Física", "PJ Atacado", "PJ Varejo", "Private", "RPPS"]</t>
         </is>
       </c>
       <c r="AN26" s="2" t="inlineStr">
@@ -7100,47 +7096,43 @@
       </c>
       <c r="AR26" s="2" t="inlineStr">
         <is>
-          <t>CAIXA EXPERTISE FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA CRÉDITO PRIVADO LONGO PRAZO - RESP LIMITADA</t>
-        </is>
-      </c>
-      <c r="AS26" s="2" t="inlineStr">
-        <is>
-          <t>*Este Fundo não está adaptado às normas vigentes para RPPS (Regimes Próprios de Previdência Social).</t>
-        </is>
-      </c>
+          <t>CAIXA EXPERT SULAMÉRICA CRÉDITO ATIVO FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA CRÉDITO PRIVADO LONGO PR</t>
+        </is>
+      </c>
+      <c r="AS26" s="2" t="inlineStr"/>
       <c r="AT26" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5156.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_7931.pdf</t>
         </is>
       </c>
       <c r="AU26" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5156.pdf</t>
+          <t>http://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_7931.pdf</t>
         </is>
       </c>
       <c r="AV26" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5156.pdf</t>
+          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_7931.pdf</t>
         </is>
       </c>
       <c r="AW26" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5156.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_7931.pdf</t>
         </is>
       </c>
       <c r="AX26" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5156.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_7931.pdf</t>
         </is>
       </c>
       <c r="AY26" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5156.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_7931.pdf</t>
         </is>
       </c>
       <c r="AZ26" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5156.pdf</t>
+          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_7931.pdf</t>
         </is>
       </c>
       <c r="BA26" s="2" t="inlineStr"/>
@@ -19608,15 +19600,19 @@
           <t>PF</t>
         </is>
       </c>
-      <c r="P75" s="4" t="inlineStr"/>
+      <c r="P75" s="4" t="inlineStr">
+        <is>
+          <t>http://www.caixa.gov.br/fundos-investimento/multimercado/estrategia-livre-mm-lp/Paginas/default.aspx</t>
+        </is>
+      </c>
       <c r="Q75" s="4" t="inlineStr">
         <is>
-          <t>35.536.472/0001-48</t>
+          <t>34.660.333/0001-69</t>
         </is>
       </c>
       <c r="R75" s="4" t="inlineStr">
         <is>
-          <t>6479</t>
+          <t>6440</t>
         </is>
       </c>
       <c r="S75" s="4" t="inlineStr">
@@ -19626,7 +19622,7 @@
       </c>
       <c r="T75" s="4" t="inlineStr">
         <is>
-          <t>0.6</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="U75" s="4" t="inlineStr">
@@ -19714,8 +19710,16 @@
           <t>100.0</t>
         </is>
       </c>
-      <c r="AL75" s="4" t="inlineStr"/>
-      <c r="AM75" s="4" t="inlineStr"/>
+      <c r="AL75" s="4" t="inlineStr">
+        <is>
+          <t>["Pessoa Física", "Private"]</t>
+        </is>
+      </c>
+      <c r="AM75" s="4" t="inlineStr">
+        <is>
+          <t>["Pessoa Física", "Private"]</t>
+        </is>
+      </c>
       <c r="AN75" s="4" t="inlineStr">
         <is>
           <t>Não</t>
@@ -19734,47 +19738,43 @@
       </c>
       <c r="AR75" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FUNCIONÁRIOS ESTRATÉGIA LIVRE FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO MULTIMERCADO LONGO PRAZO - RESPONSABI</t>
-        </is>
-      </c>
-      <c r="AS75" s="4" t="inlineStr">
-        <is>
-          <t>Fundo destinado a Funcionários e aposentados da Caixa Econômica Federal. Disponível para aplicação somente via conta corrente marcada como conta-salário empregado CAIXA.</t>
-        </is>
-      </c>
+          <t>CAIXA ESTRATÉGIA LIVRE FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO MULTIMERCADO LONGO PRAZO - RESPONSABILIDADE LIMITA</t>
+        </is>
+      </c>
+      <c r="AS75" s="4" t="inlineStr"/>
       <c r="AT75" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_6479.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_6440.pdf</t>
         </is>
       </c>
       <c r="AU75" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_6479.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_6440.pdf</t>
         </is>
       </c>
       <c r="AV75" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_6479.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_6440.pdf</t>
         </is>
       </c>
       <c r="AW75" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_6479.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_6440.pdf</t>
         </is>
       </c>
       <c r="AX75" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6479.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6440.pdf</t>
         </is>
       </c>
       <c r="AY75" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6479.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6440.pdf</t>
         </is>
       </c>
       <c r="AZ75" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_6479.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_6440.pdf</t>
         </is>
       </c>
       <c r="BA75" s="4" t="inlineStr"/>
@@ -31649,17 +31649,17 @@
       </c>
       <c r="P122" s="2" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/fundos-investimento/mutuos-privatizacao/fmp-fgts-vale-do-rio-doce-2</t>
+          <t>http://www.caixa.gov.br/fundos-investimento/mutuos-privatizacao/fmp-fgts-vale-do-rio-doce-1</t>
         </is>
       </c>
       <c r="Q122" s="2" t="inlineStr">
         <is>
-          <t>04.885.824/0001-47</t>
+          <t>04.885.818/0001-90</t>
         </is>
       </c>
       <c r="R122" s="2" t="inlineStr">
         <is>
-          <t>5206</t>
+          <t>5205</t>
         </is>
       </c>
       <c r="S122" s="2" t="inlineStr">
@@ -31669,12 +31669,12 @@
       </c>
       <c r="T122" s="2" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.9</t>
         </is>
       </c>
       <c r="U122" s="2" t="inlineStr">
         <is>
-          <t>10000.0</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="V122" s="2" t="inlineStr">
@@ -31769,7 +31769,7 @@
       </c>
       <c r="AR122" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FUNDO MÚTUO DE PRIVATIZAÇÃO - FGTS - VALE DO RIO DOCE II - RESPONSABILIDADE LIMITADA</t>
+          <t>CAIXA FUNDO MÚTUO DE PRIVATIZAÇÃO - FGTS - VALE DO RIO DOCE I - RESPONSABILIDADE LIMITADA</t>
         </is>
       </c>
       <c r="AS122" s="2" t="inlineStr">
@@ -31779,37 +31779,37 @@
       </c>
       <c r="AT122" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5206.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5205.pdf</t>
         </is>
       </c>
       <c r="AU122" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5206.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5205.pdf</t>
         </is>
       </c>
       <c r="AV122" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5206.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5205.pdf</t>
         </is>
       </c>
       <c r="AW122" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_5206.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_5205.pdf</t>
         </is>
       </c>
       <c r="AX122" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5206.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5205.pdf</t>
         </is>
       </c>
       <c r="AY122" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5206.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5205.pdf</t>
         </is>
       </c>
       <c r="AZ122" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5206.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5205.pdf</t>
         </is>
       </c>
       <c r="BA122" s="2" t="inlineStr"/>
@@ -32644,17 +32644,17 @@
       </c>
       <c r="P126" s="2" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/fundos-investimento/mutuos-privatizacao/fmp-fgts-vale-do-rio-doce-2</t>
+          <t>http://www.caixa.gov.br/fundos-investimento/mutuos-privatizacao/fmp-fgts-vale-do-rio-doce-1</t>
         </is>
       </c>
       <c r="Q126" s="2" t="inlineStr">
         <is>
-          <t>04.885.824/0001-47</t>
+          <t>04.885.818/0001-90</t>
         </is>
       </c>
       <c r="R126" s="2" t="inlineStr">
         <is>
-          <t>5206</t>
+          <t>5205</t>
         </is>
       </c>
       <c r="S126" s="2" t="inlineStr">
@@ -32664,12 +32664,12 @@
       </c>
       <c r="T126" s="2" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.9</t>
         </is>
       </c>
       <c r="U126" s="2" t="inlineStr">
         <is>
-          <t>10000.0</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="V126" s="2" t="inlineStr">
@@ -32764,7 +32764,7 @@
       </c>
       <c r="AR126" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FUNDO MÚTUO DE PRIVATIZAÇÃO - FGTS - VALE DO RIO DOCE II - RESPONSABILIDADE LIMITADA</t>
+          <t>CAIXA FUNDO MÚTUO DE PRIVATIZAÇÃO - FGTS - VALE DO RIO DOCE I - RESPONSABILIDADE LIMITADA</t>
         </is>
       </c>
       <c r="AS126" s="2" t="inlineStr">
@@ -32774,37 +32774,37 @@
       </c>
       <c r="AT126" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5206.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5205.pdf</t>
         </is>
       </c>
       <c r="AU126" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5206.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5205.pdf</t>
         </is>
       </c>
       <c r="AV126" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5206.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5205.pdf</t>
         </is>
       </c>
       <c r="AW126" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_5206.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_5205.pdf</t>
         </is>
       </c>
       <c r="AX126" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5206.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5205.pdf</t>
         </is>
       </c>
       <c r="AY126" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5206.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5205.pdf</t>
         </is>
       </c>
       <c r="AZ126" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5206.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5205.pdf</t>
         </is>
       </c>
       <c r="BA126" s="2" t="inlineStr"/>
@@ -37274,7 +37274,7 @@
       </c>
       <c r="U144" s="2" t="inlineStr">
         <is>
-          <t>1000000.0</t>
+          <t>3000000.0</t>
         </is>
       </c>
       <c r="V144" s="2" t="inlineStr">
@@ -37289,7 +37289,7 @@
       </c>
       <c r="X144" s="2" t="inlineStr">
         <is>
-          <t>100000.0</t>
+          <t>300000.0</t>
         </is>
       </c>
       <c r="Y144" s="2" t="inlineStr">
@@ -37388,17 +37388,7 @@
           <t>CAIXA TOPÁZIO CORPORATIVO FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA REFERENCIADO DI LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
         </is>
       </c>
-      <c r="AS144" s="2" t="inlineStr">
-        <is>
-          <t>Campanha "Campanha Caixa Asset Lidera RPPS" de 06/07/2026 a 31/08/2026
-Redução de Tickets
-Aplicação Inicial:
-De: R$ 3.000.000,00 para R$ 1.000.000,00
-Saldo Mínimo: 
-De: R$ 300.000,00 para R$ 100.000,00
-OBS: Após a Campanha, voltam os parâmetros originais. Saldo abaixo do mínimo pode impedir resgates parciais (somente total).</t>
-        </is>
-      </c>
+      <c r="AS144" s="2" t="inlineStr"/>
       <c r="AT144" s="2" t="inlineStr">
         <is>
           <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5189.pdf</t>
@@ -38827,12 +38817,12 @@
       </c>
       <c r="Q150" s="2" t="inlineStr">
         <is>
-          <t>10.740.670/0001-06</t>
+          <t>14.508.605/0001-00</t>
         </is>
       </c>
       <c r="R150" s="2" t="inlineStr">
         <is>
-          <t>5464</t>
+          <t>5824</t>
         </is>
       </c>
       <c r="S150" s="2" t="inlineStr">
@@ -38882,7 +38872,7 @@
       </c>
       <c r="AB150" s="2" t="inlineStr">
         <is>
-          <t>IRF-M 1</t>
+          <t>IRF-M TOTAL</t>
         </is>
       </c>
       <c r="AC150" s="2" t="inlineStr">
@@ -38907,17 +38897,17 @@
       </c>
       <c r="AG150" s="2" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="AH150" s="2" t="inlineStr">
         <is>
-          <t>17h00</t>
+          <t>16h00</t>
         </is>
       </c>
       <c r="AI150" s="2" t="inlineStr">
         <is>
-          <t>Sim · Automatico · 95%</t>
+          <t>Sim · Automatico · 90%</t>
         </is>
       </c>
       <c r="AJ150" s="2" t="inlineStr">
@@ -38927,7 +38917,7 @@
       </c>
       <c r="AK150" s="2" t="inlineStr">
         <is>
-          <t>95.0</t>
+          <t>90.0</t>
         </is>
       </c>
       <c r="AL150" s="2" t="inlineStr">
@@ -38958,58 +38948,54 @@
       </c>
       <c r="AR150" s="2" t="inlineStr">
         <is>
-          <t>CAIXA BRASIL IRF-M 1 TÍTULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA - RESPONSABILIDADE LIMITADA</t>
+          <t>CAIXA BRASIL IRF-M TÍTULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
         </is>
       </c>
       <c r="AS150" s="2" t="inlineStr">
         <is>
-          <t>1.O Fundo tem como parâmetro de rentabilidade o Índice de Renda Fixa de Mercado 1 (IRF-M 1).
-2.Para aplicação por meio de conta operação 1292, é necessário o cadastramento prévio de cotistas, conforme descrito no item Adesão, do FI612.
-3.O procedimento de inclusão da conta deverá ser realizado sempre que houver qualquer aplicação por meio de conta operação 1292, mesmo para os clientes que já realizaram o cadastramento anteriormente.
+          <t>1. O Fundo tem como parâmetro de rentabilidade o Índice de Renda Fixa de Mercado (IRF-M).
+2. Para aplicação por meio de conta operação 1292, é necessário o cadastramento prévio de cotistas, conforme descrito no item Adesão, do FI612.
+3. O procedimento de inclusão da conta deverá ser realizado sempre que houver qualquer aplicação por meio de conta operação 1292, mesmo para os clientes que já realizaram o cadastramento anteriormente.
 ¹Condições excepcionais de estorno e movimentação retroativa estão descritas no TE099.</t>
         </is>
       </c>
       <c r="AT150" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5464.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5824.pdf</t>
         </is>
       </c>
       <c r="AU150" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5464.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5824.pdf</t>
         </is>
       </c>
       <c r="AV150" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5464.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5824.pdf</t>
         </is>
       </c>
       <c r="AW150" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5464.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5824.pdf</t>
         </is>
       </c>
       <c r="AX150" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5464.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5824.pdf</t>
         </is>
       </c>
       <c r="AY150" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5464.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5824.pdf</t>
         </is>
       </c>
       <c r="AZ150" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5464.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5824.pdf</t>
         </is>
       </c>
       <c r="BA150" s="2" t="inlineStr"/>
-      <c r="BB150" s="2" t="inlineStr">
-        <is>
-          <t>https://web.microsoftstream.com/video/e092ed57-1ff7-4570-9897-57fc78b1a0c8?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
-        </is>
-      </c>
+      <c r="BB150" s="2" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" s="4" t="inlineStr">
@@ -39094,12 +39080,12 @@
       </c>
       <c r="Q151" s="4" t="inlineStr">
         <is>
-          <t>05.164.356/0001-84</t>
+          <t>03.737.206/0001-97</t>
         </is>
       </c>
       <c r="R151" s="4" t="inlineStr">
         <is>
-          <t>5462</t>
+          <t>5404</t>
         </is>
       </c>
       <c r="S151" s="4" t="inlineStr">
@@ -39154,7 +39140,7 @@
       </c>
       <c r="AC151" s="4" t="inlineStr">
         <is>
-          <t>RF 100% TPF - Longo Prazo</t>
+          <t>RF DI até 49% Crédito Privado</t>
         </is>
       </c>
       <c r="AD151" s="4" t="inlineStr">
@@ -39225,53 +39211,54 @@
       </c>
       <c r="AR151" s="4" t="inlineStr">
         <is>
-          <t>CAIXA BRASIL TÍTULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
+          <t>CAIXA BRASIL FUNDO DE INVESTIMENTO EM COTAS DE CLASSE DE FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA REFERENCIADO DI LONGO PRAZO - RESP LIMITADA</t>
         </is>
       </c>
       <c r="AS151" s="4" t="inlineStr">
         <is>
-          <t>Para aplicação no fundo é necessário o cadastramento prévio de cotistas, conforme descrito no FI657. O procedimento de inclusão da conta deverá ser realizado sempre que houver qualquer aplicação, mesmo para os clientes que já realizaram o cadsatramento anteriormente.</t>
+          <t>1. Para aplicação por meio de conta operação 003, é necessário o cadastramento prévio de cotistas, conforme descrito no item Adesão, do FI612.
+2. O procedimento de inclusão da conta deverá ser realizado sempre que houver qualquer aplicação por meio de conta operação 003, mesmo para os clientes que já realizaram o cadastramento anteriormente.</t>
         </is>
       </c>
       <c r="AT151" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5462.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5404.pdf</t>
         </is>
       </c>
       <c r="AU151" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5462.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5404.pdf</t>
         </is>
       </c>
       <c r="AV151" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5462.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5404.pdf</t>
         </is>
       </c>
       <c r="AW151" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5462.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5404.pdf</t>
         </is>
       </c>
       <c r="AX151" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5462.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5404.pdf</t>
         </is>
       </c>
       <c r="AY151" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5462.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5404.pdf</t>
         </is>
       </c>
       <c r="AZ151" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5462.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5404.pdf</t>
         </is>
       </c>
       <c r="BA151" s="4" t="inlineStr"/>
       <c r="BB151" s="4" t="inlineStr">
         <is>
-          <t>https://web.microsoftstream.com/video/91aaf70b-85c2-4cf1-b537-e42b3bd894ec?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
+          <t>https://web.microsoftstream.com/video/f88f1fc7-aac3-44df-a2a5-ce3ac05edfb3?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
     </row>
@@ -39874,12 +39861,12 @@
       </c>
       <c r="Q154" s="2" t="inlineStr">
         <is>
-          <t>10.740.670/0001-06</t>
+          <t>14.508.605/0001-00</t>
         </is>
       </c>
       <c r="R154" s="2" t="inlineStr">
         <is>
-          <t>5464</t>
+          <t>5824</t>
         </is>
       </c>
       <c r="S154" s="2" t="inlineStr">
@@ -39929,7 +39916,7 @@
       </c>
       <c r="AB154" s="2" t="inlineStr">
         <is>
-          <t>IRF-M 1</t>
+          <t>IRF-M TOTAL</t>
         </is>
       </c>
       <c r="AC154" s="2" t="inlineStr">
@@ -39954,17 +39941,17 @@
       </c>
       <c r="AG154" s="2" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="AH154" s="2" t="inlineStr">
         <is>
-          <t>17h00</t>
+          <t>16h00</t>
         </is>
       </c>
       <c r="AI154" s="2" t="inlineStr">
         <is>
-          <t>Sim · Automatico · 95%</t>
+          <t>Sim · Automatico · 90%</t>
         </is>
       </c>
       <c r="AJ154" s="2" t="inlineStr">
@@ -39974,7 +39961,7 @@
       </c>
       <c r="AK154" s="2" t="inlineStr">
         <is>
-          <t>95.0</t>
+          <t>90.0</t>
         </is>
       </c>
       <c r="AL154" s="2" t="inlineStr">
@@ -40005,58 +39992,54 @@
       </c>
       <c r="AR154" s="2" t="inlineStr">
         <is>
-          <t>CAIXA BRASIL IRF-M 1 TÍTULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA - RESPONSABILIDADE LIMITADA</t>
+          <t>CAIXA BRASIL IRF-M TÍTULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
         </is>
       </c>
       <c r="AS154" s="2" t="inlineStr">
         <is>
-          <t>1.O Fundo tem como parâmetro de rentabilidade o Índice de Renda Fixa de Mercado 1 (IRF-M 1).
-2.Para aplicação por meio de conta operação 1292, é necessário o cadastramento prévio de cotistas, conforme descrito no item Adesão, do FI612.
-3.O procedimento de inclusão da conta deverá ser realizado sempre que houver qualquer aplicação por meio de conta operação 1292, mesmo para os clientes que já realizaram o cadastramento anteriormente.
+          <t>1. O Fundo tem como parâmetro de rentabilidade o Índice de Renda Fixa de Mercado (IRF-M).
+2. Para aplicação por meio de conta operação 1292, é necessário o cadastramento prévio de cotistas, conforme descrito no item Adesão, do FI612.
+3. O procedimento de inclusão da conta deverá ser realizado sempre que houver qualquer aplicação por meio de conta operação 1292, mesmo para os clientes que já realizaram o cadastramento anteriormente.
 ¹Condições excepcionais de estorno e movimentação retroativa estão descritas no TE099.</t>
         </is>
       </c>
       <c r="AT154" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5464.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5824.pdf</t>
         </is>
       </c>
       <c r="AU154" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5464.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5824.pdf</t>
         </is>
       </c>
       <c r="AV154" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5464.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5824.pdf</t>
         </is>
       </c>
       <c r="AW154" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5464.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5824.pdf</t>
         </is>
       </c>
       <c r="AX154" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5464.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5824.pdf</t>
         </is>
       </c>
       <c r="AY154" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5464.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5824.pdf</t>
         </is>
       </c>
       <c r="AZ154" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5464.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5824.pdf</t>
         </is>
       </c>
       <c r="BA154" s="2" t="inlineStr"/>
-      <c r="BB154" s="2" t="inlineStr">
-        <is>
-          <t>https://web.microsoftstream.com/video/e092ed57-1ff7-4570-9897-57fc78b1a0c8?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
-        </is>
-      </c>
+      <c r="BB154" s="2" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" s="4" t="inlineStr">
@@ -40404,12 +40387,12 @@
       </c>
       <c r="Q156" s="2" t="inlineStr">
         <is>
-          <t>10.740.670/0001-06</t>
+          <t>14.508.605/0001-00</t>
         </is>
       </c>
       <c r="R156" s="2" t="inlineStr">
         <is>
-          <t>5464</t>
+          <t>5824</t>
         </is>
       </c>
       <c r="S156" s="2" t="inlineStr">
@@ -40459,7 +40442,7 @@
       </c>
       <c r="AB156" s="2" t="inlineStr">
         <is>
-          <t>IRF-M 1</t>
+          <t>IRF-M TOTAL</t>
         </is>
       </c>
       <c r="AC156" s="2" t="inlineStr">
@@ -40484,17 +40467,17 @@
       </c>
       <c r="AG156" s="2" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="AH156" s="2" t="inlineStr">
         <is>
-          <t>17h00</t>
+          <t>16h00</t>
         </is>
       </c>
       <c r="AI156" s="2" t="inlineStr">
         <is>
-          <t>Sim · Automatico · 95%</t>
+          <t>Sim · Automatico · 90%</t>
         </is>
       </c>
       <c r="AJ156" s="2" t="inlineStr">
@@ -40504,7 +40487,7 @@
       </c>
       <c r="AK156" s="2" t="inlineStr">
         <is>
-          <t>95.0</t>
+          <t>90.0</t>
         </is>
       </c>
       <c r="AL156" s="2" t="inlineStr">
@@ -40535,58 +40518,54 @@
       </c>
       <c r="AR156" s="2" t="inlineStr">
         <is>
-          <t>CAIXA BRASIL IRF-M 1 TÍTULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA - RESPONSABILIDADE LIMITADA</t>
+          <t>CAIXA BRASIL IRF-M TÍTULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
         </is>
       </c>
       <c r="AS156" s="2" t="inlineStr">
         <is>
-          <t>1.O Fundo tem como parâmetro de rentabilidade o Índice de Renda Fixa de Mercado 1 (IRF-M 1).
-2.Para aplicação por meio de conta operação 1292, é necessário o cadastramento prévio de cotistas, conforme descrito no item Adesão, do FI612.
-3.O procedimento de inclusão da conta deverá ser realizado sempre que houver qualquer aplicação por meio de conta operação 1292, mesmo para os clientes que já realizaram o cadastramento anteriormente.
+          <t>1. O Fundo tem como parâmetro de rentabilidade o Índice de Renda Fixa de Mercado (IRF-M).
+2. Para aplicação por meio de conta operação 1292, é necessário o cadastramento prévio de cotistas, conforme descrito no item Adesão, do FI612.
+3. O procedimento de inclusão da conta deverá ser realizado sempre que houver qualquer aplicação por meio de conta operação 1292, mesmo para os clientes que já realizaram o cadastramento anteriormente.
 ¹Condições excepcionais de estorno e movimentação retroativa estão descritas no TE099.</t>
         </is>
       </c>
       <c r="AT156" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5464.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5824.pdf</t>
         </is>
       </c>
       <c r="AU156" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5464.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5824.pdf</t>
         </is>
       </c>
       <c r="AV156" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5464.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5824.pdf</t>
         </is>
       </c>
       <c r="AW156" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5464.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5824.pdf</t>
         </is>
       </c>
       <c r="AX156" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5464.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5824.pdf</t>
         </is>
       </c>
       <c r="AY156" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5464.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5824.pdf</t>
         </is>
       </c>
       <c r="AZ156" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5464.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5824.pdf</t>
         </is>
       </c>
       <c r="BA156" s="2" t="inlineStr"/>
-      <c r="BB156" s="2" t="inlineStr">
-        <is>
-          <t>https://web.microsoftstream.com/video/e092ed57-1ff7-4570-9897-57fc78b1a0c8?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
-        </is>
-      </c>
+      <c r="BB156" s="2" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" s="4" t="inlineStr">
@@ -41452,12 +41431,12 @@
       </c>
       <c r="Q160" s="2" t="inlineStr">
         <is>
-          <t>10.740.658/0001-93</t>
+          <t>10.577.503/0001-88</t>
         </is>
       </c>
       <c r="R160" s="2" t="inlineStr">
         <is>
-          <t>5184</t>
+          <t>5568</t>
         </is>
       </c>
       <c r="S160" s="2" t="inlineStr">
@@ -41507,7 +41486,7 @@
       </c>
       <c r="AB160" s="2" t="inlineStr">
         <is>
-          <t>IMA-B TOTAL</t>
+          <t>IMA-B 5+</t>
         </is>
       </c>
       <c r="AC160" s="2" t="inlineStr">
@@ -41583,49 +41562,49 @@
       </c>
       <c r="AR160" s="2" t="inlineStr">
         <is>
-          <t>CAIXA BRASIL IMA-B TÍTULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
+          <t>CAIXA BRASIL IMA B 5+ TITULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
         </is>
       </c>
       <c r="AS160" s="2" t="inlineStr">
         <is>
-          <t>1. O Fundo tem como parâmetro de rentabilidade o Índice de Mercado ANBIMA série B (IMA-B).
+          <t>1. O Fundo tem como parâmetro de rentabilidade o Índice de Mercado da ANBIMA B 5 (IMA-B 5).
 2. Para aplicação por meio de conta operação 1292, é necessário o cadastramento prévio de cotistas, conforme descrito no item Adesão, do FI612.
 3. O procedimento de inclusão da conta deverá ser realizado sempre que houver qualquer aplicação por meio de conta operação 1292, mesmo para os clientes que já realizaram o cadastramento anteriormente.</t>
         </is>
       </c>
       <c r="AT160" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5184.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5568.pdf</t>
         </is>
       </c>
       <c r="AU160" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5184.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5568.pdf</t>
         </is>
       </c>
       <c r="AV160" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5184.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5568.pdf</t>
         </is>
       </c>
       <c r="AW160" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5184.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5568.pdf</t>
         </is>
       </c>
       <c r="AX160" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5184.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5568.pdf</t>
         </is>
       </c>
       <c r="AY160" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5184.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5568.pdf</t>
         </is>
       </c>
       <c r="AZ160" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5184.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5568.pdf</t>
         </is>
       </c>
       <c r="BA160" s="2" t="inlineStr"/>
@@ -41714,12 +41693,12 @@
       </c>
       <c r="Q161" s="4" t="inlineStr">
         <is>
-          <t>10.740.658/0001-93</t>
+          <t>10.577.503/0001-88</t>
         </is>
       </c>
       <c r="R161" s="4" t="inlineStr">
         <is>
-          <t>5184</t>
+          <t>5568</t>
         </is>
       </c>
       <c r="S161" s="4" t="inlineStr">
@@ -41769,7 +41748,7 @@
       </c>
       <c r="AB161" s="4" t="inlineStr">
         <is>
-          <t>IMA-B TOTAL</t>
+          <t>IMA-B 5+</t>
         </is>
       </c>
       <c r="AC161" s="4" t="inlineStr">
@@ -41845,49 +41824,49 @@
       </c>
       <c r="AR161" s="4" t="inlineStr">
         <is>
-          <t>CAIXA BRASIL IMA-B TÍTULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
+          <t>CAIXA BRASIL IMA B 5+ TITULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
         </is>
       </c>
       <c r="AS161" s="4" t="inlineStr">
         <is>
-          <t>1. O Fundo tem como parâmetro de rentabilidade o Índice de Mercado ANBIMA série B (IMA-B).
+          <t>1. O Fundo tem como parâmetro de rentabilidade o Índice de Mercado da ANBIMA B 5 (IMA-B 5).
 2. Para aplicação por meio de conta operação 1292, é necessário o cadastramento prévio de cotistas, conforme descrito no item Adesão, do FI612.
 3. O procedimento de inclusão da conta deverá ser realizado sempre que houver qualquer aplicação por meio de conta operação 1292, mesmo para os clientes que já realizaram o cadastramento anteriormente.</t>
         </is>
       </c>
       <c r="AT161" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5184.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5568.pdf</t>
         </is>
       </c>
       <c r="AU161" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5184.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5568.pdf</t>
         </is>
       </c>
       <c r="AV161" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5184.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5568.pdf</t>
         </is>
       </c>
       <c r="AW161" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5184.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5568.pdf</t>
         </is>
       </c>
       <c r="AX161" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5184.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5568.pdf</t>
         </is>
       </c>
       <c r="AY161" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5184.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5568.pdf</t>
         </is>
       </c>
       <c r="AZ161" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5184.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5568.pdf</t>
         </is>
       </c>
       <c r="BA161" s="4" t="inlineStr"/>
@@ -42358,12 +42337,12 @@
       </c>
       <c r="Q164" s="2" t="inlineStr">
         <is>
-          <t>10.740.658/0001-93</t>
+          <t>10.577.503/0001-88</t>
         </is>
       </c>
       <c r="R164" s="2" t="inlineStr">
         <is>
-          <t>5184</t>
+          <t>5568</t>
         </is>
       </c>
       <c r="S164" s="2" t="inlineStr">
@@ -42413,7 +42392,7 @@
       </c>
       <c r="AB164" s="2" t="inlineStr">
         <is>
-          <t>IMA-B TOTAL</t>
+          <t>IMA-B 5+</t>
         </is>
       </c>
       <c r="AC164" s="2" t="inlineStr">
@@ -42489,49 +42468,49 @@
       </c>
       <c r="AR164" s="2" t="inlineStr">
         <is>
-          <t>CAIXA BRASIL IMA-B TÍTULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
+          <t>CAIXA BRASIL IMA B 5+ TITULOS PÚBLICOS FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
         </is>
       </c>
       <c r="AS164" s="2" t="inlineStr">
         <is>
-          <t>1. O Fundo tem como parâmetro de rentabilidade o Índice de Mercado ANBIMA série B (IMA-B).
+          <t>1. O Fundo tem como parâmetro de rentabilidade o Índice de Mercado da ANBIMA B 5 (IMA-B 5).
 2. Para aplicação por meio de conta operação 1292, é necessário o cadastramento prévio de cotistas, conforme descrito no item Adesão, do FI612.
 3. O procedimento de inclusão da conta deverá ser realizado sempre que houver qualquer aplicação por meio de conta operação 1292, mesmo para os clientes que já realizaram o cadastramento anteriormente.</t>
         </is>
       </c>
       <c r="AT164" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5184.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5568.pdf</t>
         </is>
       </c>
       <c r="AU164" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5184.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5568.pdf</t>
         </is>
       </c>
       <c r="AV164" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5184.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5568.pdf</t>
         </is>
       </c>
       <c r="AW164" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5184.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5568.pdf</t>
         </is>
       </c>
       <c r="AX164" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5184.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5568.pdf</t>
         </is>
       </c>
       <c r="AY164" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5184.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5568.pdf</t>
         </is>
       </c>
       <c r="AZ164" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5184.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5568.pdf</t>
         </is>
       </c>
       <c r="BA164" s="2" t="inlineStr"/>
@@ -44535,12 +44514,12 @@
       </c>
       <c r="Q173" s="4" t="inlineStr">
         <is>
-          <t>13.058.816/0001-18</t>
+          <t>15.154.236/0001-50</t>
         </is>
       </c>
       <c r="R173" s="4" t="inlineStr">
         <is>
-          <t>5445</t>
+          <t>5842</t>
         </is>
       </c>
       <c r="S173" s="4" t="inlineStr">
@@ -44600,7 +44579,7 @@
       </c>
       <c r="AD173" s="4" t="inlineStr">
         <is>
-          <t>Aberto para captação</t>
+          <t>Fechado para captação</t>
         </is>
       </c>
       <c r="AE173" s="4" t="inlineStr">
@@ -44666,43 +44645,47 @@
       </c>
       <c r="AR173" s="4" t="inlineStr">
         <is>
-          <t>CAIXA BRASIL INDEXA IBOVESPA FUNDO DE INVESTIMENTO FINANCEIRO EM AÇÕES - RESPONSABILIDADE LIMITADA</t>
-        </is>
-      </c>
-      <c r="AS173" s="4" t="inlineStr"/>
+          <t>CAIXA BRASIL ETF IBOVESPA FUNDO DE INVESTIMENTO FINANCEIRO EM AÇÕES - RESPONSABILIDADE LIMITADA</t>
+        </is>
+      </c>
+      <c r="AS173" s="4" t="inlineStr">
+        <is>
+          <t>Fundo fechado para novas aplicações, a novos investidores e cotistas atuais a partir de 03/04/2023 (inclusive)</t>
+        </is>
+      </c>
       <c r="AT173" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5445.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5842.pdf</t>
         </is>
       </c>
       <c r="AU173" s="4" t="inlineStr">
         <is>
-          <t>http://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5445.pdf</t>
+          <t>http://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5842.pdf</t>
         </is>
       </c>
       <c r="AV173" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5445.pdf</t>
+          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5842.pdf</t>
         </is>
       </c>
       <c r="AW173" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_5445.pdf</t>
+          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/FR_5842.pdf</t>
         </is>
       </c>
       <c r="AX173" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5445.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5842.pdf</t>
         </is>
       </c>
       <c r="AY173" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5445.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5842.pdf</t>
         </is>
       </c>
       <c r="AZ173" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5445.pdf</t>
+          <t>http://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5842.pdf</t>
         </is>
       </c>
       <c r="BA173" s="4" t="inlineStr"/>

</xml_diff>

<commit_message>
Dados atualizados via Robô: 08/09/2026 14:40
</commit_message>
<xml_diff>
--- a/dados_atuais.xlsx
+++ b/dados_atuais.xlsx
@@ -839,7 +839,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>403,877</t>
+          <t>402,244</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -1099,7 +1099,7 @@
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>6.761,866</t>
+          <t>6.677,912</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
@@ -1359,7 +1359,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>742,682</t>
+          <t>771,832</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -1618,7 +1618,7 @@
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>114,934</t>
+          <t>114,933</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
@@ -1882,7 +1882,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>1.713,995</t>
+          <t>1.713,962</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -2138,7 +2138,7 @@
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>97,752</t>
+          <t>97,685</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -2646,7 +2646,7 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>65,344</t>
+          <t>65,342</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -2902,7 +2902,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>589,134</t>
+          <t>589,133</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -3278,7 +3278,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>28,018</t>
+          <t>28,009</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -3542,7 +3542,7 @@
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>121,894</t>
+          <t>121,892</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
@@ -3805,7 +3805,7 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>12,237</t>
+          <t>12,236</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -4586,7 +4586,7 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>76,881</t>
+          <t>76,859</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -5366,7 +5366,7 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>1.819,046</t>
+          <t>1.806,544</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -5620,7 +5620,7 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>125,628</t>
+          <t>125,627</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -5884,7 +5884,7 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>2.237,041</t>
+          <t>2.237,013</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -6669,7 +6669,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>967,105</t>
+          <t>967,100</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -6904,32 +6904,32 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,28232200</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>-0,001</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>0,15</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>9,48</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>14,43</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>74,377</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
@@ -7156,32 +7156,32 @@
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E27" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F27" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G27" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H27" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,14768202</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>-0,001</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>0,50</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>6,39</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>10,02</t>
         </is>
       </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>198,693</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -7412,32 +7412,32 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,21157700</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>-0,001</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>0,16</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>9,10</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>14,01</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>63,959</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
@@ -7664,32 +7664,32 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,10594560</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>-0,001</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>0,07</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>7,02</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>309,056</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -7941,7 +7941,7 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>480,264</t>
+          <t>480,261</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
@@ -8201,7 +8201,7 @@
       </c>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>182,224</t>
+          <t>182,063</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -8721,7 +8721,7 @@
       </c>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>3.460,110</t>
+          <t>3.460,052</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -9229,7 +9229,7 @@
       </c>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>568,901</t>
+          <t>568,895</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -9490,7 +9490,7 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>2.430,182</t>
+          <t>2.430,150</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
@@ -9725,32 +9725,32 @@
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E37" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F37" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G37" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,07310700</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>-0,001</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>0,13</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>9,43</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>22,520</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -9998,7 +9998,7 @@
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>856,747</t>
+          <t>856,570</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
@@ -10506,7 +10506,7 @@
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>658,494</t>
+          <t>658,478</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
@@ -10766,7 +10766,7 @@
       </c>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>118,957</t>
+          <t>118,770</t>
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr">
@@ -11022,7 +11022,7 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>3.141,881</t>
+          <t>3.141,875</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -11539,7 +11539,7 @@
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>16.769,769</t>
+          <t>16.769,367</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
@@ -12580,7 +12580,7 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>2.305,051</t>
+          <t>2.305,013</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
@@ -12844,7 +12844,7 @@
       </c>
       <c r="I49" s="4" t="inlineStr">
         <is>
-          <t>6.219,901</t>
+          <t>6.158,372</t>
         </is>
       </c>
       <c r="J49" s="4" t="inlineStr">
@@ -13104,7 +13104,7 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>71,534</t>
+          <t>71,533</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
@@ -13364,7 +13364,7 @@
       </c>
       <c r="I51" s="4" t="inlineStr">
         <is>
-          <t>14.593,850</t>
+          <t>14.593,632</t>
         </is>
       </c>
       <c r="J51" s="4" t="inlineStr">
@@ -13624,7 +13624,7 @@
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>823,683</t>
+          <t>823,680</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr">
@@ -13889,7 +13889,7 @@
       </c>
       <c r="I53" s="4" t="inlineStr">
         <is>
-          <t>17.152,889</t>
+          <t>17.152,684</t>
         </is>
       </c>
       <c r="J53" s="4" t="inlineStr">
@@ -14149,7 +14149,7 @@
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>23.357,745</t>
+          <t>23.357,185</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr">
@@ -14409,7 +14409,7 @@
       </c>
       <c r="I55" s="4" t="inlineStr">
         <is>
-          <t>9.726,717</t>
+          <t>9.726,509</t>
         </is>
       </c>
       <c r="J55" s="4" t="inlineStr">
@@ -14768,32 +14768,32 @@
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1,46331700</t>
         </is>
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F57" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G57" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H57" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>0,000</t>
+        </is>
+      </c>
+      <c r="F57" s="5" t="inlineStr">
+        <is>
+          <t>0,15</t>
+        </is>
+      </c>
+      <c r="G57" s="5" t="inlineStr">
+        <is>
+          <t>9,29</t>
+        </is>
+      </c>
+      <c r="H57" s="5" t="inlineStr">
+        <is>
+          <t>14,21</t>
         </is>
       </c>
       <c r="I57" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>65,461</t>
         </is>
       </c>
       <c r="J57" s="4" t="inlineStr">
@@ -15045,7 +15045,7 @@
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>331,342</t>
+          <t>540,035</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
@@ -15284,32 +15284,32 @@
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E59" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F59" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G59" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H59" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1.693,38752300</t>
+        </is>
+      </c>
+      <c r="E59" s="7" t="inlineStr">
+        <is>
+          <t>-0,005</t>
+        </is>
+      </c>
+      <c r="F59" s="5" t="inlineStr">
+        <is>
+          <t>0,61</t>
+        </is>
+      </c>
+      <c r="G59" s="5" t="inlineStr">
+        <is>
+          <t>8,06</t>
+        </is>
+      </c>
+      <c r="H59" s="5" t="inlineStr">
+        <is>
+          <t>12,99</t>
         </is>
       </c>
       <c r="I59" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>112,357</t>
         </is>
       </c>
       <c r="J59" s="4" t="inlineStr">
@@ -15565,7 +15565,7 @@
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>14,272</t>
+          <t>14,266</t>
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr">
@@ -16048,32 +16048,32 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E62" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F62" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G62" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H62" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,28167500</t>
+        </is>
+      </c>
+      <c r="E62" s="6" t="inlineStr">
+        <is>
+          <t>-0,006</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="inlineStr">
+        <is>
+          <t>0,44</t>
+        </is>
+      </c>
+      <c r="G62" s="3" t="inlineStr">
+        <is>
+          <t>4,94</t>
+        </is>
+      </c>
+      <c r="H62" s="3" t="inlineStr">
+        <is>
+          <t>9,96</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4,968</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr">
@@ -16812,32 +16812,32 @@
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E65" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F65" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G65" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H65" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,42746900</t>
+        </is>
+      </c>
+      <c r="E65" s="7" t="inlineStr">
+        <is>
+          <t>-0,004</t>
+        </is>
+      </c>
+      <c r="F65" s="5" t="inlineStr">
+        <is>
+          <t>2,33</t>
+        </is>
+      </c>
+      <c r="G65" s="5" t="inlineStr">
+        <is>
+          <t>4,57</t>
+        </is>
+      </c>
+      <c r="H65" s="5" t="inlineStr">
+        <is>
+          <t>13,53</t>
         </is>
       </c>
       <c r="I65" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11,464</t>
         </is>
       </c>
       <c r="J65" s="4" t="inlineStr">
@@ -17345,7 +17345,7 @@
       </c>
       <c r="I67" s="4" t="inlineStr">
         <is>
-          <t>3,375</t>
+          <t>3,371</t>
         </is>
       </c>
       <c r="J67" s="4" t="inlineStr">
@@ -17576,32 +17576,32 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E68" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F68" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G68" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H68" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>5,53543160</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="inlineStr">
+        <is>
+          <t>0,045</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
+          <t>0,60</t>
+        </is>
+      </c>
+      <c r="G68" s="3" t="inlineStr">
+        <is>
+          <t>7,87</t>
+        </is>
+      </c>
+      <c r="H68" s="3" t="inlineStr">
+        <is>
+          <t>12,89</t>
         </is>
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>32,773</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr">
@@ -17836,32 +17836,32 @@
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E69" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F69" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G69" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H69" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1.259,14977500</t>
+        </is>
+      </c>
+      <c r="E69" s="7" t="inlineStr">
+        <is>
+          <t>-0,003</t>
+        </is>
+      </c>
+      <c r="F69" s="7" t="inlineStr">
+        <is>
+          <t>-2,28</t>
+        </is>
+      </c>
+      <c r="G69" s="5" t="inlineStr">
+        <is>
+          <t>0,34</t>
+        </is>
+      </c>
+      <c r="H69" s="5" t="inlineStr">
+        <is>
+          <t>3,72</t>
         </is>
       </c>
       <c r="I69" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>37,836</t>
         </is>
       </c>
       <c r="J69" s="4" t="inlineStr">
@@ -18131,7 +18131,7 @@
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>542,857</t>
+          <t>542,340</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
@@ -18366,32 +18366,32 @@
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E71" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F71" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G71" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H71" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>2,92816400</t>
+        </is>
+      </c>
+      <c r="E71" s="7" t="inlineStr">
+        <is>
+          <t>-0,004</t>
+        </is>
+      </c>
+      <c r="F71" s="5" t="inlineStr">
+        <is>
+          <t>0,86</t>
+        </is>
+      </c>
+      <c r="G71" s="5" t="inlineStr">
+        <is>
+          <t>4,83</t>
+        </is>
+      </c>
+      <c r="H71" s="5" t="inlineStr">
+        <is>
+          <t>9,66</t>
         </is>
       </c>
       <c r="I71" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>69,267</t>
         </is>
       </c>
       <c r="J71" s="4" t="inlineStr">
@@ -18647,7 +18647,7 @@
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>30,278</t>
+          <t>30,271</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr">
@@ -18907,7 +18907,7 @@
       </c>
       <c r="I73" s="4" t="inlineStr">
         <is>
-          <t>2.462,112</t>
+          <t>2.461,910</t>
         </is>
       </c>
       <c r="J73" s="4" t="inlineStr">
@@ -19402,32 +19402,32 @@
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E75" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F75" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G75" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H75" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1.719,14265700</t>
+        </is>
+      </c>
+      <c r="E75" s="7" t="inlineStr">
+        <is>
+          <t>-0,002</t>
+        </is>
+      </c>
+      <c r="F75" s="5" t="inlineStr">
+        <is>
+          <t>0,62</t>
+        </is>
+      </c>
+      <c r="G75" s="5" t="inlineStr">
+        <is>
+          <t>8,70</t>
+        </is>
+      </c>
+      <c r="H75" s="5" t="inlineStr">
+        <is>
+          <t>13,97</t>
         </is>
       </c>
       <c r="I75" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14,625</t>
         </is>
       </c>
       <c r="J75" s="4" t="inlineStr">
@@ -19683,7 +19683,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>904,823</t>
+          <t>904,365</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr">
@@ -19918,32 +19918,32 @@
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E77" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F77" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G77" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>0,59002468</t>
+        </is>
+      </c>
+      <c r="E77" s="7" t="inlineStr">
+        <is>
+          <t>-0,005</t>
+        </is>
+      </c>
+      <c r="F77" s="5" t="inlineStr">
+        <is>
+          <t>1,27</t>
+        </is>
+      </c>
+      <c r="G77" s="7" t="inlineStr">
+        <is>
+          <t>-18,28</t>
         </is>
       </c>
       <c r="H77" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="I77" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4,711</t>
         </is>
       </c>
       <c r="J77" s="4" t="inlineStr">
@@ -20210,7 +20210,7 @@
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>713,435</t>
+          <t>713,433</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr">
@@ -20441,32 +20441,32 @@
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E79" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F79" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G79" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H79" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,41945100</t>
+        </is>
+      </c>
+      <c r="E79" s="7" t="inlineStr">
+        <is>
+          <t>-0,054</t>
+        </is>
+      </c>
+      <c r="F79" s="7" t="inlineStr">
+        <is>
+          <t>-0,63</t>
+        </is>
+      </c>
+      <c r="G79" s="5" t="inlineStr">
+        <is>
+          <t>4,66</t>
+        </is>
+      </c>
+      <c r="H79" s="5" t="inlineStr">
+        <is>
+          <t>7,53</t>
         </is>
       </c>
       <c r="I79" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>72,739</t>
         </is>
       </c>
       <c r="J79" s="4" t="inlineStr">
@@ -20709,32 +20709,32 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E80" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F80" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G80" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H80" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,52757100</t>
+        </is>
+      </c>
+      <c r="E80" s="3" t="inlineStr">
+        <is>
+          <t>0,058</t>
+        </is>
+      </c>
+      <c r="F80" s="3" t="inlineStr">
+        <is>
+          <t>0,23</t>
+        </is>
+      </c>
+      <c r="G80" s="3" t="inlineStr">
+        <is>
+          <t>5,63</t>
+        </is>
+      </c>
+      <c r="H80" s="3" t="inlineStr">
+        <is>
+          <t>11,28</t>
         </is>
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>119,968</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr">
@@ -20769,7 +20769,7 @@
       </c>
       <c r="P80" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-capital-protegido-ciclico-ii-multimercado-lp/Paginas/default.aspx</t>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/caixa-fic-fim-cap-protegido-ciclico-ii</t>
         </is>
       </c>
       <c r="Q80" s="2" t="inlineStr">
@@ -20977,32 +20977,32 @@
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E81" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F81" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G81" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H81" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>3,39528400</t>
+        </is>
+      </c>
+      <c r="E81" s="5" t="inlineStr">
+        <is>
+          <t>0,431</t>
+        </is>
+      </c>
+      <c r="F81" s="5" t="inlineStr">
+        <is>
+          <t>0,19</t>
+        </is>
+      </c>
+      <c r="G81" s="5" t="inlineStr">
+        <is>
+          <t>6,56</t>
+        </is>
+      </c>
+      <c r="H81" s="5" t="inlineStr">
+        <is>
+          <t>9,47</t>
         </is>
       </c>
       <c r="I81" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>161,712</t>
         </is>
       </c>
       <c r="J81" s="4" t="inlineStr">
@@ -21243,32 +21243,32 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E82" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F82" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G82" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H82" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,60290700</t>
+        </is>
+      </c>
+      <c r="E82" s="3" t="inlineStr">
+        <is>
+          <t>0,176</t>
+        </is>
+      </c>
+      <c r="F82" s="3" t="inlineStr">
+        <is>
+          <t>0,76</t>
+        </is>
+      </c>
+      <c r="G82" s="3" t="inlineStr">
+        <is>
+          <t>7,35</t>
+        </is>
+      </c>
+      <c r="H82" s="3" t="inlineStr">
+        <is>
+          <t>21,76</t>
         </is>
       </c>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>15,100</t>
         </is>
       </c>
       <c r="J82" s="2" t="inlineStr">
@@ -21509,32 +21509,32 @@
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E83" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F83" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G83" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H83" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>6,88795700</t>
+        </is>
+      </c>
+      <c r="E83" s="7" t="inlineStr">
+        <is>
+          <t>-0,004</t>
+        </is>
+      </c>
+      <c r="F83" s="5" t="inlineStr">
+        <is>
+          <t>0,13</t>
+        </is>
+      </c>
+      <c r="G83" s="5" t="inlineStr">
+        <is>
+          <t>7,10</t>
+        </is>
+      </c>
+      <c r="H83" s="5" t="inlineStr">
+        <is>
+          <t>12,99</t>
         </is>
       </c>
       <c r="I83" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>125,129</t>
         </is>
       </c>
       <c r="J83" s="4" t="inlineStr">
@@ -21765,32 +21765,32 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E84" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F84" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G84" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H84" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,83612400</t>
+        </is>
+      </c>
+      <c r="E84" s="6" t="inlineStr">
+        <is>
+          <t>-0,002</t>
+        </is>
+      </c>
+      <c r="F84" s="6" t="inlineStr">
+        <is>
+          <t>-0,24</t>
+        </is>
+      </c>
+      <c r="G84" s="3" t="inlineStr">
+        <is>
+          <t>3,93</t>
+        </is>
+      </c>
+      <c r="H84" s="3" t="inlineStr">
+        <is>
+          <t>9,34</t>
         </is>
       </c>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>169,741</t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr">
@@ -22021,32 +22021,32 @@
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E85" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F85" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G85" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H85" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,45500500</t>
+        </is>
+      </c>
+      <c r="E85" s="7" t="inlineStr">
+        <is>
+          <t>-0,003</t>
+        </is>
+      </c>
+      <c r="F85" s="5" t="inlineStr">
+        <is>
+          <t>0,26</t>
+        </is>
+      </c>
+      <c r="G85" s="5" t="inlineStr">
+        <is>
+          <t>5,61</t>
+        </is>
+      </c>
+      <c r="H85" s="5" t="inlineStr">
+        <is>
+          <t>11,75</t>
         </is>
       </c>
       <c r="I85" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>281,888</t>
         </is>
       </c>
       <c r="J85" s="4" t="inlineStr">
@@ -22282,32 +22282,32 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E86" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F86" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G86" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H86" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,43581600</t>
+        </is>
+      </c>
+      <c r="E86" s="6" t="inlineStr">
+        <is>
+          <t>-0,002</t>
+        </is>
+      </c>
+      <c r="F86" s="3" t="inlineStr">
+        <is>
+          <t>1,24</t>
+        </is>
+      </c>
+      <c r="G86" s="3" t="inlineStr">
+        <is>
+          <t>11,86</t>
+        </is>
+      </c>
+      <c r="H86" s="3" t="inlineStr">
+        <is>
+          <t>11,21</t>
         </is>
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12,775</t>
         </is>
       </c>
       <c r="J86" s="2" t="inlineStr">
@@ -22567,7 +22567,7 @@
       </c>
       <c r="I87" s="4" t="inlineStr">
         <is>
-          <t>96,820</t>
+          <t>96,814</t>
         </is>
       </c>
       <c r="J87" s="4" t="inlineStr">
@@ -22947,7 +22947,7 @@
       </c>
       <c r="I89" s="4" t="inlineStr">
         <is>
-          <t>4,044</t>
+          <t>4,043</t>
         </is>
       </c>
       <c r="J89" s="4" t="inlineStr">
@@ -23203,7 +23203,7 @@
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>13,541</t>
+          <t>13,533</t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr">
@@ -23712,7 +23712,7 @@
       </c>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>274,260</t>
+          <t>274,163</t>
         </is>
       </c>
       <c r="J92" s="2" t="inlineStr">
@@ -23972,7 +23972,7 @@
       </c>
       <c r="I93" s="4" t="inlineStr">
         <is>
-          <t>418,541</t>
+          <t>418,458</t>
         </is>
       </c>
       <c r="J93" s="4" t="inlineStr">
@@ -24232,7 +24232,7 @@
       </c>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t>53,832</t>
+          <t>53,820</t>
         </is>
       </c>
       <c r="J94" s="2" t="inlineStr">
@@ -24492,7 +24492,7 @@
       </c>
       <c r="I95" s="4" t="inlineStr">
         <is>
-          <t>2,094</t>
+          <t>2,083</t>
         </is>
       </c>
       <c r="J95" s="4" t="inlineStr">
@@ -24752,7 +24752,7 @@
       </c>
       <c r="I96" s="2" t="inlineStr">
         <is>
-          <t>85,108</t>
+          <t>85,100</t>
         </is>
       </c>
       <c r="J96" s="2" t="inlineStr">
@@ -25012,7 +25012,7 @@
       </c>
       <c r="I97" s="4" t="inlineStr">
         <is>
-          <t>91,934</t>
+          <t>91,885</t>
         </is>
       </c>
       <c r="J97" s="4" t="inlineStr">
@@ -25247,32 +25247,32 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E98" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F98" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G98" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H98" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,32421500</t>
+        </is>
+      </c>
+      <c r="E98" s="3" t="inlineStr">
+        <is>
+          <t>0,178</t>
+        </is>
+      </c>
+      <c r="F98" s="3" t="inlineStr">
+        <is>
+          <t>4,54</t>
+        </is>
+      </c>
+      <c r="G98" s="3" t="inlineStr">
+        <is>
+          <t>2,88</t>
+        </is>
+      </c>
+      <c r="H98" s="3" t="inlineStr">
+        <is>
+          <t>10,50</t>
         </is>
       </c>
       <c r="I98" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>295,472</t>
         </is>
       </c>
       <c r="J98" s="2" t="inlineStr">
@@ -25532,7 +25532,7 @@
       </c>
       <c r="I99" s="4" t="inlineStr">
         <is>
-          <t>107,934</t>
+          <t>107,882</t>
         </is>
       </c>
       <c r="J99" s="4" t="inlineStr">
@@ -25792,7 +25792,7 @@
       </c>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t>121,994</t>
+          <t>121,933</t>
         </is>
       </c>
       <c r="J100" s="2" t="inlineStr">
@@ -26052,7 +26052,7 @@
       </c>
       <c r="I101" s="4" t="inlineStr">
         <is>
-          <t>49,966</t>
+          <t>49,925</t>
         </is>
       </c>
       <c r="J101" s="4" t="inlineStr">
@@ -26316,7 +26316,7 @@
       </c>
       <c r="I102" s="2" t="inlineStr">
         <is>
-          <t>136,037</t>
+          <t>135,997</t>
         </is>
       </c>
       <c r="J102" s="2" t="inlineStr">
@@ -26576,7 +26576,7 @@
       </c>
       <c r="I103" s="4" t="inlineStr">
         <is>
-          <t>45,830</t>
+          <t>45,383</t>
         </is>
       </c>
       <c r="J103" s="4" t="inlineStr">
@@ -26836,7 +26836,7 @@
       </c>
       <c r="I104" s="2" t="inlineStr">
         <is>
-          <t>640,117</t>
+          <t>635,097</t>
         </is>
       </c>
       <c r="J104" s="2" t="inlineStr">
@@ -27096,7 +27096,7 @@
       </c>
       <c r="I105" s="4" t="inlineStr">
         <is>
-          <t>508,905</t>
+          <t>508,593</t>
         </is>
       </c>
       <c r="J105" s="4" t="inlineStr">
@@ -27360,7 +27360,7 @@
       </c>
       <c r="I106" s="2" t="inlineStr">
         <is>
-          <t>24,232</t>
+          <t>24,171</t>
         </is>
       </c>
       <c r="J106" s="2" t="inlineStr">
@@ -27620,7 +27620,7 @@
       </c>
       <c r="I107" s="4" t="inlineStr">
         <is>
-          <t>32,278</t>
+          <t>32,275</t>
         </is>
       </c>
       <c r="J107" s="4" t="inlineStr">
@@ -28132,7 +28132,7 @@
       </c>
       <c r="I109" s="4" t="inlineStr">
         <is>
-          <t>45,152</t>
+          <t>45,145</t>
         </is>
       </c>
       <c r="J109" s="4" t="inlineStr">
@@ -28384,7 +28384,7 @@
       </c>
       <c r="I110" s="2" t="inlineStr">
         <is>
-          <t>35,374</t>
+          <t>35,363</t>
         </is>
       </c>
       <c r="J110" s="2" t="inlineStr">
@@ -28644,7 +28644,7 @@
       </c>
       <c r="I111" s="4" t="inlineStr">
         <is>
-          <t>922,246</t>
+          <t>918,374</t>
         </is>
       </c>
       <c r="J111" s="4" t="inlineStr">
@@ -28904,7 +28904,7 @@
       </c>
       <c r="I112" s="2" t="inlineStr">
         <is>
-          <t>20,392</t>
+          <t>20,145</t>
         </is>
       </c>
       <c r="J112" s="2" t="inlineStr">
@@ -29164,7 +29164,7 @@
       </c>
       <c r="I113" s="4" t="inlineStr">
         <is>
-          <t>279,350</t>
+          <t>279,296</t>
         </is>
       </c>
       <c r="J113" s="4" t="inlineStr">
@@ -29428,7 +29428,7 @@
       </c>
       <c r="I114" s="2" t="inlineStr">
         <is>
-          <t>2,840</t>
+          <t>2,820</t>
         </is>
       </c>
       <c r="J114" s="2" t="inlineStr">
@@ -29684,7 +29684,7 @@
       </c>
       <c r="I115" s="4" t="inlineStr">
         <is>
-          <t>342,598</t>
+          <t>342,536</t>
         </is>
       </c>
       <c r="J115" s="4" t="inlineStr">
@@ -29919,32 +29919,32 @@
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E116" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F116" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G116" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H116" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1.050,92616700</t>
+        </is>
+      </c>
+      <c r="E116" s="6" t="inlineStr">
+        <is>
+          <t>-0,003</t>
+        </is>
+      </c>
+      <c r="F116" s="3" t="inlineStr">
+        <is>
+          <t>4,25</t>
+        </is>
+      </c>
+      <c r="G116" s="3" t="inlineStr">
+        <is>
+          <t>7,19</t>
+        </is>
+      </c>
+      <c r="H116" s="3" t="inlineStr">
+        <is>
+          <t>19,68</t>
         </is>
       </c>
       <c r="I116" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>8,434</t>
         </is>
       </c>
       <c r="J116" s="2" t="inlineStr">
@@ -30179,32 +30179,32 @@
       </c>
       <c r="D117" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E117" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F117" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G117" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H117" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1.548,08734700</t>
+        </is>
+      </c>
+      <c r="E117" s="7" t="inlineStr">
+        <is>
+          <t>-0,002</t>
+        </is>
+      </c>
+      <c r="F117" s="5" t="inlineStr">
+        <is>
+          <t>4,80</t>
+        </is>
+      </c>
+      <c r="G117" s="5" t="inlineStr">
+        <is>
+          <t>3,49</t>
+        </is>
+      </c>
+      <c r="H117" s="5" t="inlineStr">
+        <is>
+          <t>12,03</t>
         </is>
       </c>
       <c r="I117" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>22,229</t>
         </is>
       </c>
       <c r="J117" s="4" t="inlineStr">
@@ -30435,7 +30435,7 @@
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>180,43849600</t>
+          <t>180,43849645</t>
         </is>
       </c>
       <c r="E118" s="6" t="inlineStr">
@@ -30977,7 +30977,7 @@
       </c>
       <c r="I120" s="2" t="inlineStr">
         <is>
-          <t>1.672,911</t>
+          <t>1.672,092</t>
         </is>
       </c>
       <c r="J120" s="2" t="inlineStr">
@@ -31230,7 +31230,7 @@
       </c>
       <c r="I121" s="4" t="inlineStr">
         <is>
-          <t>754,734</t>
+          <t>752,862</t>
         </is>
       </c>
       <c r="J121" s="4" t="inlineStr">
@@ -31474,7 +31474,7 @@
       </c>
       <c r="I122" s="2" t="inlineStr">
         <is>
-          <t>740,195</t>
+          <t>739,365</t>
         </is>
       </c>
       <c r="J122" s="2" t="inlineStr">
@@ -31718,7 +31718,7 @@
       </c>
       <c r="I123" s="4" t="inlineStr">
         <is>
-          <t>112,652</t>
+          <t>112,415</t>
         </is>
       </c>
       <c r="J123" s="4" t="inlineStr">
@@ -32220,7 +32220,7 @@
       </c>
       <c r="I125" s="4" t="inlineStr">
         <is>
-          <t>653,384</t>
+          <t>653,326</t>
         </is>
       </c>
       <c r="J125" s="4" t="inlineStr">
@@ -32469,7 +32469,7 @@
       </c>
       <c r="I126" s="2" t="inlineStr">
         <is>
-          <t>447,242</t>
+          <t>447,160</t>
         </is>
       </c>
       <c r="J126" s="2" t="inlineStr">
@@ -32713,7 +32713,7 @@
       </c>
       <c r="I127" s="4" t="inlineStr">
         <is>
-          <t>744,326</t>
+          <t>743,435</t>
         </is>
       </c>
       <c r="J127" s="4" t="inlineStr">
@@ -33222,7 +33222,7 @@
       </c>
       <c r="I129" s="4" t="inlineStr">
         <is>
-          <t>225,392</t>
+          <t>216,812</t>
         </is>
       </c>
       <c r="J129" s="4" t="inlineStr">
@@ -33748,7 +33748,7 @@
       </c>
       <c r="I131" s="4" t="inlineStr">
         <is>
-          <t>807,771</t>
+          <t>807,725</t>
         </is>
       </c>
       <c r="J131" s="4" t="inlineStr">
@@ -34267,7 +34267,7 @@
       </c>
       <c r="I133" s="4" t="inlineStr">
         <is>
-          <t>96,056</t>
+          <t>95,879</t>
         </is>
       </c>
       <c r="J133" s="4" t="inlineStr">
@@ -34531,7 +34531,7 @@
       </c>
       <c r="I134" s="2" t="inlineStr">
         <is>
-          <t>8.231,271</t>
+          <t>8.002,239</t>
         </is>
       </c>
       <c r="J134" s="2" t="inlineStr">
@@ -34757,22 +34757,22 @@
       </c>
       <c r="B135" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIF SAFIRA CORPORATIVO RF LP - RESP LTDA</t>
+          <t>CAIXA FIF DIAMANTE CORP RF CRED PRIV LP - RESP LTDA</t>
         </is>
       </c>
       <c r="C135" s="4" t="inlineStr">
         <is>
-          <t>11/05/2009</t>
+          <t>06/11/2019</t>
         </is>
       </c>
       <c r="D135" s="4" t="inlineStr">
         <is>
-          <t>5,04794900</t>
+          <t>1.954,97459700</t>
         </is>
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t>0,049</t>
+          <t>0,051</t>
         </is>
       </c>
       <c r="F135" s="5" t="inlineStr">
@@ -34782,17 +34782,17 @@
       </c>
       <c r="G135" s="5" t="inlineStr">
         <is>
-          <t>9,48</t>
+          <t>9,82</t>
         </is>
       </c>
       <c r="H135" s="5" t="inlineStr">
         <is>
-          <t>14,50</t>
+          <t>15,00</t>
         </is>
       </c>
       <c r="I135" s="4" t="inlineStr">
         <is>
-          <t>3.156,286</t>
+          <t>16.935,244</t>
         </is>
       </c>
       <c r="J135" s="4" t="inlineStr">
@@ -34822,22 +34822,22 @@
       </c>
       <c r="O135" s="4" t="inlineStr">
         <is>
-          <t>PJ</t>
+          <t>PJ | TODOS</t>
         </is>
       </c>
       <c r="P135" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/referenciados/fi-safira-corporativo-rf-lp</t>
+          <t>https://www.caixa.gov.br/fundos-investimento/empresa/renda-fixa/credito-privado/caixa-fi-diamante-corporativo-rf-cred-priv-lp</t>
         </is>
       </c>
       <c r="Q135" s="4" t="inlineStr">
         <is>
-          <t>10.384.413/0001-70</t>
+          <t>29.157.520/0001-94</t>
         </is>
       </c>
       <c r="R135" s="4" t="inlineStr">
         <is>
-          <t>5148</t>
+          <t>6445</t>
         </is>
       </c>
       <c r="S135" s="4" t="inlineStr">
@@ -34847,7 +34847,7 @@
       </c>
       <c r="T135" s="4" t="inlineStr">
         <is>
-          <t>0.1</t>
+          <t>0.12</t>
         </is>
       </c>
       <c r="U135" s="4" t="inlineStr">
@@ -34892,7 +34892,7 @@
       </c>
       <c r="AC135" s="4" t="inlineStr">
         <is>
-          <t>RF 100% TPF - Longo Prazo</t>
+          <t>RF Crédito Privado permite Risco Mercado</t>
         </is>
       </c>
       <c r="AD135" s="4" t="inlineStr">
@@ -34907,7 +34907,7 @@
       </c>
       <c r="AF135" s="4" t="inlineStr">
         <is>
-          <t>GERAL</t>
+          <t>PROFISSIONAL</t>
         </is>
       </c>
       <c r="AG135" s="4" t="inlineStr">
@@ -34922,7 +34922,7 @@
       </c>
       <c r="AI135" s="4" t="inlineStr">
         <is>
-          <t>Sim · Automatico · 90%</t>
+          <t>Sim · Automatico · 95%</t>
         </is>
       </c>
       <c r="AJ135" s="4" t="inlineStr">
@@ -34932,17 +34932,17 @@
       </c>
       <c r="AK135" s="4" t="inlineStr">
         <is>
-          <t>90.0</t>
+          <t>95.0</t>
         </is>
       </c>
       <c r="AL135" s="4" t="inlineStr">
         <is>
-          <t>["Institucional", "PJ Atacado", "PJ Varejo"]</t>
+          <t>["Institucional", "PJ Atacado"]</t>
         </is>
       </c>
       <c r="AM135" s="4" t="inlineStr">
         <is>
-          <t>["Institucional", "PJ Atacado", "PJ Varejo"]</t>
+          <t>["Institucional", "PJ Atacado"]</t>
         </is>
       </c>
       <c r="AN135" s="4" t="inlineStr">
@@ -34963,49 +34963,49 @@
       </c>
       <c r="AR135" s="4" t="inlineStr">
         <is>
-          <t>CAIXA SAFIRA CORPORATIVO FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
+          <t>CAIXA DIAMANTE CORPORATIVO FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA CRÉDITO PRIVADO LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
         </is>
       </c>
       <c r="AS135" s="4" t="inlineStr"/>
       <c r="AT135" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5148.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_6445.pdf</t>
         </is>
       </c>
       <c r="AU135" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5148.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_6445.pdf</t>
         </is>
       </c>
       <c r="AV135" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5148.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_6445.pdf</t>
         </is>
       </c>
       <c r="AW135" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5148.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_6445.pdf</t>
         </is>
       </c>
       <c r="AX135" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5148.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6445.pdf</t>
         </is>
       </c>
       <c r="AY135" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5148.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6445.pdf</t>
         </is>
       </c>
       <c r="AZ135" s="4" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5148.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_6445.pdf</t>
         </is>
       </c>
       <c r="BA135" s="4" t="inlineStr"/>
       <c r="BB135" s="4" t="inlineStr">
         <is>
-          <t>https://web.microsoftstream.com/video/edcf6e85-7c1c-4dd4-9cc1-599dd69841dc?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
+          <t>https://web.microsoftstream.com/video/513ae285-b3cb-42e6-a51a-984face9af08?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
     </row>
@@ -35017,22 +35017,22 @@
       </c>
       <c r="B136" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIF DIAMANTE CORP RF CRED PRIV LP - RESP LTDA</t>
+          <t>CAIXA FIF SAFIRA CORPORATIVO RF LP - RESP LTDA</t>
         </is>
       </c>
       <c r="C136" s="2" t="inlineStr">
         <is>
-          <t>06/11/2019</t>
+          <t>11/05/2009</t>
         </is>
       </c>
       <c r="D136" s="2" t="inlineStr">
         <is>
-          <t>1.954,97459700</t>
+          <t>5,04794900</t>
         </is>
       </c>
       <c r="E136" s="3" t="inlineStr">
         <is>
-          <t>0,051</t>
+          <t>0,049</t>
         </is>
       </c>
       <c r="F136" s="3" t="inlineStr">
@@ -35042,17 +35042,17 @@
       </c>
       <c r="G136" s="3" t="inlineStr">
         <is>
-          <t>9,82</t>
+          <t>9,48</t>
         </is>
       </c>
       <c r="H136" s="3" t="inlineStr">
         <is>
-          <t>15,00</t>
+          <t>14,50</t>
         </is>
       </c>
       <c r="I136" s="2" t="inlineStr">
         <is>
-          <t>16.935,718</t>
+          <t>3.156,279</t>
         </is>
       </c>
       <c r="J136" s="2" t="inlineStr">
@@ -35082,22 +35082,22 @@
       </c>
       <c r="O136" s="2" t="inlineStr">
         <is>
-          <t>PJ | TODOS</t>
+          <t>PJ</t>
         </is>
       </c>
       <c r="P136" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/fundos-investimento/empresa/renda-fixa/credito-privado/caixa-fi-diamante-corporativo-rf-cred-priv-lp</t>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/referenciados/fi-safira-corporativo-rf-lp</t>
         </is>
       </c>
       <c r="Q136" s="2" t="inlineStr">
         <is>
-          <t>29.157.520/0001-94</t>
+          <t>10.384.413/0001-70</t>
         </is>
       </c>
       <c r="R136" s="2" t="inlineStr">
         <is>
-          <t>6445</t>
+          <t>5148</t>
         </is>
       </c>
       <c r="S136" s="2" t="inlineStr">
@@ -35107,7 +35107,7 @@
       </c>
       <c r="T136" s="2" t="inlineStr">
         <is>
-          <t>0.12</t>
+          <t>0.1</t>
         </is>
       </c>
       <c r="U136" s="2" t="inlineStr">
@@ -35152,7 +35152,7 @@
       </c>
       <c r="AC136" s="2" t="inlineStr">
         <is>
-          <t>RF Crédito Privado permite Risco Mercado</t>
+          <t>RF 100% TPF - Longo Prazo</t>
         </is>
       </c>
       <c r="AD136" s="2" t="inlineStr">
@@ -35167,7 +35167,7 @@
       </c>
       <c r="AF136" s="2" t="inlineStr">
         <is>
-          <t>PROFISSIONAL</t>
+          <t>GERAL</t>
         </is>
       </c>
       <c r="AG136" s="2" t="inlineStr">
@@ -35182,7 +35182,7 @@
       </c>
       <c r="AI136" s="2" t="inlineStr">
         <is>
-          <t>Sim · Automatico · 95%</t>
+          <t>Sim · Automatico · 90%</t>
         </is>
       </c>
       <c r="AJ136" s="2" t="inlineStr">
@@ -35192,17 +35192,17 @@
       </c>
       <c r="AK136" s="2" t="inlineStr">
         <is>
-          <t>95.0</t>
+          <t>90.0</t>
         </is>
       </c>
       <c r="AL136" s="2" t="inlineStr">
         <is>
-          <t>["Institucional", "PJ Atacado"]</t>
+          <t>["Institucional", "PJ Atacado", "PJ Varejo"]</t>
         </is>
       </c>
       <c r="AM136" s="2" t="inlineStr">
         <is>
-          <t>["Institucional", "PJ Atacado"]</t>
+          <t>["Institucional", "PJ Atacado", "PJ Varejo"]</t>
         </is>
       </c>
       <c r="AN136" s="2" t="inlineStr">
@@ -35223,49 +35223,49 @@
       </c>
       <c r="AR136" s="2" t="inlineStr">
         <is>
-          <t>CAIXA DIAMANTE CORPORATIVO FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA CRÉDITO PRIVADO LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
+          <t>CAIXA SAFIRA CORPORATIVO FUNDO DE INVESTIMENTO FINANCEIRO RENDA FIXA LONGO PRAZO - RESPONSABILIDADE LIMITADA</t>
         </is>
       </c>
       <c r="AS136" s="2" t="inlineStr"/>
       <c r="AT136" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_6445.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-laminas/LA_5148.pdf</t>
         </is>
       </c>
       <c r="AU136" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_6445.pdf</t>
+          <t>https://www.caixa.gov.br/downloads/aplicacao-financeira-regulamentos/RG_5148.pdf</t>
         </is>
       </c>
       <c r="AV136" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_6445.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-inf-com/FIC_5148.pdf</t>
         </is>
       </c>
       <c r="AW136" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_6445.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-comunicado-aos-cotistas/COM_5148.pdf</t>
         </is>
       </c>
       <c r="AX136" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_6445.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-carta-mensal/CM_5148.pdf</t>
         </is>
       </c>
       <c r="AY136" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_6445.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-laminas-comerciais/LAC_5148.pdf</t>
         </is>
       </c>
       <c r="AZ136" s="2" t="inlineStr">
         <is>
-          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_6445.pdf</t>
+          <t>https://www.caixa.gov.br/Downloads/aplicacao-financeira-termos-adesao/TA_5148.pdf</t>
         </is>
       </c>
       <c r="BA136" s="2" t="inlineStr"/>
       <c r="BB136" s="2" t="inlineStr">
         <is>
-          <t>https://web.microsoftstream.com/video/513ae285-b3cb-42e6-a51a-984face9af08?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
+          <t>https://web.microsoftstream.com/video/edcf6e85-7c1c-4dd4-9cc1-599dd69841dc?channelId=772517ff-88ae-4298-88f2-3ed5a5893c3e</t>
         </is>
       </c>
     </row>
@@ -35287,7 +35287,7 @@
       </c>
       <c r="D137" s="4" t="inlineStr">
         <is>
-          <t>1,60316300</t>
+          <t>1,60316313</t>
         </is>
       </c>
       <c r="E137" s="5" t="inlineStr">
@@ -36557,7 +36557,7 @@
       </c>
       <c r="I142" s="2" t="inlineStr">
         <is>
-          <t>14.470,394</t>
+          <t>14.012,493</t>
         </is>
       </c>
       <c r="J142" s="2" t="inlineStr">
@@ -36818,7 +36818,7 @@
       </c>
       <c r="I143" s="4" t="inlineStr">
         <is>
-          <t>16.829,613</t>
+          <t>16.829,452</t>
         </is>
       </c>
       <c r="J143" s="4" t="inlineStr">
@@ -37078,7 +37078,7 @@
       </c>
       <c r="I144" s="2" t="inlineStr">
         <is>
-          <t>3.406,225</t>
+          <t>3.406,083</t>
         </is>
       </c>
       <c r="J144" s="2" t="inlineStr">
@@ -37594,7 +37594,7 @@
       </c>
       <c r="I146" s="2" t="inlineStr">
         <is>
-          <t>32.106,984</t>
+          <t>31.681,783</t>
         </is>
       </c>
       <c r="J146" s="2" t="inlineStr">
@@ -37853,7 +37853,7 @@
       </c>
       <c r="I147" s="4" t="inlineStr">
         <is>
-          <t>2.666,500</t>
+          <t>2.633,819</t>
         </is>
       </c>
       <c r="J147" s="4" t="inlineStr">
@@ -38112,7 +38112,7 @@
       </c>
       <c r="I148" s="2" t="inlineStr">
         <is>
-          <t>17.601,138</t>
+          <t>17.465,813</t>
         </is>
       </c>
       <c r="J148" s="2" t="inlineStr">
@@ -38899,7 +38899,7 @@
       </c>
       <c r="I151" s="4" t="inlineStr">
         <is>
-          <t>3.316,320</t>
+          <t>3.316,318</t>
         </is>
       </c>
       <c r="J151" s="4" t="inlineStr">
@@ -41638,7 +41638,7 @@
       </c>
       <c r="I162" s="2" t="inlineStr">
         <is>
-          <t>12.337,986</t>
+          <t>12.337,984</t>
         </is>
       </c>
       <c r="J162" s="2" t="inlineStr">
@@ -42419,7 +42419,7 @@
       </c>
       <c r="I165" s="4" t="inlineStr">
         <is>
-          <t>1.750,120</t>
+          <t>1.779,994</t>
         </is>
       </c>
       <c r="J165" s="4" t="inlineStr">
@@ -44838,7 +44838,7 @@
       </c>
       <c r="I175" s="4" t="inlineStr">
         <is>
-          <t>304,379</t>
+          <t>304,324</t>
         </is>
       </c>
       <c r="J175" s="4" t="inlineStr">
@@ -45333,7 +45333,7 @@
       </c>
       <c r="D177" s="4" t="inlineStr">
         <is>
-          <t>11,76179600</t>
+          <t>11,76179567</t>
         </is>
       </c>
       <c r="E177" s="5" t="inlineStr">
@@ -45874,7 +45874,7 @@
       </c>
       <c r="I179" s="4" t="inlineStr">
         <is>
-          <t>756,884</t>
+          <t>749,884</t>
         </is>
       </c>
       <c r="J179" s="4" t="inlineStr">
@@ -46109,7 +46109,7 @@
       </c>
       <c r="D180" s="2" t="inlineStr">
         <is>
-          <t>3,63136900</t>
+          <t>3,63136852</t>
         </is>
       </c>
       <c r="E180" s="2" t="inlineStr">
@@ -46361,7 +46361,7 @@
       </c>
       <c r="D181" s="4" t="inlineStr">
         <is>
-          <t>2,61382100</t>
+          <t>2,61382090</t>
         </is>
       </c>
       <c r="E181" s="5" t="inlineStr">
@@ -46638,7 +46638,7 @@
       </c>
       <c r="I182" s="2" t="inlineStr">
         <is>
-          <t>4.735,182</t>
+          <t>4.735,058</t>
         </is>
       </c>
       <c r="J182" s="2" t="inlineStr">

</xml_diff>